<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 14:07:32 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T18:01:50.175909+00:00</t>
+          <t>2026-03-21T18:07:31.359037+00:00</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.3347571528630056</v>
+        <v>0.3278416641427607</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.6652428471369943</v>
+        <v>0.6721583358572394</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2369,10 +2369,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1988005554484586</v>
+        <v>0.199311411131728</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8011994445515415</v>
+        <v>0.800688588868272</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.08848333333333333</v>
+        <v>0.08818333333333332</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>121</v>
@@ -2620,10 +2620,10 @@
         <v>329</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.22244</v>
+        <v>0.22259</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.4968866666666667</v>
+        <v>0.4965866666666667</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.07708333333333335</v>
+        <v>0.07743333333333335</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>113</v>
@@ -2654,10 +2654,10 @@
         <v>301</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1754</v>
+        <v>0.1759333333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3964700000000001</v>
+        <v>0.3973700000000001</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0.0007</v>
@@ -2679,7 +2679,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.05153333333333333</v>
+        <v>0.05078333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>122</v>
@@ -2688,10 +2688,10 @@
         <v>324</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1422333333333333</v>
+        <v>0.1398333333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4480450000000001</v>
+        <v>0.4440950000000001</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0.0008</v>
@@ -2713,7 +2713,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.1411833333333333</v>
+        <v>0.1412333333333333</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>136</v>
@@ -2722,10 +2722,10 @@
         <v>291</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.3221666666666667</v>
+        <v>0.3220166666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.6981333333333335</v>
+        <v>0.6980333333333335</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2747,7 +2747,7 @@
         <v>9</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.02631666666666667</v>
+        <v>0.02616666666666667</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>118</v>
@@ -2756,10 +2756,10 @@
         <v>348</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1191166666666667</v>
+        <v>0.1188333333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.4359966666666668</v>
+        <v>0.4356216666666668</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0.0005333333333333334</v>
@@ -2781,7 +2781,7 @@
         <v>9</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.03044999999999999</v>
+        <v>0.0305</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>118</v>
@@ -2790,10 +2790,10 @@
         <v>336</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1199333333333333</v>
+        <v>0.1202666666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4638983333333334</v>
+        <v>0.4653483333333334</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.00015</v>
@@ -2815,7 +2815,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06230000000000001</v>
+        <v>0.06250000000000001</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>122</v>
@@ -2824,10 +2824,10 @@
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1749416666666666</v>
+        <v>0.1757416666666666</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4878416666666668</v>
+        <v>0.4889916666666668</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2849,7 +2849,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03453333333333333</v>
+        <v>0.03483333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>121</v>
@@ -2858,10 +2858,10 @@
         <v>330</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1396166666666666</v>
+        <v>0.1402166666666667</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.5163783333333334</v>
+        <v>0.5176533333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2892,13 +2892,13 @@
         <v>327</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1143066666666667</v>
+        <v>0.1144066666666667</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4523716666666667</v>
+        <v>0.4516549999999999</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0004</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="11">
@@ -2917,7 +2917,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.02596666666666666</v>
+        <v>0.02606666666666666</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>113</v>
@@ -2929,7 +2929,7 @@
         <v>0.08521666666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3677266666666669</v>
+        <v>0.3670933333333335</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -2951,7 +2951,7 @@
         <v>8</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.03298333333333333</v>
+        <v>0.03268333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>95</v>
@@ -2960,13 +2960,13 @@
         <v>273</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09348333333333333</v>
+        <v>0.09298333333333333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.2483666666666667</v>
+        <v>0.2462166666666667</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.02611666666666666</v>
+        <v>0.02621666666666666</v>
       </c>
     </row>
     <row r="13">
@@ -2985,22 +2985,22 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05248333333333333</v>
+        <v>0.05288333333333332</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>105</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>263</v>
+        <v>279</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.143365</v>
+        <v>0.143615</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3399033333333334</v>
+        <v>0.3405866666666668</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.003683333333333333</v>
+        <v>0.003383333333333334</v>
       </c>
     </row>
     <row r="14">
@@ -3028,13 +3028,13 @@
         <v>324</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.02338333333333334</v>
+        <v>0.02328333333333333</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.2909916666666666</v>
+        <v>0.290625</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.0011</v>
+        <v>0.00115</v>
       </c>
     </row>
     <row r="15">
@@ -3053,7 +3053,7 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02825</v>
+        <v>0.02855</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>100</v>
@@ -3062,13 +3062,13 @@
         <v>294</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.07230833333333334</v>
+        <v>0.07260833333333333</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.22815</v>
+        <v>0.22885</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.01969166666666667</v>
+        <v>0.01959166666666667</v>
       </c>
     </row>
     <row r="16">
@@ -3087,7 +3087,7 @@
         <v>8</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.023</v>
+        <v>0.0228</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>75</v>
@@ -3096,13 +3096,13 @@
         <v>246</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0535</v>
+        <v>0.053</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.1410183333333333</v>
+        <v>0.1394683333333333</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.06159166666666668</v>
+        <v>0.06234166666666668</v>
       </c>
     </row>
     <row r="17">
@@ -3130,13 +3130,13 @@
         <v>282</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.02608333333333334</v>
+        <v>0.02618333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.08419166666666668</v>
+        <v>0.08439166666666666</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.02761666666666667</v>
+        <v>0.02716666666666668</v>
       </c>
     </row>
     <row r="18">
@@ -3167,7 +3167,7 @@
         <v>0.03328333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.251425</v>
+        <v>0.251275</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0.0003666666666666667</v>
@@ -3189,7 +3189,7 @@
         <v>10</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.07675</v>
+        <v>0.07665</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>110</v>
@@ -3198,10 +3198,10 @@
         <v>281</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.1684166666666667</v>
+        <v>0.16855</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.3819733333333334</v>
+        <v>0.3819066666666667</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.003583333333333333</v>
@@ -3238,7 +3238,7 @@
         <v>0.07664166666666668</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.02318333333333334</v>
+        <v>0.02328333333333334</v>
       </c>
     </row>
     <row r="21">
@@ -3266,10 +3266,10 @@
         <v>273</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.04223333333333333</v>
+        <v>0.04233333333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2179583333333333</v>
+        <v>0.2185916666666666</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0002</v>
@@ -3300,13 +3300,13 @@
         <v>245</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.03235</v>
+        <v>0.03245</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.1213583333333333</v>
+        <v>0.121925</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02323333333333334</v>
+        <v>0.02298333333333333</v>
       </c>
     </row>
     <row r="23">
@@ -3334,10 +3334,10 @@
         <v>281</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.03039166666666666</v>
+        <v>0.03049166666666666</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1976816666666667</v>
+        <v>0.1987816666666667</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.002416666666666666</v>
@@ -3359,7 +3359,7 @@
         <v>10</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.04231666666666666</v>
+        <v>0.04241666666666667</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>103</v>
@@ -3368,13 +3368,13 @@
         <v>257</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.1079166666666666</v>
+        <v>0.1082</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.3185416666666667</v>
+        <v>0.3196416666666667</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0038</v>
+        <v>0.0036</v>
       </c>
     </row>
     <row r="25">
@@ -3393,7 +3393,7 @@
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.03475</v>
+        <v>0.03465</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>92</v>
@@ -3405,10 +3405,10 @@
         <v>0.09583333333333334</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.2478183333333333</v>
+        <v>0.2477183333333333</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02328333333333333</v>
+        <v>0.02318333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3473,7 +3473,7 @@
         <v>0.07657333333333334</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2456166666666666</v>
+        <v>0.2455166666666666</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.002075</v>
@@ -3504,10 +3504,10 @@
         <v>247</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.03651666666666666</v>
+        <v>0.03671666666666666</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2165016666666666</v>
+        <v>0.2171349999999999</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0.0062</v>
@@ -3529,7 +3529,7 @@
         <v>8</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.007849999999999999</v>
+        <v>0.00795</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>88</v>
@@ -3538,13 +3538,13 @@
         <v>197</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03285</v>
+        <v>0.0332</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1191083333333333</v>
+        <v>0.1194083333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0208</v>
+        <v>0.02075</v>
       </c>
     </row>
     <row r="30">
@@ -3575,7 +3575,7 @@
         <v>0.01371666666666667</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1285283333333333</v>
+        <v>0.1284533333333333</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0.0065</v>
@@ -3597,7 +3597,7 @@
         <v>7</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.006333333333333333</v>
+        <v>0.006283333333333333</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>86</v>
@@ -3606,13 +3606,13 @@
         <v>252</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.03275</v>
+        <v>0.0317</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.116155</v>
+        <v>0.114505</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.03271666666666667</v>
+        <v>0.03331666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3631,7 +3631,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.003116666666666666</v>
+        <v>0.003216666666666666</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>92</v>
@@ -3643,10 +3643,10 @@
         <v>0.03304</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1858416666666667</v>
+        <v>0.1869083333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.005983333333333334</v>
+        <v>0.005883333333333333</v>
       </c>
     </row>
     <row r="33">
@@ -3655,7 +3655,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
@@ -3665,22 +3665,22 @@
         <v>9</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.004583333333333333</v>
+        <v>0.004533333333333333</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02596666666666666</v>
+        <v>0.03695</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1455566666666666</v>
+        <v>0.2055266666666666</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.0063</v>
       </c>
     </row>
     <row r="34">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
@@ -3699,22 +3699,22 @@
         <v>9</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.004533333333333333</v>
+        <v>0.004483333333333334</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.03705</v>
+        <v>0.02596666666666666</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.20556</v>
+        <v>0.14529</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.0063</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>0.001566666666666667</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.05034166666666667</v>
+        <v>0.05024166666666667</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0.08269166666666666</v>
@@ -3776,10 +3776,10 @@
         <v>215</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.02723333333333333</v>
+        <v>0.02768333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1770916666666667</v>
+        <v>0.1777916666666667</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.00655</v>
@@ -3810,13 +3810,13 @@
         <v>254</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.02093333333333333</v>
+        <v>0.02103333333333333</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.07323833333333332</v>
+        <v>0.07301333333333332</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.05990000000000001</v>
+        <v>0.05980000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -3850,7 +3850,7 @@
         <v>0.04946666666666667</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1204833333333333</v>
+        <v>0.1204333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3881,10 +3881,10 @@
         <v>0.003366666666666667</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04850833333333333</v>
+        <v>0.04890833333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.042125</v>
+        <v>0.042025</v>
       </c>
     </row>
     <row r="40">
@@ -3912,13 +3912,13 @@
         <v>223</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.02101666666666667</v>
+        <v>0.02111666666666667</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.09296666666666666</v>
+        <v>0.09306666666666664</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.02163333333333333</v>
+        <v>0.02168333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -3949,10 +3949,10 @@
         <v>0.00135</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.0246</v>
+        <v>0.02455</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.03273333333333333</v>
+        <v>0.03268333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -3986,7 +3986,7 @@
         <v>0.02351666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.314275</v>
+        <v>0.3143750000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T18:07:31.359037+00:00</t>
+          <t>2026-03-21T18:11:57.663782+00:00</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.3278416641427607</v>
+        <v>0.3235832418875902</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.6721583358572394</v>
+        <v>0.6764167581124098</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.08818333333333332</v>
+        <v>0.08813333333333333</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>121</v>
@@ -2623,7 +2623,7 @@
         <v>0.22259</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.4965866666666667</v>
+        <v>0.4964366666666667</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2654,10 +2654,10 @@
         <v>301</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1759333333333333</v>
+        <v>0.1763333333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3973700000000001</v>
+        <v>0.3979200000000001</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0.0007</v>
@@ -2679,7 +2679,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.05078333333333333</v>
+        <v>0.05038333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>122</v>
@@ -2688,10 +2688,10 @@
         <v>324</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1398333333333333</v>
+        <v>0.1387333333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4440950000000001</v>
+        <v>0.4421950000000001</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0.0008</v>
@@ -2713,7 +2713,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.1412333333333333</v>
+        <v>0.1411833333333333</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>136</v>
@@ -2725,7 +2725,7 @@
         <v>0.3220166666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.6980333333333335</v>
+        <v>0.6979333333333335</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2756,7 +2756,7 @@
         <v>348</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1188333333333333</v>
+        <v>0.1190333333333333</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0.4356216666666668</v>
@@ -2781,7 +2781,7 @@
         <v>9</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0305</v>
+        <v>0.0306</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>118</v>
@@ -2790,10 +2790,10 @@
         <v>336</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1202666666666666</v>
+        <v>0.1203166666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4653483333333334</v>
+        <v>0.4658983333333334</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.00015</v>
@@ -2815,7 +2815,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06250000000000001</v>
+        <v>0.06280000000000001</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>122</v>
@@ -2824,10 +2824,10 @@
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1757416666666666</v>
+        <v>0.1761916666666666</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4889916666666668</v>
+        <v>0.4895916666666668</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2849,7 +2849,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03483333333333333</v>
+        <v>0.03493333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>121</v>
@@ -2858,10 +2858,10 @@
         <v>330</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1402166666666667</v>
+        <v>0.1406166666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.5176533333333334</v>
+        <v>0.5184533333333333</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2883,7 +2883,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.03268333333333334</v>
+        <v>0.03243333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>119</v>
@@ -2895,7 +2895,7 @@
         <v>0.1144066666666667</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4516549999999999</v>
+        <v>0.4516049999999999</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.0005</v>
@@ -2926,10 +2926,10 @@
         <v>300</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.08521666666666666</v>
+        <v>0.08506666666666667</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3670933333333335</v>
+        <v>0.3668933333333336</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -2951,7 +2951,7 @@
         <v>8</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.03268333333333333</v>
+        <v>0.03258333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>95</v>
@@ -2960,13 +2960,13 @@
         <v>273</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09298333333333333</v>
+        <v>0.09228333333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.2462166666666667</v>
+        <v>0.2447666666666667</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.02621666666666666</v>
+        <v>0.02631666666666666</v>
       </c>
     </row>
     <row r="13">
@@ -2985,7 +2985,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05288333333333332</v>
+        <v>0.05323333333333333</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>105</v>
@@ -2994,13 +2994,13 @@
         <v>279</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.143615</v>
+        <v>0.144115</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3405866666666668</v>
+        <v>0.3411366666666668</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.003383333333333334</v>
+        <v>0.003283333333333333</v>
       </c>
     </row>
     <row r="14">
@@ -3031,7 +3031,7 @@
         <v>0.02328333333333333</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.290625</v>
+        <v>0.290425</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0.00115</v>
@@ -3062,13 +3062,13 @@
         <v>294</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.07260833333333333</v>
+        <v>0.07270833333333333</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.22885</v>
+        <v>0.22915</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.01959166666666667</v>
+        <v>0.01944166666666667</v>
       </c>
     </row>
     <row r="16">
@@ -3087,7 +3087,7 @@
         <v>8</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0228</v>
+        <v>0.0225</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>75</v>
@@ -3096,13 +3096,13 @@
         <v>246</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.053</v>
+        <v>0.05213333333333332</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.1394683333333333</v>
+        <v>0.1384183333333333</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.06234166666666668</v>
+        <v>0.06254166666666668</v>
       </c>
     </row>
     <row r="17">
@@ -3121,7 +3121,7 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.01195</v>
+        <v>0.01205</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>80</v>
@@ -3130,13 +3130,13 @@
         <v>282</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.02618333333333334</v>
+        <v>0.02628333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.08439166666666666</v>
+        <v>0.08459166666666666</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.02716666666666668</v>
+        <v>0.02696666666666667</v>
       </c>
     </row>
     <row r="18">
@@ -3167,7 +3167,7 @@
         <v>0.03328333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.251275</v>
+        <v>0.251175</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0.0003666666666666667</v>
@@ -3198,10 +3198,10 @@
         <v>281</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.16855</v>
+        <v>0.16845</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.3819066666666667</v>
+        <v>0.3816566666666668</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.003583333333333333</v>
@@ -3232,13 +3232,13 @@
         <v>255</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02428333333333333</v>
+        <v>0.02438333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
         <v>0.07664166666666668</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.02328333333333334</v>
+        <v>0.02338333333333334</v>
       </c>
     </row>
     <row r="21">
@@ -3266,10 +3266,10 @@
         <v>273</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.04233333333333333</v>
+        <v>0.04253333333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2185916666666666</v>
+        <v>0.2189416666666666</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0002</v>
@@ -3303,10 +3303,10 @@
         <v>0.03245</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.121925</v>
+        <v>0.122225</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02298333333333333</v>
+        <v>0.02288333333333334</v>
       </c>
     </row>
     <row r="23">
@@ -3337,7 +3337,7 @@
         <v>0.03049166666666666</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1987816666666667</v>
+        <v>0.1991316666666667</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.002416666666666666</v>
@@ -3359,7 +3359,7 @@
         <v>10</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.04241666666666667</v>
+        <v>0.04256666666666666</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>103</v>
@@ -3368,10 +3368,10 @@
         <v>257</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.1082</v>
+        <v>0.1085833333333334</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.3196416666666667</v>
+        <v>0.3200416666666667</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.0036</v>
@@ -3408,7 +3408,7 @@
         <v>0.2477183333333333</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02318333333333333</v>
+        <v>0.02323333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3470,7 +3470,7 @@
         <v>249</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.07657333333333334</v>
+        <v>0.07647333333333334</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>0.2455166666666666</v>
@@ -3504,10 +3504,10 @@
         <v>247</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.03671666666666666</v>
+        <v>0.03681666666666666</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2171349999999999</v>
+        <v>0.2176349999999999</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0.0062</v>
@@ -3529,7 +3529,7 @@
         <v>8</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.00795</v>
+        <v>0.008</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>88</v>
@@ -3538,13 +3538,13 @@
         <v>197</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.0332</v>
+        <v>0.03333333333333334</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>0.1194083333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.02075</v>
+        <v>0.02065</v>
       </c>
     </row>
     <row r="30">
@@ -3597,7 +3597,7 @@
         <v>7</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.006283333333333333</v>
+        <v>0.006183333333333333</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>86</v>
@@ -3606,13 +3606,13 @@
         <v>252</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.0317</v>
+        <v>0.0315</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.114505</v>
+        <v>0.113305</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.03331666666666667</v>
+        <v>0.03341666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3631,7 +3631,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.003216666666666666</v>
+        <v>0.003316666666666667</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>92</v>
@@ -3640,13 +3640,13 @@
         <v>217</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03304</v>
+        <v>0.03314</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1869083333333333</v>
+        <v>0.1874583333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.005883333333333333</v>
+        <v>0.005783333333333334</v>
       </c>
     </row>
     <row r="33">
@@ -3677,10 +3677,10 @@
         <v>0.03695</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.2055266666666666</v>
+        <v>0.2055766666666666</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.0063</v>
+        <v>0.0064</v>
       </c>
     </row>
     <row r="34">
@@ -3711,7 +3711,7 @@
         <v>0.02596666666666666</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.14529</v>
+        <v>0.14524</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>0.0001</v>
@@ -3748,7 +3748,7 @@
         <v>0.05024166666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.08269166666666666</v>
+        <v>0.08279166666666667</v>
       </c>
     </row>
     <row r="36">
@@ -3779,7 +3779,7 @@
         <v>0.02768333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1777916666666667</v>
+        <v>0.1780916666666667</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.00655</v>
@@ -3813,10 +3813,10 @@
         <v>0.02103333333333333</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.07301333333333332</v>
+        <v>0.07306333333333333</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.05980000000000001</v>
+        <v>0.05990000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -3850,7 +3850,7 @@
         <v>0.04946666666666667</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1204333333333333</v>
+        <v>0.1203333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3881,10 +3881,10 @@
         <v>0.003366666666666667</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04890833333333334</v>
+        <v>0.04930833333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.042025</v>
+        <v>0.041925</v>
       </c>
     </row>
     <row r="40">
@@ -3915,7 +3915,7 @@
         <v>0.02111666666666667</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.09306666666666664</v>
+        <v>0.09286666666666665</v>
       </c>
       <c r="J40" s="5" t="n">
         <v>0.02168333333333333</v>
@@ -3949,7 +3949,7 @@
         <v>0.00135</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02455</v>
+        <v>0.02465</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.03268333333333333</v>
@@ -3986,7 +3986,7 @@
         <v>0.02351666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.3143750000000001</v>
+        <v>0.3144750000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 14:16:26 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T18:11:57.663782+00:00</t>
+          <t>2026-03-21T18:16:25.428800+00:00</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.3235832418875902</v>
+        <v>0.3224553470275923</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.6764167581124098</v>
+        <v>0.6775446529724077</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.08813333333333333</v>
+        <v>0.08818333333333332</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>121</v>
@@ -2620,10 +2620,10 @@
         <v>329</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.22259</v>
+        <v>0.22269</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.4964366666666667</v>
+        <v>0.4963866666666667</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2679,7 +2679,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.05038333333333333</v>
+        <v>0.05028333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>122</v>
@@ -2688,10 +2688,10 @@
         <v>324</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1387333333333333</v>
+        <v>0.1383333333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4421950000000001</v>
+        <v>0.4417450000000001</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0.0008</v>
@@ -2722,10 +2722,10 @@
         <v>291</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.3220166666666667</v>
+        <v>0.3222166666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.6979333333333335</v>
+        <v>0.6980333333333335</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         <v>0.1203166666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4658983333333334</v>
+        <v>0.4660983333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.00015</v>
@@ -2824,10 +2824,10 @@
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1761916666666666</v>
+        <v>0.1763916666666666</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4895916666666668</v>
+        <v>0.4896916666666668</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,7 +2861,7 @@
         <v>0.1406166666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.5184533333333333</v>
+        <v>0.5189533333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2929,7 +2929,7 @@
         <v>0.08506666666666667</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3668933333333336</v>
+        <v>0.3667933333333336</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -2951,7 +2951,7 @@
         <v>8</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.03258333333333333</v>
+        <v>0.03253333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>95</v>
@@ -2960,10 +2960,10 @@
         <v>273</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09228333333333334</v>
+        <v>0.09208333333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.2447666666666667</v>
+        <v>0.2445666666666667</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.02631666666666666</v>
@@ -2985,7 +2985,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05323333333333333</v>
+        <v>0.05333333333333332</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>105</v>
@@ -2994,10 +2994,10 @@
         <v>279</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.144115</v>
+        <v>0.144215</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3411366666666668</v>
+        <v>0.3412366666666667</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0.003283333333333333</v>
@@ -3096,10 +3096,10 @@
         <v>246</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.05213333333333332</v>
+        <v>0.05203333333333333</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.1384183333333333</v>
+        <v>0.1381183333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0.06254166666666668</v>
@@ -3136,7 +3136,7 @@
         <v>0.08459166666666666</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.02696666666666667</v>
+        <v>0.02686666666666667</v>
       </c>
     </row>
     <row r="18">
@@ -3167,7 +3167,7 @@
         <v>0.03328333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.251175</v>
+        <v>0.2510749999999999</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0.0003666666666666667</v>
@@ -3201,10 +3201,10 @@
         <v>0.16845</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.3816566666666668</v>
+        <v>0.3815566666666668</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.003583333333333333</v>
+        <v>0.003683333333333333</v>
       </c>
     </row>
     <row r="20">
@@ -3269,7 +3269,7 @@
         <v>0.04253333333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2189416666666666</v>
+        <v>0.2191416666666666</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0002</v>
@@ -3306,7 +3306,7 @@
         <v>0.122225</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02288333333333334</v>
+        <v>0.02278333333333334</v>
       </c>
     </row>
     <row r="23">
@@ -3337,7 +3337,7 @@
         <v>0.03049166666666666</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1991316666666667</v>
+        <v>0.1992316666666667</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.002416666666666666</v>
@@ -3371,7 +3371,7 @@
         <v>0.1085833333333334</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.3200416666666667</v>
+        <v>0.3201416666666667</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.0036</v>
@@ -3405,7 +3405,7 @@
         <v>0.09583333333333334</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.2477183333333333</v>
+        <v>0.2476683333333334</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>0.02323333333333333</v>
@@ -3476,7 +3476,7 @@
         <v>0.2455166666666666</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.002075</v>
+        <v>0.001975</v>
       </c>
     </row>
     <row r="28">
@@ -3544,7 +3544,7 @@
         <v>0.1194083333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.02065</v>
+        <v>0.02055</v>
       </c>
     </row>
     <row r="30">
@@ -3609,10 +3609,10 @@
         <v>0.0315</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.113305</v>
+        <v>0.113105</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.03341666666666667</v>
+        <v>0.03351666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3640,10 +3640,10 @@
         <v>217</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03314</v>
+        <v>0.03324</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1874583333333333</v>
+        <v>0.1876583333333333</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.005783333333333334</v>
@@ -3748,7 +3748,7 @@
         <v>0.05024166666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.08279166666666667</v>
+        <v>0.08280833333333333</v>
       </c>
     </row>
     <row r="36">
@@ -3884,7 +3884,7 @@
         <v>0.04930833333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.041925</v>
+        <v>0.04189166666666667</v>
       </c>
     </row>
     <row r="40">
@@ -3952,7 +3952,7 @@
         <v>0.02465</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.03268333333333333</v>
+        <v>0.03278333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -3983,10 +3983,10 @@
         <v>0.00505</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.02351666666666667</v>
+        <v>0.02346666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.3144750000000001</v>
+        <v>0.3145916666666668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 14:24:21 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1f501acd71d581d0</t>
+          <t>642a0a38c44454af</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>32f6c65cbdba97ab</t>
+          <t>1f501acd71d581d0</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T18:16:25.428800+00:00</t>
+          <t>2026-03-21T18:24:21.074213+00:00</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.3224553470275923</v>
+        <v>0.3193939181962715</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.6775446529724077</v>
+        <v>0.6806060818037285</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2130,10 +2130,14 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Michigan</t>
+        </is>
+      </c>
       <c r="F38" s="4" t="b">
         <v>0</v>
       </c>
@@ -2369,10 +2373,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.199311411131728</v>
+        <v>0.1989767127293968</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.800688588868272</v>
+        <v>0.8010232872706032</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2601,29 +2605,29 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Ellis Fleming</t>
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.08818333333333332</v>
+        <v>0.11875</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.22269</v>
+        <v>0.3115166666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.4963866666666667</v>
+        <v>0.6838116666666667</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2635,32 +2639,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Stephen Mason</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.07743333333333335</v>
+        <v>0.0581</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1763333333333333</v>
+        <v>0.15725</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3979200000000001</v>
+        <v>0.3903833333333333</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.0007</v>
+        <v>0.00555</v>
       </c>
     </row>
     <row r="4">
@@ -2669,32 +2673,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.05028333333333333</v>
+        <v>0.1293</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>324</v>
+        <v>293</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1383333333333333</v>
+        <v>0.3090166666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4417450000000001</v>
+        <v>0.6906600000000001</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.0008</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2703,32 +2707,32 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.1411833333333333</v>
+        <v>0.079</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.3222166666666667</v>
+        <v>0.2001166666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.6980333333333335</v>
+        <v>0.4748583333333333</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0</v>
+        <v>0.00045</v>
       </c>
     </row>
     <row r="6">
@@ -2737,32 +2741,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.02616666666666667</v>
+        <v>0.06313333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>348</v>
+        <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1190333333333333</v>
+        <v>0.1538083333333334</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.4356216666666668</v>
+        <v>0.37596</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.0005333333333333334</v>
+        <v>0.001033333333333333</v>
       </c>
     </row>
     <row r="7">
@@ -2771,32 +2775,32 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0306</v>
+        <v>0.04353333333333334</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>336</v>
+        <v>314</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1203166666666667</v>
+        <v>0.1256666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4660983333333333</v>
+        <v>0.4222466666666666</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.00015</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="8">
@@ -2805,32 +2809,32 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Ryan Evans</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06280000000000001</v>
+        <v>0.04465</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>280</v>
+        <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1763916666666666</v>
+        <v>0.1266166666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4896916666666668</v>
+        <v>0.3122416666666667</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0</v>
+        <v>0.00435</v>
       </c>
     </row>
     <row r="9">
@@ -2839,32 +2843,32 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ellis Fleming</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03493333333333333</v>
+        <v>0.02656666666666667</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>330</v>
+        <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1406166666666666</v>
+        <v>0.1081666666666667</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.5189533333333334</v>
+        <v>0.4536666666666667</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0</v>
+        <v>0.00045</v>
       </c>
     </row>
     <row r="10">
@@ -2873,32 +2877,32 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.03243333333333333</v>
+        <v>0.02053333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>119</v>
+        <v>117.5</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1144066666666667</v>
+        <v>0.09152500000000001</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4516049999999999</v>
+        <v>0.405675</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0005</v>
+        <v>0.0009</v>
       </c>
     </row>
     <row r="11">
@@ -2907,32 +2911,32 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.02606666666666666</v>
+        <v>0.0171</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>300</v>
+        <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.08506666666666667</v>
+        <v>0.08792499999999999</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3667933333333336</v>
+        <v>0.4345383333333333</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0</v>
+        <v>0.0004833333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -2941,32 +2945,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.03253333333333333</v>
+        <v>0.06003333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09208333333333334</v>
+        <v>0.1629916666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.2445666666666667</v>
+        <v>0.47011</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.02631666666666666</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="13">
@@ -2979,28 +2983,28 @@
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05333333333333332</v>
+        <v>0.05548333333333333</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.144215</v>
+        <v>0.1438333333333333</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3412366666666667</v>
+        <v>0.3431716666666667</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.003283333333333333</v>
+        <v>0.0019</v>
       </c>
     </row>
     <row r="14">
@@ -3009,32 +3013,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0</v>
+        <v>0.02068333333333333</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>112</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>324</v>
+        <v>307</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.02328333333333333</v>
+        <v>0.06990000000000002</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.290425</v>
+        <v>0.3282433333333333</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.00115</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3043,32 +3047,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Stephen Mason</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02855</v>
+        <v>0.02755</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>294</v>
+        <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.07270833333333333</v>
+        <v>0.08351666666666668</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.22915</v>
+        <v>0.234925</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.01944166666666667</v>
+        <v>0.02831666666666666</v>
       </c>
     </row>
     <row r="16">
@@ -3077,32 +3081,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0225</v>
+        <v>0</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>246</v>
+        <v>310</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.05203333333333333</v>
+        <v>0.0165</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.1381183333333333</v>
+        <v>0.2667766666666666</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.06254166666666668</v>
+        <v>0.00195</v>
       </c>
     </row>
     <row r="17">
@@ -3121,22 +3125,22 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.01205</v>
+        <v>0.009516666666666666</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>80</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>282</v>
+        <v>258</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.02628333333333334</v>
+        <v>0.0212</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.08459166666666666</v>
+        <v>0.07670833333333332</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.02686666666666667</v>
+        <v>0.03441666666666666</v>
       </c>
     </row>
     <row r="18">
@@ -3145,32 +3149,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
         <v>28</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.006</v>
+        <v>0.0071</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>109</v>
+        <v>70</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>274</v>
+        <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.03328333333333333</v>
+        <v>0.02678333333333334</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.2510749999999999</v>
+        <v>0.09032166666666668</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.0003666666666666667</v>
+        <v>0.07629999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -3179,32 +3183,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.07665</v>
+        <v>0.00475</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.16845</v>
+        <v>0.02795</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.3815566666666668</v>
+        <v>0.2234999999999999</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.003683333333333333</v>
+        <v>0.00045</v>
       </c>
     </row>
     <row r="20">
@@ -3213,32 +3217,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
         <v>27</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.005466666666666667</v>
+        <v>0.0631</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02438333333333333</v>
+        <v>0.145125</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.07664166666666668</v>
+        <v>0.3530550000000001</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.02338333333333334</v>
+        <v>0.003416666666666667</v>
       </c>
     </row>
     <row r="21">
@@ -3247,32 +3251,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
         <v>27</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.00325</v>
+        <v>0.03546666666666667</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>273</v>
+        <v>248</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.04253333333333333</v>
+        <v>0.1023166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2191416666666666</v>
+        <v>0.3129449999999999</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.003583333333333334</v>
       </c>
     </row>
     <row r="22">
@@ -3281,32 +3285,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.01313333333333333</v>
+        <v>0.03178333333333334</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>245</v>
+        <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.03245</v>
+        <v>0.09013333333333334</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.122225</v>
+        <v>0.2480166666666667</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02278333333333334</v>
+        <v>0.02108333333333334</v>
       </c>
     </row>
     <row r="23">
@@ -3315,32 +3319,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.006616666666666667</v>
+        <v>0.004816666666666666</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>281</v>
+        <v>260</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.03049166666666666</v>
+        <v>0.02008333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1992316666666667</v>
+        <v>0.07074166666666666</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.002416666666666666</v>
+        <v>0.02948333333333334</v>
       </c>
     </row>
     <row r="24">
@@ -3349,32 +3353,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.04256666666666666</v>
+        <v>0.001733333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.1085833333333334</v>
+        <v>0.0376</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.3201416666666667</v>
+        <v>0.2164516666666665</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0036</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="25">
@@ -3383,32 +3387,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.03465</v>
+        <v>0.009166666666666667</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.09583333333333334</v>
+        <v>0.0266</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.2476683333333334</v>
+        <v>0.110575</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02323333333333333</v>
+        <v>0.02815833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3417,32 +3421,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Ryan Evans</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.01758333333333333</v>
+        <v>0.004433333333333333</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>263</v>
+        <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.05876666666666666</v>
+        <v>0.02826666666666666</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1876333333333333</v>
+        <v>0.130495</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01648333333333334</v>
+        <v>0.003866666666666666</v>
       </c>
     </row>
     <row r="27">
@@ -3451,32 +3455,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.02411666666666667</v>
+        <v>0.00305</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>249</v>
+        <v>286</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.07647333333333334</v>
+        <v>0.01955833333333333</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2455166666666666</v>
+        <v>0.1842016666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.001975</v>
+        <v>0.001666666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3489,28 +3493,28 @@
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00445</v>
+        <v>0.00245</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>100</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.03681666666666666</v>
+        <v>0.02255833333333333</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2176349999999999</v>
+        <v>0.2044416666666667</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.0062</v>
+        <v>0.0056</v>
       </c>
     </row>
     <row r="29">
@@ -3519,32 +3523,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.008</v>
+        <v>0.01903333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>197</v>
+        <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03333333333333334</v>
+        <v>0.06365</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1194083333333333</v>
+        <v>0.2220333333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.02055</v>
+        <v>0.0046</v>
       </c>
     </row>
     <row r="30">
@@ -3553,32 +3557,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.002366666666666666</v>
+        <v>0.0072</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>266</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.01371666666666667</v>
+        <v>0.0298</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1284533333333333</v>
+        <v>0.11092</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.0065</v>
+        <v>0.03263333333333334</v>
       </c>
     </row>
     <row r="31">
@@ -3587,32 +3591,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.006183333333333333</v>
+        <v>0.00645</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>252</v>
+        <v>204</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.0315</v>
+        <v>0.0243</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.113105</v>
+        <v>0.100155</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.03351666666666667</v>
+        <v>0.020725</v>
       </c>
     </row>
     <row r="32">
@@ -3621,32 +3625,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.003316666666666667</v>
+        <v>0.00465</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03324</v>
+        <v>0.03425</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1876583333333333</v>
+        <v>0.2103833333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.005783333333333334</v>
+        <v>0.00565</v>
       </c>
     </row>
     <row r="33">
@@ -3655,32 +3659,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D33" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.004533333333333333</v>
+        <v>0.00415</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>96</v>
+        <v>87.5</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.03695</v>
+        <v>0.02334166666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.2055766666666666</v>
+        <v>0.13275</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.0064</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="34">
@@ -3689,32 +3693,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.004483333333333334</v>
+        <v>0.002133333333333333</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.02596666666666666</v>
+        <v>0.01051666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.14524</v>
+        <v>0.1042183333333333</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.01098333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3723,32 +3727,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0</v>
+        <v>0.00365</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.001566666666666667</v>
+        <v>0.03155000000000001</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.05024166666666667</v>
+        <v>0.168505</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.08280833333333333</v>
+        <v>0.007866666666666668</v>
       </c>
     </row>
     <row r="36">
@@ -3757,32 +3761,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.00615</v>
+        <v>0.0001</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.02768333333333333</v>
+        <v>0.001833333333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1780916666666667</v>
+        <v>0.04715</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.00655</v>
+        <v>0.09398333333333335</v>
       </c>
     </row>
     <row r="37">
@@ -3791,32 +3795,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
         <v>20</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00385</v>
+        <v>0.00335</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>254</v>
+        <v>209</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.02103333333333333</v>
+        <v>0.021</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.07306333333333333</v>
+        <v>0.1574983333333333</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.05990000000000001</v>
+        <v>0.0053</v>
       </c>
     </row>
     <row r="38">
@@ -3825,7 +3829,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
@@ -3835,22 +3839,22 @@
         <v>7</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.0028</v>
+        <v>0.002183333333333333</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01005</v>
+        <v>0.01585</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.04946666666666667</v>
+        <v>0.06513333333333332</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1203333333333333</v>
+        <v>0.07013333333333334</v>
       </c>
     </row>
     <row r="39">
@@ -3859,32 +3863,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
         <v>20</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0004</v>
+        <v>0.0017</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>211</v>
+        <v>248</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.003366666666666667</v>
+        <v>0.009033333333333334</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04930833333333334</v>
+        <v>0.04805333333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.04189166666666667</v>
+        <v>0.13155</v>
       </c>
     </row>
     <row r="40">
@@ -3893,32 +3897,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D40" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.003583333333333334</v>
+        <v>0.0002</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.02111666666666667</v>
+        <v>0.0023</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.09286666666666665</v>
+        <v>0.03708666666666667</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.02168333333333333</v>
+        <v>0.04766666666666666</v>
       </c>
     </row>
     <row r="41">
@@ -3927,32 +3931,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D41" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.002066666666666666</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00135</v>
+        <v>0.01136666666666667</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02465</v>
+        <v>0.06726666666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.03278333333333333</v>
+        <v>0.025625</v>
       </c>
     </row>
     <row r="42">
@@ -3965,28 +3969,28 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.0007</v>
+        <v>0.00135</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.00505</v>
+        <v>0.004683333333333334</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.02346666666666667</v>
+        <v>0.020125</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.3145916666666668</v>
+        <v>0.288575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 14:42:21 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T18:24:21.074213+00:00</t>
+          <t>2026-03-21T18:42:20.510716+00:00</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.3193939181962715</v>
+        <v>0.317882621342825</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.6806060818037285</v>
+        <v>0.682117378657175</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2373,10 +2373,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1989767127293968</v>
+        <v>0.198276868560611</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8010232872706032</v>
+        <v>0.801723131439389</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2476,10 +2476,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3032940927736555</v>
+        <v>0.304239232173541</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6967059072263444</v>
+        <v>0.6957607678264589</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.11875</v>
+        <v>0.11925</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>134</v>
@@ -2624,10 +2624,10 @@
         <v>334</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3115166666666667</v>
+        <v>0.3120166666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.6838116666666667</v>
+        <v>0.6842116666666667</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2658,10 +2658,10 @@
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.15725</v>
+        <v>0.1573</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3903833333333333</v>
+        <v>0.3909333333333333</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0.00555</v>
@@ -2692,10 +2692,10 @@
         <v>293</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3090166666666667</v>
+        <v>0.3086166666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6906600000000001</v>
+        <v>0.6904600000000001</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2726,13 +2726,13 @@
         <v>310</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.2001166666666667</v>
+        <v>0.1998666666666667</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>0.4748583333333333</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.00045</v>
+        <v>0.00035</v>
       </c>
     </row>
     <row r="6">
@@ -2751,7 +2751,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06313333333333333</v>
+        <v>0.06326666666666668</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>113</v>
@@ -2760,10 +2760,10 @@
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1538083333333334</v>
+        <v>0.1540083333333334</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.37596</v>
+        <v>0.3761100000000001</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0.001033333333333333</v>
@@ -2785,7 +2785,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.04353333333333334</v>
+        <v>0.04313333333333334</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>121</v>
@@ -2794,10 +2794,10 @@
         <v>314</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1256666666666667</v>
+        <v>0.1250166666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4222466666666666</v>
+        <v>0.4215466666666666</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0007</v>
@@ -2819,7 +2819,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.04465</v>
+        <v>0.04475</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>107</v>
@@ -2831,7 +2831,7 @@
         <v>0.1266166666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3122416666666667</v>
+        <v>0.3123416666666667</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0.00435</v>
@@ -2853,7 +2853,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02656666666666667</v>
+        <v>0.02666666666666667</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>119</v>
@@ -2862,10 +2862,10 @@
         <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1081666666666667</v>
+        <v>0.1082666666666667</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4536666666666667</v>
+        <v>0.4539166666666667</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00045</v>
@@ -2887,19 +2887,19 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.02053333333333333</v>
+        <v>0.02043333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>117.5</v>
+        <v>118</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.09152500000000001</v>
+        <v>0.09182500000000002</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.405675</v>
+        <v>0.405875</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.0009</v>
@@ -2930,10 +2930,10 @@
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.08792499999999999</v>
+        <v>0.08822499999999998</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4345383333333333</v>
+        <v>0.4346383333333333</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.0004833333333333334</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.06003333333333333</v>
+        <v>0.05993333333333332</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>122</v>
@@ -2964,10 +2964,10 @@
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1629916666666667</v>
+        <v>0.1631416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.47011</v>
+        <v>0.47031</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -2998,10 +2998,10 @@
         <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1438333333333333</v>
+        <v>0.1439333333333333</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3431716666666667</v>
+        <v>0.3433716666666667</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0.0019</v>
@@ -3023,7 +3023,7 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.02068333333333333</v>
+        <v>0.02071666666666667</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>112</v>
@@ -3035,7 +3035,7 @@
         <v>0.06990000000000002</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3282433333333333</v>
+        <v>0.3280433333333332</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3057,7 +3057,7 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02755</v>
+        <v>0.02775</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>94</v>
@@ -3066,10 +3066,10 @@
         <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.08351666666666668</v>
+        <v>0.08346666666666669</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.234925</v>
+        <v>0.2346249999999999</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.02831666666666666</v>
@@ -3100,10 +3100,10 @@
         <v>310</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0165</v>
+        <v>0.0166</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2667766666666666</v>
+        <v>0.2662766666666666</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0.00195</v>
@@ -3125,7 +3125,7 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.009516666666666666</v>
+        <v>0.009116666666666667</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>80</v>
@@ -3134,10 +3134,10 @@
         <v>258</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.0212</v>
+        <v>0.021</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.07670833333333332</v>
+        <v>0.07630833333333333</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0.03441666666666666</v>
@@ -3168,13 +3168,13 @@
         <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02678333333333334</v>
+        <v>0.02658333333333334</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.09032166666666668</v>
+        <v>0.09012166666666668</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.07629999999999999</v>
+        <v>0.07649999999999998</v>
       </c>
     </row>
     <row r="19">
@@ -3202,10 +3202,10 @@
         <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02795</v>
+        <v>0.02805</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2234999999999999</v>
+        <v>0.2234</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.00045</v>
@@ -3227,7 +3227,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.0631</v>
+        <v>0.0633</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3236,10 +3236,10 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.145125</v>
+        <v>0.145225</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3530550000000001</v>
+        <v>0.3533550000000001</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.003416666666666667</v>
@@ -3261,7 +3261,7 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03546666666666667</v>
+        <v>0.03536666666666667</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>104</v>
@@ -3270,10 +3270,10 @@
         <v>248</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1023166666666667</v>
+        <v>0.1024166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3129449999999999</v>
+        <v>0.313045</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.003583333333333334</v>
@@ -3295,7 +3295,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03178333333333334</v>
+        <v>0.03168333333333333</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>93</v>
@@ -3307,10 +3307,10 @@
         <v>0.09013333333333334</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2480166666666667</v>
+        <v>0.2479166666666666</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02108333333333334</v>
+        <v>0.02098333333333333</v>
       </c>
     </row>
     <row r="23">
@@ -3338,13 +3338,13 @@
         <v>260</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.02008333333333333</v>
+        <v>0.01988333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.07074166666666666</v>
+        <v>0.07039166666666666</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.02948333333333334</v>
+        <v>0.02963333333333334</v>
       </c>
     </row>
     <row r="24">
@@ -3363,7 +3363,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.001733333333333333</v>
+        <v>0.001666666666666666</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>108</v>
@@ -3372,10 +3372,10 @@
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.0376</v>
+        <v>0.03765</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2164516666666665</v>
+        <v>0.2166516666666665</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.0004</v>
@@ -3403,10 +3403,10 @@
         <v>82</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.0266</v>
+        <v>0.0263</v>
       </c>
       <c r="I25" s="7" t="n">
         <v>0.110575</v>
@@ -3431,7 +3431,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.004433333333333333</v>
+        <v>0.004533333333333333</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>89</v>
@@ -3440,7 +3440,7 @@
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02826666666666666</v>
+        <v>0.02846666666666666</v>
       </c>
       <c r="I26" s="5" t="n">
         <v>0.130495</v>
@@ -3477,7 +3477,7 @@
         <v>0.01955833333333333</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1842016666666667</v>
+        <v>0.1845016666666667</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.001666666666666667</v>
@@ -3511,7 +3511,7 @@
         <v>0.02255833333333333</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2044416666666667</v>
+        <v>0.2045916666666667</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0.0056</v>
@@ -3533,7 +3533,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01903333333333333</v>
+        <v>0.01913333333333334</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>102</v>
@@ -3542,10 +3542,10 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.06365</v>
+        <v>0.06375</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2220333333333333</v>
+        <v>0.2222333333333333</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.0046</v>
@@ -3576,7 +3576,7 @@
         <v>266</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0298</v>
+        <v>0.0297</v>
       </c>
       <c r="I30" s="5" t="n">
         <v>0.11092</v>
@@ -3616,7 +3616,7 @@
         <v>0.100155</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.020725</v>
+        <v>0.020675</v>
       </c>
     </row>
     <row r="32">
@@ -3644,10 +3644,10 @@
         <v>226</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03425</v>
+        <v>0.03415</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2103833333333333</v>
+        <v>0.2100333333333333</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.00565</v>
@@ -3672,16 +3672,16 @@
         <v>0.00415</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>87.5</v>
+        <v>87</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02334166666666667</v>
+        <v>0.02344166666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.13275</v>
+        <v>0.13285</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.0001</v>
@@ -3715,7 +3715,7 @@
         <v>0.01051666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.1042183333333333</v>
+        <v>0.1041183333333333</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>0.01098333333333333</v>
@@ -3752,7 +3752,7 @@
         <v>0.168505</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.007866666666666668</v>
+        <v>0.007816666666666668</v>
       </c>
     </row>
     <row r="36">
@@ -3783,10 +3783,10 @@
         <v>0.001833333333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04715</v>
+        <v>0.04735</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.09398333333333335</v>
+        <v>0.09408333333333335</v>
       </c>
     </row>
     <row r="37">
@@ -3817,7 +3817,7 @@
         <v>0.021</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1574983333333333</v>
+        <v>0.1573983333333333</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>0.0053</v>
@@ -3851,10 +3851,10 @@
         <v>0.01585</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06513333333333332</v>
+        <v>0.06523333333333332</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.07013333333333334</v>
+        <v>0.06988333333333334</v>
       </c>
     </row>
     <row r="39">
@@ -3873,7 +3873,7 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0017</v>
+        <v>0.0016</v>
       </c>
       <c r="F39" s="9" t="n">
         <v>69</v>
@@ -3888,7 +3888,7 @@
         <v>0.04805333333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.13155</v>
+        <v>0.1314</v>
       </c>
     </row>
     <row r="40">
@@ -3922,7 +3922,7 @@
         <v>0.03708666666666667</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.04766666666666666</v>
+        <v>0.04756666666666666</v>
       </c>
     </row>
     <row r="41">
@@ -3956,7 +3956,7 @@
         <v>0.06726666666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.025625</v>
+        <v>0.025425</v>
       </c>
     </row>
     <row r="42">
@@ -3975,7 +3975,7 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00135</v>
+        <v>0.00125</v>
       </c>
       <c r="F42" s="8" t="n">
         <v>53</v>
@@ -3984,13 +3984,13 @@
         <v>187</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.004683333333333334</v>
+        <v>0.004583333333333333</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.020125</v>
+        <v>0.019925</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.288575</v>
+        <v>0.289125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 14:45:42 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T18:42:20.510716+00:00</t>
+          <t>2026-03-21T18:45:41.947938+00:00</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.317882621342825</v>
+        <v>0.3172293276970683</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.682117378657175</v>
+        <v>0.6827706723029316</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2373,10 +2373,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.198276868560611</v>
+        <v>0.1997041059830182</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.801723131439389</v>
+        <v>0.8002958940169819</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2627,7 +2627,7 @@
         <v>0.3120166666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.6842116666666667</v>
+        <v>0.6843616666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2658,10 +2658,10 @@
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1573</v>
+        <v>0.1574</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3909333333333333</v>
+        <v>0.3908833333333333</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0.00555</v>
@@ -2692,10 +2692,10 @@
         <v>293</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3086166666666667</v>
+        <v>0.3088166666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6904600000000001</v>
+        <v>0.6904100000000001</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2717,7 +2717,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.079</v>
+        <v>0.0789</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
@@ -2729,10 +2729,10 @@
         <v>0.1998666666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4748583333333333</v>
+        <v>0.4746583333333333</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.00035</v>
+        <v>0.00045</v>
       </c>
     </row>
     <row r="6">
@@ -2751,7 +2751,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06326666666666668</v>
+        <v>0.06313333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>113</v>
@@ -2760,7 +2760,7 @@
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1540083333333334</v>
+        <v>0.1539083333333333</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0.3761100000000001</v>
@@ -2785,7 +2785,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.04313333333333334</v>
+        <v>0.04323333333333334</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>121</v>
@@ -2797,7 +2797,7 @@
         <v>0.1250166666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4215466666666666</v>
+        <v>0.4211966666666666</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0007</v>
@@ -2831,7 +2831,7 @@
         <v>0.1266166666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3123416666666667</v>
+        <v>0.3124416666666667</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0.00435</v>
@@ -2865,7 +2865,7 @@
         <v>0.1082666666666667</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4539166666666667</v>
+        <v>0.4536166666666667</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00045</v>
@@ -2890,16 +2890,16 @@
         <v>0.02043333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>118</v>
+        <v>117.5</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.09182500000000002</v>
+        <v>0.09152500000000001</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.405875</v>
+        <v>0.405575</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.0009</v>
@@ -2930,10 +2930,10 @@
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.08822499999999998</v>
+        <v>0.088125</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4346383333333333</v>
+        <v>0.4348383333333333</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.0004833333333333334</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.05993333333333332</v>
+        <v>0.06003333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>122</v>
@@ -2964,10 +2964,10 @@
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1631416666666667</v>
+        <v>0.1630416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.47031</v>
+        <v>0.4704099999999999</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -3004,7 +3004,7 @@
         <v>0.3433716666666667</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0019</v>
+        <v>0.00185</v>
       </c>
     </row>
     <row r="14">
@@ -3023,7 +3023,7 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.02071666666666667</v>
+        <v>0.02068333333333333</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>112</v>
@@ -3035,7 +3035,7 @@
         <v>0.06990000000000002</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3280433333333332</v>
+        <v>0.3281433333333332</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3057,7 +3057,7 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02775</v>
+        <v>0.02755</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>94</v>
@@ -3066,13 +3066,13 @@
         <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.08346666666666669</v>
+        <v>0.08321666666666669</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2346249999999999</v>
+        <v>0.2343249999999999</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.02831666666666666</v>
+        <v>0.02841666666666666</v>
       </c>
     </row>
     <row r="16">
@@ -3103,7 +3103,7 @@
         <v>0.0166</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2662766666666666</v>
+        <v>0.2664766666666666</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0.00195</v>
@@ -3125,7 +3125,7 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.009116666666666667</v>
+        <v>0.009516666666666666</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>80</v>
@@ -3134,13 +3134,13 @@
         <v>258</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.021</v>
+        <v>0.0213</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.07630833333333333</v>
+        <v>0.07670833333333332</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.03441666666666666</v>
+        <v>0.03431666666666666</v>
       </c>
     </row>
     <row r="18">
@@ -3205,7 +3205,7 @@
         <v>0.02805</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2234</v>
+        <v>0.2232999999999999</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.00045</v>
@@ -3227,7 +3227,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.0633</v>
+        <v>0.0631</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3236,13 +3236,13 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.145225</v>
+        <v>0.145125</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3533550000000001</v>
+        <v>0.3531550000000001</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.003416666666666667</v>
+        <v>0.003516666666666667</v>
       </c>
     </row>
     <row r="21">
@@ -3273,7 +3273,7 @@
         <v>0.1024166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.313045</v>
+        <v>0.313095</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.003583333333333334</v>
@@ -3307,10 +3307,10 @@
         <v>0.09013333333333334</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2479166666666666</v>
+        <v>0.2480166666666667</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02098333333333333</v>
+        <v>0.02108333333333334</v>
       </c>
     </row>
     <row r="23">
@@ -3338,13 +3338,13 @@
         <v>260</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01988333333333333</v>
+        <v>0.02008333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.07039166666666666</v>
+        <v>0.07074166666666666</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.02963333333333334</v>
+        <v>0.02953333333333334</v>
       </c>
     </row>
     <row r="24">
@@ -3363,7 +3363,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.001666666666666666</v>
+        <v>0.001733333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>108</v>
@@ -3372,7 +3372,7 @@
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03765</v>
+        <v>0.0377</v>
       </c>
       <c r="I24" s="5" t="n">
         <v>0.2166516666666665</v>
@@ -3403,16 +3403,16 @@
         <v>82</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.0263</v>
+        <v>0.0266</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.110575</v>
+        <v>0.110775</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02815833333333334</v>
+        <v>0.02805833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3434,13 +3434,13 @@
         <v>0.004533333333333333</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>89</v>
+        <v>89.5</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02846666666666666</v>
+        <v>0.02836666666666666</v>
       </c>
       <c r="I26" s="5" t="n">
         <v>0.130495</v>
@@ -3477,7 +3477,7 @@
         <v>0.01955833333333333</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1845016666666667</v>
+        <v>0.1846016666666667</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.001666666666666667</v>
@@ -3511,7 +3511,7 @@
         <v>0.02255833333333333</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2045916666666667</v>
+        <v>0.2046416666666667</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0.0056</v>
@@ -3533,7 +3533,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01913333333333334</v>
+        <v>0.01903333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>102</v>
@@ -3542,10 +3542,10 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.06375</v>
+        <v>0.06365</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2222333333333333</v>
+        <v>0.2220333333333333</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.0046</v>
@@ -3579,7 +3579,7 @@
         <v>0.0297</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.11092</v>
+        <v>0.11072</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0.03263333333333334</v>
@@ -3616,7 +3616,7 @@
         <v>0.100155</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.020675</v>
+        <v>0.020625</v>
       </c>
     </row>
     <row r="32">
@@ -3647,7 +3647,7 @@
         <v>0.03415</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2100333333333333</v>
+        <v>0.2101833333333334</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.00565</v>
@@ -3678,10 +3678,10 @@
         <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02344166666666667</v>
+        <v>0.02334166666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.13285</v>
+        <v>0.13275</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.0001</v>
@@ -3715,7 +3715,7 @@
         <v>0.01051666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.1041183333333333</v>
+        <v>0.1042183333333333</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>0.01098333333333333</v>
@@ -3752,7 +3752,7 @@
         <v>0.168505</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.007816666666666668</v>
+        <v>0.007866666666666668</v>
       </c>
     </row>
     <row r="36">
@@ -3783,10 +3783,10 @@
         <v>0.001833333333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04735</v>
+        <v>0.04715</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.09408333333333335</v>
+        <v>0.09418333333333335</v>
       </c>
     </row>
     <row r="37">
@@ -3854,7 +3854,7 @@
         <v>0.06523333333333332</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.06988333333333334</v>
+        <v>0.07018333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3922,7 +3922,7 @@
         <v>0.03708666666666667</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.04756666666666666</v>
+        <v>0.04751666666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3956,7 +3956,7 @@
         <v>0.06726666666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.025425</v>
+        <v>0.025625</v>
       </c>
     </row>
     <row r="42">
@@ -3975,7 +3975,7 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00125</v>
+        <v>0.00135</v>
       </c>
       <c r="F42" s="8" t="n">
         <v>53</v>
@@ -3984,13 +3984,13 @@
         <v>187</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.004583333333333333</v>
+        <v>0.004683333333333334</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.019925</v>
+        <v>0.020125</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.289125</v>
+        <v>0.288525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 15:00:04 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T18:46:58.096895+00:00</t>
+          <t>2026-03-21T19:00:04.138435+00:00</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr"/>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.3172293276970683</v>
+        <v>0.290417422624646</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.6827706723029316</v>
+        <v>0.709582577375354</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2476,10 +2476,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.304239232173541</v>
+        <v>0.3058865166128497</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6957607678264589</v>
+        <v>0.6941134833871503</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.11925</v>
+        <v>0.1211</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>134</v>
@@ -2624,10 +2624,10 @@
         <v>334</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3120166666666667</v>
+        <v>0.3155666666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.6843616666666666</v>
+        <v>0.6885783333333332</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2649,7 +2649,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.0581</v>
+        <v>0.0585</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>115</v>
@@ -2658,13 +2658,13 @@
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1574</v>
+        <v>0.15955</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3908833333333333</v>
+        <v>0.3932999999999999</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.00555</v>
+        <v>0.00535</v>
       </c>
     </row>
     <row r="4">
@@ -2683,7 +2683,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.1293</v>
+        <v>0.12905</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>136</v>
@@ -2692,10 +2692,10 @@
         <v>293</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3088166666666667</v>
+        <v>0.3083500000000001</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6904100000000001</v>
+        <v>0.6895766666666666</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2717,7 +2717,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.0789</v>
+        <v>0.07826666666666668</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
@@ -2726,10 +2726,10 @@
         <v>310</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1998666666666667</v>
+        <v>0.1994</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4746583333333333</v>
+        <v>0.4736583333333333</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.00045</v>
@@ -2751,7 +2751,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06313333333333333</v>
+        <v>0.06418333333333334</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>113</v>
@@ -2760,13 +2760,13 @@
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1539083333333333</v>
+        <v>0.156125</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3761100000000001</v>
+        <v>0.3780850000000001</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.001033333333333333</v>
+        <v>0.0009833333333333335</v>
       </c>
     </row>
     <row r="7">
@@ -2785,19 +2785,19 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.04323333333333334</v>
+        <v>0.03945</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>314</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1250166666666667</v>
+        <v>0.1173333333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4211966666666666</v>
+        <v>0.4102466666666667</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0007</v>
@@ -2819,7 +2819,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.04475</v>
+        <v>0.0449</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>107</v>
@@ -2828,13 +2828,13 @@
         <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1266166666666667</v>
+        <v>0.12665</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3124416666666667</v>
+        <v>0.3124833333333333</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.00435</v>
+        <v>0.0044</v>
       </c>
     </row>
     <row r="9">
@@ -2853,7 +2853,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02666666666666667</v>
+        <v>0.02638333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>119</v>
@@ -2865,7 +2865,7 @@
         <v>0.1082666666666667</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4536166666666667</v>
+        <v>0.4526166666666667</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00045</v>
@@ -2890,16 +2890,16 @@
         <v>0.02043333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>117.5</v>
+        <v>118</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.09152500000000001</v>
+        <v>0.09115833333333336</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.405575</v>
+        <v>0.4051999999999999</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.0009</v>
@@ -2921,19 +2921,19 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0171</v>
+        <v>0.0173</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.088125</v>
+        <v>0.08967499999999999</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4348383333333333</v>
+        <v>0.438755</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.0004833333333333334</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.06003333333333333</v>
+        <v>0.06083333333333332</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>122</v>
@@ -2964,10 +2964,10 @@
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1630416666666667</v>
+        <v>0.1650583333333333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4704099999999999</v>
+        <v>0.4744599999999999</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -2989,7 +2989,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05548333333333333</v>
+        <v>0.05643333333333333</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>106</v>
@@ -2998,10 +2998,10 @@
         <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1439333333333333</v>
+        <v>0.1448666666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3433716666666667</v>
+        <v>0.344805</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0.00185</v>
@@ -3032,10 +3032,10 @@
         <v>307</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.06990000000000002</v>
+        <v>0.06980000000000001</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3281433333333332</v>
+        <v>0.32751</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3057,7 +3057,7 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02755</v>
+        <v>0.027</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>94</v>
@@ -3066,13 +3066,13 @@
         <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.08321666666666669</v>
+        <v>0.08066666666666668</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2343249999999999</v>
+        <v>0.2280999999999999</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.02841666666666666</v>
+        <v>0.02936666666666666</v>
       </c>
     </row>
     <row r="16">
@@ -3094,7 +3094,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G16" s="8" t="n">
         <v>310</v>
@@ -3103,10 +3103,10 @@
         <v>0.0166</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2664766666666666</v>
+        <v>0.2661849999999999</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.00195</v>
+        <v>0.00205</v>
       </c>
     </row>
     <row r="17">
@@ -3125,7 +3125,7 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.009516666666666666</v>
+        <v>0.009666666666666665</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>80</v>
@@ -3137,10 +3137,10 @@
         <v>0.0213</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.07670833333333332</v>
+        <v>0.07748333333333332</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.03431666666666666</v>
+        <v>0.03316666666666666</v>
       </c>
     </row>
     <row r="18">
@@ -3159,22 +3159,22 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.0071</v>
+        <v>0.0068</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02658333333333334</v>
+        <v>0.02538333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.09012166666666668</v>
+        <v>0.08602166666666668</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.07649999999999998</v>
+        <v>0.07964999999999998</v>
       </c>
     </row>
     <row r="19">
@@ -3193,7 +3193,7 @@
         <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.00475</v>
+        <v>0.00495</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>108</v>
@@ -3202,10 +3202,10 @@
         <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02805</v>
+        <v>0.02775</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2232999999999999</v>
+        <v>0.2219333333333333</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.00045</v>
@@ -3236,10 +3236,10 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.145125</v>
+        <v>0.1445416666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3531550000000001</v>
+        <v>0.3526883333333334</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.003516666666666667</v>
@@ -3261,7 +3261,7 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03536666666666667</v>
+        <v>0.03546666666666667</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>104</v>
@@ -3270,13 +3270,13 @@
         <v>248</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1024166666666667</v>
+        <v>0.1033166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.313095</v>
+        <v>0.3162283333333332</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.003583333333333334</v>
+        <v>0.003483333333333334</v>
       </c>
     </row>
     <row r="22">
@@ -3295,7 +3295,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03168333333333333</v>
+        <v>0.03138333333333334</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>93</v>
@@ -3304,13 +3304,13 @@
         <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.09013333333333334</v>
+        <v>0.08976666666666668</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2480166666666667</v>
+        <v>0.2476333333333333</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02108333333333334</v>
+        <v>0.02123333333333333</v>
       </c>
     </row>
     <row r="23">
@@ -3329,7 +3329,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.004816666666666666</v>
+        <v>0.004766666666666666</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>77</v>
@@ -3338,13 +3338,13 @@
         <v>260</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.02008333333333333</v>
+        <v>0.01978333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.07074166666666666</v>
+        <v>0.07065833333333332</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.02953333333333334</v>
+        <v>0.02978333333333334</v>
       </c>
     </row>
     <row r="24">
@@ -3363,7 +3363,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.001733333333333333</v>
+        <v>0.001833333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>108</v>
@@ -3372,10 +3372,10 @@
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.0377</v>
+        <v>0.03876666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2166516666666665</v>
+        <v>0.2196933333333333</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.0004</v>
@@ -3397,7 +3397,7 @@
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.009166666666666667</v>
+        <v>0.009216666666666666</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>82</v>
@@ -3406,13 +3406,13 @@
         <v>245</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.0266</v>
+        <v>0.02685</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.110775</v>
+        <v>0.111575</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02805833333333334</v>
+        <v>0.02730833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3434,16 +3434,16 @@
         <v>0.004533333333333333</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>89.5</v>
+        <v>90</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02836666666666666</v>
+        <v>0.02851666666666666</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.130495</v>
+        <v>0.1310283333333334</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.003866666666666666</v>
@@ -3465,7 +3465,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.00305</v>
+        <v>0.00315</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>104</v>
@@ -3474,10 +3474,10 @@
         <v>286</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.01955833333333333</v>
+        <v>0.02030833333333333</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1846016666666667</v>
+        <v>0.1878016666666667</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.001666666666666667</v>
@@ -3502,19 +3502,19 @@
         <v>0.00245</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G28" s="8" t="n">
         <v>248</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.02255833333333333</v>
+        <v>0.022975</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2046416666666667</v>
+        <v>0.2064416666666667</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.0056</v>
+        <v>0.0054</v>
       </c>
     </row>
     <row r="29">
@@ -3533,7 +3533,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01903333333333333</v>
+        <v>0.01893333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>102</v>
@@ -3542,13 +3542,13 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.06365</v>
+        <v>0.0636</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2220333333333333</v>
+        <v>0.2215166666666666</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0046</v>
+        <v>0.0045</v>
       </c>
     </row>
     <row r="30">
@@ -3567,22 +3567,22 @@
         <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0072</v>
+        <v>0.00695</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>266</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0297</v>
+        <v>0.0275</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.11072</v>
+        <v>0.1049033333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03263333333333334</v>
+        <v>0.03358333333333334</v>
       </c>
     </row>
     <row r="31">
@@ -3610,13 +3610,13 @@
         <v>204</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.0243</v>
+        <v>0.02455</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.100155</v>
+        <v>0.1018216666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.020625</v>
+        <v>0.019725</v>
       </c>
     </row>
     <row r="32">
@@ -3635,7 +3635,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00465</v>
+        <v>0.00455</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>97</v>
@@ -3644,13 +3644,13 @@
         <v>226</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03415</v>
+        <v>0.03385</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2101833333333334</v>
+        <v>0.2086333333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00565</v>
+        <v>0.0056</v>
       </c>
     </row>
     <row r="33">
@@ -3678,10 +3678,10 @@
         <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02334166666666667</v>
+        <v>0.02309166666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.13275</v>
+        <v>0.1322166666666667</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.0001</v>
@@ -3712,13 +3712,13 @@
         <v>255</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.01051666666666667</v>
+        <v>0.01046666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.1042183333333333</v>
+        <v>0.1038516666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.01098333333333333</v>
+        <v>0.01088333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3737,7 +3737,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00365</v>
+        <v>0.00385</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>91</v>
@@ -3746,13 +3746,13 @@
         <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03155000000000001</v>
+        <v>0.03215</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.168505</v>
+        <v>0.1711466666666666</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.007866666666666668</v>
+        <v>0.007216666666666667</v>
       </c>
     </row>
     <row r="36">
@@ -3783,10 +3783,10 @@
         <v>0.001833333333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04715</v>
+        <v>0.0467</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.09418333333333335</v>
+        <v>0.09428333333333334</v>
       </c>
     </row>
     <row r="37">
@@ -3805,7 +3805,7 @@
         <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00335</v>
+        <v>0.00365</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>95</v>
@@ -3814,13 +3814,13 @@
         <v>209</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.021</v>
+        <v>0.0215</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1573983333333333</v>
+        <v>0.1588483333333333</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0053</v>
+        <v>0.0052</v>
       </c>
     </row>
     <row r="38">
@@ -3848,13 +3848,13 @@
         <v>257</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01585</v>
+        <v>0.01578333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06523333333333332</v>
+        <v>0.06478333333333333</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.07018333333333333</v>
+        <v>0.07038333333333334</v>
       </c>
     </row>
     <row r="39">
@@ -3882,13 +3882,13 @@
         <v>248</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.009033333333333334</v>
+        <v>0.0089</v>
       </c>
       <c r="I39" s="7" t="n">
         <v>0.04805333333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1314</v>
+        <v>0.1312</v>
       </c>
     </row>
     <row r="40">
@@ -3916,13 +3916,13 @@
         <v>208</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.0023</v>
+        <v>0.00245</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.03708666666666667</v>
+        <v>0.03733666666666667</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.04751666666666667</v>
+        <v>0.04606666666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3953,10 +3953,10 @@
         <v>0.01136666666666667</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.06726666666666667</v>
+        <v>0.06736666666666669</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.025625</v>
+        <v>0.025775</v>
       </c>
     </row>
     <row r="42">
@@ -3984,13 +3984,13 @@
         <v>187</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.004683333333333334</v>
+        <v>0.004633333333333334</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.020125</v>
+        <v>0.020075</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.288525</v>
+        <v>0.288475</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 15:20:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T19:00:04.138435+00:00</t>
+          <t>2026-03-21T19:20:07.709745+00:00</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.290417422624646</v>
+        <v>0.2530158956748701</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.709582577375354</v>
+        <v>0.7469841043251298</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2373,10 +2373,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1997041059830182</v>
+        <v>0.1979686364434314</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8002958940169819</v>
+        <v>0.8020313635565686</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2476,10 +2476,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3058865166128497</v>
+        <v>0.3085367443007756</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6941134833871503</v>
+        <v>0.6914632556992244</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2615,19 +2615,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1211</v>
+        <v>0.12435</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>334</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3155666666666667</v>
+        <v>0.3220166666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.6885783333333332</v>
+        <v>0.6941616666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2649,22 +2649,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.0585</v>
+        <v>0.0598</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.15955</v>
+        <v>0.16235</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3932999999999999</v>
+        <v>0.3982333333333333</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.00535</v>
+        <v>0.004900000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -2683,7 +2683,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.12905</v>
+        <v>0.1287</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>136</v>
@@ -2692,10 +2692,10 @@
         <v>293</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3083500000000001</v>
+        <v>0.3071833333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6895766666666666</v>
+        <v>0.6879599999999999</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2717,7 +2717,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07826666666666668</v>
+        <v>0.07801666666666668</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
@@ -2726,13 +2726,13 @@
         <v>310</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1994</v>
+        <v>0.1979166666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4736583333333333</v>
+        <v>0.4719583333333333</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.00045</v>
+        <v>0.00035</v>
       </c>
     </row>
     <row r="6">
@@ -2751,7 +2751,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06418333333333334</v>
+        <v>0.06533333333333334</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>113</v>
@@ -2760,13 +2760,13 @@
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.156125</v>
+        <v>0.1588916666666667</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3780850000000001</v>
+        <v>0.3817016666666667</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.0009833333333333335</v>
+        <v>0.0009333333333333334</v>
       </c>
     </row>
     <row r="7">
@@ -2785,22 +2785,22 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.03945</v>
+        <v>0.0352</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>314</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1173333333333333</v>
+        <v>0.10565</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4102466666666667</v>
+        <v>0.39393</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.0007</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="8">
@@ -2828,10 +2828,10 @@
         <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.12665</v>
+        <v>0.1269166666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3124833333333333</v>
+        <v>0.3124166666666667</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0.0044</v>
@@ -2853,19 +2853,19 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02638333333333333</v>
+        <v>0.02643333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1082666666666667</v>
+        <v>0.1083166666666667</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4526166666666667</v>
+        <v>0.4524999999999999</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00045</v>
@@ -2887,7 +2887,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.02043333333333333</v>
+        <v>0.02028333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>118</v>
@@ -2896,10 +2896,10 @@
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.09115833333333336</v>
+        <v>0.09107500000000002</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4051999999999999</v>
+        <v>0.4038833333333333</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.0009</v>
@@ -2921,7 +2921,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0173</v>
+        <v>0.01785</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>119</v>
@@ -2930,10 +2930,10 @@
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.08967499999999999</v>
+        <v>0.09140833333333333</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.438755</v>
+        <v>0.4438466666666666</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.0004833333333333334</v>
@@ -2955,19 +2955,19 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.06083333333333332</v>
+        <v>0.06163333333333332</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1650583333333333</v>
+        <v>0.1682583333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4744599999999999</v>
+        <v>0.4785599999999999</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -2989,19 +2989,19 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05643333333333333</v>
+        <v>0.05718333333333333</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1448666666666667</v>
+        <v>0.14615</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.344805</v>
+        <v>0.3473633333333334</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0.00185</v>
@@ -3023,19 +3023,19 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.02068333333333333</v>
+        <v>0.02038333333333333</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>112</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.06980000000000001</v>
+        <v>0.06965000000000002</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.32751</v>
+        <v>0.3261599999999999</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3057,22 +3057,22 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.027</v>
+        <v>0.02575</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.08066666666666668</v>
+        <v>0.07638333333333334</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2280999999999999</v>
+        <v>0.2189666666666666</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.02936666666666666</v>
+        <v>0.03056666666666666</v>
       </c>
     </row>
     <row r="16">
@@ -3100,13 +3100,13 @@
         <v>310</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0166</v>
+        <v>0.0165</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2661849999999999</v>
+        <v>0.264635</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.00205</v>
+        <v>0.0022</v>
       </c>
     </row>
     <row r="17">
@@ -3125,22 +3125,22 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.009666666666666665</v>
+        <v>0.009366666666666667</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>258</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.0213</v>
+        <v>0.02143333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.07748333333333332</v>
+        <v>0.07868333333333333</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.03316666666666666</v>
+        <v>0.03176666666666667</v>
       </c>
     </row>
     <row r="18">
@@ -3159,22 +3159,22 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.0068</v>
+        <v>0.0058</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02538333333333333</v>
+        <v>0.02323333333333334</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.08602166666666668</v>
+        <v>0.07938833333333334</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.07964999999999998</v>
+        <v>0.08293333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -3193,7 +3193,7 @@
         <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.00495</v>
+        <v>0.0048</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>108</v>
@@ -3202,10 +3202,10 @@
         <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02775</v>
+        <v>0.02745</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2219333333333333</v>
+        <v>0.22095</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.00045</v>
@@ -3227,7 +3227,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.0631</v>
+        <v>0.06304999999999999</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3236,13 +3236,13 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.1445416666666667</v>
+        <v>0.1438583333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3526883333333334</v>
+        <v>0.3524716666666667</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.003516666666666667</v>
+        <v>0.003716666666666666</v>
       </c>
     </row>
     <row r="21">
@@ -3261,22 +3261,22 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03546666666666667</v>
+        <v>0.03651666666666667</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G21" s="9" t="n">
         <v>248</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1033166666666667</v>
+        <v>0.1050666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3162283333333332</v>
+        <v>0.3194616666666665</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.003483333333333334</v>
+        <v>0.003383333333333333</v>
       </c>
     </row>
     <row r="22">
@@ -3295,7 +3295,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03138333333333334</v>
+        <v>0.03113333333333334</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>93</v>
@@ -3304,13 +3304,13 @@
         <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.08976666666666668</v>
+        <v>0.08971666666666668</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2476333333333333</v>
+        <v>0.2468833333333333</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02123333333333333</v>
+        <v>0.02111666666666667</v>
       </c>
     </row>
     <row r="23">
@@ -3329,7 +3329,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.004766666666666666</v>
+        <v>0.004666666666666666</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>77</v>
@@ -3338,13 +3338,13 @@
         <v>260</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01978333333333333</v>
+        <v>0.01943333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.07065833333333332</v>
+        <v>0.07025833333333333</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.02978333333333334</v>
+        <v>0.03003333333333334</v>
       </c>
     </row>
     <row r="24">
@@ -3363,7 +3363,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.001833333333333333</v>
+        <v>0.001883333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>108</v>
@@ -3372,13 +3372,13 @@
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03876666666666667</v>
+        <v>0.03995</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2196933333333333</v>
+        <v>0.2241183333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0004</v>
+        <v>0.00035</v>
       </c>
     </row>
     <row r="25">
@@ -3397,22 +3397,22 @@
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.009216666666666666</v>
+        <v>0.009316666666666668</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>82</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02685</v>
+        <v>0.02715</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.111575</v>
+        <v>0.1129083333333333</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02730833333333334</v>
+        <v>0.02600833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3431,7 +3431,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.004533333333333333</v>
+        <v>0.004633333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>90</v>
@@ -3440,13 +3440,13 @@
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02851666666666666</v>
+        <v>0.02936666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1310283333333334</v>
+        <v>0.1309783333333334</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.003866666666666666</v>
+        <v>0.004016666666666667</v>
       </c>
     </row>
     <row r="27">
@@ -3465,7 +3465,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.00315</v>
+        <v>0.0033</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>104</v>
@@ -3474,13 +3474,13 @@
         <v>286</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02030833333333333</v>
+        <v>0.02124166666666667</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1878016666666667</v>
+        <v>0.19216</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.001666666666666667</v>
+        <v>0.001416666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3508,13 +3508,13 @@
         <v>248</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.022975</v>
+        <v>0.02350833333333333</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2064416666666667</v>
+        <v>0.2111416666666667</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.0054</v>
+        <v>0.00535</v>
       </c>
     </row>
     <row r="29">
@@ -3533,7 +3533,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01893333333333333</v>
+        <v>0.01883333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>102</v>
@@ -3542,13 +3542,13 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.0636</v>
+        <v>0.0635</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2215166666666666</v>
+        <v>0.2206833333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0045</v>
+        <v>0.0044</v>
       </c>
     </row>
     <row r="30">
@@ -3567,22 +3567,22 @@
         <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.00695</v>
+        <v>0.00585</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>266</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0275</v>
+        <v>0.0244</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1049033333333333</v>
+        <v>0.0973866666666667</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03358333333333334</v>
+        <v>0.03508333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -3601,7 +3601,7 @@
         <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.00645</v>
+        <v>0.00665</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>87</v>
@@ -3610,13 +3610,13 @@
         <v>204</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.02455</v>
+        <v>0.02515</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.1018216666666667</v>
+        <v>0.1032216666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.019725</v>
+        <v>0.018975</v>
       </c>
     </row>
     <row r="32">
@@ -3635,7 +3635,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00455</v>
+        <v>0.00465</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>97</v>
@@ -3647,10 +3647,10 @@
         <v>0.03385</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2086333333333333</v>
+        <v>0.2071833333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0056</v>
+        <v>0.0057</v>
       </c>
     </row>
     <row r="33">
@@ -3678,10 +3678,10 @@
         <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02309166666666667</v>
+        <v>0.02329166666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1322166666666667</v>
+        <v>0.13175</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.0001</v>
@@ -3703,7 +3703,7 @@
         <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.002133333333333333</v>
+        <v>0.002033333333333333</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>94</v>
@@ -3715,10 +3715,10 @@
         <v>0.01046666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.1038516666666667</v>
+        <v>0.1033766666666666</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.01088333333333333</v>
+        <v>0.01098333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3737,7 +3737,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00385</v>
+        <v>0.0041</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>91</v>
@@ -3746,13 +3746,13 @@
         <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03215</v>
+        <v>0.03245000000000001</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1711466666666666</v>
+        <v>0.1736466666666666</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.007216666666666667</v>
+        <v>0.006666666666666667</v>
       </c>
     </row>
     <row r="36">
@@ -3783,10 +3783,10 @@
         <v>0.001833333333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.0467</v>
+        <v>0.0468</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.09428333333333334</v>
+        <v>0.09468333333333334</v>
       </c>
     </row>
     <row r="37">
@@ -3805,22 +3805,22 @@
         <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00365</v>
+        <v>0.0036</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G37" s="9" t="n">
         <v>209</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0215</v>
+        <v>0.0223</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1588483333333333</v>
+        <v>0.1621233333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0052</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="38">
@@ -3848,13 +3848,13 @@
         <v>257</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01578333333333333</v>
+        <v>0.01568333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
         <v>0.06478333333333333</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.07038333333333334</v>
+        <v>0.06983333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3882,13 +3882,13 @@
         <v>248</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.0089</v>
+        <v>0.008750000000000001</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04805333333333334</v>
+        <v>0.04800333333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1312</v>
+        <v>0.1308833333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3919,10 +3919,10 @@
         <v>0.00245</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.03733666666666667</v>
+        <v>0.03818666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.04606666666666667</v>
+        <v>0.04436666666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3953,10 +3953,10 @@
         <v>0.01136666666666667</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.06736666666666669</v>
+        <v>0.06740000000000003</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.025775</v>
+        <v>0.025625</v>
       </c>
     </row>
     <row r="42">
@@ -3975,7 +3975,7 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00135</v>
+        <v>0.00125</v>
       </c>
       <c r="F42" s="8" t="n">
         <v>53</v>
@@ -3984,13 +3984,13 @@
         <v>187</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.004633333333333334</v>
+        <v>0.004433333333333333</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.020075</v>
+        <v>0.019775</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.288475</v>
+        <v>0.289225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 15:28:37 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>25</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T19:20:07.709745+00:00</t>
+          <t>2026-03-21T19:28:36.728989+00:00</t>
         </is>
       </c>
     </row>
@@ -1999,10 +1999,14 @@
       </c>
       <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G34" s="5" t="inlineStr"/>
-      <c r="H34" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>0.85556916598514</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>0.14443083401486</v>
+      </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
           <t>R32_E_01</t>
@@ -2068,10 +2072,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.2530158956748701</v>
+        <v>0.2408024924172188</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.7469841043251298</v>
+        <v>0.7591975075827812</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2337,10 +2341,14 @@
       </c>
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G44" s="5" t="inlineStr"/>
-      <c r="H44" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>0.1733993715190214</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>0.8266006284809787</v>
+      </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
           <t>R32_S_03</t>
@@ -2615,19 +2623,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.12435</v>
+        <v>0.1329</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3220166666666667</v>
+        <v>0.3380666666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.6941616666666666</v>
+        <v>0.7079033333333333</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2649,22 +2657,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.0598</v>
+        <v>0.06</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.16235</v>
+        <v>0.1667833333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3982333333333333</v>
+        <v>0.4034666666666666</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.004900000000000001</v>
+        <v>0.004766666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -2683,19 +2691,19 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.1287</v>
+        <v>0.14145</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3071833333333334</v>
+        <v>0.3258833333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6879599999999999</v>
+        <v>0.7068433333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2717,22 +2725,22 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07801666666666668</v>
+        <v>0.07756666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1979166666666667</v>
+        <v>0.19805</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4719583333333333</v>
+        <v>0.4727083333333333</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.00035</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="6">
@@ -2751,7 +2759,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06533333333333334</v>
+        <v>0.06473333333333334</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>113</v>
@@ -2760,13 +2768,13 @@
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1588916666666667</v>
+        <v>0.1585083333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3817016666666667</v>
+        <v>0.3799933333333332</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.0009333333333333334</v>
+        <v>0.001016666666666667</v>
       </c>
     </row>
     <row r="7">
@@ -2785,22 +2793,22 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0352</v>
+        <v>0.03275</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.10565</v>
+        <v>0.09866666666666668</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.39393</v>
+        <v>0.3847133333333334</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.0008</v>
+        <v>0.0011</v>
       </c>
     </row>
     <row r="8">
@@ -2819,22 +2827,22 @@
         <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0449</v>
+        <v>0.046</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1269166666666667</v>
+        <v>0.1299833333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3124166666666667</v>
+        <v>0.320225</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.0044</v>
+        <v>0.00385</v>
       </c>
     </row>
     <row r="9">
@@ -2853,22 +2861,22 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02643333333333333</v>
+        <v>0.02505</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1083166666666667</v>
+        <v>0.1036833333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4524999999999999</v>
+        <v>0.4407999999999999</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00045</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -2887,22 +2895,22 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.02028333333333333</v>
+        <v>0.01953333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.09107500000000002</v>
+        <v>0.08670833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4038833333333333</v>
+        <v>0.3925833333333333</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0009</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="11">
@@ -2921,7 +2929,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.01785</v>
+        <v>0.0177</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>119</v>
@@ -2930,13 +2938,13 @@
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.09140833333333333</v>
+        <v>0.09145833333333332</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4438466666666666</v>
+        <v>0.4500133333333332</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.0004833333333333334</v>
+        <v>0.0005833333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -2955,19 +2963,19 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.06163333333333332</v>
+        <v>0.06048333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1682583333333334</v>
+        <v>0.1659416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4785599999999999</v>
+        <v>0.4704433333333333</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -2989,22 +2997,22 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05718333333333333</v>
+        <v>0.05403333333333333</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.14615</v>
+        <v>0.1441166666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3473633333333334</v>
+        <v>0.345425</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.00185</v>
+        <v>0.0017</v>
       </c>
     </row>
     <row r="14">
@@ -3023,19 +3031,19 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.02038333333333333</v>
+        <v>0.0135</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.06965000000000002</v>
+        <v>0.05525</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3261599999999999</v>
+        <v>0.3036099999999999</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3057,22 +3065,22 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02575</v>
+        <v>0.02355</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.07638333333333334</v>
+        <v>0.07110000000000001</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2189666666666666</v>
+        <v>0.2109916666666667</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.03056666666666666</v>
+        <v>0.0322</v>
       </c>
     </row>
     <row r="16">
@@ -3097,16 +3105,16 @@
         <v>111</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>310</v>
+        <v>320</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0165</v>
+        <v>0.0196</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.264635</v>
+        <v>0.2771433333333333</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.0022</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="17">
@@ -3125,22 +3133,22 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.009366666666666667</v>
+        <v>0.007533333333333333</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>258</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.02143333333333334</v>
+        <v>0.01666666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.07868333333333333</v>
+        <v>0.06560000000000001</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.03176666666666667</v>
+        <v>0.03293333333333333</v>
       </c>
     </row>
     <row r="18">
@@ -3159,7 +3167,7 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.0058</v>
+        <v>0.0054</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>68</v>
@@ -3168,13 +3176,13 @@
         <v>207</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02323333333333334</v>
+        <v>0.02188333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07938833333333334</v>
+        <v>0.07574166666666667</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.08293333333333333</v>
+        <v>0.09006666666666666</v>
       </c>
     </row>
     <row r="19">
@@ -3193,22 +3201,22 @@
         <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.0048</v>
+        <v>0.0041</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G19" s="9" t="n">
         <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02745</v>
+        <v>0.02505</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.22095</v>
+        <v>0.2108166666666667</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.00045</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="20">
@@ -3227,7 +3235,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.06304999999999999</v>
+        <v>0.06206666666666667</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3236,13 +3244,13 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.1438583333333333</v>
+        <v>0.1418416666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3524716666666667</v>
+        <v>0.3501966666666667</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.003716666666666666</v>
+        <v>0.003883333333333333</v>
       </c>
     </row>
     <row r="21">
@@ -3261,22 +3269,22 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03651666666666667</v>
+        <v>0.03795</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>105</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1050666666666667</v>
+        <v>0.1084333333333334</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3194616666666665</v>
+        <v>0.3268449999999999</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.003383333333333333</v>
+        <v>0.003133333333333333</v>
       </c>
     </row>
     <row r="22">
@@ -3295,22 +3303,22 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03113333333333334</v>
+        <v>0.03288333333333333</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.08971666666666668</v>
+        <v>0.09381666666666667</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2468833333333333</v>
+        <v>0.2548083333333333</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02111666666666667</v>
+        <v>0.01955</v>
       </c>
     </row>
     <row r="23">
@@ -3329,22 +3337,22 @@
         <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.004666666666666666</v>
+        <v>0.003083333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>260</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01943333333333333</v>
+        <v>0.01323333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.07025833333333333</v>
+        <v>0.05323333333333333</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.03003333333333334</v>
+        <v>0.0353</v>
       </c>
     </row>
     <row r="24">
@@ -3363,7 +3371,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.001883333333333333</v>
+        <v>0.001983333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>108</v>
@@ -3372,10 +3380,10 @@
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03995</v>
+        <v>0.03935</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2241183333333333</v>
+        <v>0.2228016666666666</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.00035</v>
@@ -3397,7 +3405,7 @@
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.009316666666666668</v>
+        <v>0.008183333333333334</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>82</v>
@@ -3406,13 +3414,13 @@
         <v>238</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02715</v>
+        <v>0.02468333333333333</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1129083333333333</v>
+        <v>0.1082916666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02600833333333334</v>
+        <v>0.02795833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3431,7 +3439,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.004633333333333334</v>
+        <v>0.0046</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>90</v>
@@ -3440,13 +3448,13 @@
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02936666666666667</v>
+        <v>0.02966666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1309783333333334</v>
+        <v>0.1351616666666667</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.004016666666666667</v>
+        <v>0.002816666666666667</v>
       </c>
     </row>
     <row r="27">
@@ -3465,22 +3473,22 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.0033</v>
+        <v>0.0027</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>104</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02124166666666667</v>
+        <v>0.02019166666666667</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.19216</v>
+        <v>0.1867466666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.001416666666666667</v>
+        <v>0.001766666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3499,22 +3507,22 @@
         <v>9</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00245</v>
+        <v>0.00265</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G28" s="8" t="n">
         <v>248</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.02350833333333333</v>
+        <v>0.02610833333333333</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2111416666666667</v>
+        <v>0.2257166666666666</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.00535</v>
+        <v>0.0041</v>
       </c>
     </row>
     <row r="29">
@@ -3533,22 +3541,22 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01883333333333333</v>
+        <v>0.01933333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G29" s="9" t="n">
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.0635</v>
+        <v>0.0639</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2206833333333333</v>
+        <v>0.2234833333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0044</v>
+        <v>0.0039</v>
       </c>
     </row>
     <row r="30">
@@ -3567,7 +3575,7 @@
         <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.00585</v>
+        <v>0.0052</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>86</v>
@@ -3576,13 +3584,13 @@
         <v>266</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0244</v>
+        <v>0.02258333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.0973866666666667</v>
+        <v>0.09395333333333335</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03508333333333333</v>
+        <v>0.03318333333333334</v>
       </c>
     </row>
     <row r="31">
@@ -3601,22 +3609,22 @@
         <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.00665</v>
+        <v>0.00635</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G31" s="9" t="n">
         <v>204</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.02515</v>
+        <v>0.02498333333333333</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.1032216666666667</v>
+        <v>0.105175</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.018975</v>
+        <v>0.01839166666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3635,22 +3643,22 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00465</v>
+        <v>0.0049</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03385</v>
+        <v>0.03611666666666666</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2071833333333333</v>
+        <v>0.2189333333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0057</v>
+        <v>0.00535</v>
       </c>
     </row>
     <row r="33">
@@ -3669,22 +3677,22 @@
         <v>9</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.00415</v>
+        <v>0.00365</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02329166666666667</v>
+        <v>0.02259166666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.13175</v>
+        <v>0.12965</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="34">
@@ -3712,13 +3720,13 @@
         <v>255</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.01046666666666667</v>
+        <v>0.01116666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.1033766666666666</v>
+        <v>0.106685</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.01098333333333333</v>
+        <v>0.009899999999999999</v>
       </c>
     </row>
     <row r="35">
@@ -3737,22 +3745,22 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.0041</v>
+        <v>0.0042</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G35" s="9" t="n">
         <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03245000000000001</v>
+        <v>0.03291666666666667</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1736466666666666</v>
+        <v>0.1745333333333333</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.006666666666666667</v>
+        <v>0.006633333333333334</v>
       </c>
     </row>
     <row r="36">
@@ -3780,13 +3788,13 @@
         <v>203</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.001833333333333334</v>
+        <v>0.001733333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.0468</v>
+        <v>0.04368333333333334</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.09468333333333334</v>
+        <v>0.1005833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3805,22 +3813,22 @@
         <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.0036</v>
+        <v>0.00445</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0223</v>
+        <v>0.0249</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1621233333333334</v>
+        <v>0.1759816666666667</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.005</v>
+        <v>0.0042</v>
       </c>
     </row>
     <row r="38">
@@ -3839,7 +3847,7 @@
         <v>7</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.002183333333333333</v>
+        <v>0.002133333333333333</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>73</v>
@@ -3848,13 +3856,13 @@
         <v>257</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01568333333333333</v>
+        <v>0.01543333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06478333333333333</v>
+        <v>0.06471666666666667</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.06983333333333333</v>
+        <v>0.07085</v>
       </c>
     </row>
     <row r="39">
@@ -3873,7 +3881,7 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0016</v>
+        <v>0.0015</v>
       </c>
       <c r="F39" s="9" t="n">
         <v>69</v>
@@ -3882,13 +3890,13 @@
         <v>248</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.008750000000000001</v>
+        <v>0.008883333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04800333333333334</v>
+        <v>0.04853666666666667</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1308833333333333</v>
+        <v>0.1264</v>
       </c>
     </row>
     <row r="40">
@@ -3907,22 +3915,22 @@
         <v>8</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.00025</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.00245</v>
+        <v>0.003083333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.03818666666666666</v>
+        <v>0.04126999999999999</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.04436666666666667</v>
+        <v>0.03738333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -3941,22 +3949,22 @@
         <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.002066666666666666</v>
+        <v>0.002266666666666666</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>229</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01136666666666667</v>
+        <v>0.01278333333333333</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.06740000000000003</v>
+        <v>0.07140000000000002</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.025625</v>
+        <v>0.022725</v>
       </c>
     </row>
     <row r="42">
@@ -3978,19 +3986,19 @@
         <v>0.00125</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.004433333333333333</v>
+        <v>0.0042</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.019775</v>
+        <v>0.019175</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.289225</v>
+        <v>0.288675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 15:30:45 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T19:28:36.728989+00:00</t>
+          <t>2026-03-21T19:30:44.947593+00:00</t>
         </is>
       </c>
     </row>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.85556916598514</v>
+        <v>0.8557138399715283</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.14443083401486</v>
+        <v>0.1442861600284717</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2072,10 +2072,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.2408024924172188</v>
+        <v>0.2265821050262228</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.7591975075827812</v>
+        <v>0.7734178949737772</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1329</v>
+        <v>0.1346</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>136</v>
@@ -2632,10 +2632,10 @@
         <v>344</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3380666666666667</v>
+        <v>0.3399</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7079033333333333</v>
+        <v>0.7106616666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,7 +2657,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06</v>
+        <v>0.0603</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>117</v>
@@ -2666,13 +2666,13 @@
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1667833333333333</v>
+        <v>0.1678333333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4034666666666666</v>
+        <v>0.4050166666666666</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.004766666666666667</v>
+        <v>0.004666666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.14145</v>
+        <v>0.1417</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>137</v>
@@ -2700,10 +2700,10 @@
         <v>283</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3258833333333334</v>
+        <v>0.3260833333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.7068433333333334</v>
+        <v>0.7067933333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2725,7 +2725,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07756666666666667</v>
+        <v>0.07771666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
@@ -2734,10 +2734,10 @@
         <v>313</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.19805</v>
+        <v>0.1983166666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4727083333333333</v>
+        <v>0.4720583333333333</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0003</v>
@@ -2759,19 +2759,19 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06473333333333334</v>
+        <v>0.06498333333333334</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1585083333333333</v>
+        <v>0.1591416666666667</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3799933333333332</v>
+        <v>0.3821849999999999</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0.001016666666666667</v>
@@ -2793,7 +2793,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.03275</v>
+        <v>0.0307</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>118</v>
@@ -2802,10 +2802,10 @@
         <v>313</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.09866666666666668</v>
+        <v>0.09301666666666668</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3847133333333334</v>
+        <v>0.3756633333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0011</v>
@@ -2827,7 +2827,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.046</v>
+        <v>0.0461</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>108</v>
@@ -2836,10 +2836,10 @@
         <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1299833333333333</v>
+        <v>0.1300333333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.320225</v>
+        <v>0.319825</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0.00385</v>
@@ -2861,7 +2861,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02505</v>
+        <v>0.02495</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>119</v>
@@ -2870,10 +2870,10 @@
         <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1036833333333333</v>
+        <v>0.10365</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4407999999999999</v>
+        <v>0.4400499999999999</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -2904,10 +2904,10 @@
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.08670833333333333</v>
+        <v>0.08629166666666667</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.3925833333333333</v>
+        <v>0.3918666666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.001</v>
@@ -2929,19 +2929,19 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0177</v>
+        <v>0.0179</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.09145833333333332</v>
+        <v>0.09195833333333332</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4500133333333332</v>
+        <v>0.4539716666666666</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.0005833333333333334</v>
@@ -2963,7 +2963,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.06048333333333333</v>
+        <v>0.06133333333333332</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>122</v>
@@ -2972,10 +2972,10 @@
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1659416666666667</v>
+        <v>0.168375</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4704433333333333</v>
+        <v>0.4720683333333333</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -2997,22 +2997,22 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05403333333333333</v>
+        <v>0.05423333333333333</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1441166666666667</v>
+        <v>0.1445</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.345425</v>
+        <v>0.3461750000000001</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0017</v>
+        <v>0.0016</v>
       </c>
     </row>
     <row r="14">
@@ -3031,7 +3031,7 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.0135</v>
+        <v>0.0133</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>111</v>
@@ -3040,10 +3040,10 @@
         <v>298</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.05525</v>
+        <v>0.055</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3036099999999999</v>
+        <v>0.3030599999999999</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3065,22 +3065,22 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02355</v>
+        <v>0.0225</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.07110000000000001</v>
+        <v>0.0689</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2109916666666667</v>
+        <v>0.2069583333333333</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.0322</v>
+        <v>0.03295</v>
       </c>
     </row>
     <row r="16">
@@ -3108,13 +3108,13 @@
         <v>320</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0196</v>
+        <v>0.01965</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2771433333333333</v>
+        <v>0.2765766666666665</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.002</v>
+        <v>0.0021</v>
       </c>
     </row>
     <row r="17">
@@ -3142,13 +3142,13 @@
         <v>258</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.01666666666666667</v>
+        <v>0.01676666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.06560000000000001</v>
+        <v>0.06631666666666668</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.03293333333333333</v>
+        <v>0.03208333333333333</v>
       </c>
     </row>
     <row r="18">
@@ -3167,7 +3167,7 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.0054</v>
+        <v>0.0051</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>68</v>
@@ -3176,13 +3176,13 @@
         <v>207</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02188333333333333</v>
+        <v>0.02098333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07574166666666667</v>
+        <v>0.07309166666666667</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.09006666666666666</v>
+        <v>0.09116666666666666</v>
       </c>
     </row>
     <row r="19">
@@ -3210,10 +3210,10 @@
         <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02505</v>
+        <v>0.02503333333333333</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2108166666666667</v>
+        <v>0.2101</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.00055</v>
@@ -3235,7 +3235,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.06206666666666667</v>
+        <v>0.06201666666666666</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3244,10 +3244,10 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.1418416666666667</v>
+        <v>0.142075</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3501966666666667</v>
+        <v>0.3496633333333334</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.003883333333333333</v>
@@ -3269,19 +3269,19 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03795</v>
+        <v>0.03815</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G21" s="9" t="n">
         <v>260</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1084333333333334</v>
+        <v>0.1093333333333334</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3268449999999999</v>
+        <v>0.3281949999999999</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.003133333333333333</v>
@@ -3303,7 +3303,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03288333333333333</v>
+        <v>0.03258333333333334</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>94</v>
@@ -3315,10 +3315,10 @@
         <v>0.09381666666666667</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2548083333333333</v>
+        <v>0.2547583333333333</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.01955</v>
+        <v>0.01965</v>
       </c>
     </row>
     <row r="23">
@@ -3349,10 +3349,10 @@
         <v>0.01323333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.05323333333333333</v>
+        <v>0.05300833333333334</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0353</v>
+        <v>0.0356</v>
       </c>
     </row>
     <row r="24">
@@ -3380,10 +3380,10 @@
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03935</v>
+        <v>0.03991666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2228016666666666</v>
+        <v>0.2254266666666666</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.00035</v>
@@ -3405,7 +3405,7 @@
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.008183333333333334</v>
+        <v>0.008233333333333334</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>82</v>
@@ -3414,13 +3414,13 @@
         <v>238</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02468333333333333</v>
+        <v>0.02481666666666667</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1082916666666667</v>
+        <v>0.1092916666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02795833333333334</v>
+        <v>0.02735833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3451,7 +3451,7 @@
         <v>0.02966666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1351616666666667</v>
+        <v>0.1349116666666667</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.002816666666666667</v>
@@ -3482,13 +3482,13 @@
         <v>272</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02019166666666667</v>
+        <v>0.02075833333333334</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1867466666666667</v>
+        <v>0.189205</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.001766666666666667</v>
+        <v>0.001666666666666666</v>
       </c>
     </row>
     <row r="28">
@@ -3516,10 +3516,10 @@
         <v>248</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.02610833333333333</v>
+        <v>0.026625</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2257166666666666</v>
+        <v>0.2281166666666666</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0.0041</v>
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01933333333333333</v>
+        <v>0.01923333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>103</v>
@@ -3550,13 +3550,13 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.0639</v>
+        <v>0.06351666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2234833333333333</v>
+        <v>0.2233083333333334</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0039</v>
+        <v>0.0038</v>
       </c>
     </row>
     <row r="30">
@@ -3575,7 +3575,7 @@
         <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0052</v>
+        <v>0.0048</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>86</v>
@@ -3584,13 +3584,13 @@
         <v>266</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.02258333333333333</v>
+        <v>0.0208</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.09395333333333335</v>
+        <v>0.08897000000000002</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03318333333333334</v>
+        <v>0.03378333333333334</v>
       </c>
     </row>
     <row r="31">
@@ -3609,7 +3609,7 @@
         <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.00635</v>
+        <v>0.00645</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>88</v>
@@ -3618,13 +3618,13 @@
         <v>204</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.02498333333333333</v>
+        <v>0.02538333333333333</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.105175</v>
+        <v>0.106025</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01839166666666667</v>
+        <v>0.01829166666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3652,7 +3652,7 @@
         <v>227</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03611666666666666</v>
+        <v>0.03583333333333333</v>
       </c>
       <c r="I32" s="5" t="n">
         <v>0.2189333333333333</v>
@@ -3677,7 +3677,7 @@
         <v>9</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.00365</v>
+        <v>0.0037</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>88</v>
@@ -3686,10 +3686,10 @@
         <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02259166666666667</v>
+        <v>0.02269166666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.12965</v>
+        <v>0.1290333333333334</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.0002</v>
@@ -3723,10 +3723,10 @@
         <v>0.01116666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.106685</v>
+        <v>0.1061016666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.009899999999999999</v>
+        <v>0.009999999999999998</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.0042</v>
+        <v>0.00425</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>92</v>
@@ -3754,13 +3754,13 @@
         <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03291666666666667</v>
+        <v>0.03341666666666667</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1745333333333333</v>
+        <v>0.1757666666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.006633333333333334</v>
+        <v>0.006283333333333333</v>
       </c>
     </row>
     <row r="36">
@@ -3791,10 +3791,10 @@
         <v>0.001733333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04368333333333334</v>
+        <v>0.04358333333333334</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1005833333333333</v>
+        <v>0.1001333333333334</v>
       </c>
     </row>
     <row r="37">
@@ -3813,7 +3813,7 @@
         <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00445</v>
+        <v>0.00455</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>97</v>
@@ -3822,13 +3822,13 @@
         <v>211</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0249</v>
+        <v>0.0254</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1759816666666667</v>
+        <v>0.1780483333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0042</v>
+        <v>0.00395</v>
       </c>
     </row>
     <row r="38">
@@ -3859,7 +3859,7 @@
         <v>0.01543333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06471666666666667</v>
+        <v>0.06456666666666667</v>
       </c>
       <c r="J38" s="5" t="n">
         <v>0.07085</v>
@@ -3896,7 +3896,7 @@
         <v>0.04853666666666667</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1264</v>
+        <v>0.12615</v>
       </c>
     </row>
     <row r="40">
@@ -3927,10 +3927,10 @@
         <v>0.003083333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.04126999999999999</v>
+        <v>0.04163666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.03738333333333333</v>
+        <v>0.03713333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -3961,10 +3961,10 @@
         <v>0.01278333333333333</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07140000000000002</v>
+        <v>0.07130000000000002</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.022725</v>
+        <v>0.022875</v>
       </c>
     </row>
     <row r="42">
@@ -3998,7 +3998,7 @@
         <v>0.019175</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.288675</v>
+        <v>0.288975</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 15:40:03 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T19:30:44.947593+00:00</t>
+          <t>2026-03-21T19:40:02.857817+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8557138399715283</v>
+        <v>0.8531809731462121</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1442861600284717</v>
+        <v>0.1468190268537879</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr"/>
@@ -2072,10 +2072,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.2265821050262228</v>
+        <v>0.2450111072564408</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.7734178949737772</v>
+        <v>0.7549888927435592</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1733993715190214</v>
+        <v>0.1728534619584367</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8266006284809787</v>
+        <v>0.8271465380415634</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1346</v>
+        <v>0.1323</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>136</v>
@@ -2632,10 +2632,10 @@
         <v>344</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3399</v>
+        <v>0.3371166666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7106616666666666</v>
+        <v>0.7075033333333333</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,22 +2657,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.0603</v>
+        <v>0.06005</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1678333333333333</v>
+        <v>0.1660833333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4050166666666666</v>
+        <v>0.4028833333333333</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.004666666666666667</v>
+        <v>0.004866666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.1417</v>
+        <v>0.14075</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>137</v>
@@ -2700,10 +2700,10 @@
         <v>283</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3260833333333334</v>
+        <v>0.3256833333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.7067933333333334</v>
+        <v>0.7065100000000001</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2725,7 +2725,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07771666666666667</v>
+        <v>0.07781666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
@@ -2734,10 +2734,10 @@
         <v>313</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1983166666666667</v>
+        <v>0.1979</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4720583333333333</v>
+        <v>0.4727583333333333</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0003</v>
@@ -2759,19 +2759,19 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06498333333333334</v>
+        <v>0.06463333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1591416666666667</v>
+        <v>0.1581083333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3821849999999999</v>
+        <v>0.3795433333333332</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0.001016666666666667</v>
@@ -2793,19 +2793,19 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0307</v>
+        <v>0.03345</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>313</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.09301666666666668</v>
+        <v>0.1000666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3756633333333333</v>
+        <v>0.3869466666666667</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0011</v>
@@ -2836,10 +2836,10 @@
         <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1300333333333334</v>
+        <v>0.1300833333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.319825</v>
+        <v>0.3204083333333334</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0.00385</v>
@@ -2861,7 +2861,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02495</v>
+        <v>0.02525</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>119</v>
@@ -2870,10 +2870,10 @@
         <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.10365</v>
+        <v>0.1041833333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4400499999999999</v>
+        <v>0.4411999999999999</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -2895,7 +2895,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.01953333333333333</v>
+        <v>0.01963333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>117</v>
@@ -2904,10 +2904,10 @@
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.08629166666666667</v>
+        <v>0.08710833333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.3918666666666666</v>
+        <v>0.3931166666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.001</v>
@@ -2929,19 +2929,19 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0179</v>
+        <v>0.0177</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.09195833333333332</v>
+        <v>0.09075833333333333</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4539716666666666</v>
+        <v>0.4484966666666665</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.0005833333333333334</v>
@@ -2963,7 +2963,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.06133333333333332</v>
+        <v>0.06018333333333332</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>122</v>
@@ -2972,10 +2972,10 @@
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.168375</v>
+        <v>0.1652416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4720683333333333</v>
+        <v>0.4699599999999999</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -2997,22 +2997,22 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05423333333333333</v>
+        <v>0.05383333333333332</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1445</v>
+        <v>0.1441666666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3461750000000001</v>
+        <v>0.3449883333333333</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0016</v>
+        <v>0.0017</v>
       </c>
     </row>
     <row r="14">
@@ -3031,7 +3031,7 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.0133</v>
+        <v>0.01355</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>111</v>
@@ -3040,10 +3040,10 @@
         <v>298</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.055</v>
+        <v>0.05545</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3030599999999999</v>
+        <v>0.3036099999999999</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3065,22 +3065,22 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.0225</v>
+        <v>0.02395</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.0689</v>
+        <v>0.07195000000000001</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2069583333333333</v>
+        <v>0.2123916666666666</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.03295</v>
+        <v>0.0322</v>
       </c>
     </row>
     <row r="16">
@@ -3108,13 +3108,13 @@
         <v>320</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.01965</v>
+        <v>0.0195</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2765766666666665</v>
+        <v>0.2774266666666666</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.0021</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="17">
@@ -3145,10 +3145,10 @@
         <v>0.01676666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.06631666666666668</v>
+        <v>0.06591666666666668</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.03208333333333333</v>
+        <v>0.0332</v>
       </c>
     </row>
     <row r="18">
@@ -3167,7 +3167,7 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.0051</v>
+        <v>0.00555</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>68</v>
@@ -3176,13 +3176,13 @@
         <v>207</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02098333333333333</v>
+        <v>0.02228333333333334</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07309166666666667</v>
+        <v>0.07630500000000001</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.09116666666666666</v>
+        <v>0.08901666666666666</v>
       </c>
     </row>
     <row r="19">
@@ -3210,10 +3210,10 @@
         <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02503333333333333</v>
+        <v>0.0251</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2101</v>
+        <v>0.2113666666666666</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.00055</v>
@@ -3235,7 +3235,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.06201666666666666</v>
+        <v>0.06196666666666666</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3244,10 +3244,10 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.142075</v>
+        <v>0.1417416666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3496633333333334</v>
+        <v>0.3497466666666667</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.003883333333333333</v>
@@ -3269,19 +3269,19 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03815</v>
+        <v>0.03795</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G21" s="9" t="n">
         <v>260</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1093333333333334</v>
+        <v>0.1079833333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3281949999999999</v>
+        <v>0.3262283333333332</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.003133333333333333</v>
@@ -3303,7 +3303,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03258333333333334</v>
+        <v>0.03278333333333334</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>94</v>
@@ -3315,10 +3315,10 @@
         <v>0.09381666666666667</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2547583333333333</v>
+        <v>0.2545583333333333</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.01965</v>
+        <v>0.0197</v>
       </c>
     </row>
     <row r="23">
@@ -3349,10 +3349,10 @@
         <v>0.01323333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.05300833333333334</v>
+        <v>0.05323333333333333</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0356</v>
+        <v>0.03516666666666667</v>
       </c>
     </row>
     <row r="24">
@@ -3380,10 +3380,10 @@
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03991666666666667</v>
+        <v>0.03935</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2254266666666666</v>
+        <v>0.2222516666666667</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.00035</v>
@@ -3405,7 +3405,7 @@
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.008233333333333334</v>
+        <v>0.008083333333333335</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>82</v>
@@ -3414,13 +3414,13 @@
         <v>238</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02481666666666667</v>
+        <v>0.02448333333333333</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1092916666666667</v>
+        <v>0.1082583333333333</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02735833333333334</v>
+        <v>0.02785833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3448,10 +3448,10 @@
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02966666666666667</v>
+        <v>0.02976666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1349116666666667</v>
+        <v>0.1351616666666667</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.002816666666666667</v>
@@ -3463,32 +3463,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
         <v>26</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.0027</v>
+        <v>0.00275</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>272</v>
+        <v>248</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02075833333333334</v>
+        <v>0.02610833333333333</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.189205</v>
+        <v>0.2254166666666666</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.001666666666666666</v>
+        <v>0.0042</v>
       </c>
     </row>
     <row r="28">
@@ -3497,32 +3497,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
         <v>26</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00265</v>
+        <v>0.0027</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>248</v>
+        <v>272</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.026625</v>
+        <v>0.02004166666666667</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2281166666666666</v>
+        <v>0.18626</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.0041</v>
+        <v>0.001766666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01923333333333333</v>
+        <v>0.01943333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>103</v>
@@ -3550,13 +3550,13 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.06351666666666667</v>
+        <v>0.0639</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2233083333333334</v>
+        <v>0.22395</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0038</v>
+        <v>0.0039</v>
       </c>
     </row>
     <row r="30">
@@ -3575,7 +3575,7 @@
         <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0048</v>
+        <v>0.0054</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>86</v>
@@ -3584,13 +3584,13 @@
         <v>266</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0208</v>
+        <v>0.02348333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.08897000000000002</v>
+        <v>0.09535333333333336</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03378333333333334</v>
+        <v>0.03308333333333334</v>
       </c>
     </row>
     <row r="31">
@@ -3609,7 +3609,7 @@
         <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.00645</v>
+        <v>0.00635</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>88</v>
@@ -3618,13 +3618,13 @@
         <v>204</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.02538333333333333</v>
+        <v>0.02493333333333334</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.106025</v>
+        <v>0.104905</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01829166666666667</v>
+        <v>0.01864166666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3643,19 +3643,19 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0049</v>
+        <v>0.0048</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>99</v>
+        <v>98.5</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>227</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03583333333333333</v>
+        <v>0.03621666666666666</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2189333333333333</v>
+        <v>0.21875</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.00535</v>
@@ -3677,7 +3677,7 @@
         <v>9</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.0037</v>
+        <v>0.00365</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>88</v>
@@ -3686,10 +3686,10 @@
         <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02269166666666667</v>
+        <v>0.02259166666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1290333333333334</v>
+        <v>0.1296</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.0002</v>
@@ -3720,13 +3720,13 @@
         <v>255</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.01116666666666667</v>
+        <v>0.01126666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.1061016666666667</v>
+        <v>0.106835</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.009816666666666666</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00425</v>
+        <v>0.0041</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>92</v>
@@ -3754,13 +3754,13 @@
         <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03341666666666667</v>
+        <v>0.03261666666666667</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1757666666666667</v>
+        <v>0.1739133333333333</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.006283333333333333</v>
+        <v>0.006633333333333334</v>
       </c>
     </row>
     <row r="36">
@@ -3791,10 +3791,10 @@
         <v>0.001733333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04358333333333334</v>
+        <v>0.04388333333333334</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1001333333333334</v>
+        <v>0.1005333333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3813,7 +3813,7 @@
         <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00455</v>
+        <v>0.00445</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>97</v>
@@ -3822,13 +3822,13 @@
         <v>211</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0254</v>
+        <v>0.0249</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1780483333333334</v>
+        <v>0.175265</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.00395</v>
+        <v>0.0044</v>
       </c>
     </row>
     <row r="38">
@@ -3856,13 +3856,13 @@
         <v>257</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01543333333333333</v>
+        <v>0.01533333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06456666666666667</v>
+        <v>0.06451666666666668</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.07085</v>
+        <v>0.0711</v>
       </c>
     </row>
     <row r="39">
@@ -3893,10 +3893,10 @@
         <v>0.008883333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04853666666666667</v>
+        <v>0.04863666666666668</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.12615</v>
+        <v>0.1261</v>
       </c>
     </row>
     <row r="40">
@@ -3927,10 +3927,10 @@
         <v>0.003083333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.04163666666666666</v>
+        <v>0.04121999999999999</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.03713333333333333</v>
+        <v>0.03783333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -3961,10 +3961,10 @@
         <v>0.01278333333333333</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07130000000000002</v>
+        <v>0.07160000000000002</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.022875</v>
+        <v>0.022725</v>
       </c>
     </row>
     <row r="42">
@@ -3995,10 +3995,10 @@
         <v>0.0042</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.019175</v>
+        <v>0.019125</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.288975</v>
+        <v>0.288725</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 16:00:09 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T19:40:02.857817+00:00</t>
+          <t>2026-03-21T20:00:08.526475+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8531809731462121</v>
+        <v>0.85466308992513</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1468190268537879</v>
+        <v>0.1453369100748701</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr"/>
@@ -2072,10 +2072,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.2450111072564408</v>
+        <v>0.1861362014239617</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.7549888927435592</v>
+        <v>0.8138637985760383</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1728534619584367</v>
+        <v>0.1726014237362924</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8271465380415634</v>
+        <v>0.8273985762637076</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1979686364434314</v>
+        <v>0.1984632718704647</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8020313635565686</v>
+        <v>0.8015367281295354</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2484,10 +2484,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3085367443007756</v>
+        <v>0.3093241579482524</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6914632556992244</v>
+        <v>0.6906758420517476</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1323</v>
+        <v>0.13725</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>136</v>
@@ -2632,10 +2632,10 @@
         <v>344</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3371166666666667</v>
+        <v>0.3452000000000001</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7075033333333333</v>
+        <v>0.7165283333333333</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,22 +2657,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06005</v>
+        <v>0.06135</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1660833333333333</v>
+        <v>0.1701333333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4028833333333333</v>
+        <v>0.41025</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.004866666666666667</v>
+        <v>0.004516666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.14075</v>
+        <v>0.1419</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>137</v>
@@ -2700,10 +2700,10 @@
         <v>283</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3256833333333334</v>
+        <v>0.3256083333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.7065100000000001</v>
+        <v>0.7054266666666668</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2725,7 +2725,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07781666666666667</v>
+        <v>0.07791666666666668</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
@@ -2734,10 +2734,10 @@
         <v>313</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1979</v>
+        <v>0.1983666666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4727583333333333</v>
+        <v>0.4692083333333333</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0003</v>
@@ -2759,19 +2759,19 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06463333333333333</v>
+        <v>0.06593333333333334</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1581083333333333</v>
+        <v>0.1613166666666667</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3795433333333332</v>
+        <v>0.3864433333333333</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0.001016666666666667</v>
@@ -2793,22 +2793,22 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.03345</v>
+        <v>0.02575</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>313</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1000666666666667</v>
+        <v>0.08266666666666668</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3869466666666667</v>
+        <v>0.3583133333333334</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.0011</v>
+        <v>0.0012</v>
       </c>
     </row>
     <row r="8">
@@ -2827,7 +2827,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0461</v>
+        <v>0.0458</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>108</v>
@@ -2836,13 +2836,13 @@
         <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1300833333333334</v>
+        <v>0.1292833333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3204083333333334</v>
+        <v>0.319975</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.00385</v>
+        <v>0.0039</v>
       </c>
     </row>
     <row r="9">
@@ -2861,7 +2861,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02525</v>
+        <v>0.02515</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>119</v>
@@ -2870,10 +2870,10 @@
         <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1041833333333333</v>
+        <v>0.10355</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4411999999999999</v>
+        <v>0.4374533333333333</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -2895,7 +2895,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.01963333333333333</v>
+        <v>0.01933333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>117</v>
@@ -2904,10 +2904,10 @@
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.08710833333333334</v>
+        <v>0.08590833333333332</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.3931166666666666</v>
+        <v>0.3901283333333333</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.001</v>
@@ -2929,22 +2929,22 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0177</v>
+        <v>0.0184</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.09075833333333333</v>
+        <v>0.09460833333333332</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4484966666666665</v>
+        <v>0.4597833333333331</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.0005833333333333334</v>
+        <v>0.0003833333333333333</v>
       </c>
     </row>
     <row r="12">
@@ -2963,19 +2963,19 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.06018333333333332</v>
+        <v>0.06231666666666667</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1652416666666667</v>
+        <v>0.1713916666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4699599999999999</v>
+        <v>0.4788516666666666</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -2997,22 +2997,22 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05383333333333332</v>
+        <v>0.05538333333333333</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1441666666666667</v>
+        <v>0.1476666666666666</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3449883333333333</v>
+        <v>0.3486883333333334</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0017</v>
+        <v>0.0015</v>
       </c>
     </row>
     <row r="14">
@@ -3031,7 +3031,7 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01355</v>
+        <v>0.01305</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>111</v>
@@ -3040,10 +3040,10 @@
         <v>298</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.05545</v>
+        <v>0.05468333333333333</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3036099999999999</v>
+        <v>0.3022266666666666</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3065,22 +3065,22 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02395</v>
+        <v>0.02055</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.07195000000000001</v>
+        <v>0.06386666666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2123916666666666</v>
+        <v>0.1977416666666667</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.0322</v>
+        <v>0.03415</v>
       </c>
     </row>
     <row r="16">
@@ -3108,13 +3108,13 @@
         <v>320</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0195</v>
+        <v>0.01994166666666667</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2774266666666666</v>
+        <v>0.2752683333333332</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.002</v>
+        <v>0.00225</v>
       </c>
     </row>
     <row r="17">
@@ -3133,7 +3133,7 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.007533333333333333</v>
+        <v>0.007633333333333333</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>80</v>
@@ -3142,13 +3142,13 @@
         <v>258</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.01676666666666667</v>
+        <v>0.01706666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.06591666666666668</v>
+        <v>0.06831666666666668</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.0332</v>
+        <v>0.0301</v>
       </c>
     </row>
     <row r="18">
@@ -3167,22 +3167,22 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.00555</v>
+        <v>0.0042</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>207</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02228333333333334</v>
+        <v>0.01773333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07630500000000001</v>
+        <v>0.06563833333333333</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.08901666666666666</v>
+        <v>0.09566666666666668</v>
       </c>
     </row>
     <row r="19">
@@ -3210,10 +3210,10 @@
         <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.0251</v>
+        <v>0.0248</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2113666666666666</v>
+        <v>0.20855</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.00055</v>
@@ -3235,7 +3235,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.06196666666666666</v>
+        <v>0.06191666666666666</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3244,13 +3244,13 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.1417416666666667</v>
+        <v>0.1415</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3497466666666667</v>
+        <v>0.3488250000000001</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.003883333333333333</v>
+        <v>0.0039</v>
       </c>
     </row>
     <row r="21">
@@ -3269,22 +3269,22 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03795</v>
+        <v>0.03938333333333333</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G21" s="9" t="n">
         <v>260</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1079833333333333</v>
+        <v>0.1117833333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3262283333333332</v>
+        <v>0.3314949999999999</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.003133333333333333</v>
+        <v>0.0031</v>
       </c>
     </row>
     <row r="22">
@@ -3303,7 +3303,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03278333333333334</v>
+        <v>0.03243333333333333</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>94</v>
@@ -3312,13 +3312,13 @@
         <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.09381666666666667</v>
+        <v>0.09338333333333333</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2545583333333333</v>
+        <v>0.254475</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.0197</v>
+        <v>0.0196</v>
       </c>
     </row>
     <row r="23">
@@ -3349,10 +3349,10 @@
         <v>0.01323333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.05323333333333333</v>
+        <v>0.05285833333333334</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.03516666666666667</v>
+        <v>0.03635</v>
       </c>
     </row>
     <row r="24">
@@ -3374,19 +3374,19 @@
         <v>0.001983333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03935</v>
+        <v>0.04111666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2222516666666667</v>
+        <v>0.230185</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.00035</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="25">
@@ -3405,22 +3405,22 @@
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.008083333333333335</v>
+        <v>0.008533333333333334</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G25" s="9" t="n">
         <v>238</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02448333333333333</v>
+        <v>0.02511666666666667</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1082583333333333</v>
+        <v>0.1121083333333334</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02785833333333334</v>
+        <v>0.02570833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3439,7 +3439,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.0046</v>
+        <v>0.0045</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>90</v>
@@ -3448,10 +3448,10 @@
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02976666666666667</v>
+        <v>0.02971666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1351616666666667</v>
+        <v>0.1348200000000001</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.002816666666666667</v>
@@ -3463,32 +3463,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
         <v>26</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.00275</v>
+        <v>0.0028</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>248</v>
+        <v>272</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02610833333333333</v>
+        <v>0.02125833333333334</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2254166666666666</v>
+        <v>0.1934016666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.0042</v>
+        <v>0.001366666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3497,32 +3497,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
         <v>26</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0027</v>
+        <v>0.00265</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>272</v>
+        <v>248</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.02004166666666667</v>
+        <v>0.027275</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.18626</v>
+        <v>0.233025</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.001766666666666667</v>
+        <v>0.00395</v>
       </c>
     </row>
     <row r="29">
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01943333333333333</v>
+        <v>0.01938333333333334</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>103</v>
@@ -3550,10 +3550,10 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.0639</v>
+        <v>0.06298333333333334</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.22395</v>
+        <v>0.2222083333333333</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.0039</v>
@@ -3575,22 +3575,22 @@
         <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0054</v>
+        <v>0.0038</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.02348333333333333</v>
+        <v>0.01755</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.09535333333333336</v>
+        <v>0.07877000000000002</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03308333333333334</v>
+        <v>0.03543333333333334</v>
       </c>
     </row>
     <row r="31">
@@ -3609,7 +3609,7 @@
         <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.00635</v>
+        <v>0.006583333333333333</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>88</v>
@@ -3618,13 +3618,13 @@
         <v>204</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.02493333333333334</v>
+        <v>0.02603333333333334</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.104905</v>
+        <v>0.107555</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01864166666666667</v>
+        <v>0.01735833333333333</v>
       </c>
     </row>
     <row r="32">
@@ -3643,22 +3643,22 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0048</v>
+        <v>0.0051</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>98.5</v>
+        <v>99</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>227</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03621666666666666</v>
+        <v>0.03576666666666667</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.21875</v>
+        <v>0.2174916666666666</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00535</v>
+        <v>0.00545</v>
       </c>
     </row>
     <row r="33">
@@ -3677,7 +3677,7 @@
         <v>9</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.00365</v>
+        <v>0.0037</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>88</v>
@@ -3686,10 +3686,10 @@
         <v>237</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02259166666666667</v>
+        <v>0.02250833333333333</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1296</v>
+        <v>0.1282333333333333</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.0002</v>
@@ -3711,7 +3711,7 @@
         <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.002033333333333333</v>
+        <v>0.001833333333333333</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>94</v>
@@ -3720,13 +3720,13 @@
         <v>255</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.01126666666666667</v>
+        <v>0.01115</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.106835</v>
+        <v>0.10528</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.009816666666666666</v>
+        <v>0.0101</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.0041</v>
+        <v>0.00425</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>92</v>
@@ -3754,13 +3754,13 @@
         <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03261666666666667</v>
+        <v>0.03425</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1739133333333333</v>
+        <v>0.1789633333333334</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.006633333333333334</v>
+        <v>0.005933333333333333</v>
       </c>
     </row>
     <row r="36">
@@ -3791,10 +3791,10 @@
         <v>0.001733333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04388333333333334</v>
+        <v>0.04353333333333334</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1005333333333333</v>
+        <v>0.09998333333333335</v>
       </c>
     </row>
     <row r="37">
@@ -3813,22 +3813,22 @@
         <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00445</v>
+        <v>0.00475</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G37" s="9" t="n">
         <v>211</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0249</v>
+        <v>0.02595</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.175265</v>
+        <v>0.1820816666666667</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0044</v>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="38">
@@ -3856,13 +3856,13 @@
         <v>257</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01533333333333333</v>
+        <v>0.01523333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06451666666666668</v>
+        <v>0.0645</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.0711</v>
+        <v>0.07116666666666667</v>
       </c>
     </row>
     <row r="39">
@@ -3881,7 +3881,7 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0015</v>
+        <v>0.0014</v>
       </c>
       <c r="F39" s="9" t="n">
         <v>69</v>
@@ -3890,13 +3890,13 @@
         <v>248</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.008883333333333333</v>
+        <v>0.008783333333333332</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04863666666666668</v>
+        <v>0.04823666666666667</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1261</v>
+        <v>0.1256333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3915,7 +3915,7 @@
         <v>8</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00025</v>
+        <v>0.00015</v>
       </c>
       <c r="F40" s="8" t="n">
         <v>77</v>
@@ -3927,10 +3927,10 @@
         <v>0.003083333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.04121999999999999</v>
+        <v>0.04288666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.03783333333333333</v>
+        <v>0.03528333333333334</v>
       </c>
     </row>
     <row r="41">
@@ -3958,13 +3958,13 @@
         <v>229</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01278333333333333</v>
+        <v>0.01255</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07160000000000002</v>
+        <v>0.07100000000000002</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.022725</v>
+        <v>0.023025</v>
       </c>
     </row>
     <row r="42">
@@ -3992,13 +3992,13 @@
         <v>180</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.0042</v>
+        <v>0.00425</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.019125</v>
+        <v>0.019275</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.288725</v>
+        <v>0.2887583333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 16:52:30 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T20:00:08.526475+00:00</t>
+          <t>2026-03-21T20:52:30.357516+00:00</t>
         </is>
       </c>
     </row>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.85466308992513</v>
+        <v>0.8577645953874744</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1453369100748701</v>
+        <v>0.1422354046125257</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2072,10 +2072,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.1861362014239617</v>
+        <v>0.11495857050715</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.8138637985760383</v>
+        <v>0.88504142949285</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1726014237362924</v>
+        <v>0.1710175298381005</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8273985762637076</v>
+        <v>0.8289824701618994</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1984632718704647</v>
+        <v>0.1949513304092653</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8015367281295354</v>
+        <v>0.8050486695907347</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2484,10 +2484,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3093241579482524</v>
+        <v>0.3104515028255972</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6906758420517476</v>
+        <v>0.6895484971744028</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,19 +2623,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.13725</v>
+        <v>0.1429</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>344</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3452000000000001</v>
+        <v>0.3562250000000001</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7165283333333333</v>
+        <v>0.7255616666666665</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,22 +2657,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06135</v>
+        <v>0.06370000000000001</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1701333333333333</v>
+        <v>0.1753833333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.41025</v>
+        <v>0.4183833333333332</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.004516666666666667</v>
+        <v>0.0038</v>
       </c>
     </row>
     <row r="4">
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.1419</v>
+        <v>0.1429</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>137</v>
@@ -2700,10 +2700,10 @@
         <v>283</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3256083333333334</v>
+        <v>0.325875</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.7054266666666668</v>
+        <v>0.7031850000000002</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2725,7 +2725,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07791666666666668</v>
+        <v>0.07691666666666666</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
@@ -2734,13 +2734,13 @@
         <v>313</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1983666666666667</v>
+        <v>0.1978</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4692083333333333</v>
+        <v>0.4672749999999999</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0003</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="6">
@@ -2759,22 +2759,22 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06593333333333334</v>
+        <v>0.06965</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>303</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1613166666666667</v>
+        <v>0.1659666666666666</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3864433333333333</v>
+        <v>0.3947433333333333</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.001016666666666667</v>
+        <v>0.0009166666666666668</v>
       </c>
     </row>
     <row r="7">
@@ -2793,19 +2793,19 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.02575</v>
+        <v>0.01595</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>313</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.08266666666666668</v>
+        <v>0.05926666666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3583133333333334</v>
+        <v>0.3225966666666666</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0012</v>
@@ -2827,7 +2827,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0458</v>
+        <v>0.04465</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>108</v>
@@ -2836,10 +2836,10 @@
         <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1292833333333334</v>
+        <v>0.1279333333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.319975</v>
+        <v>0.319</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0.0039</v>
@@ -2861,7 +2861,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02515</v>
+        <v>0.0248</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>119</v>
@@ -2870,10 +2870,10 @@
         <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.10355</v>
+        <v>0.1033</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4374533333333333</v>
+        <v>0.4337533333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -2895,7 +2895,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.01933333333333333</v>
+        <v>0.01908333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>117</v>
@@ -2904,10 +2904,10 @@
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.08590833333333332</v>
+        <v>0.08455833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.3901283333333333</v>
+        <v>0.3882866666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.001</v>
@@ -2929,22 +2929,22 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0184</v>
+        <v>0.01945</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>345</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.09460833333333332</v>
+        <v>0.099375</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4597833333333331</v>
+        <v>0.4746833333333333</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.0003833333333333333</v>
+        <v>0.0002833333333333333</v>
       </c>
     </row>
     <row r="12">
@@ -2963,7 +2963,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.06231666666666667</v>
+        <v>0.0645</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>123</v>
@@ -2972,10 +2972,10 @@
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1713916666666667</v>
+        <v>0.1774583333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4788516666666666</v>
+        <v>0.4916183333333333</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0001</v>
@@ -2997,22 +2997,22 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05538333333333333</v>
+        <v>0.05721666666666667</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>275</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1476666666666666</v>
+        <v>0.1526</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3486883333333334</v>
+        <v>0.355175</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0015</v>
+        <v>0.0012</v>
       </c>
     </row>
     <row r="14">
@@ -3031,7 +3031,7 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01305</v>
+        <v>0.01275</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>111</v>
@@ -3040,10 +3040,10 @@
         <v>298</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.05468333333333333</v>
+        <v>0.05428333333333332</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3022266666666666</v>
+        <v>0.2977183333333333</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3065,22 +3065,22 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.02055</v>
+        <v>0.0177</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>275</v>
+        <v>257</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.06386666666666667</v>
+        <v>0.05611666666666666</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.1977416666666667</v>
+        <v>0.1793583333333333</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.03415</v>
+        <v>0.03773333333333333</v>
       </c>
     </row>
     <row r="16">
@@ -3108,13 +3108,13 @@
         <v>320</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.01994166666666667</v>
+        <v>0.019875</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2752683333333332</v>
+        <v>0.2719099999999999</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.00225</v>
+        <v>0.0023</v>
       </c>
     </row>
     <row r="17">
@@ -3133,7 +3133,7 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.007633333333333333</v>
+        <v>0.007883333333333332</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>80</v>
@@ -3142,13 +3142,13 @@
         <v>258</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.01706666666666667</v>
+        <v>0.01766666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.06831666666666668</v>
+        <v>0.07016666666666667</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.0301</v>
+        <v>0.02426666666666667</v>
       </c>
     </row>
     <row r="18">
@@ -3157,32 +3157,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
         <v>28</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>0.0042</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>67</v>
+        <v>107</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>207</v>
+        <v>269</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01773333333333333</v>
+        <v>0.02386666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.06563833333333333</v>
+        <v>0.20625</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.09566666666666668</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="19">
@@ -3191,32 +3191,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
         <v>28</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.0041</v>
+        <v>0.0034</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>269</v>
+        <v>207</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.0248</v>
+        <v>0.0129</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.20855</v>
+        <v>0.05200833333333334</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.1034666666666667</v>
       </c>
     </row>
     <row r="20">
@@ -3235,7 +3235,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.06191666666666666</v>
+        <v>0.06156666666666667</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3244,13 +3244,13 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.1415</v>
+        <v>0.1407</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3488250000000001</v>
+        <v>0.3476750000000001</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.0039</v>
+        <v>0.00405</v>
       </c>
     </row>
     <row r="21">
@@ -3269,22 +3269,22 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03938333333333333</v>
+        <v>0.03998333333333333</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1117833333333333</v>
+        <v>0.1158833333333334</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3314949999999999</v>
+        <v>0.3406783333333331</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.0031</v>
+        <v>0.0028</v>
       </c>
     </row>
     <row r="22">
@@ -3303,7 +3303,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03243333333333333</v>
+        <v>0.03258333333333334</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>94</v>
@@ -3312,10 +3312,10 @@
         <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.09338333333333333</v>
+        <v>0.09323333333333333</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.254475</v>
+        <v>0.253775</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0196</v>
@@ -3337,7 +3337,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.003083333333333333</v>
+        <v>0.002733333333333334</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>75</v>
@@ -3346,13 +3346,13 @@
         <v>260</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01323333333333333</v>
+        <v>0.01306666666666667</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.05285833333333334</v>
+        <v>0.051675</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.03635</v>
+        <v>0.03815</v>
       </c>
     </row>
     <row r="24">
@@ -3371,7 +3371,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.001983333333333333</v>
+        <v>0.00215</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>109</v>
@@ -3380,13 +3380,13 @@
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.04111666666666667</v>
+        <v>0.04278333333333334</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.230185</v>
+        <v>0.2398016666666666</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.00025</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="25">
@@ -3414,13 +3414,13 @@
         <v>238</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02511666666666667</v>
+        <v>0.02623333333333334</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1121083333333334</v>
+        <v>0.1154916666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02570833333333334</v>
+        <v>0.02350833333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3439,7 +3439,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.0045</v>
+        <v>0.0044</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>90</v>
@@ -3448,13 +3448,13 @@
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02971666666666667</v>
+        <v>0.02961666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1348200000000001</v>
+        <v>0.1338116666666667</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.002816666666666667</v>
+        <v>0.002983333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -3473,22 +3473,22 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.0028</v>
+        <v>0.00305</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G27" s="9" t="n">
         <v>272</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02125833333333334</v>
+        <v>0.02238333333333334</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1934016666666667</v>
+        <v>0.2016633333333333</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.001366666666666667</v>
+        <v>0.00085</v>
       </c>
     </row>
     <row r="28">
@@ -3507,22 +3507,22 @@
         <v>9</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00265</v>
+        <v>0.00295</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.027275</v>
+        <v>0.02850833333333333</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.233025</v>
+        <v>0.2417333333333333</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.00395</v>
+        <v>0.003316666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01938333333333334</v>
+        <v>0.01918333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>103</v>
@@ -3550,10 +3550,10 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.06298333333333334</v>
+        <v>0.06273333333333334</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2222083333333333</v>
+        <v>0.220075</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.0039</v>
@@ -3575,22 +3575,22 @@
         <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0038</v>
+        <v>0.0014</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>258</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.01755</v>
+        <v>0.0102</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.07877000000000002</v>
+        <v>0.05968666666666666</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03543333333333334</v>
+        <v>0.03876666666666666</v>
       </c>
     </row>
     <row r="31">
@@ -3609,22 +3609,22 @@
         <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.006583333333333333</v>
+        <v>0.006983333333333333</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G31" s="9" t="n">
         <v>204</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.02603333333333334</v>
+        <v>0.02738333333333334</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.107555</v>
+        <v>0.1110416666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01735833333333333</v>
+        <v>0.015475</v>
       </c>
     </row>
     <row r="32">
@@ -3643,22 +3643,22 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0051</v>
+        <v>0.005</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>99</v>
+        <v>98.5</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>227</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03576666666666667</v>
+        <v>0.03481666666666667</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2174916666666666</v>
+        <v>0.2159833333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00545</v>
+        <v>0.0055</v>
       </c>
     </row>
     <row r="33">
@@ -3677,19 +3677,19 @@
         <v>9</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.0037</v>
+        <v>0.0035</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>88</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02250833333333333</v>
+        <v>0.02230833333333333</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1282333333333333</v>
+        <v>0.1261083333333334</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.0002</v>
@@ -3711,7 +3711,7 @@
         <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.001833333333333333</v>
+        <v>0.001633333333333333</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>94</v>
@@ -3720,13 +3720,13 @@
         <v>255</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.01115</v>
+        <v>0.01071666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.10528</v>
+        <v>0.1037216666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.0101</v>
+        <v>0.01005</v>
       </c>
     </row>
     <row r="35">
@@ -3745,22 +3745,22 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00425</v>
+        <v>0.00445</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G35" s="9" t="n">
         <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03425</v>
+        <v>0.03642500000000001</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1789633333333334</v>
+        <v>0.1847333333333334</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.005933333333333333</v>
+        <v>0.005233333333333333</v>
       </c>
     </row>
     <row r="36">
@@ -3788,13 +3788,13 @@
         <v>203</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.001733333333333333</v>
+        <v>0.001833333333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04353333333333334</v>
+        <v>0.04301666666666667</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.09998333333333335</v>
+        <v>0.1006666666666667</v>
       </c>
     </row>
     <row r="37">
@@ -3813,7 +3813,7 @@
         <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00475</v>
+        <v>0.00505</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>98</v>
@@ -3822,13 +3822,13 @@
         <v>211</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.02595</v>
+        <v>0.027225</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1820816666666667</v>
+        <v>0.1905733333333333</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0035</v>
+        <v>0.00315</v>
       </c>
     </row>
     <row r="38">
@@ -3856,13 +3856,13 @@
         <v>257</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01523333333333333</v>
+        <v>0.01538333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.0645</v>
+        <v>0.06425833333333332</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.07116666666666667</v>
+        <v>0.07036666666666666</v>
       </c>
     </row>
     <row r="39">
@@ -3881,7 +3881,7 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0014</v>
+        <v>0.0013</v>
       </c>
       <c r="F39" s="9" t="n">
         <v>69</v>
@@ -3890,13 +3890,13 @@
         <v>248</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.008783333333333332</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04823666666666667</v>
+        <v>0.04797</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1256333333333333</v>
+        <v>0.1257</v>
       </c>
     </row>
     <row r="40">
@@ -3918,7 +3918,7 @@
         <v>0.00015</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G40" s="8" t="n">
         <v>213</v>
@@ -3927,10 +3927,10 @@
         <v>0.003083333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.04288666666666666</v>
+        <v>0.04523666666666667</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.03528333333333334</v>
+        <v>0.03133333333333334</v>
       </c>
     </row>
     <row r="41">
@@ -3958,13 +3958,13 @@
         <v>229</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01255</v>
+        <v>0.01265</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07100000000000002</v>
+        <v>0.07042500000000003</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.023025</v>
+        <v>0.02300833333333334</v>
       </c>
     </row>
     <row r="42">
@@ -3992,13 +3992,13 @@
         <v>180</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.00425</v>
+        <v>0.00405</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.019275</v>
+        <v>0.01919166666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2887583333333333</v>
+        <v>0.289675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 17:00:52 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T20:52:30.357516+00:00</t>
+          <t>2026-03-21T21:00:51.699011+00:00</t>
         </is>
       </c>
     </row>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8577645953874744</v>
+        <v>0.8556016283005042</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1422354046125257</v>
+        <v>0.1443983716994957</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2069,14 +2069,10 @@
       </c>
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G36" s="5" t="n">
-        <v>0.11495857050715</v>
-      </c>
-      <c r="H36" s="5" t="n">
-        <v>0.88504142949285</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G36" s="5" t="inlineStr"/>
+      <c r="H36" s="5" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
           <t>R32_E_03</t>
@@ -2344,10 +2340,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1710175298381005</v>
+        <v>0.1687507768376464</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8289824701618994</v>
+        <v>0.8312492231623536</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2381,10 +2377,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1949513304092653</v>
+        <v>0.1952393805638805</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8050486695907347</v>
+        <v>0.8047606194361195</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2484,10 +2480,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3104515028255972</v>
+        <v>0.311170986105787</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6895484971744028</v>
+        <v>0.688829013894213</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,19 +2619,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1429</v>
+        <v>0.1181</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>344</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3562250000000001</v>
+        <v>0.3082083333333334</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7255616666666665</v>
+        <v>0.6834033333333333</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,22 +2653,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06370000000000001</v>
+        <v>0.05418333333333334</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>306</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1753833333333333</v>
+        <v>0.1523333333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4183833333333332</v>
+        <v>0.3831583333333333</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.0038</v>
+        <v>0.006266666666666666</v>
       </c>
     </row>
     <row r="4">
@@ -2691,7 +2687,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.1429</v>
+        <v>0.1418833333333333</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>137</v>
@@ -2700,10 +2696,10 @@
         <v>283</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.325875</v>
+        <v>0.3287916666666668</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.7031850000000002</v>
+        <v>0.7133166666666669</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2725,7 +2721,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07691666666666666</v>
+        <v>0.07951666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>120</v>
@@ -2734,13 +2730,13 @@
         <v>313</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1978</v>
+        <v>0.2010583333333334</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4672749999999999</v>
+        <v>0.4796666666666666</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="6">
@@ -2749,32 +2745,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
         <v>34</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06965</v>
+        <v>0.06043333333333334</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1659666666666666</v>
+        <v>0.1628666666666666</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3947433333333333</v>
+        <v>0.4767050000000001</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.0009166666666666668</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="7">
@@ -2783,32 +2779,32 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
         <v>34</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.01595</v>
+        <v>0.05723333333333332</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.05926666666666666</v>
+        <v>0.1441583333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3225966666666666</v>
+        <v>0.3571183333333333</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.0012</v>
+        <v>0.001316666666666667</v>
       </c>
     </row>
     <row r="8">
@@ -2827,7 +2823,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.04465</v>
+        <v>0.04855</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>108</v>
@@ -2836,13 +2832,13 @@
         <v>321</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1279333333333333</v>
+        <v>0.1338166666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.319</v>
+        <v>0.3263833333333334</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.0039</v>
+        <v>0.00375</v>
       </c>
     </row>
     <row r="9">
@@ -2861,7 +2857,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.0248</v>
+        <v>0.02583333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>119</v>
@@ -2870,13 +2866,13 @@
         <v>315</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1033</v>
+        <v>0.1047416666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4337533333333334</v>
+        <v>0.4513</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.00045</v>
       </c>
     </row>
     <row r="10">
@@ -2895,7 +2891,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.01908333333333333</v>
+        <v>0.02028333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>117</v>
@@ -2904,10 +2900,10 @@
         <v>345</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.08455833333333333</v>
+        <v>0.08980833333333335</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.3882866666666666</v>
+        <v>0.4017416666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.001</v>
@@ -2929,22 +2925,22 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.01945</v>
+        <v>0.01465</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.099375</v>
+        <v>0.07897500000000002</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4746833333333333</v>
+        <v>0.4133716666666667</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.0002833333333333333</v>
+        <v>0.0005833333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -2963,22 +2959,22 @@
         <v>10</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.0645</v>
+        <v>0.05193333333333332</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>270</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1774583333333334</v>
+        <v>0.1470083333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4916183333333333</v>
+        <v>0.4353499999999999</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="13">
@@ -2997,22 +2993,22 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05721666666666667</v>
+        <v>0.04933333333333334</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1526</v>
+        <v>0.1327166666666666</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.355175</v>
+        <v>0.3255250000000001</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0012</v>
+        <v>0.0025</v>
       </c>
     </row>
     <row r="14">
@@ -3031,7 +3027,7 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01275</v>
+        <v>0.01303333333333333</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>111</v>
@@ -3040,10 +3036,10 @@
         <v>298</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.05428333333333332</v>
+        <v>0.05536666666666666</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.2977183333333333</v>
+        <v>0.31169</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3065,22 +3061,22 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.0177</v>
+        <v>0.0302</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.05611666666666666</v>
+        <v>0.09488333333333333</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.1793583333333333</v>
+        <v>0.2618083333333333</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.03773333333333333</v>
+        <v>0.02401666666666667</v>
       </c>
     </row>
     <row r="16">
@@ -3102,19 +3098,19 @@
         <v>0</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>111</v>
+        <v>111.5</v>
       </c>
       <c r="G16" s="8" t="n">
         <v>320</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.019875</v>
+        <v>0.01946666666666667</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2719099999999999</v>
+        <v>0.2843850000000001</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.0023</v>
+        <v>0.00175</v>
       </c>
     </row>
     <row r="17">
@@ -3123,7 +3119,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
@@ -3133,22 +3129,22 @@
         <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.007883333333333332</v>
+        <v>0.00915</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>258</v>
+        <v>223</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.01766666666666667</v>
+        <v>0.03365</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.07016666666666667</v>
+        <v>0.10869</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.02426666666666667</v>
+        <v>0.06734999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -3157,32 +3153,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
         <v>28</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.0042</v>
+        <v>0.006966666666666667</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02386666666666667</v>
+        <v>0.01581666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.20625</v>
+        <v>0.05761666666666666</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.00055</v>
+        <v>0.04436666666666667</v>
       </c>
     </row>
     <row r="19">
@@ -3191,32 +3187,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
         <v>28</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.0034</v>
+        <v>0.00425</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>65</v>
+        <v>107</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>207</v>
+        <v>269</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.0129</v>
+        <v>0.02595</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.05200833333333334</v>
+        <v>0.2176</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.1034666666666667</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="20">
@@ -3235,7 +3231,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.06156666666666667</v>
+        <v>0.06405</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3244,13 +3240,13 @@
         <v>271</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.1407</v>
+        <v>0.145825</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3476750000000001</v>
+        <v>0.3555883333333334</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.00405</v>
+        <v>0.003283333333333333</v>
       </c>
     </row>
     <row r="21">
@@ -3269,22 +3265,22 @@
         <v>10</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03998333333333333</v>
+        <v>0.03443333333333333</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1158833333333334</v>
+        <v>0.1000666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3406783333333331</v>
+        <v>0.306845</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.0028</v>
+        <v>0.004383333333333334</v>
       </c>
     </row>
     <row r="22">
@@ -3303,22 +3299,22 @@
         <v>9</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03258333333333334</v>
+        <v>0.03288333333333333</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.09323333333333333</v>
+        <v>0.0944</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.253775</v>
+        <v>0.2570083333333333</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.0196</v>
+        <v>0.01956666666666667</v>
       </c>
     </row>
     <row r="23">
@@ -3337,7 +3333,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.002733333333333334</v>
+        <v>0.003366666666666666</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>75</v>
@@ -3346,13 +3342,13 @@
         <v>260</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01306666666666667</v>
+        <v>0.01348333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.051675</v>
+        <v>0.05353166666666666</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.03815</v>
+        <v>0.03048333333333334</v>
       </c>
     </row>
     <row r="24">
@@ -3371,22 +3367,22 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.00215</v>
+        <v>0.001283333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>268</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.04278333333333334</v>
+        <v>0.03231666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2398016666666666</v>
+        <v>0.1942333333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="25">
@@ -3405,22 +3401,22 @@
         <v>9</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.008533333333333334</v>
+        <v>0.007316666666666667</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G25" s="9" t="n">
         <v>238</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02623333333333334</v>
+        <v>0.02203333333333334</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1154916666666667</v>
+        <v>0.09917500000000001</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02350833333333334</v>
+        <v>0.03529166666666667</v>
       </c>
     </row>
     <row r="26">
@@ -3439,22 +3435,22 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.0044</v>
+        <v>0.00505</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>90</v>
+        <v>90.5</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>284</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02961666666666667</v>
+        <v>0.0305</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1338116666666667</v>
+        <v>0.1381533333333334</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.002983333333333333</v>
+        <v>0.002216666666666667</v>
       </c>
     </row>
     <row r="27">
@@ -3463,32 +3459,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
         <v>26</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.00305</v>
+        <v>0.00225</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>272</v>
+        <v>248</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02238333333333334</v>
+        <v>0.022125</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2016633333333333</v>
+        <v>0.2014083333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.00085</v>
+        <v>0.00545</v>
       </c>
     </row>
     <row r="28">
@@ -3497,32 +3493,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
         <v>26</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00295</v>
+        <v>0.00205</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.02850833333333333</v>
+        <v>0.01544166666666667</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.2417333333333333</v>
+        <v>0.1606283333333333</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.003316666666666667</v>
+        <v>0.002866666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -3541,7 +3537,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.01918333333333333</v>
+        <v>0.02111666666666667</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>103</v>
@@ -3550,13 +3546,13 @@
         <v>249</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.06273333333333334</v>
+        <v>0.06513333333333333</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.220075</v>
+        <v>0.2309833333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0039</v>
+        <v>0.00385</v>
       </c>
     </row>
     <row r="30">
@@ -3575,22 +3571,22 @@
         <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0014</v>
+        <v>0.01</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0102</v>
+        <v>0.04240000000000001</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.05968666666666666</v>
+        <v>0.1481183333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03876666666666666</v>
+        <v>0.02605</v>
       </c>
     </row>
     <row r="31">
@@ -3599,32 +3595,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
         <v>23</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.006983333333333333</v>
+        <v>0.0049</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>204</v>
+        <v>227</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.02738333333333334</v>
+        <v>0.03618333333333333</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.1110416666666667</v>
+        <v>0.2241666666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.015475</v>
+        <v>0.0048</v>
       </c>
     </row>
     <row r="32">
@@ -3633,32 +3629,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
         <v>23</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.005</v>
+        <v>0.00475</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>98.5</v>
+        <v>85</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>227</v>
+        <v>204</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03481666666666667</v>
+        <v>0.02133333333333333</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2159833333333333</v>
+        <v>0.09511499999999999</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0055</v>
+        <v>0.024425</v>
       </c>
     </row>
     <row r="33">
@@ -3677,7 +3673,7 @@
         <v>9</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.0035</v>
+        <v>0.004083333333333334</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>88</v>
@@ -3686,13 +3682,13 @@
         <v>225</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.02230833333333333</v>
+        <v>0.023775</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1261083333333334</v>
+        <v>0.1343916666666667</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="34">
@@ -3711,22 +3707,22 @@
         <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.001633333333333333</v>
+        <v>0.002083333333333333</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>255</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.01071666666666667</v>
+        <v>0.01106666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.1037216666666667</v>
+        <v>0.1096766666666666</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.01005</v>
+        <v>0.009766666666666667</v>
       </c>
     </row>
     <row r="35">
@@ -3745,22 +3741,22 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00445</v>
+        <v>0.00325</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G35" s="9" t="n">
         <v>223</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03642500000000001</v>
+        <v>0.02716666666666666</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1847333333333334</v>
+        <v>0.1557666666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.005233333333333333</v>
+        <v>0.009950000000000001</v>
       </c>
     </row>
     <row r="36">
@@ -3788,13 +3784,13 @@
         <v>203</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.001833333333333334</v>
+        <v>0.001733333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04301666666666667</v>
+        <v>0.04526666666666666</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1006666666666667</v>
+        <v>0.1007333333333334</v>
       </c>
     </row>
     <row r="37">
@@ -3813,22 +3809,22 @@
         <v>9</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00505</v>
+        <v>0.00395</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="G37" s="9" t="n">
         <v>211</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.027225</v>
+        <v>0.0203</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1905733333333333</v>
+        <v>0.1573316666666666</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.00315</v>
+        <v>0.0056</v>
       </c>
     </row>
     <row r="38">
@@ -3847,7 +3843,7 @@
         <v>7</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.002133333333333333</v>
+        <v>0.002233333333333333</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>73</v>
@@ -3856,13 +3852,13 @@
         <v>257</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01538333333333333</v>
+        <v>0.0162</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06425833333333332</v>
+        <v>0.066125</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.07036666666666666</v>
+        <v>0.07096666666666666</v>
       </c>
     </row>
     <row r="39">
@@ -3881,7 +3877,7 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0013</v>
+        <v>0.0016</v>
       </c>
       <c r="F39" s="9" t="n">
         <v>69</v>
@@ -3890,13 +3886,13 @@
         <v>248</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.008333333333333333</v>
+        <v>0.009433333333333334</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04797</v>
+        <v>0.04955333333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1257</v>
+        <v>0.1257333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3915,22 +3911,22 @@
         <v>8</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00015</v>
+        <v>0.0002</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G40" s="8" t="n">
         <v>213</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.003083333333333333</v>
+        <v>0.002233333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.04523666666666667</v>
+        <v>0.03588666666666667</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.03133333333333334</v>
+        <v>0.04888333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -3949,7 +3945,7 @@
         <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.002266666666666666</v>
+        <v>0.002366666666666666</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>80</v>
@@ -3958,13 +3954,13 @@
         <v>229</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01265</v>
+        <v>0.01303333333333333</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07042500000000003</v>
+        <v>0.07261666666666668</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.02300833333333334</v>
+        <v>0.022175</v>
       </c>
     </row>
     <row r="42">
@@ -3983,7 +3979,7 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00125</v>
+        <v>0.00115</v>
       </c>
       <c r="F42" s="8" t="n">
         <v>54</v>
@@ -3992,13 +3988,13 @@
         <v>180</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.00405</v>
+        <v>0.0042</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.01919166666666667</v>
+        <v>0.0196</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.289675</v>
+        <v>0.287525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 17:15:47 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>642a0a38c44454af</t>
+          <t>beb794c701680ae0</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>1f501acd71d581d0</t>
+          <t>642a0a38c44454af</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Round of 32: Michigan State over Louisville</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T21:00:51.699011+00:00</t>
+          <t>2026-03-21T21:15:46.805556+00:00</t>
         </is>
       </c>
     </row>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8556016283005042</v>
+        <v>0.8531332211889067</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1443983716994957</v>
+        <v>0.1468667788110933</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2064,10 +2064,14 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Michigan State</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="b">
         <v>0</v>
       </c>
@@ -2340,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1687507768376464</v>
+        <v>0.1679202050040954</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8312492231623536</v>
+        <v>0.8320797949959046</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2480,10 +2484,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.311170986105787</v>
+        <v>0.3112515180769795</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.688829013894213</v>
+        <v>0.6887484819230205</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2613,25 +2617,25 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1181</v>
+        <v>0.1560166666666667</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3082083333333334</v>
+        <v>0.3826833333333334</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.6834033333333333</v>
+        <v>0.7536</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2647,28 +2651,28 @@
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.05418333333333334</v>
+        <v>0.06981666666666667</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1523333333333333</v>
+        <v>0.179125</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.3831583333333333</v>
+        <v>0.4307766666666668</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.006266666666666666</v>
+        <v>0.00225</v>
       </c>
     </row>
     <row r="4">
@@ -2677,32 +2681,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.1418833333333333</v>
+        <v>0.07488333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.3287916666666668</v>
+        <v>0.1738583333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.7133166666666669</v>
+        <v>0.4118066666666667</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0</v>
+        <v>0.0009333333333333332</v>
       </c>
     </row>
     <row r="5">
@@ -2711,32 +2715,32 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07951666666666667</v>
+        <v>0.02055</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.2010583333333334</v>
+        <v>0.1117666666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4796666666666666</v>
+        <v>0.5020433333333332</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0003</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="6">
@@ -2745,32 +2749,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06043333333333334</v>
+        <v>0.14085</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>315</v>
+        <v>297</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1628666666666666</v>
+        <v>0.3253366666666666</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.4767050000000001</v>
+        <v>0.7012166666666667</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.0008</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2779,32 +2783,32 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.05723333333333332</v>
+        <v>0.08011666666666667</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>303</v>
+        <v>323</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1441583333333333</v>
+        <v>0.1934666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3571183333333333</v>
+        <v>0.4493066666666667</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.001316666666666667</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="8">
@@ -2813,32 +2817,32 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ryan Evans</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.04855</v>
+        <v>0.06836666666666667</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>321</v>
+        <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1338166666666667</v>
+        <v>0.1871033333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3263833333333334</v>
+        <v>0.4981433333333334</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.00375</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2847,32 +2851,32 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.02583333333333333</v>
+        <v>0.05888333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>315</v>
+        <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1047416666666666</v>
+        <v>0.1531533333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4513</v>
+        <v>0.3518416666666667</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00045</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="10">
@@ -2881,32 +2885,32 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.02028333333333333</v>
+        <v>0.0028</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>345</v>
+        <v>319</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.08980833333333335</v>
+        <v>0.03040000000000001</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4017416666666666</v>
+        <v>0.2723666666666666</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.001</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="11">
@@ -2915,32 +2919,32 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Ryan Evans</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.01465</v>
+        <v>0.04333333333333333</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>341</v>
+        <v>281</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.07897500000000002</v>
+        <v>0.1249</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4133716666666667</v>
+        <v>0.3149</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.0005833333333333334</v>
+        <v>0.003783333333333333</v>
       </c>
     </row>
     <row r="12">
@@ -2949,32 +2953,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.05193333333333332</v>
+        <v>0.02498333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>270</v>
+        <v>320</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1470083333333334</v>
+        <v>0.1016416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4353499999999999</v>
+        <v>0.43965</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.001083333333333334</v>
       </c>
     </row>
     <row r="13">
@@ -2983,32 +2987,32 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.04933333333333334</v>
+        <v>0.01635</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>266</v>
+        <v>336</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1327166666666666</v>
+        <v>0.08476666666666666</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3255250000000001</v>
+        <v>0.3921733333333334</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0025</v>
+        <v>0.00115</v>
       </c>
     </row>
     <row r="14">
@@ -3017,32 +3021,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01303333333333333</v>
+        <v>0.0077</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.05536666666666666</v>
+        <v>0.02065</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.31169</v>
+        <v>0.07633333333333334</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0</v>
+        <v>0.01833333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -3051,32 +3055,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.0302</v>
+        <v>0.04033333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>275</v>
+        <v>245</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.09488333333333333</v>
+        <v>0.1214916666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2618083333333333</v>
+        <v>0.35356</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.02401666666666667</v>
+        <v>0.00225</v>
       </c>
     </row>
     <row r="16">
@@ -3085,32 +3089,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0</v>
+        <v>0.009833333333333333</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>111.5</v>
+        <v>112</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.01946666666666667</v>
+        <v>0.050525</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2843850000000001</v>
+        <v>0.3029583333333333</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.00175</v>
+        <v>8.333333333333333e-05</v>
       </c>
     </row>
     <row r="17">
@@ -3119,32 +3123,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.00915</v>
+        <v>0.002233333333333334</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>73</v>
+        <v>111</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>223</v>
+        <v>268</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.03365</v>
+        <v>0.04363333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.10869</v>
+        <v>0.2412666666666667</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.06734999999999999</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="18">
@@ -3153,32 +3157,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.006966666666666667</v>
+        <v>0.01223333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01581666666666667</v>
+        <v>0.04561666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.05761666666666666</v>
+        <v>0.1492916666666667</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.04436666666666667</v>
+        <v>0.0432</v>
       </c>
     </row>
     <row r="19">
@@ -3187,32 +3191,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.00425</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>269</v>
+        <v>242</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02595</v>
+        <v>0.03065</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2176</v>
+        <v>0.1183</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.01875</v>
       </c>
     </row>
     <row r="20">
@@ -3221,32 +3225,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.06405</v>
+        <v>0.004466666666666667</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.145825</v>
+        <v>0.02902500000000001</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3555883333333334</v>
+        <v>0.2180766666666666</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.003283333333333333</v>
+        <v>0.0006833333333333334</v>
       </c>
     </row>
     <row r="21">
@@ -3255,32 +3259,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.03443333333333333</v>
+        <v>0.003783333333333333</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.1000666666666667</v>
+        <v>0.03326999999999999</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.306845</v>
+        <v>0.2594666666666666</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.004383333333333334</v>
+        <v>0.002625</v>
       </c>
     </row>
     <row r="22">
@@ -3289,32 +3293,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.03288333333333333</v>
+        <v>0</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>256</v>
+        <v>314</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.0944</v>
+        <v>0.01955</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2570083333333333</v>
+        <v>0.272765</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.01956666666666667</v>
+        <v>0.0015</v>
       </c>
     </row>
     <row r="23">
@@ -3323,32 +3327,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.003366666666666666</v>
+        <v>0.003283333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01348333333333333</v>
+        <v>0.01915</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.05353166666666666</v>
+        <v>0.2045583333333333</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.03048333333333334</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -3357,32 +3361,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.001283333333333333</v>
+        <v>0.00175</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>268</v>
+        <v>180</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03231666666666667</v>
+        <v>0.00545</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1942333333333333</v>
+        <v>0.03218333333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0007</v>
+        <v>0.1213</v>
       </c>
     </row>
     <row r="25">
@@ -3391,32 +3395,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.007316666666666667</v>
+        <v>0.06205</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>238</v>
+        <v>276</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02203333333333334</v>
+        <v>0.1370666666666666</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.09917500000000001</v>
+        <v>0.3458066666666666</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.03529166666666667</v>
+        <v>0.004033333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3425,32 +3429,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.00505</v>
+        <v>0.02653333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>90.5</v>
+        <v>94</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>284</v>
+        <v>239</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.0305</v>
+        <v>0.08498333333333334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1381533333333334</v>
+        <v>0.2393999999999999</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.002216666666666667</v>
+        <v>0.01833333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -3459,32 +3463,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.00225</v>
+        <v>0.007483333333333334</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>248</v>
+        <v>198</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.022125</v>
+        <v>0.0277</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2014083333333334</v>
+        <v>0.1219333333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.00545</v>
+        <v>0.01304166666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3493,32 +3497,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00205</v>
+        <v>0.00255</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01544166666666667</v>
+        <v>0.01415</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1606283333333333</v>
+        <v>0.05032500000000001</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.002866666666666667</v>
+        <v>0.03807499999999999</v>
       </c>
     </row>
     <row r="29">
@@ -3527,32 +3531,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D29" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.02111666666666667</v>
+        <v>0.00635</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>249</v>
+        <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.06513333333333333</v>
+        <v>0.03958333333333332</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2309833333333333</v>
+        <v>0.19235</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.00385</v>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="30">
@@ -3561,32 +3565,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.01</v>
+        <v>0.0035</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.04240000000000001</v>
+        <v>0.03023333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1481183333333333</v>
+        <v>0.1281183333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.02605</v>
+        <v>0.00305</v>
       </c>
     </row>
     <row r="31">
@@ -3595,32 +3599,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D31" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.0049</v>
+        <v>0.0174</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>227</v>
+        <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.03618333333333333</v>
+        <v>0.062</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2241666666666667</v>
+        <v>0.2182066666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.0048</v>
+        <v>0.001866666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3629,32 +3633,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00475</v>
+        <v>0.005233333333333333</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.02133333333333333</v>
+        <v>0.03017</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.09511499999999999</v>
+        <v>0.2004316666666666</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.024425</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="33">
@@ -3663,32 +3667,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.004083333333333334</v>
+        <v>5e-05</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.023775</v>
+        <v>0.003</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1343916666666667</v>
+        <v>0.05073333333333333</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.02561666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3697,32 +3701,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.002083333333333333</v>
+        <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>255</v>
+        <v>224</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.01106666666666667</v>
+        <v>0.0013</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.1096766666666666</v>
+        <v>0.032125</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.009766666666666667</v>
+        <v>0.04168333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3731,32 +3735,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D35" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00325</v>
+        <v>0.00545</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.02716666666666666</v>
+        <v>0.03203333333333334</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1557666666666667</v>
+        <v>0.2014733333333333</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.009950000000000001</v>
+        <v>0.0056</v>
       </c>
     </row>
     <row r="36">
@@ -3765,32 +3769,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.0025</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>203</v>
+        <v>236</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.001733333333333333</v>
+        <v>0.01971666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04526666666666666</v>
+        <v>0.1258533333333333</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1007333333333334</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="37">
@@ -3799,32 +3803,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00395</v>
+        <v>0.001233333333333333</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>211</v>
+        <v>250</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0203</v>
+        <v>0.007566666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1573316666666666</v>
+        <v>0.1058</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0056</v>
+        <v>0.009133333333333334</v>
       </c>
     </row>
     <row r="38">
@@ -3833,32 +3837,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.002233333333333333</v>
+        <v>0.0001</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>257</v>
+        <v>207</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.0162</v>
+        <v>0.0014</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.066125</v>
+        <v>0.03945000000000001</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.07096666666666666</v>
+        <v>0.09453333333333336</v>
       </c>
     </row>
     <row r="39">
@@ -3867,7 +3871,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
@@ -3877,22 +3881,22 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0016</v>
+        <v>0.002</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.009433333333333334</v>
+        <v>0.01513333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04955333333333334</v>
+        <v>0.06471666666666667</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1257333333333333</v>
+        <v>0.07368333333333334</v>
       </c>
     </row>
     <row r="40">
@@ -3901,32 +3905,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
         <v>20</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.00185</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>213</v>
+        <v>253</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.002233333333333333</v>
+        <v>0.00835</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.03588666666666667</v>
+        <v>0.0425</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.04888333333333333</v>
+        <v>0.126225</v>
       </c>
     </row>
     <row r="41">
@@ -3945,22 +3949,22 @@
         <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.002366666666666666</v>
+        <v>0.0026</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01303333333333333</v>
+        <v>0.01485</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07261666666666668</v>
+        <v>0.07385833333333333</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.022175</v>
+        <v>0.0217</v>
       </c>
     </row>
     <row r="42">
@@ -3979,22 +3983,22 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00115</v>
+        <v>0.00065</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.0042</v>
+        <v>0.00355</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.0196</v>
+        <v>0.02033333333333334</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.287525</v>
+        <v>0.2952</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 17:20:03 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Round of 32: Michigan State over Louisville</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T21:15:46.805556+00:00</t>
+          <t>2026-03-21T21:20:02.679962+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8531332211889067</v>
+        <v>0.8519264996299132</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1468667788110933</v>
+        <v>0.1480735003700867</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1952393805638805</v>
+        <v>0.1935705489429316</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8047606194361195</v>
+        <v>0.8064294510570685</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1560166666666667</v>
+        <v>0.1561166666666667</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>140</v>
@@ -2635,7 +2635,7 @@
         <v>0.3826833333333334</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7536</v>
+        <v>0.7534000000000001</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2669,7 +2669,7 @@
         <v>0.179125</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4307766666666668</v>
+        <v>0.4306766666666668</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0.00225</v>
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07488333333333333</v>
+        <v>0.07498333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>117</v>
@@ -2700,10 +2700,10 @@
         <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1738583333333333</v>
+        <v>0.1740083333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4118066666666667</v>
+        <v>0.4120066666666667</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0.0009333333333333332</v>
@@ -2737,7 +2737,7 @@
         <v>0.1117666666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5020433333333332</v>
+        <v>0.5018933333333332</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0002</v>
@@ -2759,7 +2759,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.14085</v>
+        <v>0.14075</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>138</v>
@@ -2768,7 +2768,7 @@
         <v>297</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3253366666666666</v>
+        <v>0.3252366666666666</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0.7012166666666667</v>
@@ -2793,7 +2793,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.08011666666666667</v>
+        <v>0.08016666666666666</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>119</v>
@@ -2805,7 +2805,7 @@
         <v>0.1934666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4493066666666667</v>
+        <v>0.4495400000000001</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0002</v>
@@ -2827,7 +2827,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06836666666666667</v>
+        <v>0.06831666666666668</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>126</v>
@@ -2836,10 +2836,10 @@
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1871033333333333</v>
+        <v>0.1872033333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4981433333333334</v>
+        <v>0.4983433333333334</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,7 +2861,7 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.05888333333333333</v>
+        <v>0.05898333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>108</v>
@@ -2870,10 +2870,10 @@
         <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1531533333333333</v>
+        <v>0.1532033333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3518416666666667</v>
+        <v>0.3519416666666667</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00055</v>
@@ -2907,7 +2907,7 @@
         <v>0.03040000000000001</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2723666666666666</v>
+        <v>0.2722666666666667</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.0008</v>
@@ -2941,7 +2941,7 @@
         <v>0.1249</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3149</v>
+        <v>0.3148</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.003783333333333333</v>
@@ -2975,7 +2975,7 @@
         <v>0.1016416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.43965</v>
+        <v>0.43975</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.001083333333333334</v>
@@ -3006,13 +3006,13 @@
         <v>336</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08476666666666666</v>
+        <v>0.08486666666666666</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3921733333333334</v>
+        <v>0.3922733333333334</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.00115</v>
+        <v>0.0011</v>
       </c>
     </row>
     <row r="14">
@@ -3031,7 +3031,7 @@
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.0077</v>
+        <v>0.00775</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>82</v>
@@ -3040,13 +3040,13 @@
         <v>290</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.02065</v>
+        <v>0.02085</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>0.07633333333333334</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01833333333333334</v>
+        <v>0.01848333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -3065,7 +3065,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.04033333333333334</v>
+        <v>0.04028333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>109</v>
@@ -3077,7 +3077,7 @@
         <v>0.1214916666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.35356</v>
+        <v>0.35376</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00225</v>
@@ -3111,7 +3111,7 @@
         <v>0.050525</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3029583333333333</v>
+        <v>0.3030083333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>8.333333333333333e-05</v>
@@ -3179,10 +3179,10 @@
         <v>0.04561666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1492916666666667</v>
+        <v>0.1495416666666667</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.0432</v>
+        <v>0.04305</v>
       </c>
     </row>
     <row r="19">
@@ -3201,7 +3201,7 @@
         <v>9</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0098</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>85</v>
@@ -3210,10 +3210,10 @@
         <v>242</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03065</v>
+        <v>0.03045</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1183</v>
+        <v>0.1181</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.01875</v>
@@ -3247,7 +3247,7 @@
         <v>0.02902500000000001</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2180766666666666</v>
+        <v>0.2180599999999999</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.0006833333333333334</v>
@@ -3269,7 +3269,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.003783333333333333</v>
+        <v>0.003683333333333334</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
@@ -3315,7 +3315,7 @@
         <v>0.01955</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.272765</v>
+        <v>0.2726150000000001</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0015</v>
@@ -3349,7 +3349,7 @@
         <v>0.01915</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2045583333333333</v>
+        <v>0.2046583333333334</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -3386,7 +3386,7 @@
         <v>0.03218333333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.1213</v>
+        <v>0.1211</v>
       </c>
     </row>
     <row r="25">
@@ -3417,7 +3417,7 @@
         <v>0.1370666666666666</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3458066666666666</v>
+        <v>0.3459566666666666</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>0.004033333333333333</v>
@@ -3451,7 +3451,7 @@
         <v>0.08498333333333334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2393999999999999</v>
+        <v>0.2394499999999999</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.01833333333333333</v>
@@ -3485,7 +3485,7 @@
         <v>0.0277</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1219333333333334</v>
+        <v>0.1218333333333334</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.01304166666666667</v>
@@ -3516,13 +3516,13 @@
         <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01415</v>
+        <v>0.01395</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.05032500000000001</v>
+        <v>0.049925</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.03807499999999999</v>
+        <v>0.03812499999999999</v>
       </c>
     </row>
     <row r="29">
@@ -3553,7 +3553,7 @@
         <v>0.03958333333333332</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.19235</v>
+        <v>0.1921</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.0035</v>
@@ -3587,7 +3587,7 @@
         <v>0.03023333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1281183333333333</v>
+        <v>0.1280516666666666</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0.00305</v>
@@ -3621,7 +3621,7 @@
         <v>0.062</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2182066666666667</v>
+        <v>0.2184066666666667</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0.001866666666666667</v>
@@ -3652,10 +3652,10 @@
         <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03017</v>
+        <v>0.03007</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2004316666666666</v>
+        <v>0.2002316666666667</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.004</v>
@@ -3680,7 +3680,7 @@
         <v>5e-05</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>80</v>
+        <v>79.5</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>218</v>
@@ -3723,7 +3723,7 @@
         <v>0.0013</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.032125</v>
+        <v>0.032225</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>0.04168333333333333</v>
@@ -3754,10 +3754,10 @@
         <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03203333333333334</v>
+        <v>0.03213333333333334</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.2014733333333333</v>
+        <v>0.2013733333333333</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0.0056</v>
@@ -3791,7 +3791,7 @@
         <v>0.01971666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1258533333333333</v>
+        <v>0.1259533333333333</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0002</v>
@@ -3825,7 +3825,7 @@
         <v>0.007566666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1058</v>
+        <v>0.10565</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>0.009133333333333334</v>
@@ -3862,7 +3862,7 @@
         <v>0.03945000000000001</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.09453333333333336</v>
+        <v>0.09433333333333337</v>
       </c>
     </row>
     <row r="39">
@@ -3893,10 +3893,10 @@
         <v>0.01513333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.06471666666666667</v>
+        <v>0.06481666666666668</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.07368333333333334</v>
+        <v>0.07358333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3930,7 +3930,7 @@
         <v>0.0425</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.126225</v>
+        <v>0.126325</v>
       </c>
     </row>
     <row r="41">
@@ -3958,10 +3958,10 @@
         <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01485</v>
+        <v>0.01495</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07385833333333333</v>
+        <v>0.07410833333333333</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.0217</v>
@@ -3992,13 +3992,13 @@
         <v>185</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.00355</v>
+        <v>0.00335</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.02033333333333334</v>
+        <v>0.02013333333333333</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2952</v>
+        <v>0.2956</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 17:40:07 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T21:20:02.679962+00:00</t>
+          <t>2026-03-21T21:40:07.350900+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8519264996299132</v>
+        <v>0.8247885391457197</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1480735003700867</v>
+        <v>0.1752114608542804</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1679202050040954</v>
+        <v>0.1671455482448929</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8320797949959046</v>
+        <v>0.8328544517551071</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1935705489429316</v>
+        <v>0.1932345091971844</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8064294510570685</v>
+        <v>0.8067654908028156</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2484,10 +2484,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3112515180769795</v>
+        <v>0.312028614752377</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6887484819230205</v>
+        <v>0.6879713852476229</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1561166666666667</v>
+        <v>0.1558166666666667</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>140</v>
@@ -2632,10 +2632,10 @@
         <v>360</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3826833333333334</v>
+        <v>0.3835166666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7534000000000001</v>
+        <v>0.7539166666666668</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,19 +2657,19 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06981666666666667</v>
+        <v>0.07031666666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>120</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.179125</v>
+        <v>0.1796083333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4306766666666668</v>
+        <v>0.4322466666666668</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0.00225</v>
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07498333333333333</v>
+        <v>0.07488333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>117</v>
@@ -2700,10 +2700,10 @@
         <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1740083333333333</v>
+        <v>0.1737583333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4120066666666667</v>
+        <v>0.4103266666666666</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0.0009333333333333332</v>
@@ -2725,7 +2725,7 @@
         <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.02055</v>
+        <v>0.02</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>123</v>
@@ -2734,10 +2734,10 @@
         <v>326</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1117666666666667</v>
+        <v>0.1093833333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5018933333333332</v>
+        <v>0.4970433333333332</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0002</v>
@@ -2759,7 +2759,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.14075</v>
+        <v>0.1387</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>138</v>
@@ -2768,10 +2768,10 @@
         <v>297</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3252366666666666</v>
+        <v>0.3212366666666666</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.7012166666666667</v>
+        <v>0.6967500000000002</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.08016666666666666</v>
+        <v>0.07941666666666666</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>119</v>
@@ -2802,10 +2802,10 @@
         <v>323</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1934666666666667</v>
+        <v>0.1921333333333334</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4495400000000001</v>
+        <v>0.4468733333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0002</v>
@@ -2827,7 +2827,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06831666666666668</v>
+        <v>0.06871666666666668</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>126</v>
@@ -2836,10 +2836,10 @@
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1872033333333333</v>
+        <v>0.1881033333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4983433333333334</v>
+        <v>0.5003933333333335</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,7 +2861,7 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.05898333333333333</v>
+        <v>0.05943333333333332</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>108</v>
@@ -2870,13 +2870,13 @@
         <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1532033333333333</v>
+        <v>0.15332</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3519416666666667</v>
+        <v>0.3517833333333333</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.00065</v>
       </c>
     </row>
     <row r="10">
@@ -2895,7 +2895,7 @@
         <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0028</v>
+        <v>0.00285</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>114</v>
@@ -2904,13 +2904,13 @@
         <v>319</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.03040000000000001</v>
+        <v>0.03030000000000001</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2722666666666667</v>
+        <v>0.2714666666666666</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0008</v>
+        <v>0.00095</v>
       </c>
     </row>
     <row r="11">
@@ -2929,7 +2929,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04333333333333333</v>
+        <v>0.04308333333333333</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>108</v>
@@ -2938,13 +2938,13 @@
         <v>281</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1249</v>
+        <v>0.1255166666666667</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3148</v>
+        <v>0.31685</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.003783333333333333</v>
+        <v>0.003683333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -2963,7 +2963,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02498333333333333</v>
+        <v>0.02533333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>120</v>
@@ -2972,10 +2972,10 @@
         <v>320</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1016416666666667</v>
+        <v>0.1022416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.43975</v>
+        <v>0.4405833333333334</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.001083333333333334</v>
@@ -2997,7 +2997,7 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.01635</v>
+        <v>0.0166</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>119</v>
@@ -3006,10 +3006,10 @@
         <v>336</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08486666666666666</v>
+        <v>0.08606666666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3922733333333334</v>
+        <v>0.3943016666666667</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0.0011</v>
@@ -3031,22 +3031,22 @@
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.00775</v>
+        <v>0.00885</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G14" s="8" t="n">
         <v>290</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.02085</v>
+        <v>0.02315000000000001</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.07633333333333334</v>
+        <v>0.0825</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01848333333333334</v>
+        <v>0.01803333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -3065,7 +3065,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.04028333333333334</v>
+        <v>0.04083333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>109</v>
@@ -3074,10 +3074,10 @@
         <v>245</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.1214916666666667</v>
+        <v>0.1227416666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.35376</v>
+        <v>0.3551766666666666</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00225</v>
@@ -3099,7 +3099,7 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.009833333333333333</v>
+        <v>0.009683333333333334</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>112</v>
@@ -3108,10 +3108,10 @@
         <v>300</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.050525</v>
+        <v>0.050275</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3030083333333333</v>
+        <v>0.303625</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>8.333333333333333e-05</v>
@@ -3133,7 +3133,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.002233333333333334</v>
+        <v>0.002333333333333334</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>111</v>
@@ -3142,10 +3142,10 @@
         <v>268</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04363333333333334</v>
+        <v>0.04388333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2412666666666667</v>
+        <v>0.2409166666666666</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0.00025</v>
@@ -3176,13 +3176,13 @@
         <v>261</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.04561666666666667</v>
+        <v>0.04591666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1495416666666667</v>
+        <v>0.1503916666666666</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.04305</v>
+        <v>0.0428</v>
       </c>
     </row>
     <row r="19">
@@ -3201,7 +3201,7 @@
         <v>9</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.0098</v>
+        <v>0.00975</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>85</v>
@@ -3210,13 +3210,13 @@
         <v>242</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03045</v>
+        <v>0.03061666666666667</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1181</v>
+        <v>0.1190333333333334</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.01875</v>
+        <v>0.01865</v>
       </c>
     </row>
     <row r="20">
@@ -3244,10 +3244,10 @@
         <v>276</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02902500000000001</v>
+        <v>0.02937500000000001</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2180599999999999</v>
+        <v>0.2193099999999999</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.0006833333333333334</v>
@@ -3269,7 +3269,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.003683333333333334</v>
+        <v>0.003783333333333333</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
@@ -3278,13 +3278,13 @@
         <v>259</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.03326999999999999</v>
+        <v>0.03293666666666666</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2594666666666666</v>
+        <v>0.2587666666666666</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.002625</v>
+        <v>0.002725</v>
       </c>
     </row>
     <row r="22">
@@ -3312,10 +3312,10 @@
         <v>314</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.01955</v>
+        <v>0.0197</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2726150000000001</v>
+        <v>0.2734350000000001</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0015</v>
@@ -3337,7 +3337,7 @@
         <v>8</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.003283333333333333</v>
+        <v>0.003633333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>108</v>
@@ -3346,13 +3346,13 @@
         <v>271</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01915</v>
+        <v>0.02025</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2046583333333334</v>
+        <v>0.2065166666666667</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="24">
@@ -3380,13 +3380,13 @@
         <v>180</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.00545</v>
+        <v>0.00535</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.03218333333333333</v>
+        <v>0.03211666666666666</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.1211</v>
+        <v>0.11985</v>
       </c>
     </row>
     <row r="25">
@@ -3405,7 +3405,7 @@
         <v>10</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.06205</v>
+        <v>0.06185</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>109</v>
@@ -3414,10 +3414,10 @@
         <v>276</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.1370666666666666</v>
+        <v>0.1367166666666667</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3459566666666666</v>
+        <v>0.3441899999999999</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>0.004033333333333333</v>
@@ -3439,22 +3439,22 @@
         <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.02653333333333334</v>
+        <v>0.02643333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>239</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.08498333333333334</v>
+        <v>0.08434999999999999</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2394499999999999</v>
+        <v>0.2380166666666667</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01833333333333333</v>
+        <v>0.01853333333333334</v>
       </c>
     </row>
     <row r="27">
@@ -3473,7 +3473,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.007483333333333334</v>
+        <v>0.007383333333333335</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>91</v>
@@ -3482,13 +3482,13 @@
         <v>198</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0277</v>
+        <v>0.0275</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1218333333333334</v>
+        <v>0.1207</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01304166666666667</v>
+        <v>0.01329166666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3507,7 +3507,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00255</v>
+        <v>0.0024</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>75</v>
@@ -3516,13 +3516,13 @@
         <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01395</v>
+        <v>0.0137</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.049925</v>
+        <v>0.04972500000000001</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.03812499999999999</v>
+        <v>0.03787499999999999</v>
       </c>
     </row>
     <row r="29">
@@ -3550,10 +3550,10 @@
         <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03958333333333332</v>
+        <v>0.03938333333333333</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1921</v>
+        <v>0.1906166666666667</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.0035</v>
@@ -3575,7 +3575,7 @@
         <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0035</v>
+        <v>0.0037</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>90</v>
@@ -3587,10 +3587,10 @@
         <v>0.03023333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1280516666666666</v>
+        <v>0.1284516666666666</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.00305</v>
+        <v>0.00295</v>
       </c>
     </row>
     <row r="31">
@@ -3609,7 +3609,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.0174</v>
+        <v>0.01765</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>104</v>
@@ -3618,13 +3618,13 @@
         <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.062</v>
+        <v>0.063</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2184066666666667</v>
+        <v>0.2202933333333333</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.001866666666666667</v>
+        <v>0.001766666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3643,7 +3643,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.005233333333333333</v>
+        <v>0.005083333333333333</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>99</v>
@@ -3652,10 +3652,10 @@
         <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03007</v>
+        <v>0.02937</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2002316666666667</v>
+        <v>0.1988016666666667</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.004</v>
@@ -3680,7 +3680,7 @@
         <v>5e-05</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>79.5</v>
+        <v>79</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>218</v>
@@ -3689,10 +3689,10 @@
         <v>0.003</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05073333333333333</v>
+        <v>0.05064999999999999</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02561666666666666</v>
+        <v>0.02611666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3720,13 +3720,13 @@
         <v>224</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0013</v>
+        <v>0.00125</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.032225</v>
+        <v>0.032025</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.04168333333333333</v>
+        <v>0.04228333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00545</v>
+        <v>0.00575</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>98</v>
@@ -3754,13 +3754,13 @@
         <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03213333333333334</v>
+        <v>0.03175</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.2013733333333333</v>
+        <v>0.1998466666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.0056</v>
+        <v>0.0057</v>
       </c>
     </row>
     <row r="36">
@@ -3788,10 +3788,10 @@
         <v>236</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01971666666666667</v>
+        <v>0.01976666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1259533333333333</v>
+        <v>0.1247233333333333</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0002</v>
@@ -3822,13 +3822,13 @@
         <v>250</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.007566666666666667</v>
+        <v>0.007766666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.10565</v>
+        <v>0.106545</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.009133333333333334</v>
+        <v>0.008933333333333335</v>
       </c>
     </row>
     <row r="38">
@@ -3850,7 +3850,7 @@
         <v>0.0001</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G38" s="8" t="n">
         <v>207</v>
@@ -3859,10 +3859,10 @@
         <v>0.0014</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.03945000000000001</v>
+        <v>0.04048333333333334</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.09433333333333337</v>
+        <v>0.09233333333333336</v>
       </c>
     </row>
     <row r="39">
@@ -3890,13 +3890,13 @@
         <v>254</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01513333333333333</v>
+        <v>0.01498333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.06481666666666668</v>
+        <v>0.06461666666666667</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.07358333333333333</v>
+        <v>0.07443333333333334</v>
       </c>
     </row>
     <row r="40">
@@ -3915,7 +3915,7 @@
         <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00185</v>
+        <v>0.00195</v>
       </c>
       <c r="F40" s="8" t="n">
         <v>69</v>
@@ -3924,13 +3924,13 @@
         <v>253</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.00835</v>
+        <v>0.008449999999999999</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.0425</v>
+        <v>0.0428</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.126325</v>
+        <v>0.125425</v>
       </c>
     </row>
     <row r="41">
@@ -3949,7 +3949,7 @@
         <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.0026</v>
+        <v>0.00245</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>81</v>
@@ -3958,13 +3958,13 @@
         <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01495</v>
+        <v>0.01465</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07410833333333333</v>
+        <v>0.07325833333333334</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.0217</v>
+        <v>0.02175</v>
       </c>
     </row>
     <row r="42">
@@ -3995,10 +3995,10 @@
         <v>0.00335</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.02013333333333333</v>
+        <v>0.01993333333333333</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2956</v>
+        <v>0.29845</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 18:01:00 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T21:40:07.350900+00:00</t>
+          <t>2026-03-21T22:01:00.058685+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8247885391457197</v>
+        <v>0.8822709529859037</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1752114608542804</v>
+        <v>0.1177290470140962</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1671455482448929</v>
+        <v>0.1674779918985809</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8328544517551071</v>
+        <v>0.8325220081014191</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1932345091971844</v>
+        <v>0.2008656676452992</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8067654908028156</v>
+        <v>0.7991343323547009</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1558166666666667</v>
+        <v>0.1554333333333333</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>140</v>
@@ -2632,10 +2632,10 @@
         <v>360</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3835166666666667</v>
+        <v>0.3830333333333333</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7539166666666668</v>
+        <v>0.7543333333333335</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,22 +2657,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.07031666666666667</v>
+        <v>0.06961666666666666</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>120</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1796083333333333</v>
+        <v>0.178925</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4322466666666668</v>
+        <v>0.4298016666666667</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.00225</v>
+        <v>0.00235</v>
       </c>
     </row>
     <row r="4">
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07488333333333333</v>
+        <v>0.07463333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>117</v>
@@ -2700,13 +2700,13 @@
         <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1737583333333333</v>
+        <v>0.1736583333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4103266666666666</v>
+        <v>0.4137566666666667</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.0009333333333333332</v>
+        <v>0.0009</v>
       </c>
     </row>
     <row r="5">
@@ -2725,22 +2725,22 @@
         <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.02</v>
+        <v>0.02128333333333333</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>326</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1093833333333333</v>
+        <v>0.1138</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4970433333333332</v>
+        <v>0.5066933333333331</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="6">
@@ -2759,7 +2759,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.1387</v>
+        <v>0.1432833333333333</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>138</v>
@@ -2768,10 +2768,10 @@
         <v>297</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3212366666666666</v>
+        <v>0.3302333333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.6967500000000002</v>
+        <v>0.7056833333333333</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.07941666666666666</v>
+        <v>0.08041666666666666</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>119</v>
@@ -2802,13 +2802,13 @@
         <v>323</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1921333333333334</v>
+        <v>0.1939833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4468733333333333</v>
+        <v>0.4507500000000001</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="8">
@@ -2827,19 +2827,19 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06871666666666668</v>
+        <v>0.0677</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1881033333333333</v>
+        <v>0.1856333333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5003933333333335</v>
+        <v>0.4953516666666667</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,7 +2861,7 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.05943333333333332</v>
+        <v>0.05848333333333332</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>108</v>
@@ -2870,13 +2870,13 @@
         <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.15332</v>
+        <v>0.1524666666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3517833333333333</v>
+        <v>0.3510083333333334</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00065</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="10">
@@ -2895,7 +2895,7 @@
         <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.00285</v>
+        <v>0.00275</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>114</v>
@@ -2904,13 +2904,13 @@
         <v>319</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.03030000000000001</v>
+        <v>0.03040000000000001</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2714666666666666</v>
+        <v>0.2722666666666667</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.00095</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="11">
@@ -2929,7 +2929,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04308333333333333</v>
+        <v>0.04323333333333334</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>108</v>
@@ -2938,13 +2938,13 @@
         <v>281</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1255166666666667</v>
+        <v>0.1247</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.31685</v>
+        <v>0.3144666666666667</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.003683333333333334</v>
+        <v>0.003783333333333333</v>
       </c>
     </row>
     <row r="12">
@@ -2963,7 +2963,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02533333333333333</v>
+        <v>0.02458333333333334</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>120</v>
@@ -2972,10 +2972,10 @@
         <v>320</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1022416666666667</v>
+        <v>0.09975833333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4405833333333334</v>
+        <v>0.4374333333333334</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.001083333333333334</v>
@@ -2997,7 +2997,7 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.0166</v>
+        <v>0.01605</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>119</v>
@@ -3006,13 +3006,13 @@
         <v>336</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08606666666666667</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3943016666666667</v>
+        <v>0.3901333333333334</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0011</v>
+        <v>0.00125</v>
       </c>
     </row>
     <row r="14">
@@ -3031,22 +3031,22 @@
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.00885</v>
+        <v>0.0069</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>290</v>
+        <v>248</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.02315000000000001</v>
+        <v>0.01885</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.0825</v>
+        <v>0.07112499999999999</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01803333333333334</v>
+        <v>0.01881666666666667</v>
       </c>
     </row>
     <row r="15">
@@ -3065,7 +3065,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.04083333333333334</v>
+        <v>0.04023333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>109</v>
@@ -3074,10 +3074,10 @@
         <v>245</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.1227416666666667</v>
+        <v>0.1204916666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3551766666666666</v>
+        <v>0.3521766666666666</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00225</v>
@@ -3099,19 +3099,19 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.009683333333333334</v>
+        <v>0.01003333333333333</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>112</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.050275</v>
+        <v>0.049775</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.303625</v>
+        <v>0.3023666666666666</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>8.333333333333333e-05</v>
@@ -3133,7 +3133,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.002333333333333334</v>
+        <v>0.002233333333333334</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>111</v>
@@ -3142,10 +3142,10 @@
         <v>268</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04388333333333334</v>
+        <v>0.04353333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2409166666666666</v>
+        <v>0.2399583333333333</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0.00025</v>
@@ -3167,7 +3167,7 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.01223333333333333</v>
+        <v>0.01193333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>86</v>
@@ -3176,13 +3176,13 @@
         <v>261</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.04591666666666667</v>
+        <v>0.04526666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1503916666666666</v>
+        <v>0.1482416666666667</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.0428</v>
+        <v>0.0441</v>
       </c>
     </row>
     <row r="19">
@@ -3201,7 +3201,7 @@
         <v>9</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.00975</v>
+        <v>0.0103</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>85</v>
@@ -3210,13 +3210,13 @@
         <v>242</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03061666666666667</v>
+        <v>0.03105</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1190333333333334</v>
+        <v>0.1191</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.01865</v>
+        <v>0.01906666666666667</v>
       </c>
     </row>
     <row r="20">
@@ -3235,7 +3235,7 @@
         <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.004466666666666667</v>
+        <v>0.00425</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>108</v>
@@ -3244,10 +3244,10 @@
         <v>276</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02937500000000001</v>
+        <v>0.02830833333333334</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2193099999999999</v>
+        <v>0.2161433333333333</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.0006833333333333334</v>
@@ -3269,7 +3269,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.003783333333333333</v>
+        <v>0.003833333333333334</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
@@ -3278,13 +3278,13 @@
         <v>259</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.03293666666666666</v>
+        <v>0.03398333333333332</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2587666666666666</v>
+        <v>0.2623083333333333</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.002725</v>
+        <v>0.00265</v>
       </c>
     </row>
     <row r="22">
@@ -3312,10 +3312,10 @@
         <v>314</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.0197</v>
+        <v>0.0198</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2734350000000001</v>
+        <v>0.2737083333333333</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0015</v>
@@ -3337,7 +3337,7 @@
         <v>8</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.003633333333333333</v>
+        <v>0.003233333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>108</v>
@@ -3346,13 +3346,13 @@
         <v>271</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.02025</v>
+        <v>0.01836666666666667</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2065166666666667</v>
+        <v>0.200625</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -3380,13 +3380,13 @@
         <v>180</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.00535</v>
+        <v>0.00545</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.03211666666666666</v>
+        <v>0.03158333333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.11985</v>
+        <v>0.123</v>
       </c>
     </row>
     <row r="25">
@@ -3405,7 +3405,7 @@
         <v>10</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.06185</v>
+        <v>0.0618</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>109</v>
@@ -3414,13 +3414,13 @@
         <v>276</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.1367166666666667</v>
+        <v>0.1375833333333333</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3441899999999999</v>
+        <v>0.3468999999999999</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.004033333333333333</v>
+        <v>0.003733333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3439,22 +3439,22 @@
         <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.02643333333333334</v>
+        <v>0.02653333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>239</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.08434999999999999</v>
+        <v>0.08563333333333334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2380166666666667</v>
+        <v>0.2401749999999999</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01853333333333334</v>
+        <v>0.01778333333333334</v>
       </c>
     </row>
     <row r="27">
@@ -3473,7 +3473,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.007383333333333335</v>
+        <v>0.007583333333333334</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>91</v>
@@ -3482,13 +3482,13 @@
         <v>198</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0275</v>
+        <v>0.02835</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1207</v>
+        <v>0.1231833333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01329166666666667</v>
+        <v>0.01271666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3507,7 +3507,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0024</v>
+        <v>0.00265</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>75</v>
@@ -3516,13 +3516,13 @@
         <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.0137</v>
+        <v>0.0142</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.04972500000000001</v>
+        <v>0.05090833333333334</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.03787499999999999</v>
+        <v>0.03829999999999999</v>
       </c>
     </row>
     <row r="29">
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.00635</v>
+        <v>0.00655</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>94</v>
@@ -3550,13 +3550,13 @@
         <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03938333333333333</v>
+        <v>0.03961666666666665</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1906166666666667</v>
+        <v>0.19305</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0035</v>
+        <v>0.0034</v>
       </c>
     </row>
     <row r="30">
@@ -3575,7 +3575,7 @@
         <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0037</v>
+        <v>0.0035</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>90</v>
@@ -3584,13 +3584,13 @@
         <v>284</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.03023333333333334</v>
+        <v>0.03005000000000001</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1284516666666666</v>
+        <v>0.127585</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.00295</v>
+        <v>0.0031</v>
       </c>
     </row>
     <row r="31">
@@ -3609,7 +3609,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.01765</v>
+        <v>0.01725</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>104</v>
@@ -3618,13 +3618,13 @@
         <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.063</v>
+        <v>0.06161666666666666</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2202933333333333</v>
+        <v>0.21649</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.001766666666666667</v>
+        <v>0.001916666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3643,22 +3643,22 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.005083333333333333</v>
+        <v>0.005483333333333333</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.02937</v>
+        <v>0.03045</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1988016666666667</v>
+        <v>0.2019316666666667</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.004</v>
+        <v>0.00375</v>
       </c>
     </row>
     <row r="33">
@@ -3680,7 +3680,7 @@
         <v>5e-05</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>218</v>
@@ -3689,10 +3689,10 @@
         <v>0.003</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05064999999999999</v>
+        <v>0.05101666666666666</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02611666666666666</v>
+        <v>0.02491666666666667</v>
       </c>
     </row>
     <row r="34">
@@ -3720,13 +3720,13 @@
         <v>224</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.00125</v>
+        <v>0.0014</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.032025</v>
+        <v>0.03310833333333333</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.04228333333333333</v>
+        <v>0.04113333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00575</v>
+        <v>0.0052</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>98</v>
@@ -3754,13 +3754,13 @@
         <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03175</v>
+        <v>0.03218333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1998466666666667</v>
+        <v>0.2024483333333333</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.0057</v>
+        <v>0.0055</v>
       </c>
     </row>
     <row r="36">
@@ -3779,7 +3779,7 @@
         <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.0025</v>
+        <v>0.0026</v>
       </c>
       <c r="F36" s="8" t="n">
         <v>88</v>
@@ -3788,10 +3788,10 @@
         <v>236</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01976666666666667</v>
+        <v>0.01985</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1247233333333333</v>
+        <v>0.12738</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0002</v>
@@ -3822,13 +3822,13 @@
         <v>250</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.007766666666666667</v>
+        <v>0.007366666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.106545</v>
+        <v>0.10495</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.008933333333333335</v>
+        <v>0.009433333333333334</v>
       </c>
     </row>
     <row r="38">
@@ -3850,7 +3850,7 @@
         <v>0.0001</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G38" s="8" t="n">
         <v>207</v>
@@ -3859,10 +3859,10 @@
         <v>0.0014</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.04048333333333334</v>
+        <v>0.03863333333333334</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.09233333333333336</v>
+        <v>0.0977666666666667</v>
       </c>
     </row>
     <row r="39">
@@ -3890,13 +3890,13 @@
         <v>254</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01498333333333333</v>
+        <v>0.01508333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.06461666666666667</v>
+        <v>0.06494999999999999</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.07443333333333334</v>
+        <v>0.07283333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3915,7 +3915,7 @@
         <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00195</v>
+        <v>0.00185</v>
       </c>
       <c r="F40" s="8" t="n">
         <v>69</v>
@@ -3924,13 +3924,13 @@
         <v>253</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.008449999999999999</v>
+        <v>0.00825</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.0428</v>
+        <v>0.0425</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.125425</v>
+        <v>0.12795</v>
       </c>
     </row>
     <row r="41">
@@ -3949,7 +3949,7 @@
         <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.00245</v>
+        <v>0.0026</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>81</v>
@@ -3958,13 +3958,13 @@
         <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01465</v>
+        <v>0.01495</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07325833333333334</v>
+        <v>0.07494166666666666</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.02175</v>
+        <v>0.02135</v>
       </c>
     </row>
     <row r="42">
@@ -3983,22 +3983,22 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00065</v>
+        <v>0.00085</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>185</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.00335</v>
+        <v>0.00395</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.01993333333333333</v>
+        <v>0.02083333333333334</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.29845</v>
+        <v>0.2903</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 18:24:02 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T22:01:00.058685+00:00</t>
+          <t>2026-03-21T22:24:01.897148+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8822709529859037</v>
+        <v>0.8521002889680528</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1177290470140962</v>
+        <v>0.1478997110319473</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1674779918985809</v>
+        <v>0.1662357816377033</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8325220081014191</v>
+        <v>0.8337642183622967</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.2008656676452992</v>
+        <v>0.1872230695809393</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.7991343323547009</v>
+        <v>0.8127769304190607</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2484,10 +2484,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.312028614752377</v>
+        <v>0.3139572100143057</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6879713852476229</v>
+        <v>0.6860427899856943</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1554333333333333</v>
+        <v>0.1568</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>140</v>
@@ -2632,10 +2632,10 @@
         <v>360</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3830333333333333</v>
+        <v>0.3836833333333334</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7543333333333335</v>
+        <v>0.7545500000000001</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,7 +2657,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06961666666666666</v>
+        <v>0.06981666666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>120</v>
@@ -2666,13 +2666,13 @@
         <v>294</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.178925</v>
+        <v>0.179125</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4298016666666667</v>
+        <v>0.4313766666666668</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.00235</v>
+        <v>0.00225</v>
       </c>
     </row>
     <row r="4">
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07463333333333333</v>
+        <v>0.07518333333333332</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>117</v>
@@ -2700,13 +2700,13 @@
         <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1736583333333333</v>
+        <v>0.1742083333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4137566666666667</v>
+        <v>0.4132066666666667</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.0009</v>
+        <v>0.0009333333333333332</v>
       </c>
     </row>
     <row r="5">
@@ -2725,22 +2725,22 @@
         <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.02128333333333333</v>
+        <v>0.0205</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>326</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1138</v>
+        <v>0.1120666666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5066933333333331</v>
+        <v>0.5019933333333332</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="6">
@@ -2759,7 +2759,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.1432833333333333</v>
+        <v>0.1406</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>138</v>
@@ -2768,10 +2768,10 @@
         <v>297</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3302333333333333</v>
+        <v>0.3249866666666666</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.7056833333333333</v>
+        <v>0.7015666666666667</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.08041666666666666</v>
+        <v>0.0801</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>119</v>
@@ -2802,13 +2802,13 @@
         <v>323</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1939833333333333</v>
+        <v>0.1935666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4507500000000001</v>
+        <v>0.4496233333333333</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="8">
@@ -2827,19 +2827,19 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0677</v>
+        <v>0.06856666666666668</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1856333333333333</v>
+        <v>0.1869533333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4953516666666667</v>
+        <v>0.4977933333333334</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,7 +2861,7 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.05848333333333332</v>
+        <v>0.05908333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>108</v>
@@ -2870,13 +2870,13 @@
         <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1524666666666666</v>
+        <v>0.1537533333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3510083333333334</v>
+        <v>0.3516583333333334</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.00065</v>
       </c>
     </row>
     <row r="10">
@@ -2895,7 +2895,7 @@
         <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.00275</v>
+        <v>0.0028</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>114</v>
@@ -2907,7 +2907,7 @@
         <v>0.03040000000000001</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2722666666666667</v>
+        <v>0.2711333333333333</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.0008</v>
@@ -2929,7 +2929,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04323333333333334</v>
+        <v>0.04341666666666667</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>108</v>
@@ -2938,10 +2938,10 @@
         <v>281</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1247</v>
+        <v>0.1253</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3144666666666667</v>
+        <v>0.3156</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.003783333333333333</v>
@@ -2963,7 +2963,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02458333333333334</v>
+        <v>0.02503333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>120</v>
@@ -2972,13 +2972,13 @@
         <v>320</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09975833333333334</v>
+        <v>0.1020916666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4374333333333334</v>
+        <v>0.4409</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.001083333333333334</v>
+        <v>0.0009833333333333335</v>
       </c>
     </row>
     <row r="13">
@@ -2997,7 +2997,7 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.01605</v>
+        <v>0.01665</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>119</v>
@@ -3006,13 +3006,13 @@
         <v>336</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08359999999999999</v>
+        <v>0.08526666666666666</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3901333333333334</v>
+        <v>0.3938233333333334</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.00125</v>
+        <v>0.0011</v>
       </c>
     </row>
     <row r="14">
@@ -3031,22 +3031,22 @@
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.0069</v>
+        <v>0.00735</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>82</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>248</v>
+        <v>290</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.01885</v>
+        <v>0.02005</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.07112499999999999</v>
+        <v>0.07398333333333333</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01881666666666667</v>
+        <v>0.01868333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -3065,7 +3065,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.04023333333333334</v>
+        <v>0.04018333333333333</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>109</v>
@@ -3074,10 +3074,10 @@
         <v>245</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.1204916666666667</v>
+        <v>0.1214416666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3521766666666666</v>
+        <v>0.3537933333333333</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00225</v>
@@ -3099,19 +3099,19 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.01003333333333333</v>
+        <v>0.009633333333333332</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>112</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.049775</v>
+        <v>0.050025</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3023666666666666</v>
+        <v>0.3038583333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>8.333333333333333e-05</v>
@@ -3133,7 +3133,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.002233333333333334</v>
+        <v>0.002083333333333333</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>111</v>
@@ -3142,10 +3142,10 @@
         <v>268</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04353333333333334</v>
+        <v>0.04373333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2399583333333333</v>
+        <v>0.24055</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0.00025</v>
@@ -3167,7 +3167,7 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.01193333333333333</v>
+        <v>0.01208333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>86</v>
@@ -3176,13 +3176,13 @@
         <v>261</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.04526666666666667</v>
+        <v>0.04551666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1482416666666667</v>
+        <v>0.1495916666666667</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.0441</v>
+        <v>0.04315</v>
       </c>
     </row>
     <row r="19">
@@ -3201,7 +3201,7 @@
         <v>9</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.0103</v>
+        <v>0.0095</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>85</v>
@@ -3210,13 +3210,13 @@
         <v>242</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03105</v>
+        <v>0.0297</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1191</v>
+        <v>0.11605</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.01906666666666667</v>
+        <v>0.01875</v>
       </c>
     </row>
     <row r="20">
@@ -3235,7 +3235,7 @@
         <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.00425</v>
+        <v>0.004466666666666667</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>108</v>
@@ -3244,10 +3244,10 @@
         <v>276</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02830833333333334</v>
+        <v>0.02882500000000001</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2161433333333333</v>
+        <v>0.2183933333333333</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.0006833333333333334</v>
@@ -3269,7 +3269,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.003833333333333334</v>
+        <v>0.003683333333333334</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
@@ -3278,13 +3278,13 @@
         <v>259</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.03398333333333332</v>
+        <v>0.03326999999999999</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2623083333333333</v>
+        <v>0.2601999999999999</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.00265</v>
+        <v>0.002625</v>
       </c>
     </row>
     <row r="22">
@@ -3312,10 +3312,10 @@
         <v>314</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.0198</v>
+        <v>0.01975</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2737083333333333</v>
+        <v>0.2730983333333334</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0015</v>
@@ -3346,10 +3346,10 @@
         <v>271</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01836666666666667</v>
+        <v>0.01905</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.200625</v>
+        <v>0.20445</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -3383,10 +3383,10 @@
         <v>0.00545</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.03158333333333333</v>
+        <v>0.03218333333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.123</v>
+        <v>0.12105</v>
       </c>
     </row>
     <row r="25">
@@ -3405,7 +3405,7 @@
         <v>10</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.0618</v>
+        <v>0.06205</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>109</v>
@@ -3414,13 +3414,13 @@
         <v>276</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.1375833333333333</v>
+        <v>0.1375666666666666</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3468999999999999</v>
+        <v>0.3466066666666666</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.003733333333333333</v>
+        <v>0.004033333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3448,13 +3448,13 @@
         <v>239</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.08563333333333334</v>
+        <v>0.08478333333333334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2401749999999999</v>
+        <v>0.2393999999999999</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01778333333333334</v>
+        <v>0.01833333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -3473,7 +3473,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.007583333333333334</v>
+        <v>0.007483333333333334</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>91</v>
@@ -3482,13 +3482,13 @@
         <v>198</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02835</v>
+        <v>0.0277</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1231833333333334</v>
+        <v>0.1217083333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01271666666666667</v>
+        <v>0.01299166666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3507,7 +3507,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00265</v>
+        <v>0.00245</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>75</v>
@@ -3516,13 +3516,13 @@
         <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.0142</v>
+        <v>0.013</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.05090833333333334</v>
+        <v>0.04790000000000001</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.03829999999999999</v>
+        <v>0.03837499999999999</v>
       </c>
     </row>
     <row r="29">
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.00655</v>
+        <v>0.0063</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>94</v>
@@ -3550,13 +3550,13 @@
         <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03961666666666665</v>
+        <v>0.03938333333333333</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.19305</v>
+        <v>0.1916</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0034</v>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="30">
@@ -3584,13 +3584,13 @@
         <v>284</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.03005000000000001</v>
+        <v>0.03023333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.127585</v>
+        <v>0.1284016666666666</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.0031</v>
+        <v>0.00295</v>
       </c>
     </row>
     <row r="31">
@@ -3609,7 +3609,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.01725</v>
+        <v>0.01755</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>104</v>
@@ -3618,13 +3618,13 @@
         <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.06161666666666666</v>
+        <v>0.0622</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.21649</v>
+        <v>0.2191066666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.001916666666666667</v>
+        <v>0.001666666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3643,22 +3643,22 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.005483333333333333</v>
+        <v>0.005233333333333333</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03045</v>
+        <v>0.02997</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2019316666666667</v>
+        <v>0.2002066666666667</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00375</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="33">
@@ -3680,7 +3680,7 @@
         <v>5e-05</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>80</v>
+        <v>79.5</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>218</v>
@@ -3689,10 +3689,10 @@
         <v>0.003</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05101666666666666</v>
+        <v>0.05068333333333333</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02491666666666667</v>
+        <v>0.02556666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3720,13 +3720,13 @@
         <v>224</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0014</v>
+        <v>0.0013</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03310833333333333</v>
+        <v>0.032225</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.04113333333333333</v>
+        <v>0.04158333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.0052</v>
+        <v>0.00545</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>98</v>
@@ -3754,10 +3754,10 @@
         <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03218333333333333</v>
+        <v>0.03213333333333334</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.2024483333333333</v>
+        <v>0.2010233333333333</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0.0055</v>
@@ -3779,7 +3779,7 @@
         <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.0026</v>
+        <v>0.00245</v>
       </c>
       <c r="F36" s="8" t="n">
         <v>88</v>
@@ -3788,10 +3788,10 @@
         <v>236</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01985</v>
+        <v>0.01976666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.12738</v>
+        <v>0.1258033333333333</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0002</v>
@@ -3822,13 +3822,13 @@
         <v>250</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.007366666666666667</v>
+        <v>0.007566666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.10495</v>
+        <v>0.1056</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.009433333333333334</v>
+        <v>0.009033333333333334</v>
       </c>
     </row>
     <row r="38">
@@ -3859,10 +3859,10 @@
         <v>0.0014</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.03863333333333334</v>
+        <v>0.03935</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.0977666666666667</v>
+        <v>0.09433333333333337</v>
       </c>
     </row>
     <row r="39">
@@ -3890,13 +3890,13 @@
         <v>254</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01508333333333333</v>
+        <v>0.01513333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.06494999999999999</v>
+        <v>0.06501666666666668</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.07283333333333333</v>
+        <v>0.07298333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3924,13 +3924,13 @@
         <v>253</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.00825</v>
+        <v>0.00835</v>
       </c>
       <c r="I40" s="5" t="n">
         <v>0.0425</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.12795</v>
+        <v>0.126025</v>
       </c>
     </row>
     <row r="41">
@@ -3958,10 +3958,10 @@
         <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01495</v>
+        <v>0.01505</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07494166666666666</v>
+        <v>0.07425833333333334</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.02135</v>
@@ -3983,22 +3983,22 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00085</v>
+        <v>0.00065</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>185</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.00395</v>
+        <v>0.00325</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.02083333333333334</v>
+        <v>0.01923333333333333</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2903</v>
+        <v>0.29705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 18:40:09 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T22:24:01.897148+00:00</t>
+          <t>2026-03-21T22:40:08.564535+00:00</t>
         </is>
       </c>
     </row>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8521002889680528</v>
+        <v>0.8485275315915585</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1478997110319473</v>
+        <v>0.1514724684084416</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1662357816377033</v>
+        <v>0.1652690617944636</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8337642183622967</v>
+        <v>0.8347309382055365</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1872230695809393</v>
+        <v>0.1660175086632202</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8127769304190607</v>
+        <v>0.8339824913367798</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2484,10 +2484,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3139572100143057</v>
+        <v>0.3135868253614602</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6860427899856943</v>
+        <v>0.6864131746385398</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1568</v>
+        <v>0.1563</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>140</v>
@@ -2632,10 +2632,10 @@
         <v>360</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3836833333333334</v>
+        <v>0.381825</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7545500000000001</v>
+        <v>0.7536333333333335</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,7 +2657,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06981666666666667</v>
+        <v>0.06996666666666666</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>120</v>
@@ -2666,13 +2666,13 @@
         <v>294</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.179125</v>
+        <v>0.178625</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4313766666666668</v>
+        <v>0.43046</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.00225</v>
+        <v>0.0022</v>
       </c>
     </row>
     <row r="4">
@@ -2691,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07518333333333332</v>
+        <v>0.07553333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>117</v>
@@ -2700,10 +2700,10 @@
         <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1742083333333333</v>
+        <v>0.1752583333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4132066666666667</v>
+        <v>0.4153233333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0.0009333333333333332</v>
@@ -2725,7 +2725,7 @@
         <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.0205</v>
+        <v>0.02065</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>123</v>
@@ -2734,10 +2734,10 @@
         <v>326</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1120666666666667</v>
+        <v>0.1116416666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5019933333333332</v>
+        <v>0.5020599999999998</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0002</v>
@@ -2759,7 +2759,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.1406</v>
+        <v>0.13965</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>138</v>
@@ -2768,10 +2768,10 @@
         <v>297</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3249866666666666</v>
+        <v>0.32412</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.7015666666666667</v>
+        <v>0.7001833333333334</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0801</v>
+        <v>0.08055</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>119</v>
@@ -2802,10 +2802,10 @@
         <v>323</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1935666666666667</v>
+        <v>0.1946166666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4496233333333333</v>
+        <v>0.4519066666666667</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0002</v>
@@ -2827,7 +2827,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06856666666666668</v>
+        <v>0.06861666666666667</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>126</v>
@@ -2836,10 +2836,10 @@
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1869533333333333</v>
+        <v>0.1872533333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4977933333333334</v>
+        <v>0.4989266666666667</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,7 +2861,7 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.05908333333333333</v>
+        <v>0.05968333333333332</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>108</v>
@@ -2870,10 +2870,10 @@
         <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1537533333333333</v>
+        <v>0.1547866666666667</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3516583333333334</v>
+        <v>0.353125</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00065</v>
@@ -2904,13 +2904,13 @@
         <v>319</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.03040000000000001</v>
+        <v>0.03023333333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2711333333333333</v>
+        <v>0.2713833333333333</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0008</v>
+        <v>0.00085</v>
       </c>
     </row>
     <row r="11">
@@ -2929,7 +2929,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04341666666666667</v>
+        <v>0.04351666666666667</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>108</v>
@@ -2938,13 +2938,13 @@
         <v>281</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1253</v>
+        <v>0.1254</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3156</v>
+        <v>0.31495</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.003783333333333333</v>
+        <v>0.003683333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -2963,7 +2963,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02503333333333333</v>
+        <v>0.02523333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>120</v>
@@ -2972,13 +2972,13 @@
         <v>320</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1020916666666667</v>
+        <v>0.1034416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4409</v>
+        <v>0.4441666666666667</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.0009833333333333335</v>
+        <v>0.0009333333333333334</v>
       </c>
     </row>
     <row r="13">
@@ -2997,7 +2997,7 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.01665</v>
+        <v>0.01725</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>119</v>
@@ -3006,13 +3006,13 @@
         <v>336</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08526666666666666</v>
+        <v>0.08679999999999999</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3938233333333334</v>
+        <v>0.3971066666666666</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0011</v>
+        <v>0.00105</v>
       </c>
     </row>
     <row r="14">
@@ -3031,7 +3031,7 @@
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.00735</v>
+        <v>0.00695</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>82</v>
@@ -3040,13 +3040,13 @@
         <v>290</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.02005</v>
+        <v>0.0193</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.07398333333333333</v>
+        <v>0.07201666666666666</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01868333333333334</v>
+        <v>0.01878333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -3065,7 +3065,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.04018333333333333</v>
+        <v>0.04003333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>109</v>
@@ -3074,10 +3074,10 @@
         <v>245</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.1214416666666667</v>
+        <v>0.1213416666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3537933333333333</v>
+        <v>0.3533766666666666</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00225</v>
@@ -3099,7 +3099,7 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.009633333333333332</v>
+        <v>0.009533333333333333</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>112</v>
@@ -3108,10 +3108,10 @@
         <v>300</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.050025</v>
+        <v>0.050575</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3038583333333333</v>
+        <v>0.3048416666666666</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>8.333333333333333e-05</v>
@@ -3145,7 +3145,7 @@
         <v>0.04373333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.24055</v>
+        <v>0.2411666666666666</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0.00025</v>
@@ -3167,7 +3167,7 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.01208333333333333</v>
+        <v>0.01243333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>86</v>
@@ -3176,13 +3176,13 @@
         <v>261</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.04551666666666667</v>
+        <v>0.04586666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1495916666666667</v>
+        <v>0.1502916666666667</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.04315</v>
+        <v>0.04175</v>
       </c>
     </row>
     <row r="19">
@@ -3201,19 +3201,19 @@
         <v>9</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.0095</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G19" s="9" t="n">
         <v>242</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.0297</v>
+        <v>0.02756666666666666</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.11605</v>
+        <v>0.1123333333333334</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.01875</v>
@@ -3244,10 +3244,10 @@
         <v>276</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02882500000000001</v>
+        <v>0.028875</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2183933333333333</v>
+        <v>0.2187266666666667</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.0006833333333333334</v>
@@ -3269,7 +3269,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.003683333333333334</v>
+        <v>0.003583333333333334</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
@@ -3278,13 +3278,13 @@
         <v>259</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.03326999999999999</v>
+        <v>0.03291999999999999</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2601999999999999</v>
+        <v>0.2591499999999999</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.002625</v>
+        <v>0.002575</v>
       </c>
     </row>
     <row r="22">
@@ -3312,10 +3312,10 @@
         <v>314</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.01975</v>
+        <v>0.0193</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2730983333333334</v>
+        <v>0.2724150000000001</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0015</v>
@@ -3337,7 +3337,7 @@
         <v>8</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.003233333333333333</v>
+        <v>0.003333333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>108</v>
@@ -3346,13 +3346,13 @@
         <v>271</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01905</v>
+        <v>0.01925</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.20445</v>
+        <v>0.2049833333333334</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="24">
@@ -3383,10 +3383,10 @@
         <v>0.00545</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.03218333333333333</v>
+        <v>0.03208333333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.12105</v>
+        <v>0.11945</v>
       </c>
     </row>
     <row r="25">
@@ -3405,7 +3405,7 @@
         <v>10</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.06205</v>
+        <v>0.0624</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>109</v>
@@ -3414,13 +3414,13 @@
         <v>276</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.1375666666666666</v>
+        <v>0.1381916666666667</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3466066666666666</v>
+        <v>0.3477399999999999</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.004033333333333333</v>
+        <v>0.003833333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3442,19 +3442,19 @@
         <v>0.02653333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>239</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.08478333333333334</v>
+        <v>0.08481666666666668</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2393999999999999</v>
+        <v>0.2388666666666666</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01833333333333333</v>
+        <v>0.01798333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -3473,7 +3473,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.007483333333333334</v>
+        <v>0.007583333333333334</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>91</v>
@@ -3485,10 +3485,10 @@
         <v>0.0277</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1217083333333334</v>
+        <v>0.1216416666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01299166666666667</v>
+        <v>0.01309166666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3507,7 +3507,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00245</v>
+        <v>0.00235</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>75</v>
@@ -3516,13 +3516,13 @@
         <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.013</v>
+        <v>0.01205</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.04790000000000001</v>
+        <v>0.04555000000000001</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.03837499999999999</v>
+        <v>0.03937499999999999</v>
       </c>
     </row>
     <row r="29">
@@ -3550,13 +3550,13 @@
         <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03938333333333333</v>
+        <v>0.03965</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>0.1916</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0035</v>
+        <v>0.0034</v>
       </c>
     </row>
     <row r="30">
@@ -3584,10 +3584,10 @@
         <v>284</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.03023333333333334</v>
+        <v>0.03043333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1284016666666666</v>
+        <v>0.1283183333333333</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0.00295</v>
@@ -3609,7 +3609,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.01755</v>
+        <v>0.0176</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>104</v>
@@ -3618,13 +3618,13 @@
         <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.0622</v>
+        <v>0.06294166666666666</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2191066666666667</v>
+        <v>0.21999</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.001666666666666667</v>
+        <v>0.001566666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3643,7 +3643,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.005233333333333333</v>
+        <v>0.005033333333333333</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>99</v>
@@ -3652,10 +3652,10 @@
         <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.02997</v>
+        <v>0.02962</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.2002066666666667</v>
+        <v>0.1999566666666667</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.004</v>
@@ -3680,7 +3680,7 @@
         <v>5e-05</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>79.5</v>
+        <v>79</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>218</v>
@@ -3689,10 +3689,10 @@
         <v>0.003</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05068333333333333</v>
+        <v>0.05034999999999999</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02556666666666666</v>
+        <v>0.02586666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3720,13 +3720,13 @@
         <v>224</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0013</v>
+        <v>0.0014</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.032225</v>
+        <v>0.03209166666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.04158333333333333</v>
+        <v>0.04153333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00545</v>
+        <v>0.00555</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>98</v>
@@ -3754,10 +3754,10 @@
         <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03213333333333334</v>
+        <v>0.03208333333333334</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.2010233333333333</v>
+        <v>0.1995233333333334</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0.0055</v>
@@ -3788,10 +3788,10 @@
         <v>236</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01976666666666667</v>
+        <v>0.01986666666666666</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1258033333333333</v>
+        <v>0.1255366666666666</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0002</v>
@@ -3822,10 +3822,10 @@
         <v>250</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.007566666666666667</v>
+        <v>0.007316666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1056</v>
+        <v>0.10515</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>0.009033333333333334</v>
@@ -3859,10 +3859,10 @@
         <v>0.0014</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.03935</v>
+        <v>0.03950000000000001</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.09433333333333337</v>
+        <v>0.09398333333333336</v>
       </c>
     </row>
     <row r="39">
@@ -3890,13 +3890,13 @@
         <v>254</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01513333333333333</v>
+        <v>0.01538333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.06501666666666668</v>
+        <v>0.06536666666666667</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.07298333333333333</v>
+        <v>0.07103333333333334</v>
       </c>
     </row>
     <row r="40">
@@ -3927,10 +3927,10 @@
         <v>0.00835</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.0425</v>
+        <v>0.04251666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.126025</v>
+        <v>0.126225</v>
       </c>
     </row>
     <row r="41">
@@ -3958,13 +3958,13 @@
         <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01505</v>
+        <v>0.01486666666666667</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07425833333333334</v>
+        <v>0.07415833333333334</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.02135</v>
+        <v>0.0203</v>
       </c>
     </row>
     <row r="42">
@@ -3983,7 +3983,7 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00065</v>
+        <v>0.00055</v>
       </c>
       <c r="F42" s="8" t="n">
         <v>53</v>
@@ -3992,13 +3992,13 @@
         <v>185</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.00325</v>
+        <v>0.00275</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.01923333333333333</v>
+        <v>0.01753333333333333</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.29705</v>
+        <v>0.3028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 19:03:15 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T22:40:08.564535+00:00</t>
+          <t>2026-03-21T23:03:14.704086+00:00</t>
         </is>
       </c>
     </row>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.8485275315915585</v>
+        <v>0.7764810236180187</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.1514724684084416</v>
+        <v>0.2235189763819813</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1652690617944636</v>
+        <v>0.1651388802254331</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8347309382055365</v>
+        <v>0.8348611197745669</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1660175086632202</v>
+        <v>0.07057959088592061</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.8339824913367798</v>
+        <v>0.9294204091140793</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2484,10 +2484,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3135868253614602</v>
+        <v>0.3135519465323415</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6864131746385398</v>
+        <v>0.6864480534676586</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1563</v>
+        <v>0.1558666666666667</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>140</v>
@@ -2632,10 +2632,10 @@
         <v>360</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.381825</v>
+        <v>0.3792416666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7536333333333335</v>
+        <v>0.75077</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,22 +2657,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06996666666666666</v>
+        <v>0.06953333333333332</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>120</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.178625</v>
+        <v>0.1780083333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.43046</v>
+        <v>0.4317016666666667</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.0022</v>
+        <v>0.00195</v>
       </c>
     </row>
     <row r="4">
@@ -2691,22 +2691,22 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07553333333333333</v>
+        <v>0.07863333333333332</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>117</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1752583333333333</v>
+        <v>0.179975</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4153233333333334</v>
+        <v>0.4218166666666666</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.0009333333333333332</v>
+        <v>0.0004833333333333334</v>
       </c>
     </row>
     <row r="5">
@@ -2725,7 +2725,7 @@
         <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.02065</v>
+        <v>0.01905</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>123</v>
@@ -2734,10 +2734,10 @@
         <v>326</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1116416666666667</v>
+        <v>0.1080083333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5020599999999998</v>
+        <v>0.4930883333333333</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0002</v>
@@ -2759,19 +2759,19 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.13965</v>
+        <v>0.13115</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>297</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.32412</v>
+        <v>0.3113533333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.7001833333333334</v>
+        <v>0.6868000000000002</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2793,19 +2793,19 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.08055</v>
+        <v>0.0814</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>119</v>
+        <v>119.5</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>323</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1946166666666667</v>
+        <v>0.19815</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4519066666666667</v>
+        <v>0.45566</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0.0002</v>
@@ -2827,7 +2827,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06861666666666667</v>
+        <v>0.07020000000000001</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>126</v>
@@ -2836,10 +2836,10 @@
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1872533333333333</v>
+        <v>0.1924033333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4989266666666667</v>
+        <v>0.5043433333333334</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,22 +2861,22 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.05968333333333332</v>
+        <v>0.06391666666666666</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1547866666666667</v>
+        <v>0.1602533333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.353125</v>
+        <v>0.358525</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00065</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="10">
@@ -2895,7 +2895,7 @@
         <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0028</v>
+        <v>0.00305</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>114</v>
@@ -2907,10 +2907,10 @@
         <v>0.03023333333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2713833333333333</v>
+        <v>0.270325</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.00085</v>
+        <v>0.00105</v>
       </c>
     </row>
     <row r="11">
@@ -2929,7 +2929,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04351666666666667</v>
+        <v>0.04261666666666667</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>108</v>
@@ -2938,13 +2938,13 @@
         <v>281</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1254</v>
+        <v>0.1244166666666667</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.31495</v>
+        <v>0.3143833333333333</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.003683333333333334</v>
+        <v>0.003283333333333333</v>
       </c>
     </row>
     <row r="12">
@@ -2963,22 +2963,22 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02523333333333333</v>
+        <v>0.02715</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>320</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1034416666666667</v>
+        <v>0.111925</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4441666666666667</v>
+        <v>0.4591916666666668</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.0009333333333333334</v>
+        <v>0.0004833333333333333</v>
       </c>
     </row>
     <row r="13">
@@ -2997,22 +2997,22 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.01725</v>
+        <v>0.0192</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08679999999999999</v>
+        <v>0.09359999999999999</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3971066666666666</v>
+        <v>0.4160233333333335</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.00105</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="14">
@@ -3031,22 +3031,22 @@
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.00695</v>
+        <v>0.008149999999999999</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>82</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>290</v>
+        <v>250</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.0193</v>
+        <v>0.01938333333333334</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.07201666666666666</v>
+        <v>0.07188333333333331</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01878333333333334</v>
+        <v>0.01798333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -3065,7 +3065,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.04003333333333334</v>
+        <v>0.04066666666666667</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>109</v>
@@ -3074,13 +3074,13 @@
         <v>245</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.1213416666666667</v>
+        <v>0.1216916666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3533766666666666</v>
+        <v>0.3535916666666666</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.00225</v>
+        <v>0.00215</v>
       </c>
     </row>
     <row r="16">
@@ -3099,22 +3099,22 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.009533333333333333</v>
+        <v>0.009383333333333332</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G16" s="8" t="n">
         <v>300</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.050575</v>
+        <v>0.050325</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3048416666666666</v>
+        <v>0.310375</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>8.333333333333333e-05</v>
+        <v>5e-05</v>
       </c>
     </row>
     <row r="17">
@@ -3133,7 +3133,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.002083333333333333</v>
+        <v>0.001833333333333333</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>111</v>
@@ -3142,13 +3142,13 @@
         <v>268</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04373333333333334</v>
+        <v>0.04483333333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2411666666666666</v>
+        <v>0.2447249999999999</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.00025</v>
+        <v>0.00015</v>
       </c>
     </row>
     <row r="18">
@@ -3167,22 +3167,22 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.01243333333333333</v>
+        <v>0.01263333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>261</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.04586666666666667</v>
+        <v>0.04806666666666666</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1502916666666667</v>
+        <v>0.1572416666666666</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.04175</v>
+        <v>0.0365</v>
       </c>
     </row>
     <row r="19">
@@ -3201,22 +3201,22 @@
         <v>9</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.004983333333333334</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02756666666666666</v>
+        <v>0.01978333333333333</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1123333333333334</v>
+        <v>0.09887499999999999</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.01875</v>
+        <v>0.02035</v>
       </c>
     </row>
     <row r="20">
@@ -3235,22 +3235,22 @@
         <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.004466666666666667</v>
+        <v>0.004483333333333334</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G20" s="8" t="n">
         <v>276</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.028875</v>
+        <v>0.02915833333333334</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2187266666666667</v>
+        <v>0.2239166666666667</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.0006833333333333334</v>
+        <v>0.0002833333333333333</v>
       </c>
     </row>
     <row r="21">
@@ -3269,7 +3269,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.003583333333333334</v>
+        <v>0.003433333333333333</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
@@ -3278,13 +3278,13 @@
         <v>259</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.03291999999999999</v>
+        <v>0.03118666666666666</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2591499999999999</v>
+        <v>0.2519833333333333</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.002575</v>
+        <v>0.002708333333333333</v>
       </c>
     </row>
     <row r="22">
@@ -3312,13 +3312,13 @@
         <v>314</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.0193</v>
+        <v>0.0191</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2724150000000001</v>
+        <v>0.2683233333333334</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.0015</v>
+        <v>0.0016</v>
       </c>
     </row>
     <row r="23">
@@ -3337,7 +3337,7 @@
         <v>8</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.003333333333333333</v>
+        <v>0.003933333333333334</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>108</v>
@@ -3346,13 +3346,13 @@
         <v>271</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01925</v>
+        <v>0.0209</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2049833333333334</v>
+        <v>0.2135333333333334</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.00065</v>
       </c>
     </row>
     <row r="24">
@@ -3380,13 +3380,13 @@
         <v>180</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.00545</v>
+        <v>0.0054</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.03208333333333333</v>
+        <v>0.033</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.11945</v>
+        <v>0.1089</v>
       </c>
     </row>
     <row r="25">
@@ -3405,22 +3405,22 @@
         <v>10</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.0624</v>
+        <v>0.06411666666666667</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G25" s="9" t="n">
         <v>276</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.1381916666666667</v>
+        <v>0.1412916666666667</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3477399999999999</v>
+        <v>0.3512816666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.003833333333333333</v>
+        <v>0.003133333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3439,7 +3439,7 @@
         <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.02653333333333334</v>
+        <v>0.02578333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>93</v>
@@ -3448,13 +3448,13 @@
         <v>239</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.08481666666666668</v>
+        <v>0.08201666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2388666666666666</v>
+        <v>0.23385</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01798333333333333</v>
+        <v>0.01768333333333334</v>
       </c>
     </row>
     <row r="27">
@@ -3473,22 +3473,22 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.007583333333333334</v>
+        <v>0.006783333333333334</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G27" s="9" t="n">
         <v>198</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0277</v>
+        <v>0.0272</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1216416666666667</v>
+        <v>0.118225</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01309166666666667</v>
+        <v>0.01335833333333333</v>
       </c>
     </row>
     <row r="28">
@@ -3507,22 +3507,22 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00235</v>
+        <v>0.0011</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G28" s="8" t="n">
         <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01205</v>
+        <v>0.007183333333333334</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.04555000000000001</v>
+        <v>0.03193333333333333</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.03937499999999999</v>
+        <v>0.04139166666666666</v>
       </c>
     </row>
     <row r="29">
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.0063</v>
+        <v>0.00605</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>94</v>
@@ -3550,10 +3550,10 @@
         <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03965</v>
+        <v>0.03858333333333333</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1916</v>
+        <v>0.18915</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.0034</v>
@@ -3575,7 +3575,7 @@
         <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0035</v>
+        <v>0.0038</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>90</v>
@@ -3584,13 +3584,13 @@
         <v>284</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.03043333333333334</v>
+        <v>0.03023333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1283183333333333</v>
+        <v>0.1293433333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.00295</v>
+        <v>0.00265</v>
       </c>
     </row>
     <row r="31">
@@ -3609,22 +3609,22 @@
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.0176</v>
+        <v>0.0185</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G31" s="9" t="n">
         <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.06294166666666666</v>
+        <v>0.067175</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.21999</v>
+        <v>0.2276133333333333</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.001566666666666667</v>
+        <v>0.001016666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3643,7 +3643,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.005033333333333333</v>
+        <v>0.004716666666666667</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>99</v>
@@ -3652,13 +3652,13 @@
         <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.02962</v>
+        <v>0.02652</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1999566666666667</v>
+        <v>0.1910083333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.004</v>
+        <v>0.0038</v>
       </c>
     </row>
     <row r="33">
@@ -3686,13 +3686,13 @@
         <v>218</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.003</v>
+        <v>0.00305</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05034999999999999</v>
+        <v>0.0486</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02586666666666666</v>
+        <v>0.02691666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3714,19 +3714,19 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>224</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0014</v>
+        <v>0.0012</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03209166666666667</v>
+        <v>0.03139500000000001</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.04153333333333333</v>
+        <v>0.0428</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00555</v>
+        <v>0.00585</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>98</v>
@@ -3754,13 +3754,13 @@
         <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03208333333333334</v>
+        <v>0.03061666666666667</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1995233333333334</v>
+        <v>0.1939166666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.0055</v>
+        <v>0.00565</v>
       </c>
     </row>
     <row r="36">
@@ -3779,19 +3779,19 @@
         <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.00245</v>
+        <v>0.00255</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G36" s="8" t="n">
         <v>236</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01986666666666666</v>
+        <v>0.01966666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1255366666666666</v>
+        <v>0.123115</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0002</v>
@@ -3813,7 +3813,7 @@
         <v>8</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.001233333333333333</v>
+        <v>0.0009333333333333332</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>96</v>
@@ -3825,10 +3825,10 @@
         <v>0.007316666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.10515</v>
+        <v>0.1059666666666667</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.009033333333333334</v>
+        <v>0.008800000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -3850,19 +3850,19 @@
         <v>0.0001</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G38" s="8" t="n">
         <v>207</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.0014</v>
+        <v>0.0012</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.03950000000000001</v>
+        <v>0.0418</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.09398333333333336</v>
+        <v>0.0864</v>
       </c>
     </row>
     <row r="39">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
@@ -3881,22 +3881,22 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.002</v>
+        <v>0.0021</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01538333333333333</v>
+        <v>0.0083</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.06536666666666667</v>
+        <v>0.04289999999999999</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.07103333333333334</v>
+        <v>0.1253583333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
@@ -3915,22 +3915,22 @@
         <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00185</v>
+        <v>0.00195</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.00835</v>
+        <v>0.01553333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.04251666666666666</v>
+        <v>0.06595000000000001</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.126225</v>
+        <v>0.06478333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -3949,7 +3949,7 @@
         <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.0026</v>
+        <v>0.0024</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>81</v>
@@ -3958,13 +3958,13 @@
         <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01486666666666667</v>
+        <v>0.01441666666666667</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07415833333333334</v>
+        <v>0.07297499999999998</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.0203</v>
+        <v>0.01765</v>
       </c>
     </row>
     <row r="42">
@@ -3983,22 +3983,22 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.00055</v>
+        <v>0.0002</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>185</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.00275</v>
+        <v>0.0011</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.01753333333333333</v>
+        <v>0.0109</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.3028</v>
+        <v>0.3347333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 19:24:23 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T23:03:14.704086+00:00</t>
+          <t>2026-03-21T23:24:22.602479+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
@@ -2002,10 +2002,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0.7764810236180187</v>
+        <v>0.9711510996858042</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.2235189763819813</v>
+        <v>0.02884890031419595</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2344,10 +2344,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1651388802254331</v>
+        <v>0.1644146760095708</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8348611197745669</v>
+        <v>0.8355853239904292</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2381,10 +2381,10 @@
         <v>1</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.07057959088592061</v>
+        <v>0.04866293008447869</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>0.9294204091140793</v>
+        <v>0.9513370699155212</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2484,10 +2484,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3135519465323415</v>
+        <v>0.3161041999464038</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6864480534676586</v>
+        <v>0.6838958000535962</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,19 +2623,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1558666666666667</v>
+        <v>0.1549833333333333</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>360</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3792416666666667</v>
+        <v>0.3765916666666668</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.75077</v>
+        <v>0.7497366666666667</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,22 +2657,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06953333333333332</v>
+        <v>0.06713333333333332</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1780083333333333</v>
+        <v>0.1736083333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4317016666666667</v>
+        <v>0.4243683333333333</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.00195</v>
+        <v>0.002333333333333334</v>
       </c>
     </row>
     <row r="4">
@@ -2691,22 +2691,22 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07863333333333332</v>
+        <v>0.08233333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.179975</v>
+        <v>0.1873416666666666</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4218166666666666</v>
+        <v>0.4368883333333333</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.0004833333333333334</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="5">
@@ -2725,22 +2725,22 @@
         <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.01905</v>
+        <v>0.02213333333333333</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>326</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1080083333333333</v>
+        <v>0.122125</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4930883333333333</v>
+        <v>0.5248633333333335</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="6">
@@ -2759,19 +2759,19 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.13115</v>
+        <v>0.1481333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>297</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3113533333333333</v>
+        <v>0.3387666666666667</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.6868000000000002</v>
+        <v>0.716625</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2793,22 +2793,22 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0814</v>
+        <v>0.0856</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>119.5</v>
+        <v>120</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>323</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.19815</v>
+        <v>0.2083166666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.45566</v>
+        <v>0.4750766666666668</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -2827,19 +2827,19 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.07020000000000001</v>
+        <v>0.06508333333333333</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1924033333333333</v>
+        <v>0.1808833333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5043433333333334</v>
+        <v>0.4909933333333333</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,22 +2861,22 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.06391666666666666</v>
+        <v>0.06133333333333332</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1602533333333333</v>
+        <v>0.1593166666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.358525</v>
+        <v>0.3596</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.00035</v>
       </c>
     </row>
     <row r="10">
@@ -2895,22 +2895,22 @@
         <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.00305</v>
+        <v>0.0029</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>319</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.03023333333333334</v>
+        <v>0.02955</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.270325</v>
+        <v>0.273325</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.00105</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="11">
@@ -2929,22 +2929,22 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04261666666666667</v>
+        <v>0.04201666666666667</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>281</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1244166666666667</v>
+        <v>0.1229333333333334</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3143833333333333</v>
+        <v>0.30855</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.003283333333333333</v>
+        <v>0.003716666666666667</v>
       </c>
     </row>
     <row r="12">
@@ -2963,22 +2963,22 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02715</v>
+        <v>0.0252</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>320</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.111925</v>
+        <v>0.105825</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4591916666666668</v>
+        <v>0.4525000000000002</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.0004833333333333333</v>
+        <v>0.0003833333333333333</v>
       </c>
     </row>
     <row r="13">
@@ -2997,19 +2997,19 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.0192</v>
+        <v>0.0173</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>341</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.09359999999999999</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.4160233333333335</v>
+        <v>0.4066816666666668</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0.00075</v>
@@ -3031,22 +3031,22 @@
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.008149999999999999</v>
+        <v>0.0021</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.01938333333333334</v>
+        <v>0.005666666666666667</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.07188333333333331</v>
+        <v>0.02535833333333333</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01798333333333334</v>
+        <v>0.02228333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -3065,22 +3065,22 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.04066666666666667</v>
+        <v>0.03698333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>245</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.1216916666666667</v>
+        <v>0.1140416666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3535916666666666</v>
+        <v>0.340075</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.00215</v>
+        <v>0.0024</v>
       </c>
     </row>
     <row r="16">
@@ -3099,19 +3099,19 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.009383333333333332</v>
+        <v>0.009333333333333332</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.050325</v>
+        <v>0.04979166666666667</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.310375</v>
+        <v>0.3112583333333332</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>5e-05</v>
@@ -3133,22 +3133,22 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.001833333333333333</v>
+        <v>0.001633333333333333</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>268</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04483333333333334</v>
+        <v>0.04225</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2447249999999999</v>
+        <v>0.240125</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.00015</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="18">
@@ -3167,22 +3167,22 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.01263333333333333</v>
+        <v>0.01133333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>261</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.04806666666666666</v>
+        <v>0.0459</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1572416666666666</v>
+        <v>0.151725</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.0365</v>
+        <v>0.03813333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -3191,32 +3191,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
         <v>30</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.004983333333333334</v>
+        <v>0.003816666666666667</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>224</v>
+        <v>276</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.01978333333333333</v>
+        <v>0.02630833333333334</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.09887499999999999</v>
+        <v>0.2103166666666666</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.02035</v>
+        <v>0.0001833333333333333</v>
       </c>
     </row>
     <row r="20">
@@ -3225,32 +3225,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
         <v>30</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.004483333333333334</v>
+        <v>0.003783333333333333</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>276</v>
+        <v>224</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02915833333333334</v>
+        <v>0.01495</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2239166666666667</v>
+        <v>0.08700833333333333</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.0002833333333333333</v>
+        <v>0.02313333333333334</v>
       </c>
     </row>
     <row r="21">
@@ -3269,7 +3269,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.003433333333333333</v>
+        <v>0.00345</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
@@ -3278,13 +3278,13 @@
         <v>259</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.03118666666666666</v>
+        <v>0.03324999999999999</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2519833333333333</v>
+        <v>0.2630416666666667</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.002708333333333333</v>
+        <v>0.00205</v>
       </c>
     </row>
     <row r="22">
@@ -3306,19 +3306,19 @@
         <v>0</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>314</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.0191</v>
+        <v>0.01845</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2683233333333334</v>
+        <v>0.2685733333333334</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.0016</v>
+        <v>0.00165</v>
       </c>
     </row>
     <row r="23">
@@ -3337,22 +3337,22 @@
         <v>8</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.003933333333333334</v>
+        <v>0.003033333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>271</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.0209</v>
+        <v>0.01705</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2135333333333334</v>
+        <v>0.1929083333333333</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.00065</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="24">
@@ -3371,22 +3371,22 @@
         <v>6</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.00175</v>
+        <v>0.00145</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>180</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.0054</v>
+        <v>0.0051</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.033</v>
+        <v>0.03108333333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.1089</v>
+        <v>0.11915</v>
       </c>
     </row>
     <row r="25">
@@ -3405,7 +3405,7 @@
         <v>10</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.06411666666666667</v>
+        <v>0.06513333333333333</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>110</v>
@@ -3414,13 +3414,13 @@
         <v>276</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.1412916666666667</v>
+        <v>0.146825</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3512816666666667</v>
+        <v>0.3649816666666666</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.003133333333333333</v>
+        <v>0.002183333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3439,22 +3439,22 @@
         <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.02578333333333334</v>
+        <v>0.02638333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>239</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.08201666666666667</v>
+        <v>0.08531666666666668</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.23385</v>
+        <v>0.2413083333333333</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01768333333333334</v>
+        <v>0.01528333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -3473,22 +3473,22 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.006783333333333334</v>
+        <v>0.008</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G27" s="9" t="n">
         <v>198</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0272</v>
+        <v>0.02958333333333333</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.118225</v>
+        <v>0.1289666666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01335833333333333</v>
+        <v>0.01078333333333333</v>
       </c>
     </row>
     <row r="28">
@@ -3507,7 +3507,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0011</v>
+        <v>0.0009</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>72</v>
@@ -3516,13 +3516,13 @@
         <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.007183333333333334</v>
+        <v>0.006333333333333333</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.03193333333333333</v>
+        <v>0.02646666666666667</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.04139166666666666</v>
+        <v>0.04638333333333331</v>
       </c>
     </row>
     <row r="29">
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.00605</v>
+        <v>0.0063</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>94</v>
@@ -3550,13 +3550,13 @@
         <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03858333333333333</v>
+        <v>0.03988333333333333</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.18915</v>
+        <v>0.19625</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0034</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="30">
@@ -3575,22 +3575,22 @@
         <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0038</v>
+        <v>0.0031</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>284</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.03023333333333334</v>
+        <v>0.029</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1293433333333333</v>
+        <v>0.124885</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.00265</v>
+        <v>0.00285</v>
       </c>
     </row>
     <row r="31">
@@ -3609,22 +3609,22 @@
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.0185</v>
+        <v>0.0173</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G31" s="9" t="n">
         <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.067175</v>
+        <v>0.06214166666666665</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2276133333333333</v>
+        <v>0.2167683333333333</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.001016666666666667</v>
+        <v>0.001616666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3643,7 +3643,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.004716666666666667</v>
+        <v>0.005283333333333333</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>99</v>
@@ -3652,13 +3652,13 @@
         <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.02652</v>
+        <v>0.03018333333333333</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1910083333333333</v>
+        <v>0.203605</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0038</v>
+        <v>0.00345</v>
       </c>
     </row>
     <row r="33">
@@ -3677,7 +3677,7 @@
         <v>8</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>5e-05</v>
+        <v>0.00015</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>79</v>
@@ -3686,13 +3686,13 @@
         <v>218</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.00305</v>
+        <v>0.00295</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.0486</v>
+        <v>0.04953333333333333</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02691666666666666</v>
+        <v>0.02266666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3714,19 +3714,19 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>224</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0012</v>
+        <v>0.0019</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03139500000000001</v>
+        <v>0.03588666666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.0428</v>
+        <v>0.03721666666666667</v>
       </c>
     </row>
     <row r="35">
@@ -3745,7 +3745,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00585</v>
+        <v>0.00555</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>98</v>
@@ -3754,13 +3754,13 @@
         <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03061666666666667</v>
+        <v>0.03165</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1939166666666667</v>
+        <v>0.2021466666666666</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.00565</v>
+        <v>0.0052</v>
       </c>
     </row>
     <row r="36">
@@ -3779,19 +3779,19 @@
         <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.00255</v>
+        <v>0.00285</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G36" s="8" t="n">
         <v>236</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01966666666666667</v>
+        <v>0.0211</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.123115</v>
+        <v>0.1332366666666667</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0002</v>
@@ -3813,22 +3813,22 @@
         <v>8</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.0009333333333333332</v>
+        <v>0.0007833333333333333</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G37" s="9" t="n">
         <v>250</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.007316666666666667</v>
+        <v>0.006166666666666668</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1059666666666667</v>
+        <v>0.09859166666666665</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0101</v>
       </c>
     </row>
     <row r="38">
@@ -3850,19 +3850,19 @@
         <v>0.0001</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G38" s="8" t="n">
         <v>207</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.0012</v>
+        <v>0.0011</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.0418</v>
+        <v>0.03655</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.0864</v>
+        <v>0.1019</v>
       </c>
     </row>
     <row r="39">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
@@ -3881,22 +3881,22 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0021</v>
+        <v>0.0022</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.0083</v>
+        <v>0.01663333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04289999999999999</v>
+        <v>0.06947500000000001</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1253583333333333</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="40">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
@@ -3915,22 +3915,22 @@
         <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00195</v>
+        <v>0.00185</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.01553333333333333</v>
+        <v>0.0075</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.06595000000000001</v>
+        <v>0.04086666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.06478333333333333</v>
+        <v>0.1358</v>
       </c>
     </row>
     <row r="41">
@@ -3949,22 +3949,22 @@
         <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.0024</v>
+        <v>0.00295</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01441666666666667</v>
+        <v>0.01681666666666667</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07297499999999998</v>
+        <v>0.08035</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.01765</v>
+        <v>0.01396666666666667</v>
       </c>
     </row>
     <row r="42">
@@ -3983,22 +3983,22 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>185</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.0011</v>
+        <v>0.0009</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.0109</v>
+        <v>0.00945</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.3347333333333333</v>
+        <v>0.3138333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 19:41:47 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T23:24:22.602479+00:00</t>
+          <t>2026-03-21T23:41:46.491384+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,19 +1994,15 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G34" s="5" t="n">
-        <v>0.9711510996858042</v>
-      </c>
-      <c r="H34" s="5" t="n">
-        <v>0.02884890031419595</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="5" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr">
         <is>
           <t>R32_E_01</t>
@@ -2064,7 +2060,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2130,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2299,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2332,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2344,10 +2340,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1644146760095708</v>
+        <v>0.1645711189902212</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.8355853239904292</v>
+        <v>0.8354288810097787</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -2373,19 +2369,15 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="G45" s="7" t="n">
-        <v>0.04866293008447869</v>
-      </c>
-      <c r="H45" s="7" t="n">
-        <v>0.9513370699155212</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G45" s="7" t="inlineStr"/>
+      <c r="H45" s="7" t="inlineStr"/>
       <c r="I45" s="2" t="inlineStr">
         <is>
           <t>R32_S_04</t>
@@ -2443,7 +2435,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2468,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2484,10 +2476,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.3161041999464038</v>
+        <v>0.2080924211990313</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.6838958000535962</v>
+        <v>0.7919075788009687</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2623,19 +2615,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1549833333333333</v>
+        <v>0.1311166666666667</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>360</v>
+        <v>326</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3765916666666668</v>
+        <v>0.3420166666666666</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7497366666666667</v>
+        <v>0.7262083333333335</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2657,22 +2649,22 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06713333333333332</v>
+        <v>0.06416666666666666</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1736083333333333</v>
+        <v>0.1608</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4243683333333333</v>
+        <v>0.4012800000000001</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.002333333333333334</v>
+        <v>0.00225</v>
       </c>
     </row>
     <row r="4">
@@ -2691,22 +2683,22 @@
         <v>10</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.08233333333333333</v>
+        <v>0.07038333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G4" s="8" t="n">
         <v>300</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1873416666666666</v>
+        <v>0.1653916666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4368883333333333</v>
+        <v>0.39346</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.001333333333333333</v>
       </c>
     </row>
     <row r="5">
@@ -2725,19 +2717,19 @@
         <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.02213333333333333</v>
+        <v>0.02023333333333333</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>326</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.122125</v>
+        <v>0.1072916666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5248633333333335</v>
+        <v>0.4836433333333333</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0001</v>
@@ -2759,19 +2751,19 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.1481333333333333</v>
+        <v>0.1491</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3387666666666667</v>
+        <v>0.3374116666666667</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.716625</v>
+        <v>0.7140000000000001</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2793,7 +2785,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0856</v>
+        <v>0.08521666666666666</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>120</v>
@@ -2802,13 +2794,13 @@
         <v>323</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.2083166666666666</v>
+        <v>0.20255</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4750766666666668</v>
+        <v>0.4574666666666666</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="8">
@@ -2827,19 +2819,19 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06508333333333333</v>
+        <v>0.07468333333333334</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>280</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1808833333333333</v>
+        <v>0.2028366666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4909933333333333</v>
+        <v>0.5220766666666669</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2861,22 +2853,22 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.06133333333333332</v>
+        <v>0.06015</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>288</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1593166666666666</v>
+        <v>0.1585533333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3596</v>
+        <v>0.3648166666666667</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00035</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="10">
@@ -2895,22 +2887,22 @@
         <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0029</v>
+        <v>0.00335</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>319</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.02955</v>
+        <v>0.03540833333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.273325</v>
+        <v>0.2907666666666667</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0008</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="11">
@@ -2929,22 +2921,22 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04201666666666667</v>
+        <v>0.03558333333333333</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>281</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1229333333333334</v>
+        <v>0.1097833333333333</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.30855</v>
+        <v>0.2871666666666666</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.003716666666666667</v>
+        <v>0.004866666666666667</v>
       </c>
     </row>
     <row r="12">
@@ -2963,22 +2955,22 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.0252</v>
+        <v>0.02496666666666667</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>320</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.105825</v>
+        <v>0.09865</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4525000000000002</v>
+        <v>0.4221950000000001</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.0003833333333333333</v>
+        <v>0.001183333333333333</v>
       </c>
     </row>
     <row r="13">
@@ -2997,22 +2989,22 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.0173</v>
+        <v>0.0164</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.08253333333333332</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.4066816666666668</v>
+        <v>0.377465</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.00075</v>
+        <v>0.0017</v>
       </c>
     </row>
     <row r="14">
@@ -3031,22 +3023,22 @@
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.0021</v>
+        <v>0.01245</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>245</v>
+        <v>290</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.005666666666666667</v>
+        <v>0.03155833333333333</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.02535833333333333</v>
+        <v>0.09929166666666665</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.02228333333333334</v>
+        <v>0.01713333333333333</v>
       </c>
     </row>
     <row r="15">
@@ -3065,22 +3057,22 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.03698333333333334</v>
+        <v>0.04371666666666667</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>245</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.1140416666666667</v>
+        <v>0.1242666666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.340075</v>
+        <v>0.3526933333333333</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.0024</v>
+        <v>0.0027</v>
       </c>
     </row>
     <row r="16">
@@ -3099,22 +3091,22 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.009333333333333332</v>
+        <v>0.0107</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.04979166666666667</v>
+        <v>0.04814999999999999</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3112583333333332</v>
+        <v>0.291395</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>5e-05</v>
+        <v>0.0001833333333333333</v>
       </c>
     </row>
     <row r="17">
@@ -3133,22 +3125,22 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.001633333333333333</v>
+        <v>0.002933333333333333</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04225</v>
+        <v>0.04725833333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.240125</v>
+        <v>0.2584033333333332</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="18">
@@ -3157,32 +3149,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
         <v>30</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.01133333333333333</v>
+        <v>0.01415</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.0459</v>
+        <v>0.03958333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.151725</v>
+        <v>0.13525</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.03813333333333333</v>
+        <v>0.01865</v>
       </c>
     </row>
     <row r="19">
@@ -3191,32 +3183,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
         <v>30</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.003816666666666667</v>
+        <v>0.01343333333333333</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>276</v>
+        <v>261</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02630833333333334</v>
+        <v>0.04906666666666667</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2103166666666666</v>
+        <v>0.158175</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.0001833333333333333</v>
+        <v>0.0399</v>
       </c>
     </row>
     <row r="20">
@@ -3225,32 +3217,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
         <v>30</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.003783333333333333</v>
+        <v>0.005016666666666668</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>224</v>
+        <v>276</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.01495</v>
+        <v>0.02927500000000001</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.08700833333333333</v>
+        <v>0.2151349999999999</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.02313333333333334</v>
+        <v>0.001033333333333333</v>
       </c>
     </row>
     <row r="21">
@@ -3269,22 +3261,22 @@
         <v>9</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.00345</v>
+        <v>0.004433333333333333</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.03324999999999999</v>
+        <v>0.03372833333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2630416666666667</v>
+        <v>0.2532</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.00205</v>
+        <v>0.003225</v>
       </c>
     </row>
     <row r="22">
@@ -3306,19 +3298,19 @@
         <v>0</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>314</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.01845</v>
+        <v>0.02</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2685733333333334</v>
+        <v>0.2693200000000001</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.00165</v>
+        <v>0.001866666666666667</v>
       </c>
     </row>
     <row r="23">
@@ -3337,22 +3329,22 @@
         <v>8</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.003033333333333333</v>
+        <v>0.004283333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>271</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01705</v>
+        <v>0.02338333333333334</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1929083333333333</v>
+        <v>0.2219366666666667</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0007</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="24">
@@ -3371,22 +3363,22 @@
         <v>6</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.00145</v>
+        <v>0.00175</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>180</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.0051</v>
+        <v>0.00545</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.03108333333333333</v>
+        <v>0.03643333333333334</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.11915</v>
+        <v>0.1100666666666667</v>
       </c>
     </row>
     <row r="25">
@@ -3405,22 +3397,22 @@
         <v>10</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.06513333333333333</v>
+        <v>0.06086666666666667</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G25" s="9" t="n">
         <v>276</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.146825</v>
+        <v>0.1312</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3649816666666666</v>
+        <v>0.3301083333333333</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.002183333333333333</v>
+        <v>0.00515</v>
       </c>
     </row>
     <row r="26">
@@ -3439,22 +3431,22 @@
         <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.02638333333333334</v>
+        <v>0.02933333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>239</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.08531666666666668</v>
+        <v>0.09271666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2413083333333333</v>
+        <v>0.2535666666666667</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01528333333333333</v>
+        <v>0.01775</v>
       </c>
     </row>
     <row r="27">
@@ -3473,22 +3465,22 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.008</v>
+        <v>0.006983333333333334</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G27" s="9" t="n">
         <v>198</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.02958333333333333</v>
+        <v>0.0273</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1289666666666667</v>
+        <v>0.1166166666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01078333333333333</v>
+        <v>0.01449166666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3507,22 +3499,22 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0009</v>
+        <v>0.00375</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G28" s="8" t="n">
         <v>258</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.006333333333333333</v>
+        <v>0.0177</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.02646666666666667</v>
+        <v>0.06203333333333334</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.04638333333333331</v>
+        <v>0.03747499999999999</v>
       </c>
     </row>
     <row r="29">
@@ -3541,22 +3533,22 @@
         <v>9</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.0063</v>
+        <v>0.0073</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G29" s="9" t="n">
         <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03988333333333333</v>
+        <v>0.04466666666666666</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.19625</v>
+        <v>0.2054</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.003</v>
+        <v>0.0029</v>
       </c>
     </row>
     <row r="30">
@@ -3575,22 +3567,22 @@
         <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0031</v>
+        <v>0.00225</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>89</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>284</v>
+        <v>260</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.029</v>
+        <v>0.0222</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.124885</v>
+        <v>0.1011516666666667</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.00285</v>
+        <v>0.003533333333333334</v>
       </c>
     </row>
     <row r="31">
@@ -3609,7 +3601,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.0173</v>
+        <v>0.01788333333333333</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>104</v>
@@ -3618,13 +3610,13 @@
         <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.06214166666666665</v>
+        <v>0.062025</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2167683333333333</v>
+        <v>0.2140266666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.001616666666666667</v>
+        <v>0.002616666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3643,22 +3635,22 @@
         <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.005283333333333333</v>
+        <v>0.005983333333333333</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03018333333333333</v>
+        <v>0.03258666666666666</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.203605</v>
+        <v>0.213835</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00345</v>
+        <v>0.00355</v>
       </c>
     </row>
     <row r="33">
@@ -3677,10 +3669,10 @@
         <v>8</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.00015</v>
+        <v>0.0001</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>218</v>
@@ -3689,10 +3681,10 @@
         <v>0.00295</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.04953333333333333</v>
+        <v>0.049675</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02266666666666666</v>
+        <v>0.02771666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3714,19 +3706,19 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>224</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0019</v>
+        <v>0.0014</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03588666666666667</v>
+        <v>0.03039166666666666</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.03721666666666667</v>
+        <v>0.04666666666666667</v>
       </c>
     </row>
     <row r="35">
@@ -3745,22 +3737,22 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00555</v>
+        <v>0.00595</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G35" s="9" t="n">
         <v>234</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03165</v>
+        <v>0.03733333333333332</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.2021466666666666</v>
+        <v>0.21608</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.0052</v>
+        <v>0.004883333333333333</v>
       </c>
     </row>
     <row r="36">
@@ -3779,19 +3771,19 @@
         <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.00285</v>
+        <v>0.00235</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G36" s="8" t="n">
         <v>236</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.0211</v>
+        <v>0.02011666666666666</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1332366666666667</v>
+        <v>0.1219</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0002</v>
@@ -3813,22 +3805,22 @@
         <v>8</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.0007833333333333333</v>
+        <v>0.001183333333333333</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G37" s="9" t="n">
         <v>250</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.006166666666666668</v>
+        <v>0.008691666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.09859166666666665</v>
+        <v>0.107395</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0101</v>
+        <v>0.0094</v>
       </c>
     </row>
     <row r="38">
@@ -3847,22 +3839,22 @@
         <v>6</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="G38" s="8" t="n">
         <v>207</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.0011</v>
+        <v>0.0018</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.03655</v>
+        <v>0.04501666666666668</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1019</v>
+        <v>0.08153333333333335</v>
       </c>
     </row>
     <row r="39">
@@ -3871,7 +3863,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
@@ -3881,22 +3873,22 @@
         <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0022</v>
+        <v>0.002</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01663333333333333</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.06947500000000001</v>
+        <v>0.04198333333333333</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.055</v>
+        <v>0.1316083333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3905,7 +3897,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
@@ -3915,22 +3907,22 @@
         <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00185</v>
+        <v>0.002</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.0075</v>
+        <v>0.01446666666666667</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.04086666666666666</v>
+        <v>0.06198333333333333</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1358</v>
+        <v>0.08555</v>
       </c>
     </row>
     <row r="41">
@@ -3949,22 +3941,22 @@
         <v>8</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.00295</v>
+        <v>0.00245</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>221</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.01681666666666667</v>
+        <v>0.0138</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.08035</v>
+        <v>0.07017500000000002</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.01396666666666667</v>
+        <v>0.02625000000000001</v>
       </c>
     </row>
     <row r="42">
@@ -3983,22 +3975,22 @@
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.0012</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>185</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.0009</v>
+        <v>0.0057</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.00945</v>
+        <v>0.02688333333333333</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.3138333333333333</v>
+        <v>0.2905333333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 20:00:34 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>beb794c701680ae0</t>
+          <t>7c39954d7e69400c</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>642a0a38c44454af</t>
+          <t>beb794c701680ae0</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>27</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21T23:41:46.491384+00:00</t>
+          <t>2026-03-22T00:00:33.369382+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,10 +1994,14 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr"/>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Duke</t>
+        </is>
+      </c>
       <c r="F34" s="4" t="b">
         <v>0</v>
       </c>
@@ -2060,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2130,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2299,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2332,19 +2336,15 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G44" s="5" t="n">
-        <v>0.1645711189902212</v>
-      </c>
-      <c r="H44" s="5" t="n">
-        <v>0.8354288810097787</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G44" s="5" t="inlineStr"/>
+      <c r="H44" s="5" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
         <is>
           <t>R32_S_03</t>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2476,10 +2476,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.2080924211990313</v>
+        <v>0.4008903706569034</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.7919075788009687</v>
+        <v>0.5991096293430965</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2615,19 +2615,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1311166666666667</v>
+        <v>0.1735333333333333</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3420166666666666</v>
+        <v>0.3958083333333333</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7262083333333335</v>
+        <v>0.7542550000000001</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2639,32 +2639,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Stephen Mason</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
         <v>40</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.06416666666666666</v>
+        <v>0.07498333333333333</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>117</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>302</v>
+        <v>324</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1608</v>
+        <v>0.1751</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4012800000000001</v>
+        <v>0.4155783333333334</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.00225</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -2673,32 +2673,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Stephen Mason</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07038333333333333</v>
+        <v>0.07078333333333334</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1653916666666667</v>
+        <v>0.1896416666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.39346</v>
+        <v>0.4449499999999999</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.001333333333333333</v>
+        <v>0.00245</v>
       </c>
     </row>
     <row r="5">
@@ -2711,28 +2711,28 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.02023333333333333</v>
+        <v>0.0235</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1072916666666667</v>
+        <v>0.1299916666666666</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4836433333333333</v>
+        <v>0.5342116666666669</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.00015</v>
       </c>
     </row>
     <row r="6">
@@ -2745,25 +2745,25 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.1491</v>
+        <v>0.1368166666666667</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3374116666666667</v>
+        <v>0.3175083333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.7140000000000001</v>
+        <v>0.7046116666666666</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2779,28 +2779,28 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.08521666666666666</v>
+        <v>0.07666666666666666</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.20255</v>
+        <v>0.1850666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4574666666666666</v>
+        <v>0.4468033333333333</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.0001</v>
+        <v>5e-05</v>
       </c>
     </row>
     <row r="8">
@@ -2819,19 +2819,19 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.07468333333333334</v>
+        <v>0.06253333333333333</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.2028366666666667</v>
+        <v>0.1635833333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5220766666666669</v>
+        <v>0.4752900000000002</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2853,22 +2853,22 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.06015</v>
+        <v>0.0463</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>288</v>
+        <v>264</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1585533333333333</v>
+        <v>0.1386</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3648166666666667</v>
+        <v>0.333295</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.0007</v>
+        <v>0.0011</v>
       </c>
     </row>
     <row r="10">
@@ -2887,22 +2887,22 @@
         <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.00335</v>
+        <v>0.0019</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.03540833333333334</v>
+        <v>0.02383333333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2907666666666667</v>
+        <v>0.26107</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0007</v>
+        <v>0.00165</v>
       </c>
     </row>
     <row r="11">
@@ -2921,22 +2921,22 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.03558333333333333</v>
+        <v>0.04926666666666666</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1097833333333333</v>
+        <v>0.1332833333333333</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.2871666666666666</v>
+        <v>0.3322166666666665</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.004866666666666667</v>
+        <v>0.0052</v>
       </c>
     </row>
     <row r="12">
@@ -2955,22 +2955,22 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02496666666666667</v>
+        <v>0.02028333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>119</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09865</v>
+        <v>0.09502500000000003</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4221950000000001</v>
+        <v>0.4334549999999999</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.001183333333333333</v>
+        <v>0.0009166666666666666</v>
       </c>
     </row>
     <row r="13">
@@ -2989,22 +2989,22 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.0164</v>
+        <v>0.0146</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>336</v>
+        <v>347</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08253333333333332</v>
+        <v>0.08094999999999999</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.377465</v>
+        <v>0.3797083333333333</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0017</v>
+        <v>0.0009333333333333332</v>
       </c>
     </row>
     <row r="14">
@@ -3020,25 +3020,25 @@
         <v>32</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01245</v>
+        <v>0.00305</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>290</v>
+        <v>253</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.03155833333333333</v>
+        <v>0.01355</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.09929166666666665</v>
+        <v>0.05841666666666665</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01713333333333333</v>
+        <v>0.01641666666666667</v>
       </c>
     </row>
     <row r="15">
@@ -3047,32 +3047,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.04371666666666667</v>
+        <v>0.00275</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.1242666666666667</v>
+        <v>0.03285</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3526933333333333</v>
+        <v>0.2645083333333335</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.0027</v>
+        <v>0.00295</v>
       </c>
     </row>
     <row r="16">
@@ -3081,32 +3081,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
         <v>31</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0107</v>
+        <v>0.03385</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>295</v>
+        <v>252</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.04814999999999999</v>
+        <v>0.1122333333333334</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.291395</v>
+        <v>0.34249</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.0001833333333333333</v>
+        <v>0.0028</v>
       </c>
     </row>
     <row r="17">
@@ -3115,29 +3115,29 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
         <v>31</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.002933333333333333</v>
+        <v>0.0215</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>278</v>
+        <v>294</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04725833333333334</v>
+        <v>0.07275</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2584033333333332</v>
+        <v>0.3304699999999998</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0.0001</v>
@@ -3149,32 +3149,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.01415</v>
+        <v>0.001483333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>242</v>
+        <v>270</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.03958333333333333</v>
+        <v>0.040325</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.13525</v>
+        <v>0.2262916666666666</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.01865</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="19">
@@ -3183,32 +3183,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
         <v>30</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.01343333333333333</v>
+        <v>0.01573333333333333</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.04906666666666667</v>
+        <v>0.03765</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.158175</v>
+        <v>0.1345833333333334</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.0399</v>
+        <v>0.01763333333333333</v>
       </c>
     </row>
     <row r="20">
@@ -3217,32 +3217,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
         <v>30</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.005016666666666668</v>
+        <v>0.01093333333333333</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02927500000000001</v>
+        <v>0.04433333333333334</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2151349999999999</v>
+        <v>0.139925</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.001033333333333333</v>
+        <v>0.05256666666666666</v>
       </c>
     </row>
     <row r="21">
@@ -3251,32 +3251,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
         <v>30</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.004433333333333333</v>
+        <v>0.002966666666666667</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>256</v>
+        <v>280</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.03372833333333333</v>
+        <v>0.02298333333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2532</v>
+        <v>0.2131916666666665</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.003225</v>
+        <v>0.00185</v>
       </c>
     </row>
     <row r="22">
@@ -3285,32 +3285,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
         <v>29</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0</v>
+        <v>0.06301666666666668</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>314</v>
+        <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.02</v>
+        <v>0.1434666666666667</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2693200000000001</v>
+        <v>0.3511666666666666</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.001866666666666667</v>
+        <v>0.00445</v>
       </c>
     </row>
     <row r="23">
@@ -3319,32 +3319,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.004283333333333333</v>
+        <v>0.02928333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>271</v>
+        <v>255</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.02338333333333334</v>
+        <v>0.0839</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2219366666666667</v>
+        <v>0.2392166666666666</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0004</v>
+        <v>0.01891666666666667</v>
       </c>
     </row>
     <row r="24">
@@ -3353,32 +3353,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.00175</v>
+        <v>0.007283333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>180</v>
+        <v>207</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.00545</v>
+        <v>0.03344999999999999</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.03643333333333334</v>
+        <v>0.1310416666666666</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.1100666666666667</v>
+        <v>0.00975</v>
       </c>
     </row>
     <row r="25">
@@ -3387,32 +3387,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.06086666666666667</v>
+        <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>276</v>
+        <v>302</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.1312</v>
+        <v>0.02115</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.3301083333333333</v>
+        <v>0.2748916666666666</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.00515</v>
+        <v>0.001716666666666667</v>
       </c>
     </row>
     <row r="26">
@@ -3421,32 +3421,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.02933333333333334</v>
+        <v>0.004933333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>239</v>
+        <v>216</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.09271666666666667</v>
+        <v>0.03649166666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2535666666666667</v>
+        <v>0.1870016666666667</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01775</v>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="27">
@@ -3455,32 +3455,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D27" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.006983333333333334</v>
+        <v>0.002333333333333334</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>198</v>
+        <v>268</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0273</v>
+        <v>0.01758333333333334</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1166166666666667</v>
+        <v>0.17579</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01449166666666667</v>
+        <v>0.00105</v>
       </c>
     </row>
     <row r="28">
@@ -3489,32 +3489,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00375</v>
+        <v>0.00165</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>258</v>
+        <v>173</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.0177</v>
+        <v>0.004933333333333334</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.06203333333333334</v>
+        <v>0.031355</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.03747499999999999</v>
+        <v>0.1399666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -3523,32 +3523,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.0073</v>
+        <v>0.006083333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>216</v>
+        <v>252</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.04466666666666666</v>
+        <v>0.02486666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2054</v>
+        <v>0.08625833333333335</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0029</v>
+        <v>0.03236666666666667</v>
       </c>
     </row>
     <row r="30">
@@ -3567,22 +3567,22 @@
         <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.00225</v>
+        <v>0.00525</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0222</v>
+        <v>0.03368333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1011516666666667</v>
+        <v>0.1418166666666667</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.003533333333333334</v>
+        <v>0.00375</v>
       </c>
     </row>
     <row r="31">
@@ -3591,32 +3591,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D31" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.01788333333333333</v>
+        <v>0.0051</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>250</v>
+        <v>206</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.062025</v>
+        <v>0.02988333333333334</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2140266666666667</v>
+        <v>0.19435</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.002616666666666667</v>
+        <v>0.004216666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3625,32 +3625,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.005983333333333333</v>
+        <v>0.0003</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03258666666666666</v>
+        <v>0.003783333333333333</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.213835</v>
+        <v>0.05161666666666666</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00355</v>
+        <v>0.02468333333333333</v>
       </c>
     </row>
     <row r="33">
@@ -3659,32 +3659,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>0.0001</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.00295</v>
+        <v>0.00275</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.049675</v>
+        <v>0.04001166666666667</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02771666666666666</v>
+        <v>0.03391666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3693,32 +3693,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0</v>
+        <v>0.0035</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0014</v>
+        <v>0.0199</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03039166666666666</v>
+        <v>0.129275</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.04666666666666667</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="35">
@@ -3731,28 +3731,28 @@
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D35" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00595</v>
+        <v>0.00295</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03733333333333332</v>
+        <v>0.03103333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.21608</v>
+        <v>0.1993866666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.004883333333333333</v>
+        <v>0.0063</v>
       </c>
     </row>
     <row r="36">
@@ -3761,32 +3761,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D36" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.00235</v>
+        <v>0.01473333333333333</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.02011666666666666</v>
+        <v>0.05655833333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1219</v>
+        <v>0.20369</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.0049</v>
       </c>
     </row>
     <row r="37">
@@ -3805,22 +3805,22 @@
         <v>8</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.001183333333333333</v>
+        <v>0.0008</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>250</v>
+        <v>267</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.008691666666666667</v>
+        <v>0.006466666666666667</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.107395</v>
+        <v>0.09585</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0094</v>
+        <v>0.01176666666666666</v>
       </c>
     </row>
     <row r="38">
@@ -3829,32 +3829,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.00195</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>207</v>
+        <v>242</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.0018</v>
+        <v>0.01428333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.04501666666666668</v>
+        <v>0.06468333333333333</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.08153333333333335</v>
+        <v>0.06663333333333334</v>
       </c>
     </row>
     <row r="39">
@@ -3863,32 +3863,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.002</v>
+        <v>0.00315</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>253</v>
+        <v>225</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.01468333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.04198333333333333</v>
+        <v>0.07412333333333332</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1316083333333333</v>
+        <v>0.02428333333333334</v>
       </c>
     </row>
     <row r="40">
@@ -3897,32 +3897,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.002</v>
+        <v>0.00015</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>249</v>
+        <v>207</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.01446666666666667</v>
+        <v>0.001433333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.06198333333333333</v>
+        <v>0.03082</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.08555</v>
+        <v>0.1173666666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3931,32 +3931,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D41" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.00245</v>
+        <v>0.0018</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.0138</v>
+        <v>0.007633333333333334</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.07017500000000002</v>
+        <v>0.04046666666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.02625000000000001</v>
+        <v>0.1325</v>
       </c>
     </row>
     <row r="42">
@@ -3969,28 +3969,28 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.0012</v>
+        <v>0.0022</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.0057</v>
+        <v>0.007</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.02688333333333333</v>
+        <v>0.03186666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2905333333333334</v>
+        <v>0.2501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 20:20:06 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>25</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T00:00:33.369382+00:00</t>
+          <t>2026-03-22T00:20:05.851341+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -2476,10 +2476,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.4008903706569034</v>
+        <v>0.4020426864735876</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.5991096293430965</v>
+        <v>0.5979573135264125</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1735333333333333</v>
+        <v>0.1737333333333333</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>140</v>
@@ -2624,10 +2624,10 @@
         <v>335</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3958083333333333</v>
+        <v>0.3960083333333333</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7542550000000001</v>
+        <v>0.7548550000000001</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2649,7 +2649,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.07498333333333333</v>
+        <v>0.07493333333333334</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>117</v>
@@ -2661,7 +2661,7 @@
         <v>0.1751</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4155783333333334</v>
+        <v>0.4156283333333334</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -2695,7 +2695,7 @@
         <v>0.1896416666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4449499999999999</v>
+        <v>0.4453499999999999</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0.00245</v>
@@ -2729,7 +2729,7 @@
         <v>0.1299916666666666</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5342116666666669</v>
+        <v>0.5344616666666668</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.00015</v>
@@ -2751,7 +2751,7 @@
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.1368166666666667</v>
+        <v>0.1366166666666667</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>137</v>
@@ -2760,10 +2760,10 @@
         <v>292</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3175083333333333</v>
+        <v>0.3172083333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.7046116666666666</v>
+        <v>0.7045116666666666</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2794,10 +2794,10 @@
         <v>308</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1850666666666667</v>
+        <v>0.1848666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4468033333333333</v>
+        <v>0.4464033333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>5e-05</v>
@@ -2828,10 +2828,10 @@
         <v>283</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1635833333333334</v>
+        <v>0.1634833333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4752900000000002</v>
+        <v>0.4749900000000001</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
         <v>0.1386</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.333295</v>
+        <v>0.333195</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.0011</v>
@@ -2899,7 +2899,7 @@
         <v>0.02383333333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.26107</v>
+        <v>0.26077</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.00165</v>
@@ -2921,7 +2921,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04926666666666666</v>
+        <v>0.04936666666666666</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>109</v>
@@ -2930,10 +2930,10 @@
         <v>276</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1332833333333333</v>
+        <v>0.1334833333333333</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3322166666666665</v>
+        <v>0.3325166666666666</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0.0052</v>
@@ -2967,7 +2967,7 @@
         <v>0.09502500000000003</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4334549999999999</v>
+        <v>0.4335549999999999</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0009166666666666666</v>
@@ -2998,10 +2998,10 @@
         <v>347</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08094999999999999</v>
+        <v>0.08105</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3797083333333333</v>
+        <v>0.3797583333333333</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0.0009333333333333332</v>
@@ -3069,7 +3069,7 @@
         <v>0.03285</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2645083333333335</v>
+        <v>0.2647083333333334</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00295</v>
@@ -3103,7 +3103,7 @@
         <v>0.1122333333333334</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.34249</v>
+        <v>0.34239</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0.0028</v>
@@ -3171,7 +3171,7 @@
         <v>0.040325</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.2262916666666666</v>
+        <v>0.2261416666666666</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0.00025</v>
@@ -3202,7 +3202,7 @@
         <v>267</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03765</v>
+        <v>0.03775</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>0.1345833333333334</v>
@@ -3236,10 +3236,10 @@
         <v>262</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.04433333333333334</v>
+        <v>0.04423333333333334</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.139925</v>
+        <v>0.139825</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.05256666666666666</v>
@@ -3304,13 +3304,13 @@
         <v>256</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.1434666666666667</v>
+        <v>0.1435666666666667</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.3511666666666666</v>
+        <v>0.3513666666666667</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.00445</v>
+        <v>0.00435</v>
       </c>
     </row>
     <row r="23">
@@ -3329,7 +3329,7 @@
         <v>9</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.02928333333333333</v>
+        <v>0.02923333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>92</v>
@@ -3338,13 +3338,13 @@
         <v>255</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.0839</v>
+        <v>0.0838</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2392166666666666</v>
+        <v>0.2390166666666666</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.01891666666666667</v>
+        <v>0.01896666666666667</v>
       </c>
     </row>
     <row r="24">
@@ -3372,10 +3372,10 @@
         <v>207</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03344999999999999</v>
+        <v>0.03355</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1310416666666666</v>
+        <v>0.1311416666666667</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.00975</v>
@@ -3443,7 +3443,7 @@
         <v>0.03649166666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1870016666666667</v>
+        <v>0.1867016666666667</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.0035</v>
@@ -3474,10 +3474,10 @@
         <v>268</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.01758333333333334</v>
+        <v>0.01748333333333334</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.17579</v>
+        <v>0.17564</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.00105</v>
@@ -3514,7 +3514,7 @@
         <v>0.031355</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.1399666666666667</v>
+        <v>0.1400666666666666</v>
       </c>
     </row>
     <row r="29">
@@ -3576,13 +3576,13 @@
         <v>261</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.03368333333333334</v>
+        <v>0.03378333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1418166666666667</v>
+        <v>0.1419166666666667</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.00375</v>
+        <v>0.0037</v>
       </c>
     </row>
     <row r="31">
@@ -3613,7 +3613,7 @@
         <v>0.02988333333333334</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.19435</v>
+        <v>0.19405</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0.004216666666666667</v>
@@ -3783,7 +3783,7 @@
         <v>0.05655833333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.20369</v>
+        <v>0.20379</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0049</v>
@@ -3851,7 +3851,7 @@
         <v>0.01428333333333333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06468333333333333</v>
+        <v>0.06473333333333332</v>
       </c>
       <c r="J38" s="5" t="n">
         <v>0.06663333333333334</v>
@@ -3922,7 +3922,7 @@
         <v>0.03082</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1173666666666667</v>
+        <v>0.1175166666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3956,7 +3956,7 @@
         <v>0.04046666666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.1325</v>
+        <v>0.13235</v>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 20:43:29 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>7c39954d7e69400c</t>
+          <t>519ed8091a1b1179</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>beb794c701680ae0</t>
+          <t>7c39954d7e69400c</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T00:20:05.851341+00:00</t>
+          <t>2026-03-22T00:43:29.117862+00:00</t>
         </is>
       </c>
     </row>
@@ -2369,10 +2369,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
       <c r="F45" s="6" t="b">
         <v>0</v>
       </c>
@@ -2476,10 +2480,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.4020426864735876</v>
+        <v>0.4519295154173104</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.5979573135264125</v>
+        <v>0.5480704845826897</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2605,32 +2609,32 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Ellis Fleming</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1737333333333333</v>
+        <v>0.08601666666666666</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>140</v>
+        <v>119</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>335</v>
+        <v>306</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.3960083333333333</v>
+        <v>0.1929666666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.7548550000000001</v>
+        <v>0.4524733333333334</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="3">
@@ -2639,32 +2643,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Ellis Fleming</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>10</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.07493333333333334</v>
+        <v>0.1749</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>324</v>
+        <v>346</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1751</v>
+        <v>0.40782</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4156283333333334</v>
+        <v>0.7746916666666667</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2683,22 +2687,22 @@
         <v>9</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07078333333333334</v>
+        <v>0.07528333333333333</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>319</v>
+        <v>336</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1896416666666667</v>
+        <v>0.2035116666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4453499999999999</v>
+        <v>0.4614766666666666</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.00245</v>
+        <v>0.00222</v>
       </c>
     </row>
     <row r="5">
@@ -2707,32 +2711,32 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.0235</v>
+        <v>0.07316666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1299916666666666</v>
+        <v>0.1962416666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5344616666666668</v>
+        <v>0.4563916666666667</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.00015</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="6">
@@ -2741,32 +2745,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.1366166666666667</v>
+        <v>0.02105</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>292</v>
+        <v>346</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3172083333333333</v>
+        <v>0.1264666666666667</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.7045116666666666</v>
+        <v>0.5438283333333332</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0</v>
+        <v>0.0001333333333333333</v>
       </c>
     </row>
     <row r="7">
@@ -2775,7 +2779,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
@@ -2785,22 +2789,22 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.07666666666666666</v>
+        <v>0.1297</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1848666666666667</v>
+        <v>0.3052833333333334</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4464033333333333</v>
+        <v>0.6850133333333333</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>5e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -2809,32 +2813,32 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.06253333333333333</v>
+        <v>0.05985000000000001</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1634833333333334</v>
+        <v>0.15055</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.4749900000000001</v>
+        <v>0.34494</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0</v>
+        <v>0.0005833333333333334</v>
       </c>
     </row>
     <row r="9">
@@ -2843,7 +2847,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
@@ -2853,22 +2857,22 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.0463</v>
+        <v>0.0586</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>264</v>
+        <v>290</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1386</v>
+        <v>0.163575</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.333195</v>
+        <v>0.4670766666666668</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.0011</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2877,32 +2881,32 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0019</v>
+        <v>0.02223333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>304</v>
+        <v>333</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.02383333333333333</v>
+        <v>0.1090833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.26077</v>
+        <v>0.4800166666666668</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.00165</v>
+        <v>0.00015</v>
       </c>
     </row>
     <row r="11">
@@ -2911,32 +2915,32 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Ryan Evans</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.04936666666666666</v>
+        <v>0.02055</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>276</v>
+        <v>349</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.1334833333333333</v>
+        <v>0.08904166666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3325166666666666</v>
+        <v>0.4203433333333333</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.0052</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="12">
@@ -2945,32 +2949,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02028333333333333</v>
+        <v>0.00135</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09502500000000003</v>
+        <v>0.01995</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4335549999999999</v>
+        <v>0.2453950000000001</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.0009166666666666666</v>
+        <v>0.00165</v>
       </c>
     </row>
     <row r="13">
@@ -2979,7 +2983,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Ryan Evans</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
@@ -2989,22 +2993,22 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.0146</v>
+        <v>0.05325</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>347</v>
+        <v>274</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.08105</v>
+        <v>0.1442916666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3797583333333333</v>
+        <v>0.3494333333333333</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0009333333333333332</v>
+        <v>0.0046</v>
       </c>
     </row>
     <row r="14">
@@ -3013,32 +3017,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.00305</v>
+        <v>0.01868333333333333</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>253</v>
+        <v>306</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.01355</v>
+        <v>0.069025</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.05841666666666665</v>
+        <v>0.3498916666666667</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.01641666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3047,32 +3051,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
         <v>32</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.00275</v>
+        <v>0.0115</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.03285</v>
+        <v>0.04739166666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.2647083333333334</v>
+        <v>0.146825</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.00295</v>
+        <v>0.0415</v>
       </c>
     </row>
     <row r="16">
@@ -3081,32 +3085,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.03385</v>
+        <v>0.00225</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.1122333333333334</v>
+        <v>0.03038333333333333</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.34239</v>
+        <v>0.2566349999999999</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.0028</v>
+        <v>0.002466666666666666</v>
       </c>
     </row>
     <row r="17">
@@ -3115,32 +3119,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.0215</v>
+        <v>0</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>294</v>
+        <v>227</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.07275</v>
+        <v>6.666666666666666e-05</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.3304699999999998</v>
+        <v>0.008475</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.02283666666666667</v>
       </c>
     </row>
     <row r="18">
@@ -3149,32 +3153,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
         <v>31</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.001483333333333333</v>
+        <v>0.06633333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.040325</v>
+        <v>0.152425</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.2261416666666666</v>
+        <v>0.3835333333333333</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.00025</v>
+        <v>0.00205</v>
       </c>
     </row>
     <row r="19">
@@ -3183,32 +3187,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.01573333333333333</v>
+        <v>0.03441666666666666</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03775</v>
+        <v>0.1119333333333333</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1345833333333334</v>
+        <v>0.3417116666666667</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.01763333333333333</v>
+        <v>0.00235</v>
       </c>
     </row>
     <row r="20">
@@ -3217,32 +3221,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.01093333333333333</v>
+        <v>0.0019</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.04423333333333334</v>
+        <v>0.03484166666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.139825</v>
+        <v>0.2151983333333333</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.05256666666666666</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="21">
@@ -3261,22 +3265,22 @@
         <v>8</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.002966666666666667</v>
+        <v>0.00315</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>106</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02298333333333333</v>
+        <v>0.02218333333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2131916666666665</v>
+        <v>0.2129249999999999</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.00185</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="22">
@@ -3285,32 +3289,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.06301666666666668</v>
+        <v>0.0012</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>256</v>
+        <v>220</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.1435666666666667</v>
+        <v>0.009533333333333335</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.3513666666666667</v>
+        <v>0.07571166666666668</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.00435</v>
+        <v>0.02215</v>
       </c>
     </row>
     <row r="23">
@@ -3329,22 +3333,22 @@
         <v>9</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.02923333333333333</v>
+        <v>0.02358333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.0838</v>
+        <v>0.075375</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2390166666666666</v>
+        <v>0.2314916666666667</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.01896666666666667</v>
+        <v>0.01907</v>
       </c>
     </row>
     <row r="24">
@@ -3363,7 +3367,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.007283333333333333</v>
+        <v>0.00685</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>92</v>
@@ -3372,13 +3376,13 @@
         <v>207</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03355</v>
+        <v>0.03388333333333333</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1311416666666667</v>
+        <v>0.1320333333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.00975</v>
+        <v>0.01000333333333333</v>
       </c>
     </row>
     <row r="25">
@@ -3400,19 +3404,19 @@
         <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>302</v>
+        <v>322</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02115</v>
+        <v>0.01808333333333333</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.2748916666666666</v>
+        <v>0.264865</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.001716666666666667</v>
+        <v>0.0017</v>
       </c>
     </row>
     <row r="26">
@@ -3431,22 +3435,22 @@
         <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.004933333333333334</v>
+        <v>0.006033333333333333</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>216</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.03649166666666667</v>
+        <v>0.03351666666666666</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1867016666666667</v>
+        <v>0.1779083333333333</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.0035</v>
+        <v>0.0041</v>
       </c>
     </row>
     <row r="27">
@@ -3465,22 +3469,22 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.002333333333333334</v>
+        <v>0.00245</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>105</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.01748333333333334</v>
+        <v>0.01465833333333333</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.17564</v>
+        <v>0.1702533333333333</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.00105</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="28">
@@ -3499,22 +3503,22 @@
         <v>6</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00165</v>
+        <v>0.00125</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.004933333333333334</v>
+        <v>0.005116666666666666</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.031355</v>
+        <v>0.03016166666666666</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.1400666666666666</v>
+        <v>0.1302833333333333</v>
       </c>
     </row>
     <row r="29">
@@ -3530,25 +3534,25 @@
         <v>27</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.006083333333333333</v>
+        <v>0.0007333333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.02486666666666667</v>
+        <v>0.0069</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.08625833333333335</v>
+        <v>0.03205833333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.03236666666666667</v>
+        <v>0.04102499999999999</v>
       </c>
     </row>
     <row r="30">
@@ -3557,32 +3561,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
         <v>26</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.00525</v>
+        <v>0.0169</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>261</v>
+        <v>246</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.03378333333333334</v>
+        <v>0.05775333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1419166666666667</v>
+        <v>0.2242633333333334</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.0037</v>
+        <v>0.00195</v>
       </c>
     </row>
     <row r="31">
@@ -3601,22 +3605,22 @@
         <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.0051</v>
+        <v>0.005933333333333334</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.02988333333333334</v>
+        <v>0.0251</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.19405</v>
+        <v>0.174135</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.004216666666666667</v>
+        <v>0.00385</v>
       </c>
     </row>
     <row r="32">
@@ -3625,7 +3629,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
@@ -3635,22 +3639,22 @@
         <v>8</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0003</v>
+        <v>0.00465</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>220</v>
+        <v>257</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.003783333333333333</v>
+        <v>0.03715</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.05161666666666666</v>
+        <v>0.1568416666666666</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.02468333333333333</v>
+        <v>0.0046</v>
       </c>
     </row>
     <row r="33">
@@ -3669,22 +3673,22 @@
         <v>6</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>82</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.00275</v>
+        <v>0.00242</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.04001166666666667</v>
+        <v>0.03923333333333333</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.03391666666666666</v>
+        <v>0.02947</v>
       </c>
     </row>
     <row r="34">
@@ -3693,32 +3697,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.0035</v>
+        <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0199</v>
+        <v>0.003025</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.129275</v>
+        <v>0.04992666666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.00025</v>
+        <v>0.02366666666666667</v>
       </c>
     </row>
     <row r="35">
@@ -3737,22 +3741,22 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00295</v>
+        <v>0.004033333333333333</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.03103333333333333</v>
+        <v>0.02614999999999999</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1993866666666667</v>
+        <v>0.1816516666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.0063</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="36">
@@ -3761,32 +3765,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D36" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.01473333333333333</v>
+        <v>0.00375</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.05655833333333334</v>
+        <v>0.02290333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.20379</v>
+        <v>0.1363966666666666</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.0049</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -3795,32 +3799,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.0008</v>
+        <v>0.0023</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.006466666666666667</v>
+        <v>0.02048333333333333</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.09585</v>
+        <v>0.073975</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.01176666666666666</v>
+        <v>0.04344166666666666</v>
       </c>
     </row>
     <row r="38">
@@ -3829,32 +3833,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.00195</v>
+        <v>0.00325</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>242</v>
+        <v>221</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01428333333333333</v>
+        <v>0.01715</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.06473333333333332</v>
+        <v>0.08225000000000002</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.06663333333333334</v>
+        <v>0.01673333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3863,32 +3867,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D39" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.00315</v>
+        <v>0.001</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>225</v>
+        <v>264</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01468333333333333</v>
+        <v>0.006083333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.07412333333333332</v>
+        <v>0.09309333333333331</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.02428333333333334</v>
+        <v>0.010475</v>
       </c>
     </row>
     <row r="40">
@@ -3907,22 +3911,22 @@
         <v>6</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G40" s="8" t="n">
         <v>207</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.001433333333333333</v>
+        <v>0.0005833333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.03082</v>
+        <v>0.02955</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1175166666666667</v>
+        <v>0.11785</v>
       </c>
     </row>
     <row r="41">
@@ -3941,22 +3945,22 @@
         <v>7</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.0018</v>
+        <v>0.0019</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.007633333333333334</v>
+        <v>0.0071</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.04046666666666667</v>
+        <v>0.04351666666666666</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.13235</v>
+        <v>0.13605</v>
       </c>
     </row>
     <row r="42">
@@ -3972,25 +3976,25 @@
         <v>18</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.0022</v>
+        <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>189</v>
+        <v>103</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.007</v>
+        <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.03186666666666666</v>
+        <v>0.004408333333333333</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2501</v>
+        <v>0.2971916666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 21:05:57 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T00:43:29.117862+00:00</t>
+          <t>2026-03-22T01:05:56.636899+00:00</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2480,10 +2480,10 @@
         <v>1</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.4519295154173104</v>
+        <v>0.6863507404965623</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.5480704845826897</v>
+        <v>0.3136492595034376</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -2619,19 +2619,19 @@
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.08601666666666666</v>
+        <v>0.08735</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>306</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.1929666666666667</v>
+        <v>0.19745</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.4524733333333334</v>
+        <v>0.4685866666666667</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0.0004</v>
@@ -2653,19 +2653,19 @@
         <v>10</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1749</v>
+        <v>0.2350333333333333</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>346</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.40782</v>
+        <v>0.5076533333333335</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.7746916666666667</v>
+        <v>0.8500166666666668</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2687,22 +2687,22 @@
         <v>9</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.07528333333333333</v>
+        <v>0.092</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="G4" s="8" t="n">
         <v>336</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2035116666666667</v>
+        <v>0.2487366666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4614766666666666</v>
+        <v>0.53995</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.00222</v>
+        <v>0.00122</v>
       </c>
     </row>
     <row r="5">
@@ -2721,19 +2721,19 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.07316666666666667</v>
+        <v>0.05091666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>118</v>
+        <v>114.5</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>337</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1962416666666667</v>
+        <v>0.1561333333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4563916666666667</v>
+        <v>0.4095433333333333</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0001</v>
@@ -2755,22 +2755,22 @@
         <v>9</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.02105</v>
+        <v>0.0196</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>346</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1264666666666667</v>
+        <v>0.1268083333333334</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.5438283333333332</v>
+        <v>0.5632283333333333</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.0001333333333333333</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="7">
@@ -2789,19 +2789,19 @@
         <v>10</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.1297</v>
+        <v>0.1037</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G7" s="9" t="n">
         <v>294</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.3052833333333334</v>
+        <v>0.25875</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.6850133333333333</v>
+        <v>0.6412633333333334</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2823,22 +2823,22 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.05985000000000001</v>
+        <v>0.05258333333333333</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>275</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.15055</v>
+        <v>0.1288333333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.34494</v>
+        <v>0.3043150000000001</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.0005833333333333334</v>
+        <v>0.0007833333333333334</v>
       </c>
     </row>
     <row r="9">
@@ -2857,19 +2857,19 @@
         <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.0586</v>
+        <v>0.0465</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>290</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.163575</v>
+        <v>0.13385</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4670766666666668</v>
+        <v>0.4192016666666668</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2891,22 +2891,22 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.02223333333333333</v>
+        <v>0.02038333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>333</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1090833333333333</v>
+        <v>0.10835</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4800166666666668</v>
+        <v>0.4995316666666668</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2925,22 +2925,22 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.02055</v>
+        <v>0.02018333333333333</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G11" s="9" t="n">
         <v>349</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.08904166666666666</v>
+        <v>0.09092500000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4203433333333333</v>
+        <v>0.4379833333333334</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="12">
@@ -2959,22 +2959,22 @@
         <v>7</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.00135</v>
+        <v>0.00095</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>323</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.01995</v>
+        <v>0.01223333333333333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.2453950000000001</v>
+        <v>0.2015416666666666</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.00165</v>
+        <v>0.00245</v>
       </c>
     </row>
     <row r="13">
@@ -2993,22 +2993,22 @@
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.05325</v>
+        <v>0.06884999999999999</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1442916666666667</v>
+        <v>0.1824083333333333</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3494333333333333</v>
+        <v>0.4205916666666666</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0046</v>
+        <v>0.0033</v>
       </c>
     </row>
     <row r="14">
@@ -3027,19 +3027,19 @@
         <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01868333333333333</v>
+        <v>0.01781666666666667</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G14" s="8" t="n">
         <v>306</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.069025</v>
+        <v>0.07094166666666668</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3498916666666667</v>
+        <v>0.3646583333333333</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3061,22 +3061,22 @@
         <v>7</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.0115</v>
+        <v>0.008</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.04739166666666667</v>
+        <v>0.03883333333333333</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.146825</v>
+        <v>0.1219916666666667</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.0415</v>
+        <v>0.05295</v>
       </c>
     </row>
     <row r="16">
@@ -3095,22 +3095,22 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.00225</v>
+        <v>0.0018</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G16" s="8" t="n">
         <v>249</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.03038333333333333</v>
+        <v>0.03053333333333334</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2566349999999999</v>
+        <v>0.2697749999999999</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.002466666666666666</v>
+        <v>0.002416666666666666</v>
       </c>
     </row>
     <row r="17">
@@ -3138,13 +3138,13 @@
         <v>227</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>6.666666666666666e-05</v>
+        <v>0.0001166666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.008475</v>
+        <v>0.009350000000000001</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.02283666666666667</v>
+        <v>0.01817</v>
       </c>
     </row>
     <row r="18">
@@ -3163,22 +3163,22 @@
         <v>10</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.06633333333333333</v>
+        <v>0.06668333333333333</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>264</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.152425</v>
+        <v>0.1556833333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.3835333333333333</v>
+        <v>0.3960750000000001</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.00205</v>
+        <v>0.0018</v>
       </c>
     </row>
     <row r="19">
@@ -3197,22 +3197,22 @@
         <v>10</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.03441666666666666</v>
+        <v>0.03188333333333333</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G19" s="9" t="n">
         <v>263</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.1119333333333333</v>
+        <v>0.1150666666666667</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.3417116666666667</v>
+        <v>0.3542033333333334</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.00235</v>
+        <v>0.0017</v>
       </c>
     </row>
     <row r="20">
@@ -3231,22 +3231,22 @@
         <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.0019</v>
+        <v>0.00105</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G20" s="8" t="n">
         <v>279</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.03484166666666667</v>
+        <v>0.02761666666666666</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2151983333333333</v>
+        <v>0.1793666666666667</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.00015</v>
       </c>
     </row>
     <row r="21">
@@ -3265,19 +3265,19 @@
         <v>8</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.00315</v>
+        <v>0.0029</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G21" s="9" t="n">
         <v>278</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02218333333333333</v>
+        <v>0.02286666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2129249999999999</v>
+        <v>0.2266983333333334</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0002</v>
@@ -3299,7 +3299,7 @@
         <v>8</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.0012</v>
+        <v>0.00115</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>80</v>
@@ -3308,13 +3308,13 @@
         <v>220</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.009533333333333335</v>
+        <v>0.009650000000000001</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.07571166666666668</v>
+        <v>0.07851999999999999</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.02215</v>
+        <v>0.01851666666666667</v>
       </c>
     </row>
     <row r="23">
@@ -3333,22 +3333,22 @@
         <v>9</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.02358333333333333</v>
+        <v>0.0144</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>248</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.075375</v>
+        <v>0.0548</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2314916666666667</v>
+        <v>0.2009000000000001</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.01907</v>
+        <v>0.02315333333333333</v>
       </c>
     </row>
     <row r="24">
@@ -3367,22 +3367,22 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.00685</v>
+        <v>0.0068</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>207</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03388333333333333</v>
+        <v>0.03514999999999999</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1320333333333333</v>
+        <v>0.14055</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.01000333333333333</v>
+        <v>0.008153333333333334</v>
       </c>
     </row>
     <row r="25">
@@ -3404,19 +3404,19 @@
         <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G25" s="9" t="n">
         <v>322</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.01808333333333333</v>
+        <v>0.01803333333333333</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.264865</v>
+        <v>0.2771</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.0017</v>
+        <v>0.0009</v>
       </c>
     </row>
     <row r="26">
@@ -3435,22 +3435,22 @@
         <v>9</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.006033333333333333</v>
+        <v>0.003583333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.03351666666666666</v>
+        <v>0.02043333333333333</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1779083333333333</v>
+        <v>0.1369233333333333</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.0041</v>
+        <v>0.005233333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -3469,22 +3469,22 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.00245</v>
+        <v>0.0016</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="G27" s="9" t="n">
         <v>267</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.01465833333333333</v>
+        <v>0.01008333333333333</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1702533333333333</v>
+        <v>0.1345983333333333</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.0005</v>
+        <v>0.0014</v>
       </c>
     </row>
     <row r="28">
@@ -3503,22 +3503,22 @@
         <v>6</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00125</v>
+        <v>0.0009</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G28" s="8" t="n">
         <v>199</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.005116666666666666</v>
+        <v>0.0038</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.03016166666666666</v>
+        <v>0.02095833333333334</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.1302833333333333</v>
+        <v>0.1595833333333333</v>
       </c>
     </row>
     <row r="29">
@@ -3546,13 +3546,13 @@
         <v>240</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.0069</v>
+        <v>0.0068</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.03205833333333333</v>
+        <v>0.03290833333333334</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.04102499999999999</v>
+        <v>0.03360833333333334</v>
       </c>
     </row>
     <row r="30">
@@ -3571,22 +3571,22 @@
         <v>9</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0169</v>
+        <v>0.0171</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>246</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.05775333333333333</v>
+        <v>0.05900333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.2242633333333334</v>
+        <v>0.2319133333333334</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.00195</v>
+        <v>0.0016</v>
       </c>
     </row>
     <row r="31">
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
         <v>26</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.005933333333333334</v>
+        <v>0.008</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>96</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>211</v>
+        <v>264</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.0251</v>
+        <v>0.05565</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.174135</v>
+        <v>0.2169833333333333</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.00385</v>
+        <v>0.0029</v>
       </c>
     </row>
     <row r="32">
@@ -3629,32 +3629,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
         <v>26</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00465</v>
+        <v>0.0035</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>257</v>
+        <v>211</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.03715</v>
+        <v>0.01796666666666667</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1568416666666666</v>
+        <v>0.1395833333333334</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0046</v>
+        <v>0.00565</v>
       </c>
     </row>
     <row r="33">
@@ -3676,19 +3676,19 @@
         <v>0</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.00242</v>
+        <v>0.00227</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.03923333333333333</v>
+        <v>0.041275</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02947</v>
+        <v>0.02552</v>
       </c>
     </row>
     <row r="34">
@@ -3716,13 +3716,13 @@
         <v>222</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.003025</v>
+        <v>0.002766666666666667</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.04992666666666667</v>
+        <v>0.05148500000000002</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02366666666666667</v>
+        <v>0.021</v>
       </c>
     </row>
     <row r="35">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
@@ -3741,22 +3741,22 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.004033333333333333</v>
+        <v>0.0037</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.02614999999999999</v>
+        <v>0.02283666666666666</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1816516666666667</v>
+        <v>0.1397466666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
@@ -3775,22 +3775,22 @@
         <v>9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.00375</v>
+        <v>0.0025</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.02290333333333333</v>
+        <v>0.01616666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1363966666666666</v>
+        <v>0.14984</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0</v>
+        <v>0.0062</v>
       </c>
     </row>
     <row r="37">
@@ -3809,7 +3809,7 @@
         <v>7</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.0023</v>
+        <v>0.00205</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>75</v>
@@ -3818,13 +3818,13 @@
         <v>271</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.02048333333333333</v>
+        <v>0.02033333333333334</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.073975</v>
+        <v>0.07413333333333331</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.04344166666666666</v>
+        <v>0.03869166666666667</v>
       </c>
     </row>
     <row r="38">
@@ -3843,7 +3843,7 @@
         <v>8</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.00325</v>
+        <v>0.00315</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>81</v>
@@ -3852,13 +3852,13 @@
         <v>221</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01715</v>
+        <v>0.016</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.08225000000000002</v>
+        <v>0.08496666666666668</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.01673333333333333</v>
+        <v>0.01441666666666667</v>
       </c>
     </row>
     <row r="39">
@@ -3877,22 +3877,22 @@
         <v>8</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.001</v>
+        <v>0.00065</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G39" s="9" t="n">
         <v>264</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.006083333333333333</v>
+        <v>0.006283333333333333</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.09309333333333331</v>
+        <v>0.0982933333333333</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.010475</v>
+        <v>0.009258333333333334</v>
       </c>
     </row>
     <row r="40">
@@ -3914,19 +3914,19 @@
         <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.0005833333333333333</v>
+        <v>0.0003833333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.02955</v>
+        <v>0.02141666666666667</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.11785</v>
+        <v>0.1461</v>
       </c>
     </row>
     <row r="41">
@@ -3945,7 +3945,7 @@
         <v>7</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.0019</v>
+        <v>0.002</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>66</v>
@@ -3954,13 +3954,13 @@
         <v>247</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.0071</v>
+        <v>0.0078</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.04351666666666666</v>
+        <v>0.04533333333333333</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.13605</v>
+        <v>0.1209333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -3991,10 +3991,10 @@
         <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.004408333333333333</v>
+        <v>0.0047</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2971916666666667</v>
+        <v>0.2713416666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 21:20:44 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>519ed8091a1b1179</t>
+          <t>164b5778cca71ffb</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>7c39954d7e69400c</t>
+          <t>519ed8091a1b1179</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Round of 32: Texas over Gonzaga</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T01:05:56.636899+00:00</t>
+          <t>2026-03-22T01:20:43.984578+00:00</t>
         </is>
       </c>
     </row>
@@ -2472,19 +2472,19 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
       <c r="F48" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G48" s="5" t="n">
-        <v>0.6863507404965623</v>
-      </c>
-      <c r="H48" s="5" t="n">
-        <v>0.3136492595034376</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr"/>
       <c r="I48" s="3" t="inlineStr">
         <is>
           <t>R32_W_03</t>
@@ -2609,32 +2609,32 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Ellis Fleming</t>
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.08735</v>
+        <v>0.3216333333333333</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>306</v>
+        <v>360</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.19745</v>
+        <v>0.63855</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.4685866666666667</v>
+        <v>0.9404749999999998</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2643,29 +2643,29 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Ellis Fleming</t>
+          <t>Stephen Mason</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.2350333333333333</v>
+        <v>0.1084333333333334</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>346</v>
+        <v>320</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.5076533333333335</v>
+        <v>0.3062</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.8500166666666668</v>
+        <v>0.6386833333333336</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2677,32 +2677,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Stephen Mason</t>
+          <t>Ryan Evans</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.092</v>
+        <v>0.08586666666666666</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>336</v>
+        <v>294</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2487366666666667</v>
+        <v>0.2242083333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.53995</v>
+        <v>0.5122533333333333</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.00122</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2711,29 +2711,29 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.05091666666666667</v>
+        <v>0.09088333333333333</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>114.5</v>
+        <v>121</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>337</v>
+        <v>324</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1561333333333333</v>
+        <v>0.2054916666666667</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4095433333333333</v>
+        <v>0.4843716666666666</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0.0001</v>
@@ -2745,32 +2745,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.0196</v>
+        <v>0.02573333333333334</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1268083333333334</v>
+        <v>0.1104833333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.5632283333333333</v>
+        <v>0.3549683333333333</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2779,32 +2779,32 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.1037</v>
+        <v>0.01783333333333333</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>294</v>
+        <v>334</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.25875</v>
+        <v>0.1318666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.6412633333333334</v>
+        <v>0.5799566666666667</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0</v>
+        <v>5e-05</v>
       </c>
     </row>
     <row r="8">
@@ -2813,32 +2813,32 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.05258333333333333</v>
+        <v>0.0143</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1288333333333334</v>
+        <v>0.08604166666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3043150000000001</v>
+        <v>0.2997533333333334</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.0007833333333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2847,29 +2847,29 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.0465</v>
+        <v>0.06731666666666666</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.13385</v>
+        <v>0.1974833333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4192016666666668</v>
+        <v>0.5961033333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2881,32 +2881,32 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.02038333333333333</v>
+        <v>0.0411</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>333</v>
+        <v>268</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.10835</v>
+        <v>0.1040083333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4995316666666668</v>
+        <v>0.2575616666666666</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="11">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
@@ -2925,22 +2925,22 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.02018333333333333</v>
+        <v>0.02725</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>349</v>
+        <v>267</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.09092500000000001</v>
+        <v>0.09158333333333335</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4379833333333334</v>
+        <v>0.3514016666666668</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2949,32 +2949,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.00095</v>
+        <v>0.02176666666666667</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>323</v>
+        <v>339</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.01223333333333333</v>
+        <v>0.1106333333333333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.2015416666666666</v>
+        <v>0.5238633333333332</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.00245</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2983,32 +2983,32 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ryan Evans</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.06884999999999999</v>
+        <v>0.01888333333333333</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>278</v>
+        <v>334</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1824083333333333</v>
+        <v>0.09326666666666668</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.4205916666666666</v>
+        <v>0.4513333333333336</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0033</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="14">
@@ -3017,32 +3017,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01781666666666667</v>
+        <v>0</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>306</v>
+        <v>329</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.07094166666666668</v>
+        <v>0.00015</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3646583333333333</v>
+        <v>0.1383416666666667</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0</v>
+        <v>0.0032</v>
       </c>
     </row>
     <row r="15">
@@ -3051,32 +3051,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.008</v>
+        <v>0.01406666666666667</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.03883333333333333</v>
+        <v>0.07041666666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.1219916666666667</v>
+        <v>0.3831316666666668</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.05295</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3095,22 +3095,22 @@
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0018</v>
+        <v>0.0028</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>249</v>
+        <v>266</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.03053333333333334</v>
+        <v>0.03265</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2697749999999999</v>
+        <v>0.2898116666666665</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.002416666666666666</v>
+        <v>0.00095</v>
       </c>
     </row>
     <row r="17">
@@ -3119,32 +3119,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
         <v>32</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0</v>
+        <v>0.00195</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.0001166666666666667</v>
+        <v>0.01898333333333333</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.009350000000000001</v>
+        <v>0.08337</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.01817</v>
+        <v>0.06783333333333333</v>
       </c>
     </row>
     <row r="18">
@@ -3153,32 +3153,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.06668333333333333</v>
+        <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>264</v>
+        <v>234</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.1556833333333333</v>
+        <v>0</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.3960750000000001</v>
+        <v>0.01391</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.0018</v>
+        <v>0.01265</v>
       </c>
     </row>
     <row r="19">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
@@ -3197,22 +3197,22 @@
         <v>10</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.03188333333333333</v>
+        <v>0.06571666666666666</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.1150666666666667</v>
+        <v>0.1525583333333333</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.3542033333333334</v>
+        <v>0.407755</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.0017</v>
+        <v>0.001233333333333333</v>
       </c>
     </row>
     <row r="20">
@@ -3221,32 +3221,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
         <v>31</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.00105</v>
+        <v>0.03</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>279</v>
+        <v>251</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02761666666666666</v>
+        <v>0.1188666666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.1793666666666667</v>
+        <v>0.3749283333333332</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.00015</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="21">
@@ -3255,32 +3255,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.0029</v>
+        <v>0</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02286666666666667</v>
+        <v>0.02248333333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2266983333333334</v>
+        <v>0.1320666666666666</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="22">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
@@ -3299,22 +3299,22 @@
         <v>8</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.00115</v>
+        <v>0.0019</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>220</v>
+        <v>283</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.009650000000000001</v>
+        <v>0.02441666666666667</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.07851999999999999</v>
+        <v>0.2456316666666667</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.01851666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -3323,32 +3323,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.0144</v>
+        <v>0.001</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.0548</v>
+        <v>0.0075</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2009000000000001</v>
+        <v>0.08437500000000001</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.02315333333333333</v>
+        <v>0.01358333333333333</v>
       </c>
     </row>
     <row r="24">
@@ -3367,22 +3367,22 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.0068</v>
+        <v>0.00715</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>207</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03514999999999999</v>
+        <v>0.03693333333333333</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.14055</v>
+        <v>0.1532750000000001</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.008153333333333334</v>
+        <v>0.007033333333333334</v>
       </c>
     </row>
     <row r="25">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
@@ -3401,22 +3401,22 @@
         <v>8</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0</v>
+        <v>0.0044</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>322</v>
+        <v>224</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.01803333333333333</v>
+        <v>0.03073333333333334</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.2771</v>
+        <v>0.1607433333333333</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.0009</v>
+        <v>0.02708333333333334</v>
       </c>
     </row>
     <row r="26">
@@ -3425,32 +3425,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.003583333333333334</v>
+        <v>0</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>87</v>
+        <v>114</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>206</v>
+        <v>336</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02043333333333333</v>
+        <v>0.02115</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1369233333333333</v>
+        <v>0.3025616666666666</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.005233333333333333</v>
+        <v>0.0009</v>
       </c>
     </row>
     <row r="27">
@@ -3459,32 +3459,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
         <v>28</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.0016</v>
+        <v>0.0009</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>267</v>
+        <v>189</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.01008333333333333</v>
+        <v>0.00275</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1345983333333333</v>
+        <v>0.009508333333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.0014</v>
+        <v>0.2084166666666666</v>
       </c>
     </row>
     <row r="28">
@@ -3493,32 +3493,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
         <v>28</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0009</v>
+        <v>0.00035</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>56</v>
+        <v>97</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>199</v>
+        <v>266</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.0038</v>
+        <v>0.005466666666666667</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.02095833333333334</v>
+        <v>0.09282999999999998</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.1595833333333333</v>
+        <v>0.0018</v>
       </c>
     </row>
     <row r="29">
@@ -3527,32 +3527,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.0007333333333333333</v>
+        <v>0.0003333333333333333</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>240</v>
+        <v>203</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.0068</v>
+        <v>0.006266666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.03290833333333334</v>
+        <v>0.08702500000000001</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.03360833333333334</v>
+        <v>0.0054</v>
       </c>
     </row>
     <row r="30">
@@ -3561,32 +3561,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0171</v>
+        <v>0.00115</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>246</v>
+        <v>261</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.05900333333333333</v>
+        <v>0.007583333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.2319133333333334</v>
+        <v>0.03525833333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.0016</v>
+        <v>0.02335</v>
       </c>
     </row>
     <row r="31">
@@ -3595,32 +3595,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
         <v>26</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.008</v>
+        <v>0.01623333333333333</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.05565</v>
+        <v>0.05603333333333332</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2169833333333333</v>
+        <v>0.2369316666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.0029</v>
+        <v>0.0009</v>
       </c>
     </row>
     <row r="32">
@@ -3636,25 +3636,25 @@
         <v>26</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0035</v>
+        <v>0.00065</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.01796666666666667</v>
+        <v>0.007875</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1395833333333334</v>
+        <v>0.1018583333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00565</v>
+        <v>0.008133333333333333</v>
       </c>
     </row>
     <row r="33">
@@ -3663,32 +3663,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
         <v>26</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0</v>
+        <v>0.00015</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>223</v>
+        <v>204</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.00227</v>
+        <v>0.003416666666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.041275</v>
+        <v>0.050535</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02552</v>
+        <v>0.01688333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -3697,32 +3697,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
         <v>26</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0</v>
+        <v>5e-05</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.002766666666666667</v>
+        <v>0.001383333333333333</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.05148500000000002</v>
+        <v>0.03747833333333334</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.021</v>
+        <v>0.02513333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3741,19 +3741,19 @@
         <v>9</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.0037</v>
+        <v>0.00385</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>89</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.02283666666666666</v>
+        <v>0.02335</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1397466666666667</v>
+        <v>0.14598</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0</v>
@@ -3772,25 +3772,25 @@
         <v>25</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.0025</v>
+        <v>0.00015</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01616666666666667</v>
+        <v>0.004891666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.14984</v>
+        <v>0.1125166666666667</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.0062</v>
+        <v>0.01255</v>
       </c>
     </row>
     <row r="37">
@@ -3809,22 +3809,22 @@
         <v>7</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00205</v>
+        <v>0.0012</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>75</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>271</v>
+        <v>237</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.02033333333333334</v>
+        <v>0.01608333333333333</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.07413333333333331</v>
+        <v>0.07205833333333332</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.03869166666666667</v>
+        <v>0.0317</v>
       </c>
     </row>
     <row r="38">
@@ -3843,22 +3843,22 @@
         <v>8</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.00315</v>
+        <v>0.0024</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>81</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.016</v>
+        <v>0.01481666666666667</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.08496666666666668</v>
+        <v>0.083785</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.01441666666666667</v>
+        <v>0.01043333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3877,22 +3877,22 @@
         <v>8</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.00065</v>
+        <v>0.0009</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.006283333333333333</v>
+        <v>0.005891666666666667</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.0982933333333333</v>
+        <v>0.1093916666666667</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.009258333333333334</v>
+        <v>0.005816666666666667</v>
       </c>
     </row>
     <row r="40">
@@ -3908,25 +3908,25 @@
         <v>21</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.0003833333333333333</v>
+        <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.02141666666666667</v>
+        <v>0.01041666666666667</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1461</v>
+        <v>0.1808</v>
       </c>
     </row>
     <row r="41">
@@ -3945,22 +3945,22 @@
         <v>7</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.002</v>
+        <v>0.0017</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.0078</v>
+        <v>0.007433333333333334</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.04533333333333333</v>
+        <v>0.04771666666666666</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.1209333333333333</v>
+        <v>0.09715000000000001</v>
       </c>
     </row>
     <row r="42">
@@ -3985,16 +3985,16 @@
         <v>52</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.0047</v>
+        <v>0.006083333333333333</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2713416666666666</v>
+        <v>0.2352666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 21:40:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Round of 32: Texas over Gonzaga</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T01:20:43.984578+00:00</t>
+          <t>2026-03-22T01:40:07.669177+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 22:02:14 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T01:40:07.669177+00:00</t>
+          <t>2026-03-22T02:02:12.540678+00:00</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 22:28:44 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leaderboard'!$A$1:$J$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>164b5778cca71ffb</t>
+          <t>165dfae70dd42676</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>519ed8091a1b1179</t>
+          <t>164b5778cca71ffb</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Round of 32: Illinois over VCU</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T02:02:12.540678+00:00</t>
+          <t>2026-03-22T02:28:44.284204+00:00</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2336,10 +2336,14 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Illinois</t>
+        </is>
+      </c>
       <c r="F44" s="4" t="b">
         <v>0</v>
       </c>
@@ -2524,8 +2528,41 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Sweet 16</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Illinois vs Houston</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G50" s="5" t="inlineStr"/>
+      <c r="H50" s="5" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>R16_S_02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I49"/>
+  <autoFilter ref="A1:I50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2613,25 +2650,25 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3216333333333333</v>
+        <v>0.3500833333333334</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>360</v>
+        <v>349</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.63855</v>
+        <v>0.6759666666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9404749999999998</v>
+        <v>0.9517333333333334</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2647,25 +2684,25 @@
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1084333333333334</v>
+        <v>0.1176916666666667</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>134</v>
+        <v>137.5</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.3062</v>
+        <v>0.3307166666666667</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6386833333333336</v>
+        <v>0.6707633333333333</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2681,28 +2718,28 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.08586666666666666</v>
+        <v>0.09734166666666669</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2242083333333333</v>
+        <v>0.251875</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5122533333333333</v>
+        <v>0.5457666666666666</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="5">
@@ -2721,22 +2758,22 @@
         <v>10</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.09088333333333333</v>
+        <v>0.08086666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.2054916666666667</v>
+        <v>0.1838</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4843716666666666</v>
+        <v>0.4700666666666667</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="6">
@@ -2745,29 +2782,29 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.02573333333333334</v>
+        <v>0.01561666666666667</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>305</v>
+        <v>262</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1104833333333333</v>
+        <v>0.09752499999999999</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3549683333333333</v>
+        <v>0.3251749999999999</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2779,32 +2816,32 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.01783333333333333</v>
+        <v>0.06853333333333332</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>334</v>
+        <v>290</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1318666666666667</v>
+        <v>0.2144416666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.5799566666666667</v>
+        <v>0.6348666666666666</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>5e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -2813,29 +2850,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0143</v>
+        <v>0.0216</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>264</v>
+        <v>332</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.08604166666666667</v>
+        <v>0.09845000000000001</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.2997533333333334</v>
+        <v>0.3329166666666667</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2847,32 +2884,32 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.06731666666666666</v>
+        <v>0.01698333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>284</v>
+        <v>336</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1974833333333333</v>
+        <v>0.1194833333333334</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.5961033333333334</v>
+        <v>0.5699500000000002</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0</v>
+        <v>3.333333333333333e-05</v>
       </c>
     </row>
     <row r="10">
@@ -2891,22 +2928,22 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0411</v>
+        <v>0.03570833333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>98</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>268</v>
+        <v>288</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1040083333333333</v>
+        <v>0.09398333333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2575616666666666</v>
+        <v>0.2405666666666667</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.00055</v>
+        <v>0.0006833333333333334</v>
       </c>
     </row>
     <row r="11">
@@ -2915,29 +2952,29 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.02725</v>
+        <v>0</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>267</v>
+        <v>285</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.09158333333333335</v>
+        <v>0.03291666666666667</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3514016666666668</v>
+        <v>0.3134416666666666</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -2949,32 +2986,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02176666666666667</v>
+        <v>0.002533333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>339</v>
+        <v>250</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1106333333333333</v>
+        <v>0.03953333333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.5238633333333332</v>
+        <v>0.32585</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="13">
@@ -2983,32 +3020,32 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
         <v>35</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.01888333333333333</v>
+        <v>0.0301</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>334</v>
+        <v>267</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.09326666666666668</v>
+        <v>0.1262833333333333</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.4513333333333336</v>
+        <v>0.3917583333333333</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0002</v>
+        <v>3.333333333333333e-05</v>
       </c>
     </row>
     <row r="14">
@@ -3017,32 +3054,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0</v>
+        <v>0.025275</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>329</v>
+        <v>282</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.00015</v>
+        <v>0.087475</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.1383416666666667</v>
+        <v>0.3384383333333335</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.0032</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3051,29 +3088,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.01406666666666667</v>
+        <v>0.0167</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.07041666666666667</v>
+        <v>0.09762500000000002</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3831316666666668</v>
+        <v>0.4969466666666666</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3085,32 +3122,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0028</v>
+        <v>0.01468333333333333</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>266</v>
+        <v>337</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.03265</v>
+        <v>0.0852666666666667</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2898116666666665</v>
+        <v>0.4304416666666666</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.00095</v>
+        <v>0.0001333333333333333</v>
       </c>
     </row>
     <row r="17">
@@ -3119,32 +3156,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.00195</v>
+        <v>0</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>75</v>
+        <v>103</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>241</v>
+        <v>313</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.01898333333333333</v>
+        <v>8.333333333333333e-05</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.08337</v>
+        <v>0.127075</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.06783333333333333</v>
+        <v>0.00335</v>
       </c>
     </row>
     <row r="18">
@@ -3153,32 +3190,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0</v>
+        <v>0.00495</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0</v>
+        <v>0.03315833333333334</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.01391</v>
+        <v>0.1698583333333333</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.01265</v>
+        <v>0.01918333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -3187,32 +3224,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.06571666666666666</v>
+        <v>0</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>273</v>
+        <v>318</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.1525583333333333</v>
+        <v>0.02826666666666667</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.407755</v>
+        <v>0.3446416666666666</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.001233333333333333</v>
+        <v>0.0005833333333333333</v>
       </c>
     </row>
     <row r="20">
@@ -3221,32 +3258,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.03</v>
+        <v>0.0017</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.1188666666666667</v>
+        <v>0.01908333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3749283333333332</v>
+        <v>0.07628333333333333</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.0005</v>
+        <v>0.07270000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -3255,32 +3292,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>267</v>
+        <v>225</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02248333333333333</v>
+        <v>0</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.1320666666666666</v>
+        <v>0.01264166666666667</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.0004</v>
+        <v>0.01158333333333333</v>
       </c>
     </row>
     <row r="22">
@@ -3289,32 +3326,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.0019</v>
+        <v>0.06133333333333334</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.02441666666666667</v>
+        <v>0.143975</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2456316666666667</v>
+        <v>0.3798416666666666</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0</v>
+        <v>0.00155</v>
       </c>
     </row>
     <row r="23">
@@ -3323,32 +3360,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>226</v>
+        <v>265</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.0075</v>
+        <v>0.01905</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.08437500000000001</v>
+        <v>0.1269916666666667</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.01358333333333333</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="24">
@@ -3357,32 +3394,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.00715</v>
+        <v>0.01630833333333333</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>207</v>
+        <v>264</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03693333333333333</v>
+        <v>0.060325</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1532750000000001</v>
+        <v>0.2580749999999999</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.007033333333333334</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="25">
@@ -3391,32 +3428,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.0044</v>
+        <v>0.002</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>82</v>
+        <v>109</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>224</v>
+        <v>272</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.03073333333333334</v>
+        <v>0.02121666666666666</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1607433333333333</v>
+        <v>0.2314299999999999</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.02708333333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3425,32 +3462,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0</v>
+        <v>0.0012</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>336</v>
+        <v>204</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02115</v>
+        <v>0.01049166666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.3025616666666666</v>
+        <v>0.119775</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.0009</v>
+        <v>0.00405</v>
       </c>
     </row>
     <row r="27">
@@ -3459,32 +3496,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.0009</v>
+        <v>0.0008</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>189</v>
+        <v>223</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.00275</v>
+        <v>0.0076</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.009508333333333334</v>
+        <v>0.07798333333333336</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.2084166666666666</v>
+        <v>0.01443333333333333</v>
       </c>
     </row>
     <row r="28">
@@ -3493,32 +3530,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00035</v>
+        <v>0.0002</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>266</v>
+        <v>226</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.005466666666666667</v>
+        <v>0.002666666666666667</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.09282999999999998</v>
+        <v>0.06288333333333333</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.0018</v>
+        <v>0.01166666666666667</v>
       </c>
     </row>
     <row r="29">
@@ -3527,32 +3564,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D29" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.0003333333333333333</v>
+        <v>0.00725</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.006266666666666667</v>
+        <v>0.03233333333333334</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.08702500000000001</v>
+        <v>0.1397916666666667</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0054</v>
+        <v>0.007416666666666667</v>
       </c>
     </row>
     <row r="30">
@@ -3561,32 +3598,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.00115</v>
+        <v>0.0002333333333333333</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>261</v>
+        <v>228</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.007583333333333334</v>
+        <v>0.004508333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.03525833333333333</v>
+        <v>0.1266833333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.02335</v>
+        <v>0.00615</v>
       </c>
     </row>
     <row r="31">
@@ -3595,32 +3632,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.01623333333333333</v>
+        <v>0.0005</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.05603333333333332</v>
+        <v>0.0047</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.2369316666666667</v>
+        <v>0.08441333333333334</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.0009</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="32">
@@ -3629,32 +3666,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00065</v>
+        <v>0.0005</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>203</v>
+        <v>190</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.007875</v>
+        <v>0.0021</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1018583333333333</v>
+        <v>0.007933333333333332</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.008133333333333333</v>
+        <v>0.2256333333333333</v>
       </c>
     </row>
     <row r="33">
@@ -3663,32 +3700,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D33" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.003416666666666667</v>
+        <v>0.005783333333333333</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.050535</v>
+        <v>0.08367499999999999</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.01688333333333333</v>
+        <v>0.006866666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3697,32 +3734,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>5e-05</v>
+        <v>0.002083333333333333</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.001383333333333333</v>
+        <v>0.01503333333333333</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03747833333333334</v>
+        <v>0.08735833333333334</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02513333333333333</v>
+        <v>0.00755</v>
       </c>
     </row>
     <row r="35">
@@ -3731,32 +3768,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00385</v>
+        <v>0.00055</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>231</v>
+        <v>270</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.02335</v>
+        <v>0.009291666666666667</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.14598</v>
+        <v>0.1277166666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0</v>
+        <v>0.004566666666666667</v>
       </c>
     </row>
     <row r="36">
@@ -3765,32 +3802,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.004891666666666667</v>
+        <v>0</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.1125166666666667</v>
+        <v>0.002208333333333333</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.01255</v>
+        <v>0.03135</v>
       </c>
     </row>
     <row r="37">
@@ -3799,32 +3836,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.0012</v>
+        <v>0.00015</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.01608333333333333</v>
+        <v>0.0013</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.07205833333333332</v>
+        <v>0.03666666666666667</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.0317</v>
+        <v>0.02638333333333333</v>
       </c>
     </row>
     <row r="38">
@@ -3833,32 +3870,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.0024</v>
+        <v>0.002775</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.01481666666666667</v>
+        <v>0.019525</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.083785</v>
+        <v>0.1382083333333333</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.01043333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -3867,32 +3904,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0009</v>
+        <v>0.0026</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>261</v>
+        <v>223</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.005891666666666667</v>
+        <v>0.01066666666666667</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.1093916666666667</v>
+        <v>0.053925</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.005816666666666667</v>
+        <v>0.07711666666666668</v>
       </c>
     </row>
     <row r="40">
@@ -3901,32 +3938,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0</v>
+        <v>0.00115</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>192</v>
+        <v>254</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0</v>
+        <v>0.0133</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.01041666666666667</v>
+        <v>0.07055</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1808</v>
+        <v>0.0347</v>
       </c>
     </row>
     <row r="41">
@@ -3935,32 +3972,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D41" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.0017</v>
+        <v>0</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>248</v>
+        <v>192</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.007433333333333334</v>
+        <v>0.0001</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.04771666666666666</v>
+        <v>0.01070833333333333</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.09715000000000001</v>
+        <v>0.1851166666666666</v>
       </c>
     </row>
     <row r="42">
@@ -3985,16 +4022,16 @@
         <v>52</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="H42" s="5" t="n">
         <v>0.0001</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.006083333333333333</v>
+        <v>0.004</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2352666666666667</v>
+        <v>0.2433166666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 22:49:39 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Round of 32: Illinois over VCU</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T02:28:44.284204+00:00</t>
+          <t>2026-03-22T02:49:38.269966+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 23:05:56 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T02:49:38.269966+00:00</t>
+          <t>2026-03-22T03:05:56.149754+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-21 23:28:33 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T03:05:56.149754+00:00</t>
+          <t>2026-03-22T03:28:32.945256+00:00</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 10:33:42 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/21/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/20/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/22/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/21/all-conf</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>44</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>165dfae70dd42676</t>
+          <t>f18ca837ac5d50d9</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>164b5778cca71ffb</t>
+          <t>165dfae70dd42676</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>40</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>22</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T03:42:05.457139+00:00</t>
+          <t>2026-03-22T14:33:41.935526+00:00</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2303,10 +2303,14 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Nebraska</t>
+        </is>
+      </c>
       <c r="F43" s="6" t="b">
         <v>0</v>
       </c>
@@ -2336,7 +2340,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2373,7 +2377,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2410,15 +2414,19 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G46" s="5" t="inlineStr"/>
-      <c r="H46" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>0.8522683568135787</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>0.1477316431864213</v>
+      </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
           <t>R32_W_01</t>
@@ -2443,10 +2451,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Arkansas</t>
+        </is>
+      </c>
       <c r="F47" s="6" t="b">
         <v>0</v>
       </c>
@@ -2476,7 +2488,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2513,7 +2525,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -2650,25 +2662,25 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3500833333333334</v>
+        <v>0.3190833333333334</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>349</v>
+        <v>329</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6759666666666667</v>
+        <v>0.6526416666666666</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9517333333333334</v>
+        <v>0.9468066666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2680,29 +2692,29 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Stephen Mason</t>
+          <t>Ryan Evans</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1176916666666667</v>
+        <v>0.1385666666666666</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>137.5</v>
+        <v>130</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>305</v>
+        <v>292</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.3307166666666667</v>
+        <v>0.32535</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6707633333333333</v>
+        <v>0.6652366666666667</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2714,32 +2726,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Ryan Evans</t>
+          <t>Stephen Mason</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.09734166666666669</v>
+        <v>0.08456666666666666</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>299</v>
+        <v>310</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.251875</v>
+        <v>0.2569833333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5457666666666666</v>
+        <v>0.5962500000000001</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2748,32 +2760,32 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.08086666666666667</v>
+        <v>0.01378333333333333</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>320</v>
+        <v>227</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1838</v>
+        <v>0.07988333333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4700666666666667</v>
+        <v>0.303665</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2782,29 +2794,29 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.01561666666666667</v>
+        <v>0.06038333333333334</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.09752499999999999</v>
+        <v>0.1879666666666666</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.3251749999999999</v>
+        <v>0.5999316666666668</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2816,29 +2828,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.06853333333333332</v>
+        <v>0.04246666666666667</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>290</v>
+        <v>259</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.2144416666666666</v>
+        <v>0.1320833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.6348666666666666</v>
+        <v>0.4254816666666669</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2854,25 +2866,25 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0216</v>
+        <v>0.0136</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>332</v>
+        <v>278</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.09845000000000001</v>
+        <v>0.05803333333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3329166666666667</v>
+        <v>0.2759416666666666</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2888,28 +2900,28 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.01698333333333333</v>
+        <v>0.01295</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>336</v>
+        <v>300</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1194833333333334</v>
+        <v>0.10125</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.5699500000000002</v>
+        <v>0.5414950000000003</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.333333333333333e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2918,32 +2930,32 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.03570833333333333</v>
+        <v>0.1205333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.09398333333333334</v>
+        <v>0.2684833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.2405666666666667</v>
+        <v>0.6018733333333334</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0006833333333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2956,25 +2968,25 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>285</v>
+        <v>250</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.03291666666666667</v>
+        <v>0.02985</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3134416666666666</v>
+        <v>0.2761116666666666</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -2986,32 +2998,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.002533333333333333</v>
+        <v>0.04118333333333334</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>250</v>
+        <v>271</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.03953333333333334</v>
+        <v>0.10345</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.32585</v>
+        <v>0.2597533333333332</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.00075</v>
+        <v>0.00065</v>
       </c>
     </row>
     <row r="13">
@@ -3020,32 +3032,32 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.0301</v>
+        <v>0.01475</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>111</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>267</v>
+        <v>304</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.1262833333333333</v>
+        <v>0.0771</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3917583333333333</v>
+        <v>0.4064400000000001</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>3.333333333333333e-05</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="14">
@@ -3054,29 +3066,29 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.025275</v>
+        <v>0.01425</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.087475</v>
+        <v>0.09035000000000003</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.3384383333333335</v>
+        <v>0.4551400000000002</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3088,32 +3100,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.0167</v>
+        <v>0.03498333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.09762500000000002</v>
+        <v>0.11015</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.4969466666666666</v>
+        <v>0.34957</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="16">
@@ -3122,32 +3134,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.01468333333333333</v>
+        <v>0</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>337</v>
+        <v>280</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0852666666666667</v>
+        <v>0</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.4304416666666666</v>
+        <v>0.1056583333333333</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.0001333333333333333</v>
+        <v>0.004383333333333334</v>
       </c>
     </row>
     <row r="17">
@@ -3156,32 +3168,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0</v>
+        <v>0.05256666666666666</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>313</v>
+        <v>252</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>8.333333333333333e-05</v>
+        <v>0.2191833333333333</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.127075</v>
+        <v>0.5744583333333336</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.00335</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3190,32 +3202,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.00495</v>
+        <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>86</v>
+        <v>107.5</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>224</v>
+        <v>281</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.03315833333333334</v>
+        <v>0.01825</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1698583333333333</v>
+        <v>0.3167616666666666</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.01918333333333333</v>
+        <v>0.00015</v>
       </c>
     </row>
     <row r="19">
@@ -3224,32 +3236,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E19" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>117</v>
+        <v>64</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>318</v>
+        <v>173</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02826666666666667</v>
+        <v>0</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.3446416666666666</v>
+        <v>0.007133333333333334</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.0005833333333333333</v>
+        <v>0.01429166666666667</v>
       </c>
     </row>
     <row r="20">
@@ -3258,32 +3270,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.0017</v>
+        <v>0.007883333333333334</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>252</v>
+        <v>226</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.01908333333333333</v>
+        <v>0.05826666666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.07628333333333333</v>
+        <v>0.2632966666666667</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.07270000000000001</v>
+        <v>0.009633333333333332</v>
       </c>
     </row>
     <row r="21">
@@ -3292,32 +3304,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0</v>
+        <v>0.00825</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.01264166666666667</v>
+        <v>0.06273166666666667</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.01158333333333333</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="22">
@@ -3326,32 +3338,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.06133333333333334</v>
+        <v>0.01223333333333333</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>274</v>
+        <v>203</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.143975</v>
+        <v>0.04919999999999999</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.3798416666666666</v>
+        <v>0.2388516666666666</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.00155</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="23">
@@ -3360,32 +3372,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0</v>
+        <v>0.001933333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>265</v>
+        <v>241</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01905</v>
+        <v>0.0164</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1269916666666667</v>
+        <v>0.206015</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0005</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -3394,32 +3406,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.01630833333333333</v>
+        <v>0.004</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>264</v>
+        <v>197</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.060325</v>
+        <v>0.03466666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2580749999999999</v>
+        <v>0.1628583333333334</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0003</v>
+        <v>0.0037</v>
       </c>
     </row>
     <row r="25">
@@ -3428,29 +3440,29 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.002</v>
+        <v>0.0012</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>272</v>
+        <v>210</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.02121666666666666</v>
+        <v>0.01245</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.2314299999999999</v>
+        <v>0.137285</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>0</v>
@@ -3462,32 +3474,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.0012</v>
+        <v>0.001</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.01049166666666667</v>
+        <v>0.0158</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.119775</v>
+        <v>0.2321</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.00405</v>
+        <v>0.002066666666666666</v>
       </c>
     </row>
     <row r="27">
@@ -3496,32 +3508,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.0008</v>
+        <v>0.0002</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0076</v>
+        <v>0.00375</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.07798333333333336</v>
+        <v>0.07245</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01443333333333333</v>
+        <v>0.002283333333333333</v>
       </c>
     </row>
     <row r="28">
@@ -3530,32 +3542,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.0011</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>226</v>
+        <v>182</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.002666666666666667</v>
+        <v>0.01233333333333333</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.06288333333333333</v>
+        <v>0.08643333333333335</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.01166666666666667</v>
+        <v>0.006233333333333334</v>
       </c>
     </row>
     <row r="29">
@@ -3564,32 +3576,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.00725</v>
+        <v>0</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>95</v>
+        <v>59</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>205</v>
+        <v>167</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.03233333333333334</v>
+        <v>0</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1397916666666667</v>
+        <v>0.0025</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.007416666666666667</v>
+        <v>0.02694166666666667</v>
       </c>
     </row>
     <row r="30">
@@ -3598,32 +3610,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0002333333333333333</v>
+        <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>228</v>
+        <v>164</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.004508333333333334</v>
+        <v>0.0003833333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1266833333333333</v>
+        <v>0.023235</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.00615</v>
+        <v>0.03351666666666666</v>
       </c>
     </row>
     <row r="31">
@@ -3632,32 +3644,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>253</v>
+        <v>203</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.0047</v>
+        <v>0.01675833333333333</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.08441333333333334</v>
+        <v>0.1258116666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -3666,32 +3678,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>5</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0005</v>
+        <v>0.00165</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>190</v>
+        <v>224</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.0021</v>
+        <v>0.01578333333333333</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.007933333333333332</v>
+        <v>0.06108333333333334</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.2256333333333333</v>
+        <v>0.136075</v>
       </c>
     </row>
     <row r="33">
@@ -3700,32 +3712,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.005783333333333333</v>
+        <v>0.01016666666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.08367499999999999</v>
+        <v>0.06361666666666667</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.006866666666666666</v>
+        <v>0.04986666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3734,32 +3746,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.002083333333333333</v>
+        <v>0.00135</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>223</v>
+        <v>209</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.01503333333333333</v>
+        <v>0.014525</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.08735833333333334</v>
+        <v>0.15638</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.00755</v>
+        <v>0.002833333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3768,32 +3780,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.00065</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.009291666666666667</v>
+        <v>0.003983333333333334</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.1277166666666667</v>
+        <v>0.05794166666666666</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.004566666666666667</v>
+        <v>0.02643333333333334</v>
       </c>
     </row>
     <row r="36">
@@ -3802,32 +3814,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>222</v>
+        <v>172</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0</v>
+        <v>0.001016666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.002208333333333333</v>
+        <v>0.03671833333333333</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.03135</v>
+        <v>0.0237</v>
       </c>
     </row>
     <row r="37">
@@ -3836,32 +3848,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.00015</v>
+        <v>0.0001</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0013</v>
+        <v>0.004575</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.03666666666666667</v>
+        <v>0.1657483333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.02638333333333333</v>
+        <v>0.00615</v>
       </c>
     </row>
     <row r="38">
@@ -3870,32 +3882,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.002775</v>
+        <v>0</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>234</v>
+        <v>192</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.019525</v>
+        <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.1382083333333333</v>
+        <v>0.0139</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0</v>
+        <v>0.10935</v>
       </c>
     </row>
     <row r="39">
@@ -3904,32 +3916,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.0026</v>
+        <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>223</v>
+        <v>129</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.01066666666666667</v>
+        <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.053925</v>
+        <v>0.0007833333333333333</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.07711666666666668</v>
+        <v>0.2358666666666666</v>
       </c>
     </row>
     <row r="40">
@@ -3938,32 +3950,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D40" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.00115</v>
+        <v>0.0002833333333333333</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>254</v>
+        <v>228</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.0133</v>
+        <v>0.00555</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.07055</v>
+        <v>0.07956000000000001</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.0347</v>
+        <v>0.006791666666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3972,32 +3984,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D41" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0</v>
+        <v>0.00135</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>192</v>
+        <v>241</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.004933333333333334</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.01070833333333333</v>
+        <v>0.03494166666666666</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.1851166666666666</v>
+        <v>0.08119999999999999</v>
       </c>
     </row>
     <row r="42">
@@ -4019,19 +4031,19 @@
         <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.004</v>
+        <v>0.00805</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2433166666666666</v>
+        <v>0.2164333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 12:00:04 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T14:33:41.935526+00:00</t>
+          <t>2026-03-22T16:00:04.035381+00:00</t>
         </is>
       </c>
     </row>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8522683568135787</v>
+        <v>0.8516603694614894</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1477316431864213</v>
+        <v>0.1483396305385106</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2668,7 +2668,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3190833333333334</v>
+        <v>0.3188333333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>150</v>
@@ -2677,10 +2677,10 @@
         <v>329</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6526416666666666</v>
+        <v>0.6524416666666666</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9468066666666666</v>
+        <v>0.9467066666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2702,7 +2702,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1385666666666666</v>
+        <v>0.1386666666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>130</v>
@@ -2714,7 +2714,7 @@
         <v>0.32535</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6652366666666667</v>
+        <v>0.6653366666666667</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2745,7 +2745,7 @@
         <v>310</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2569833333333333</v>
+        <v>0.2568833333333334</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>0.5962500000000001</v>
@@ -2782,7 +2782,7 @@
         <v>0.07988333333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.303665</v>
+        <v>0.303615</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2813,7 +2813,7 @@
         <v>258</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1879666666666666</v>
+        <v>0.1881666666666666</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0.5999316666666668</v>
@@ -2850,7 +2850,7 @@
         <v>0.1320833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4254816666666669</v>
+        <v>0.4252816666666668</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2884,7 +2884,7 @@
         <v>0.05803333333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.2759416666666666</v>
+        <v>0.2762416666666666</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2915,7 +2915,7 @@
         <v>300</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.10125</v>
+        <v>0.10115</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>0.5414950000000003</v>
@@ -2940,7 +2940,7 @@
         <v>10</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.1205333333333333</v>
+        <v>0.1204333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>124</v>
@@ -2949,7 +2949,7 @@
         <v>278</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.2684833333333333</v>
+        <v>0.2683833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>0.6018733333333334</v>
@@ -3110,7 +3110,7 @@
         <v>9</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.03498333333333334</v>
+        <v>0.03523333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>104</v>
@@ -3119,10 +3119,10 @@
         <v>310</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.11015</v>
+        <v>0.11055</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.34957</v>
+        <v>0.34997</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00075</v>
@@ -3187,10 +3187,10 @@
         <v>252</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.2191833333333333</v>
+        <v>0.2190833333333333</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.5744583333333336</v>
+        <v>0.5741583333333335</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3215,7 +3215,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>107.5</v>
+        <v>108</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>281</v>
@@ -3224,7 +3224,7 @@
         <v>0.01825</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.3167616666666666</v>
+        <v>0.3166616666666666</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0.00015</v>
@@ -3292,7 +3292,7 @@
         <v>0.05826666666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2632966666666667</v>
+        <v>0.2629966666666667</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.009633333333333332</v>
@@ -3323,10 +3323,10 @@
         <v>211</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.00825</v>
+        <v>0.00835</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.06273166666666667</v>
+        <v>0.06303166666666667</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0005</v>
@@ -3360,7 +3360,7 @@
         <v>0.04919999999999999</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2388516666666666</v>
+        <v>0.2386516666666667</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0001</v>
@@ -3385,7 +3385,7 @@
         <v>0.001933333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>99</v>
+        <v>99.5</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>241</v>
@@ -3530,7 +3530,7 @@
         <v>0.00375</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.07245</v>
+        <v>0.07255</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.002283333333333333</v>
@@ -3663,7 +3663,7 @@
         <v>203</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.01675833333333333</v>
+        <v>0.01665833333333333</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0.1258116666666667</v>
@@ -3703,7 +3703,7 @@
         <v>0.06108333333333334</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.136075</v>
+        <v>0.136025</v>
       </c>
     </row>
     <row r="33">
@@ -3768,7 +3768,7 @@
         <v>0.014525</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.15638</v>
+        <v>0.15618</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>0.002833333333333333</v>
@@ -3836,7 +3836,7 @@
         <v>0.001016666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.03671833333333333</v>
+        <v>0.03666833333333333</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0237</v>
@@ -3870,7 +3870,7 @@
         <v>0.004575</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1657483333333334</v>
+        <v>0.1656483333333334</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>0.00615</v>
@@ -3904,10 +3904,10 @@
         <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.0139</v>
+        <v>0.014</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.10935</v>
+        <v>0.10925</v>
       </c>
     </row>
     <row r="39">
@@ -4006,7 +4006,7 @@
         <v>0.004933333333333334</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.03494166666666666</v>
+        <v>0.03524166666666666</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.08119999999999999</v>
@@ -4043,7 +4043,7 @@
         <v>0.00805</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2164333333333333</v>
+        <v>0.2165833333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 12:32:42 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T16:00:04.035381+00:00</t>
+          <t>2026-03-22T16:32:41.535406+00:00</t>
         </is>
       </c>
     </row>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8516603694614894</v>
+        <v>0.8523019056693478</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1483396305385106</v>
+        <v>0.1476980943306522</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -2668,7 +2668,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3188333333333334</v>
+        <v>0.3190833333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>150</v>
@@ -2677,10 +2677,10 @@
         <v>329</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6524416666666666</v>
+        <v>0.6526416666666666</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9467066666666666</v>
+        <v>0.9468066666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2702,7 +2702,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1386666666666667</v>
+        <v>0.1385666666666666</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>130</v>
@@ -2714,7 +2714,7 @@
         <v>0.32535</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6653366666666667</v>
+        <v>0.6652366666666667</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2745,7 +2745,7 @@
         <v>310</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2568833333333334</v>
+        <v>0.2569833333333333</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>0.5962500000000001</v>
@@ -2782,7 +2782,7 @@
         <v>0.07988333333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.303615</v>
+        <v>0.303665</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2813,7 +2813,7 @@
         <v>258</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1881666666666666</v>
+        <v>0.1879666666666666</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0.5999316666666668</v>
@@ -2850,7 +2850,7 @@
         <v>0.1320833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4252816666666668</v>
+        <v>0.4254816666666669</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2884,7 +2884,7 @@
         <v>0.05803333333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.2762416666666666</v>
+        <v>0.2759416666666666</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2915,7 +2915,7 @@
         <v>300</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.10115</v>
+        <v>0.10125</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>0.5414950000000003</v>
@@ -2940,7 +2940,7 @@
         <v>10</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.1204333333333333</v>
+        <v>0.1205333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>124</v>
@@ -2949,7 +2949,7 @@
         <v>278</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.2683833333333333</v>
+        <v>0.2684833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>0.6018733333333334</v>
@@ -3110,7 +3110,7 @@
         <v>9</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.03523333333333334</v>
+        <v>0.03498333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>104</v>
@@ -3119,10 +3119,10 @@
         <v>310</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.11055</v>
+        <v>0.11015</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.34997</v>
+        <v>0.34957</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00075</v>
@@ -3187,10 +3187,10 @@
         <v>252</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.2190833333333333</v>
+        <v>0.2191833333333333</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.5741583333333335</v>
+        <v>0.5744583333333336</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3215,7 +3215,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>108</v>
+        <v>107.5</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>281</v>
@@ -3224,7 +3224,7 @@
         <v>0.01825</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.3166616666666666</v>
+        <v>0.3167616666666666</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0.00015</v>
@@ -3292,7 +3292,7 @@
         <v>0.05826666666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2629966666666667</v>
+        <v>0.2632966666666667</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.009633333333333332</v>
@@ -3323,10 +3323,10 @@
         <v>211</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.00835</v>
+        <v>0.00825</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.06303166666666667</v>
+        <v>0.06273166666666667</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0005</v>
@@ -3360,7 +3360,7 @@
         <v>0.04919999999999999</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2386516666666667</v>
+        <v>0.2388516666666666</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0001</v>
@@ -3385,7 +3385,7 @@
         <v>0.001933333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>99.5</v>
+        <v>99</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>241</v>
@@ -3530,7 +3530,7 @@
         <v>0.00375</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.07255</v>
+        <v>0.07245</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.002283333333333333</v>
@@ -3663,7 +3663,7 @@
         <v>203</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.01665833333333333</v>
+        <v>0.01675833333333333</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0.1258116666666667</v>
@@ -3703,7 +3703,7 @@
         <v>0.06108333333333334</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.136025</v>
+        <v>0.136075</v>
       </c>
     </row>
     <row r="33">
@@ -3768,7 +3768,7 @@
         <v>0.014525</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.15618</v>
+        <v>0.15638</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>0.002833333333333333</v>
@@ -3836,7 +3836,7 @@
         <v>0.001016666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.03666833333333333</v>
+        <v>0.03671833333333333</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0237</v>
@@ -3870,7 +3870,7 @@
         <v>0.004575</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1656483333333334</v>
+        <v>0.1657483333333334</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>0.00615</v>
@@ -3904,10 +3904,10 @@
         <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.014</v>
+        <v>0.0139</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.10925</v>
+        <v>0.10935</v>
       </c>
     </row>
     <row r="39">
@@ -4006,7 +4006,7 @@
         <v>0.004933333333333334</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.03524166666666666</v>
+        <v>0.03494166666666666</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.08119999999999999</v>
@@ -4043,7 +4043,7 @@
         <v>0.00805</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2165833333333333</v>
+        <v>0.2164333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 13:20:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T17:00:08.173904+00:00</t>
+          <t>2026-03-22T17:20:08.220556+00:00</t>
         </is>
       </c>
     </row>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8523019056693478</v>
+        <v>0.8517321586216384</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1476980943306522</v>
+        <v>0.1482678413783616</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2668,7 +2668,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3190833333333334</v>
+        <v>0.3188333333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>150</v>
@@ -2677,10 +2677,10 @@
         <v>329</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6526416666666666</v>
+        <v>0.6524416666666666</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9468066666666666</v>
+        <v>0.9467066666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2702,7 +2702,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1385666666666666</v>
+        <v>0.1386666666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>130</v>
@@ -2714,7 +2714,7 @@
         <v>0.32535</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6652366666666667</v>
+        <v>0.6653366666666667</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2745,7 +2745,7 @@
         <v>310</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2569833333333333</v>
+        <v>0.2568833333333334</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>0.5962500000000001</v>
@@ -2782,7 +2782,7 @@
         <v>0.07988333333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.303665</v>
+        <v>0.303615</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2813,7 +2813,7 @@
         <v>258</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1879666666666666</v>
+        <v>0.1881666666666666</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0.5999316666666668</v>
@@ -2850,7 +2850,7 @@
         <v>0.1320833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4254816666666669</v>
+        <v>0.4252816666666668</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2884,7 +2884,7 @@
         <v>0.05803333333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.2759416666666666</v>
+        <v>0.2762416666666666</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2915,7 +2915,7 @@
         <v>300</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.10125</v>
+        <v>0.10115</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>0.5414950000000003</v>
@@ -2940,7 +2940,7 @@
         <v>10</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.1205333333333333</v>
+        <v>0.1204333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>124</v>
@@ -2949,7 +2949,7 @@
         <v>278</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.2684833333333333</v>
+        <v>0.2683833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>0.6018733333333334</v>
@@ -3110,7 +3110,7 @@
         <v>9</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.03498333333333334</v>
+        <v>0.03523333333333334</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>104</v>
@@ -3119,10 +3119,10 @@
         <v>310</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.11015</v>
+        <v>0.11055</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.34957</v>
+        <v>0.34997</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00075</v>
@@ -3187,10 +3187,10 @@
         <v>252</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.2191833333333333</v>
+        <v>0.2190833333333333</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.5744583333333336</v>
+        <v>0.5741583333333335</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3215,7 +3215,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>107.5</v>
+        <v>108</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>281</v>
@@ -3224,7 +3224,7 @@
         <v>0.01825</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.3167616666666666</v>
+        <v>0.3166616666666666</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0.00015</v>
@@ -3292,7 +3292,7 @@
         <v>0.05826666666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2632966666666667</v>
+        <v>0.2629966666666667</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.009633333333333332</v>
@@ -3323,10 +3323,10 @@
         <v>211</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.00825</v>
+        <v>0.00835</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.06273166666666667</v>
+        <v>0.06303166666666667</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0005</v>
@@ -3360,7 +3360,7 @@
         <v>0.04919999999999999</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2388516666666666</v>
+        <v>0.2386516666666667</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0001</v>
@@ -3385,7 +3385,7 @@
         <v>0.001933333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>99</v>
+        <v>99.5</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>241</v>
@@ -3530,7 +3530,7 @@
         <v>0.00375</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.07245</v>
+        <v>0.07255</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.002283333333333333</v>
@@ -3663,7 +3663,7 @@
         <v>203</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.01675833333333333</v>
+        <v>0.01665833333333333</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0.1258116666666667</v>
@@ -3703,7 +3703,7 @@
         <v>0.06108333333333334</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.136075</v>
+        <v>0.136025</v>
       </c>
     </row>
     <row r="33">
@@ -3768,7 +3768,7 @@
         <v>0.014525</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.15638</v>
+        <v>0.15618</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>0.002833333333333333</v>
@@ -3836,7 +3836,7 @@
         <v>0.001016666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.03671833333333333</v>
+        <v>0.03666833333333333</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0237</v>
@@ -3870,7 +3870,7 @@
         <v>0.004575</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1657483333333334</v>
+        <v>0.1656483333333334</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>0.00615</v>
@@ -3904,10 +3904,10 @@
         <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.0139</v>
+        <v>0.014</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.10935</v>
+        <v>0.10925</v>
       </c>
     </row>
     <row r="39">
@@ -4006,7 +4006,7 @@
         <v>0.004933333333333334</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.03494166666666666</v>
+        <v>0.03524166666666666</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.08119999999999999</v>
@@ -4043,7 +4043,7 @@
         <v>0.00805</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2164333333333333</v>
+        <v>0.2165833333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 13:40:09 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T17:20:08.220556+00:00</t>
+          <t>2026-03-22T17:40:09.400192+00:00</t>
         </is>
       </c>
     </row>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8517321586216384</v>
+        <v>0.8510012560261497</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1482678413783616</v>
+        <v>0.1489987439738503</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2702,7 +2702,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1386666666666667</v>
+        <v>0.1387666666666666</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>130</v>
@@ -2736,7 +2736,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.08456666666666666</v>
+        <v>0.08446666666666666</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>124</v>
@@ -3292,7 +3292,7 @@
         <v>0.05826666666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2629966666666667</v>
+        <v>0.2628966666666667</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.009633333333333332</v>
@@ -3385,7 +3385,7 @@
         <v>0.001933333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>99.5</v>
+        <v>100</v>
       </c>
       <c r="G23" s="9" t="n">
         <v>241</v>
@@ -3836,7 +3836,7 @@
         <v>0.001016666666666667</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.03666833333333333</v>
+        <v>0.03676833333333333</v>
       </c>
       <c r="J36" s="5" t="n">
         <v>0.0237</v>
@@ -3941,7 +3941,7 @@
         <v>0.0007833333333333333</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.2358666666666666</v>
+        <v>0.2358166666666666</v>
       </c>
     </row>
     <row r="40">
@@ -4043,7 +4043,7 @@
         <v>0.00805</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2165833333333333</v>
+        <v>0.2166333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 14:22:30 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T18:04:38.819366+00:00</t>
+          <t>2026-03-22T18:22:30.345685+00:00</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8510012560261497</v>
+        <v>0.8506692616155107</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1489987439738503</v>
+        <v>0.1493307383844894</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -2714,7 +2714,7 @@
         <v>0.32535</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6653366666666667</v>
+        <v>0.6654366666666667</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2745,10 +2745,10 @@
         <v>310</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2568833333333334</v>
+        <v>0.2567833333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5962500000000001</v>
+        <v>0.5960500000000001</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2779,10 +2779,10 @@
         <v>227</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.07988333333333333</v>
+        <v>0.07998333333333334</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.303615</v>
+        <v>0.303715</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2813,7 +2813,7 @@
         <v>258</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1881666666666666</v>
+        <v>0.1882666666666666</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0.5999316666666668</v>
@@ -2918,7 +2918,7 @@
         <v>0.10115</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.5414950000000003</v>
+        <v>0.5415950000000003</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -3088,7 +3088,7 @@
         <v>0.09035000000000003</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.4551400000000002</v>
+        <v>0.4552733333333335</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3122,7 +3122,7 @@
         <v>0.11055</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.34997</v>
+        <v>0.35007</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0.00075</v>
@@ -3156,7 +3156,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.1056583333333333</v>
+        <v>0.1057583333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0.004383333333333334</v>
@@ -3224,7 +3224,7 @@
         <v>0.01825</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.3166616666666666</v>
+        <v>0.3165616666666665</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0.00015</v>
@@ -3258,7 +3258,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.007133333333333334</v>
+        <v>0.007166666666666668</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0.01429166666666667</v>
@@ -3292,7 +3292,7 @@
         <v>0.05826666666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2628966666666667</v>
+        <v>0.2627966666666667</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.009633333333333332</v>
@@ -3394,7 +3394,7 @@
         <v>0.0164</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.206015</v>
+        <v>0.2061483333333334</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0</v>
@@ -3428,7 +3428,7 @@
         <v>0.03466666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1628583333333334</v>
+        <v>0.1627583333333333</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0.0037</v>
@@ -3635,7 +3635,7 @@
         <v>0.023235</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03351666666666666</v>
+        <v>0.03341666666666666</v>
       </c>
     </row>
     <row r="31">
@@ -3737,7 +3737,7 @@
         <v>0.06361666666666667</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.04986666666666666</v>
+        <v>0.04976666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -3870,7 +3870,7 @@
         <v>0.004575</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1656483333333334</v>
+        <v>0.1655483333333334</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>0.00615</v>
@@ -3941,7 +3941,7 @@
         <v>0.0007833333333333333</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.2358166666666666</v>
+        <v>0.2357666666666666</v>
       </c>
     </row>
     <row r="40">
@@ -3969,10 +3969,10 @@
         <v>228</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.00555</v>
+        <v>0.00545</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.07956000000000001</v>
+        <v>0.07946</v>
       </c>
       <c r="J40" s="5" t="n">
         <v>0.006791666666666667</v>
@@ -4006,7 +4006,7 @@
         <v>0.004933333333333334</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.03524166666666666</v>
+        <v>0.03514166666666666</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.08119999999999999</v>
@@ -4043,7 +4043,7 @@
         <v>0.00805</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2166333333333333</v>
+        <v>0.2168833333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 14:41:48 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leaderboard'!$A$1:$J$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>f18ca837ac5d50d9</t>
+          <t>a02614466dbdf7f2</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>165dfae70dd42676</t>
+          <t>f18ca837ac5d50d9</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T18:22:30.345685+00:00</t>
+          <t>2026-03-22T18:41:48.048576+00:00</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8506692616155107</v>
+        <v>0.8508454771567467</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1493307383844894</v>
+        <v>0.1491545228432533</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2525,10 +2525,14 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Purdue</t>
+        </is>
+      </c>
       <c r="F49" s="6" t="b">
         <v>0</v>
       </c>
@@ -2573,8 +2577,41 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Sweet 16</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Texas vs Purdue</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G51" s="7" t="inlineStr"/>
+      <c r="H51" s="7" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>R16_W_02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I50"/>
+  <autoFilter ref="A1:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2662,25 +2699,25 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3188333333333334</v>
+        <v>0.3368666666666668</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6524416666666666</v>
+        <v>0.6806166666666666</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9467066666666666</v>
+        <v>0.9671666666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2696,25 +2733,25 @@
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1387666666666666</v>
+        <v>0.158875</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>292</v>
+        <v>311</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.32535</v>
+        <v>0.3371166666666667</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6654366666666667</v>
+        <v>0.6797333333333335</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2730,25 +2767,25 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.08446666666666666</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2567833333333334</v>
+        <v>0.2680333333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5960500000000001</v>
+        <v>0.6122033333333333</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2760,29 +2797,29 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.01378333333333333</v>
+        <v>0.05425</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>227</v>
+        <v>259</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.07998333333333334</v>
+        <v>0.16865</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.303715</v>
+        <v>0.4779433333333334</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2798,25 +2835,25 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.06038333333333334</v>
+        <v>0.01163333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>123</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1882666666666666</v>
+        <v>0.1032833333333334</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.5999316666666668</v>
+        <v>0.5192000000000001</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2828,29 +2865,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.04246666666666667</v>
+        <v>0.0171</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>259</v>
+        <v>309</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1320833333333333</v>
+        <v>0.1155333333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4252816666666668</v>
+        <v>0.5891683333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2862,29 +2899,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0136</v>
+        <v>0.1481583333333333</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.05803333333333333</v>
+        <v>0.3028833333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.2762416666666666</v>
+        <v>0.6342699999999999</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2896,29 +2933,29 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.01295</v>
+        <v>0</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>300</v>
+        <v>257</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.10115</v>
+        <v>0.03041666666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.5415950000000003</v>
+        <v>0.31798</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2930,29 +2967,29 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.1204333333333333</v>
+        <v>0.01906666666666667</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>278</v>
+        <v>292</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.2683833333333333</v>
+        <v>0.1055</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.6018733333333334</v>
+        <v>0.4998150000000002</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -2964,29 +3001,29 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0</v>
+        <v>0.01571666666666667</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>250</v>
+        <v>316</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.02985</v>
+        <v>0.08755000000000002</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.2761116666666666</v>
+        <v>0.4503549999999999</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -2998,32 +3035,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.04118333333333334</v>
+        <v>0.0373</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>271</v>
+        <v>294</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.10345</v>
+        <v>0.1316916666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.2597533333333332</v>
+        <v>0.3877983333333333</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.00065</v>
+        <v>5e-05</v>
       </c>
     </row>
     <row r="13">
@@ -3032,32 +3069,32 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.01475</v>
+        <v>0.0072</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>304</v>
+        <v>247</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.0771</v>
+        <v>0.05221666666666668</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.4064400000000001</v>
+        <v>0.2208883333333333</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -3066,32 +3103,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01425</v>
+        <v>0</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.09035000000000003</v>
+        <v>0.0001</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.4552733333333335</v>
+        <v>0.11752</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0</v>
+        <v>0.00115</v>
       </c>
     </row>
     <row r="15">
@@ -3100,32 +3137,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.03523333333333334</v>
+        <v>0.06243333333333333</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>310</v>
+        <v>271</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.11055</v>
+        <v>0.2502666666666666</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.35007</v>
+        <v>0.6115166666666667</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.00075</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3134,32 +3171,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>280</v>
+        <v>295</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0</v>
+        <v>0.02396666666666667</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.1057583333333333</v>
+        <v>0.3389333333333331</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.004383333333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3168,29 +3205,29 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.05256666666666666</v>
+        <v>0.0073</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>252</v>
+        <v>293</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.2190833333333333</v>
+        <v>0.03841666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.5741583333333335</v>
+        <v>0.2007483333333333</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3202,32 +3239,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>281</v>
+        <v>203</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01825</v>
+        <v>0.009283333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.3165616666666665</v>
+        <v>0.07144833333333336</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -3236,32 +3273,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0</v>
+        <v>0.015975</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>173</v>
+        <v>209</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0</v>
+        <v>0.067025</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.007166666666666668</v>
+        <v>0.2713249999999999</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.01429166666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -3270,32 +3307,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.007883333333333334</v>
+        <v>0.00195</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>226</v>
+        <v>244</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.05826666666666667</v>
+        <v>0.02593333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2627966666666667</v>
+        <v>0.2353783333333333</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.009633333333333332</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -3304,32 +3341,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0</v>
+        <v>0.0047</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.00835</v>
+        <v>0.04201666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.06303166666666667</v>
+        <v>0.1902683333333333</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.0005</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="22">
@@ -3338,32 +3375,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.01223333333333333</v>
+        <v>0.0015</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>99</v>
+        <v>106.5</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>203</v>
+        <v>221</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.04919999999999999</v>
+        <v>0.0205</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2386516666666667</v>
+        <v>0.2725899999999999</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="23">
@@ -3372,29 +3409,29 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.001933333333333333</v>
+        <v>0.00055</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>241</v>
+        <v>221</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.0164</v>
+        <v>0.004866666666666667</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2061483333333334</v>
+        <v>0.09238166666666668</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0</v>
@@ -3406,32 +3443,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.004</v>
+        <v>0.0007</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03466666666666667</v>
+        <v>0.01081666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1627583333333333</v>
+        <v>0.1089583333333334</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0037</v>
+        <v>0.001783333333333333</v>
       </c>
     </row>
     <row r="25">
@@ -3440,32 +3477,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.0012</v>
+        <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>210</v>
+        <v>164</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.01245</v>
+        <v>0.0004333333333333333</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.137285</v>
+        <v>0.03656666666666666</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0</v>
+        <v>0.009350000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -3474,32 +3511,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>97</v>
+        <v>64</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>213</v>
+        <v>169</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.0158</v>
+        <v>0</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2321</v>
+        <v>0.002783333333333333</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.002066666666666666</v>
+        <v>0.0169</v>
       </c>
     </row>
     <row r="27">
@@ -3508,32 +3545,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.00315</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.00375</v>
+        <v>0.04166666666666666</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.07255</v>
+        <v>0.21039</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.002283333333333333</v>
+        <v>0.0112</v>
       </c>
     </row>
     <row r="28">
@@ -3542,32 +3579,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0011</v>
+        <v>0.0019</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>182</v>
+        <v>208</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01233333333333333</v>
+        <v>0.01955</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.08643333333333335</v>
+        <v>0.1780083333333334</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.006233333333333334</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="29">
@@ -3576,32 +3613,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0</v>
+        <v>5e-05</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>59</v>
+        <v>99</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>167</v>
+        <v>236</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0</v>
+        <v>0.007699999999999999</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.0025</v>
+        <v>0.1850033333333333</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.02694166666666667</v>
+        <v>0.00185</v>
       </c>
     </row>
     <row r="30">
@@ -3610,32 +3647,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0</v>
+        <v>0.00025</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>164</v>
+        <v>204</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0003833333333333333</v>
+        <v>0.006133333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.023235</v>
+        <v>0.09010666666666665</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.03341666666666666</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -3644,32 +3681,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.001</v>
+        <v>0.0002</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>203</v>
+        <v>182</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.01665833333333333</v>
+        <v>0.006958333333333335</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.1258116666666667</v>
+        <v>0.06000833333333335</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0</v>
+        <v>0.01051666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3678,32 +3715,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00165</v>
+        <v>0.00015</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>62</v>
+        <v>96</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.01578333333333333</v>
+        <v>0.005633333333333333</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.06108333333333334</v>
+        <v>0.09575833333333332</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.136025</v>
+        <v>0.001783333333333334</v>
       </c>
     </row>
     <row r="33">
@@ -3712,32 +3749,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>222</v>
+        <v>166</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.01016666666666667</v>
+        <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.06361666666666667</v>
+        <v>0.0005666666666666666</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.04976666666666666</v>
+        <v>0.02493333333333334</v>
       </c>
     </row>
     <row r="34">
@@ -3746,32 +3783,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.00135</v>
+        <v>0.000775</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.014525</v>
+        <v>0.009458333333333332</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.15618</v>
+        <v>0.08118333333333334</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.002833333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -3780,32 +3817,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00065</v>
+        <v>0.00055</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>180</v>
+        <v>243</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.003983333333333334</v>
+        <v>0.01228333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.05794166666666666</v>
+        <v>0.04171666666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.02643333333333334</v>
+        <v>0.1422</v>
       </c>
     </row>
     <row r="36">
@@ -3814,32 +3851,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>172</v>
+        <v>213</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.001016666666666667</v>
+        <v>0.0091</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.03676833333333333</v>
+        <v>0.05491166666666666</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.0237</v>
+        <v>0.05215833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3848,32 +3885,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>226</v>
+        <v>177</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.004575</v>
+        <v>0.00095</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.1655483333333334</v>
+        <v>0.03443333333333333</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.00615</v>
+        <v>0.03323333333333333</v>
       </c>
     </row>
     <row r="38">
@@ -3882,32 +3919,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E38" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.014</v>
+        <v>0.02234833333333333</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.10925</v>
+        <v>0.02478333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3916,32 +3953,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>129</v>
+        <v>192</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.0007833333333333333</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.2357666666666666</v>
+        <v>0.1133583333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3950,32 +3987,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.0002833333333333333</v>
+        <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>228</v>
+        <v>129</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.00545</v>
+        <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.07946</v>
+        <v>0.0006666666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.006791666666666667</v>
+        <v>0.2313916666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3994,22 +4031,22 @@
         <v>7</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.00135</v>
+        <v>0.0008</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>68</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.004933333333333334</v>
+        <v>0.00315</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.03514166666666666</v>
+        <v>0.02539166666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.08119999999999999</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="42">
@@ -4031,19 +4068,19 @@
         <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>110</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.00805</v>
+        <v>0.003866666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2168833333333333</v>
+        <v>0.2305583333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 15:05:50 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T18:41:48.048576+00:00</t>
+          <t>2026-03-22T19:05:49.762603+00:00</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8508454771567467</v>
+        <v>0.8513113723242769</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1491545228432533</v>
+        <v>0.1486886276757231</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2748,10 +2748,10 @@
         <v>311</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.3371166666666667</v>
+        <v>0.3372166666666667</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6797333333333335</v>
+        <v>0.6796333333333334</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2782,7 +2782,7 @@
         <v>308</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2680333333333334</v>
+        <v>0.2681333333333334</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>0.6122033333333333</v>
@@ -2807,7 +2807,7 @@
         <v>8</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.05425</v>
+        <v>0.05435</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>122</v>
@@ -2850,7 +2850,7 @@
         <v>239</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1032833333333334</v>
+        <v>0.1031833333333333</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0.5192000000000001</v>
@@ -2887,7 +2887,7 @@
         <v>0.1155333333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.5891683333333333</v>
+        <v>0.5892683333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2909,7 +2909,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.1481583333333333</v>
+        <v>0.1482583333333334</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>133</v>
@@ -2955,7 +2955,7 @@
         <v>0.03041666666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.31798</v>
+        <v>0.3181133333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2977,7 +2977,7 @@
         <v>8</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.01906666666666667</v>
+        <v>0.01896666666666667</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>122</v>
@@ -3023,7 +3023,7 @@
         <v>0.08755000000000002</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4503549999999999</v>
+        <v>0.4504883333333332</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3045,7 +3045,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.0373</v>
+        <v>0.0372</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>114</v>
@@ -3054,10 +3054,10 @@
         <v>294</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1316916666666667</v>
+        <v>0.1315916666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3877983333333333</v>
+        <v>0.3876983333333333</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>5e-05</v>
@@ -3091,7 +3091,7 @@
         <v>0.05221666666666668</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.2208883333333333</v>
+        <v>0.220855</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3125,7 +3125,7 @@
         <v>0.0001</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.11752</v>
+        <v>0.11742</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0.00115</v>
@@ -3193,7 +3193,7 @@
         <v>0.02396666666666667</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3389333333333331</v>
+        <v>0.3389999999999998</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3227,7 +3227,7 @@
         <v>0.03841666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2007483333333333</v>
+        <v>0.2004483333333333</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3261,7 +3261,7 @@
         <v>0.009283333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07144833333333336</v>
+        <v>0.07134833333333336</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3295,7 +3295,7 @@
         <v>0.067025</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2713249999999999</v>
+        <v>0.2712916666666666</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3329,7 +3329,7 @@
         <v>0.02593333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2353783333333333</v>
+        <v>0.2354116666666666</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0</v>
@@ -3570,7 +3570,7 @@
         <v>0.21039</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.0112</v>
+        <v>0.01115</v>
       </c>
     </row>
     <row r="28">
@@ -3635,7 +3635,7 @@
         <v>0.007699999999999999</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1850033333333333</v>
+        <v>0.1851033333333333</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.00185</v>
@@ -3839,7 +3839,7 @@
         <v>0.01228333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.04171666666666667</v>
+        <v>0.04181666666666667</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0.1422</v>
@@ -3944,7 +3944,7 @@
         <v>0.02234833333333333</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.02478333333333333</v>
+        <v>0.02483333333333334</v>
       </c>
     </row>
     <row r="39">
@@ -4043,10 +4043,10 @@
         <v>0.00315</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02539166666666667</v>
+        <v>0.02549166666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.091</v>
+        <v>0.0911</v>
       </c>
     </row>
     <row r="42">
@@ -4080,7 +4080,7 @@
         <v>0.003866666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2305583333333333</v>
+        <v>0.2304583333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 15:26:53 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T19:05:49.762603+00:00</t>
+          <t>2026-03-22T19:26:52.948377+00:00</t>
         </is>
       </c>
     </row>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8513113723242769</v>
+        <v>0.8521261599970271</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1486886276757231</v>
+        <v>0.1478738400029729</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2739,7 +2739,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.158875</v>
+        <v>0.158825</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>137</v>
@@ -2748,7 +2748,7 @@
         <v>311</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.3372166666666667</v>
+        <v>0.3371166666666667</v>
       </c>
       <c r="I3" s="7" t="n">
         <v>0.6796333333333334</v>
@@ -2773,7 +2773,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.09105000000000001</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>131</v>
@@ -2785,7 +2785,7 @@
         <v>0.2681333333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6122033333333333</v>
+        <v>0.6121033333333333</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2816,7 +2816,7 @@
         <v>259</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.16865</v>
+        <v>0.16875</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>0.4779433333333334</v>
@@ -2921,7 +2921,7 @@
         <v>0.3028833333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.6342699999999999</v>
+        <v>0.6343366666666665</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2955,7 +2955,7 @@
         <v>0.03041666666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3181133333333334</v>
+        <v>0.3181800000000001</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2989,7 +2989,7 @@
         <v>0.1055</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4998150000000002</v>
+        <v>0.4997150000000002</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3045,7 +3045,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.0372</v>
+        <v>0.0371</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>114</v>
@@ -3054,10 +3054,10 @@
         <v>294</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1315916666666667</v>
+        <v>0.1314916666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3876983333333333</v>
+        <v>0.3876483333333333</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>5e-05</v>
@@ -3091,7 +3091,7 @@
         <v>0.05221666666666668</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.220855</v>
+        <v>0.220755</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3159,7 +3159,7 @@
         <v>0.2502666666666666</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.6115166666666667</v>
+        <v>0.6117499999999999</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3224,10 +3224,10 @@
         <v>293</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.03841666666666666</v>
+        <v>0.03831666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2004483333333333</v>
+        <v>0.2002483333333333</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3261,7 +3261,7 @@
         <v>0.009283333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07134833333333336</v>
+        <v>0.07114833333333336</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3363,7 +3363,7 @@
         <v>0.04201666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.1902683333333333</v>
+        <v>0.1901683333333333</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -3397,7 +3397,7 @@
         <v>0.0205</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2725899999999999</v>
+        <v>0.2724733333333332</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.0008</v>
@@ -3536,7 +3536,7 @@
         <v>0.002783333333333333</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.0169</v>
+        <v>0.01695</v>
       </c>
     </row>
     <row r="27">
@@ -3564,13 +3564,13 @@
         <v>226</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.04176666666666666</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.21039</v>
+        <v>0.2104233333333333</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01115</v>
+        <v>0.01105</v>
       </c>
     </row>
     <row r="28">
@@ -3601,7 +3601,7 @@
         <v>0.01955</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1780083333333334</v>
+        <v>0.1782083333333334</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0.0004</v>
@@ -3703,7 +3703,7 @@
         <v>0.006958333333333335</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.06000833333333335</v>
+        <v>0.06010833333333335</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0.01051666666666667</v>
@@ -3774,7 +3774,7 @@
         <v>0.0005666666666666666</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02493333333333334</v>
+        <v>0.02498333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -3802,7 +3802,7 @@
         <v>196</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.009458333333333332</v>
+        <v>0.009558333333333334</v>
       </c>
       <c r="I34" s="5" t="n">
         <v>0.08118333333333334</v>
@@ -3839,7 +3839,7 @@
         <v>0.01228333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.04181666666666667</v>
+        <v>0.04188333333333333</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0.1422</v>
@@ -3907,7 +3907,7 @@
         <v>0.00095</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.03443333333333333</v>
+        <v>0.03453333333333333</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>0.03323333333333333</v>
@@ -4077,7 +4077,7 @@
         <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.003866666666666667</v>
+        <v>0.003966666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
         <v>0.2304583333333333</v>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 16:01:34 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T19:46:02.892932+00:00</t>
+          <t>2026-03-22T20:01:33.644405+00:00</t>
         </is>
       </c>
     </row>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8521261599970271</v>
+        <v>0.8300181025500823</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1478738400029729</v>
+        <v>0.1699818974499177</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2705,7 +2705,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3368666666666668</v>
+        <v>0.3348333333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>155</v>
@@ -2714,10 +2714,10 @@
         <v>319</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6806166666666666</v>
+        <v>0.6785666666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9671666666666666</v>
+        <v>0.96655</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2739,7 +2739,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.158825</v>
+        <v>0.1588916666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>137</v>
@@ -2748,10 +2748,10 @@
         <v>311</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.3371166666666667</v>
+        <v>0.3380666666666666</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6796333333333334</v>
+        <v>0.6798916666666667</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2773,7 +2773,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.09105000000000001</v>
+        <v>0.09021666666666668</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>131</v>
@@ -2782,10 +2782,10 @@
         <v>308</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2681333333333334</v>
+        <v>0.2669333333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6121033333333333</v>
+        <v>0.6108366666666666</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2807,7 +2807,7 @@
         <v>8</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.05435</v>
+        <v>0.05415</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>122</v>
@@ -2816,10 +2816,10 @@
         <v>259</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.16875</v>
+        <v>0.1676</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4779433333333334</v>
+        <v>0.4767600000000001</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2841,19 +2841,19 @@
         <v>7</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.01163333333333333</v>
+        <v>0.01193333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>239</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1031833333333333</v>
+        <v>0.1040333333333334</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.5192000000000001</v>
+        <v>0.5204666666666667</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2875,7 +2875,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0171</v>
+        <v>0.0169</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>126</v>
@@ -2884,10 +2884,10 @@
         <v>309</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1155333333333333</v>
+        <v>0.1148833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.5892683333333333</v>
+        <v>0.5875183333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2909,7 +2909,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.1482583333333334</v>
+        <v>0.1472083333333334</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>133</v>
@@ -2918,10 +2918,10 @@
         <v>283</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.3028833333333334</v>
+        <v>0.3015666666666668</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.6343366666666665</v>
+        <v>0.6328366666666666</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2952,10 +2952,10 @@
         <v>257</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.03041666666666666</v>
+        <v>0.02996666666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3181800000000001</v>
+        <v>0.3171133333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2977,7 +2977,7 @@
         <v>8</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.01896666666666667</v>
+        <v>0.01911666666666667</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>122</v>
@@ -2986,10 +2986,10 @@
         <v>292</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1055</v>
+        <v>0.1060833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4997150000000002</v>
+        <v>0.5008400000000003</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
         <v>8</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.01571666666666667</v>
+        <v>0.01531666666666667</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>120</v>
@@ -3020,10 +3020,10 @@
         <v>316</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.08755000000000002</v>
+        <v>0.08685000000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4504883333333332</v>
+        <v>0.4487549999999999</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3045,19 +3045,19 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.0371</v>
+        <v>0.04075</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>294</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1314916666666667</v>
+        <v>0.1365916666666666</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3876483333333333</v>
+        <v>0.3929316666666667</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>5e-05</v>
@@ -3088,10 +3088,10 @@
         <v>247</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.05221666666666668</v>
+        <v>0.05245</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.220755</v>
+        <v>0.2218066666666667</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3116,16 +3116,16 @@
         <v>0</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G14" s="8" t="n">
         <v>284</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.11742</v>
+        <v>0.1182033333333333</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0.00115</v>
@@ -3147,7 +3147,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.06243333333333333</v>
+        <v>0.06168333333333333</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>128</v>
@@ -3156,10 +3156,10 @@
         <v>271</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.2502666666666666</v>
+        <v>0.2472166666666666</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.6117499999999999</v>
+        <v>0.607325</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3190,10 +3190,10 @@
         <v>295</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.02396666666666667</v>
+        <v>0.02391666666666667</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3389999999999998</v>
+        <v>0.3376166666666666</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3215,19 +3215,19 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.0073</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>293</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.03831666666666667</v>
+        <v>0.04201666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2002483333333333</v>
+        <v>0.2062983333333334</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3258,10 +3258,10 @@
         <v>203</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.009283333333333333</v>
+        <v>0.01033333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07114833333333336</v>
+        <v>0.07757333333333334</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3283,7 +3283,7 @@
         <v>8</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.015975</v>
+        <v>0.015875</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>108</v>
@@ -3292,10 +3292,10 @@
         <v>209</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.067025</v>
+        <v>0.066625</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2712916666666666</v>
+        <v>0.2703749999999999</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3317,19 +3317,19 @@
         <v>7</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.00195</v>
+        <v>0.00205</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G20" s="8" t="n">
         <v>244</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02593333333333333</v>
+        <v>0.02603333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2354116666666666</v>
+        <v>0.2367616666666666</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0</v>
@@ -3351,19 +3351,19 @@
         <v>7</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.0047</v>
+        <v>0.00475</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G21" s="9" t="n">
         <v>203</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.04201666666666667</v>
+        <v>0.04221666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.1901683333333333</v>
+        <v>0.1909016666666666</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0.0005999999999999999</v>
@@ -3388,19 +3388,19 @@
         <v>0.0015</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>106.5</v>
+        <v>107</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>221</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.0205</v>
+        <v>0.02015</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2724733333333332</v>
+        <v>0.2719233333333332</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.0008</v>
+        <v>0.00075</v>
       </c>
     </row>
     <row r="23">
@@ -3431,7 +3431,7 @@
         <v>0.004866666666666667</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.09238166666666668</v>
+        <v>0.09288333333333335</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0</v>
@@ -3462,13 +3462,13 @@
         <v>185</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.01081666666666667</v>
+        <v>0.01066666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1089583333333334</v>
+        <v>0.107875</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.001783333333333333</v>
+        <v>0.001733333333333333</v>
       </c>
     </row>
     <row r="25">
@@ -3499,10 +3499,10 @@
         <v>0.0004333333333333333</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.03656666666666666</v>
+        <v>0.03678333333333332</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.009350000000000001</v>
+        <v>0.009050000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -3536,7 +3536,7 @@
         <v>0.002783333333333333</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01695</v>
+        <v>0.01675</v>
       </c>
     </row>
     <row r="27">
@@ -3555,7 +3555,7 @@
         <v>8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.00315</v>
+        <v>0.0029</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>93</v>
@@ -3564,13 +3564,13 @@
         <v>226</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.04176666666666666</v>
+        <v>0.04071666666666666</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2104233333333333</v>
+        <v>0.2078</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01105</v>
+        <v>0.0113</v>
       </c>
     </row>
     <row r="28">
@@ -3598,10 +3598,10 @@
         <v>208</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01955</v>
+        <v>0.01915</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1782083333333334</v>
+        <v>0.1756416666666667</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0.0004</v>
@@ -3632,10 +3632,10 @@
         <v>236</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.007699999999999999</v>
+        <v>0.007499999999999999</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1851033333333333</v>
+        <v>0.18267</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.00185</v>
@@ -3660,7 +3660,7 @@
         <v>0.00025</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>204</v>
@@ -3669,7 +3669,7 @@
         <v>0.006133333333333334</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.09010666666666665</v>
+        <v>0.09060833333333333</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0</v>
@@ -3700,13 +3700,13 @@
         <v>182</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.006958333333333335</v>
+        <v>0.006858333333333334</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.06010833333333335</v>
+        <v>0.05960833333333335</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01051666666666667</v>
+        <v>0.01071666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3728,19 +3728,19 @@
         <v>0.00015</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>226</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.005633333333333333</v>
+        <v>0.005433333333333333</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.09575833333333332</v>
+        <v>0.09495833333333333</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.001783333333333334</v>
+        <v>0.001883333333333333</v>
       </c>
     </row>
     <row r="33">
@@ -3774,7 +3774,7 @@
         <v>0.0005666666666666666</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02498333333333333</v>
+        <v>0.02473333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -3802,10 +3802,10 @@
         <v>196</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.009558333333333334</v>
+        <v>0.009458333333333332</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.08118333333333334</v>
+        <v>0.08083333333333333</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>0</v>
@@ -3839,10 +3839,10 @@
         <v>0.01228333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.04188333333333333</v>
+        <v>0.04161666666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.1422</v>
+        <v>0.14195</v>
       </c>
     </row>
     <row r="36">
@@ -3870,13 +3870,13 @@
         <v>213</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.0091</v>
+        <v>0.0094</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.05491166666666666</v>
+        <v>0.05509500000000001</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.05215833333333333</v>
+        <v>0.05140833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3904,13 +3904,13 @@
         <v>177</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.00095</v>
+        <v>0.00085</v>
       </c>
       <c r="I37" s="7" t="n">
+        <v>0.03373333333333334</v>
+      </c>
+      <c r="J37" s="7" t="n">
         <v>0.03453333333333333</v>
-      </c>
-      <c r="J37" s="7" t="n">
-        <v>0.03323333333333333</v>
       </c>
     </row>
     <row r="38">
@@ -3941,10 +3941,10 @@
         <v>0.0003</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.02234833333333333</v>
+        <v>0.02203333333333333</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.02483333333333334</v>
+        <v>0.02473333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3975,10 +3975,10 @@
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0089</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1133583333333333</v>
+        <v>0.1123083333333333</v>
       </c>
     </row>
     <row r="40">
@@ -4012,7 +4012,7 @@
         <v>0.0006666666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.2313916666666667</v>
+        <v>0.2311416666666667</v>
       </c>
     </row>
     <row r="41">
@@ -4034,19 +4034,19 @@
         <v>0.0008</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>230</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00315</v>
+        <v>0.00365</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02549166666666667</v>
+        <v>0.02789166666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.0911</v>
+        <v>0.08975</v>
       </c>
     </row>
     <row r="42">
@@ -4077,10 +4077,10 @@
         <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.003966666666666667</v>
+        <v>0.003766666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2304583333333333</v>
+        <v>0.2332083333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 16:20:13 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T20:01:33.644405+00:00</t>
+          <t>2026-03-22T20:20:13.263390+00:00</t>
         </is>
       </c>
     </row>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8300181025500823</v>
+        <v>0.8286944729158215</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1699818974499177</v>
+        <v>0.1713055270841785</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2705,7 +2705,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3348333333333334</v>
+        <v>0.3346333333333333</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>155</v>
@@ -2714,10 +2714,10 @@
         <v>319</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6785666666666667</v>
+        <v>0.6781666666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.96655</v>
+        <v>0.9665</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2739,7 +2739,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1588916666666667</v>
+        <v>0.1587916666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>137</v>
@@ -2748,10 +2748,10 @@
         <v>311</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.3380666666666666</v>
+        <v>0.3379666666666666</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6798916666666667</v>
+        <v>0.6799416666666668</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2773,7 +2773,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.09021666666666668</v>
+        <v>0.09011666666666668</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>131</v>
@@ -2782,7 +2782,7 @@
         <v>308</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2669333333333334</v>
+        <v>0.2668333333333334</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>0.6108366666666666</v>
@@ -2816,7 +2816,7 @@
         <v>259</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1676</v>
+        <v>0.1675</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>0.4767600000000001</v>
@@ -2850,10 +2850,10 @@
         <v>239</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1040333333333334</v>
+        <v>0.1041333333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.5204666666666667</v>
+        <v>0.5203666666666668</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2887,7 +2887,7 @@
         <v>0.1148833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.5875183333333333</v>
+        <v>0.5873683333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2918,10 +2918,10 @@
         <v>283</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.3015666666666668</v>
+        <v>0.3015166666666668</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.6328366666666666</v>
+        <v>0.6326366666666666</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2955,7 +2955,7 @@
         <v>0.02996666666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3171133333333334</v>
+        <v>0.3169133333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2986,10 +2986,10 @@
         <v>292</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1060833333333333</v>
+        <v>0.1061833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5008400000000003</v>
+        <v>0.5009900000000003</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
         <v>0.08685000000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4487549999999999</v>
+        <v>0.4486549999999999</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3045,7 +3045,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.04075</v>
+        <v>0.04105</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>115</v>
@@ -3054,10 +3054,10 @@
         <v>294</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1365916666666666</v>
+        <v>0.1371416666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3929316666666667</v>
+        <v>0.3930816666666667</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>5e-05</v>
@@ -3088,10 +3088,10 @@
         <v>247</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.05245</v>
+        <v>0.05235</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.2218066666666667</v>
+        <v>0.2218566666666667</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3147,7 +3147,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.06168333333333333</v>
+        <v>0.06158333333333332</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>128</v>
@@ -3156,10 +3156,10 @@
         <v>271</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.2472166666666666</v>
+        <v>0.2470166666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.607325</v>
+        <v>0.607025</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3215,7 +3215,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>97</v>
@@ -3224,10 +3224,10 @@
         <v>293</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04201666666666666</v>
+        <v>0.04231666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2062983333333334</v>
+        <v>0.2066983333333333</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3258,10 +3258,10 @@
         <v>203</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01033333333333333</v>
+        <v>0.01043333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07757333333333334</v>
+        <v>0.07827333333333335</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3397,7 +3397,7 @@
         <v>0.02015</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2719233333333332</v>
+        <v>0.2717233333333332</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.00075</v>
@@ -3564,10 +3564,10 @@
         <v>226</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.04071666666666666</v>
+        <v>0.04051666666666667</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2078</v>
+        <v>0.2077</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.0113</v>
@@ -3635,7 +3635,7 @@
         <v>0.007499999999999999</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.18267</v>
+        <v>0.18227</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.00185</v>
@@ -3876,7 +3876,7 @@
         <v>0.05509500000000001</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.05140833333333333</v>
+        <v>0.05130833333333332</v>
       </c>
     </row>
     <row r="37">
@@ -3910,7 +3910,7 @@
         <v>0.03373333333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.03453333333333333</v>
+        <v>0.03463333333333333</v>
       </c>
     </row>
     <row r="38">
@@ -4012,7 +4012,7 @@
         <v>0.0006666666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.2311416666666667</v>
+        <v>0.2310416666666666</v>
       </c>
     </row>
     <row r="41">
@@ -4040,10 +4040,10 @@
         <v>230</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00365</v>
+        <v>0.00375</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02789166666666667</v>
+        <v>0.02819166666666667</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.08975</v>
@@ -4080,7 +4080,7 @@
         <v>0.003766666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2332083333333334</v>
+        <v>0.2333083333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 16:40:52 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T20:20:13.263390+00:00</t>
+          <t>2026-03-22T20:40:52.343574+00:00</t>
         </is>
       </c>
     </row>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8286944729158215</v>
+        <v>0.8300647101568199</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1713055270841785</v>
+        <v>0.1699352898431801</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2705,7 +2705,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3346333333333333</v>
+        <v>0.3348333333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>155</v>
@@ -2714,10 +2714,10 @@
         <v>319</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6781666666666667</v>
+        <v>0.6785666666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9665</v>
+        <v>0.96655</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2739,7 +2739,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1587916666666667</v>
+        <v>0.1588916666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>137</v>
@@ -2748,10 +2748,10 @@
         <v>311</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.3379666666666666</v>
+        <v>0.3380666666666666</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6799416666666668</v>
+        <v>0.6798916666666667</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2773,7 +2773,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.09011666666666668</v>
+        <v>0.09021666666666668</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>131</v>
@@ -2782,7 +2782,7 @@
         <v>308</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2668333333333334</v>
+        <v>0.2669333333333334</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>0.6108366666666666</v>
@@ -2816,7 +2816,7 @@
         <v>259</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1675</v>
+        <v>0.1676</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>0.4767600000000001</v>
@@ -2850,10 +2850,10 @@
         <v>239</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1041333333333333</v>
+        <v>0.1040333333333334</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.5203666666666668</v>
+        <v>0.5204666666666667</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2887,7 +2887,7 @@
         <v>0.1148833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.5873683333333333</v>
+        <v>0.5875183333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2918,10 +2918,10 @@
         <v>283</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.3015166666666668</v>
+        <v>0.3015666666666668</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.6326366666666666</v>
+        <v>0.6328366666666666</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2955,7 +2955,7 @@
         <v>0.02996666666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3169133333333334</v>
+        <v>0.3171133333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -2986,10 +2986,10 @@
         <v>292</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1061833333333333</v>
+        <v>0.1060833333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5009900000000003</v>
+        <v>0.5008400000000003</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
         <v>0.08685000000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4486549999999999</v>
+        <v>0.4487549999999999</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3045,7 +3045,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.04105</v>
+        <v>0.04075</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>115</v>
@@ -3054,10 +3054,10 @@
         <v>294</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1371416666666667</v>
+        <v>0.1365916666666666</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3930816666666667</v>
+        <v>0.3929316666666667</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>5e-05</v>
@@ -3088,10 +3088,10 @@
         <v>247</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.05235</v>
+        <v>0.05245</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.2218566666666667</v>
+        <v>0.2218066666666667</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3147,7 +3147,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.06158333333333332</v>
+        <v>0.06168333333333333</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>128</v>
@@ -3156,10 +3156,10 @@
         <v>271</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.2470166666666667</v>
+        <v>0.2472166666666666</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.607025</v>
+        <v>0.607325</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3215,7 +3215,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>97</v>
@@ -3224,10 +3224,10 @@
         <v>293</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04231666666666666</v>
+        <v>0.04201666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2066983333333333</v>
+        <v>0.2062983333333334</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3258,10 +3258,10 @@
         <v>203</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01043333333333333</v>
+        <v>0.01033333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07827333333333335</v>
+        <v>0.07757333333333334</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3397,7 +3397,7 @@
         <v>0.02015</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2717233333333332</v>
+        <v>0.2719233333333332</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0.00075</v>
@@ -3564,10 +3564,10 @@
         <v>226</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.04051666666666667</v>
+        <v>0.04071666666666666</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2077</v>
+        <v>0.2078</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0.0113</v>
@@ -3635,7 +3635,7 @@
         <v>0.007499999999999999</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.18227</v>
+        <v>0.18267</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.00185</v>
@@ -3876,7 +3876,7 @@
         <v>0.05509500000000001</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.05130833333333332</v>
+        <v>0.05140833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3910,7 +3910,7 @@
         <v>0.03373333333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.03463333333333333</v>
+        <v>0.03453333333333333</v>
       </c>
     </row>
     <row r="38">
@@ -4012,7 +4012,7 @@
         <v>0.0006666666666666666</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.2310416666666666</v>
+        <v>0.2311416666666667</v>
       </c>
     </row>
     <row r="41">
@@ -4040,10 +4040,10 @@
         <v>230</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00375</v>
+        <v>0.00365</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02819166666666667</v>
+        <v>0.02789166666666667</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.08975</v>
@@ -4080,7 +4080,7 @@
         <v>0.003766666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2333083333333333</v>
+        <v>0.2332083333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 17:04:02 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>a02614466dbdf7f2</t>
+          <t>d47a3783c781a135</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>f18ca837ac5d50d9</t>
+          <t>a02614466dbdf7f2</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Round of 32: Iowa State over Kentucky</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T20:40:52.343574+00:00</t>
+          <t>2026-03-22T21:04:02.141168+00:00</t>
         </is>
       </c>
     </row>
@@ -2237,10 +2237,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Iowa State</t>
+        </is>
+      </c>
       <c r="F41" s="6" t="b">
         <v>0</v>
       </c>
@@ -2422,10 +2426,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8300647101568199</v>
+        <v>0.8306909087400456</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1699352898431801</v>
+        <v>0.1693090912599544</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2699,25 +2703,25 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3348333333333334</v>
+        <v>0.4323083333333334</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.6785666666666667</v>
+        <v>0.7574249999999999</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.96655</v>
+        <v>0.975725</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2736,22 +2740,22 @@
         <v>65</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1588916666666667</v>
+        <v>0.05474166666666666</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>311</v>
+        <v>260</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.3380666666666666</v>
+        <v>0.2057583333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.6798916666666667</v>
+        <v>0.5801499999999999</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2773,19 +2777,19 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.09021666666666668</v>
+        <v>0.087675</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2669333333333334</v>
+        <v>0.2641533333333334</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6108366666666666</v>
+        <v>0.5877833333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2797,29 +2801,29 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.05415</v>
+        <v>0.01789166666666667</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>259</v>
+        <v>241</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1676</v>
+        <v>0.1393249999999999</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4767600000000001</v>
+        <v>0.5732916666666665</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2831,29 +2835,29 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
         <v>57</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.01193333333333333</v>
+        <v>0.04978333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1040333333333334</v>
+        <v>0.1491033333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.5204666666666667</v>
+        <v>0.4369683333333333</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2865,29 +2869,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0169</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>309</v>
+        <v>257</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1148833333333333</v>
+        <v>0.04401666666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.5875183333333333</v>
+        <v>0.3795483333333334</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2899,29 +2903,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.1472083333333334</v>
+        <v>0.02319166666666667</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.3015666666666668</v>
+        <v>0.12987</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.6328366666666666</v>
+        <v>0.5554333333333333</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2933,32 +2937,32 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0</v>
+        <v>0.03498333333333334</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.02996666666666666</v>
+        <v>0.09213333333333337</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3171133333333334</v>
+        <v>0.3271400000000001</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0</v>
+        <v>0.00015</v>
       </c>
     </row>
     <row r="10">
@@ -2967,29 +2971,29 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.01911666666666667</v>
+        <v>0.0136</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1060833333333333</v>
+        <v>0.1015083333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5008400000000003</v>
+        <v>0.5394866666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3001,29 +3005,29 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.01531666666666667</v>
+        <v>0.008733333333333333</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>316</v>
+        <v>238</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.08685000000000001</v>
+        <v>0.06686666666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4487549999999999</v>
+        <v>0.2408083333333334</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3035,32 +3039,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.04075</v>
+        <v>0</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.1365916666666666</v>
+        <v>0.0002333333333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3929316666666667</v>
+        <v>0.1367333333333333</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>5e-05</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="13">
@@ -3069,29 +3073,29 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.0072</v>
+        <v>0.145625</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>95</v>
+        <v>131</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>247</v>
+        <v>277</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.05245</v>
+        <v>0.291395</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.2218066666666667</v>
+        <v>0.6029166666666667</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3103,32 +3107,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0</v>
+        <v>0.07591666666666665</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>103</v>
+        <v>131</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.3095116666666667</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.1182033333333333</v>
+        <v>0.6615500000000002</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.00115</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3137,29 +3141,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.06168333333333333</v>
+        <v>0</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.2472166666666666</v>
+        <v>0.02902500000000001</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.607325</v>
+        <v>0.3858199999999999</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3171,29 +3175,29 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0</v>
+        <v>0.01436666666666667</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.02391666666666667</v>
+        <v>0.07782500000000001</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.3376166666666666</v>
+        <v>0.4056083333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3209,25 +3213,25 @@
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0105</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04201666666666666</v>
+        <v>0.05011666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2062983333333334</v>
+        <v>0.2382666666666667</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3243,7 +3247,7 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>6</v>
@@ -3252,16 +3256,16 @@
         <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01033333333333333</v>
+        <v>0.01195</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.07757333333333334</v>
+        <v>0.09866666666666664</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3273,29 +3277,29 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.015875</v>
+        <v>0.002733333333333333</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>209</v>
+        <v>246</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.066625</v>
+        <v>0.03078333333333334</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2703749999999999</v>
+        <v>0.2724816666666667</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3307,32 +3311,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.00205</v>
+        <v>0.00525</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>244</v>
+        <v>198</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.02603333333333333</v>
+        <v>0.04966666666666666</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2367616666666666</v>
+        <v>0.2301833333333333</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0</v>
+        <v>0.00035</v>
       </c>
     </row>
     <row r="21">
@@ -3341,32 +3345,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.00475</v>
+        <v>0.0015</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.04221666666666667</v>
+        <v>0.02844166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.1909016666666666</v>
+        <v>0.3145566666666668</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -3375,32 +3379,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.0015</v>
+        <v>0.00045</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>221</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.02015</v>
+        <v>0.0062</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.2719233333333332</v>
+        <v>0.1019833333333333</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.00075</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -3409,32 +3413,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.001383333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>221</v>
+        <v>185</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.004866666666666667</v>
+        <v>0.01348333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.09288333333333335</v>
+        <v>0.1170916666666667</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0</v>
+        <v>0.00025</v>
       </c>
     </row>
     <row r="24">
@@ -3443,32 +3447,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.0007</v>
+        <v>0.01376666666666667</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>185</v>
+        <v>211</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.01066666666666667</v>
+        <v>0.06420000000000002</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.107875</v>
+        <v>0.2431749999999999</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.001733333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -3477,32 +3481,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.0004333333333333333</v>
+        <v>0</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.03678333333333332</v>
+        <v>0.003066666666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.009050000000000001</v>
+        <v>0.009266666666666666</v>
       </c>
     </row>
     <row r="26">
@@ -3511,32 +3515,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0</v>
+        <v>0.00295</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>169</v>
+        <v>210</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0</v>
+        <v>0.02465833333333333</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.002783333333333333</v>
+        <v>0.2179750000000001</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01675</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="27">
@@ -3545,32 +3549,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.0029</v>
+        <v>0</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>226</v>
+        <v>164</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.04071666666666666</v>
+        <v>0.0005166666666666666</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.2078</v>
+        <v>0.02998333333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.0113</v>
+        <v>0.01151666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3579,32 +3583,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0019</v>
+        <v>0.00015</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01915</v>
+        <v>0.006016666666666667</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1756416666666667</v>
+        <v>0.1000166666666667</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3613,32 +3617,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>5e-05</v>
+        <v>0.00025</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>99</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.007499999999999999</v>
+        <v>0.007616666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.18267</v>
+        <v>0.1108866666666666</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.00185</v>
+        <v>0.002016666666666667</v>
       </c>
     </row>
     <row r="30">
@@ -3647,32 +3651,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.00025</v>
+        <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.006133333333333334</v>
+        <v>0.005033333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.09060833333333333</v>
+        <v>0.1008833333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0</v>
+        <v>0.01518333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -3681,32 +3685,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.006858333333333334</v>
+        <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.05960833333333335</v>
+        <v>0.001066666666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01071666666666667</v>
+        <v>0.01676666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3715,32 +3719,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" s="5" t="n">
         <v>0.00015</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.005433333333333333</v>
+        <v>0.007766666666666667</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.09495833333333333</v>
+        <v>0.1573366666666667</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.001883333333333333</v>
+        <v>0.00155</v>
       </c>
     </row>
     <row r="33">
@@ -3749,32 +3753,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
         <v>35</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0</v>
+        <v>0.005383333333333333</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.0005666666666666666</v>
+        <v>0.05215833333333333</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.02473333333333333</v>
+        <v>0.01208333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -3783,32 +3787,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.000775</v>
+        <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>196</v>
+        <v>171</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.009458333333333332</v>
+        <v>0.0027</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.08083333333333333</v>
+        <v>0.03795</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0</v>
+        <v>0.02638333333333334</v>
       </c>
     </row>
     <row r="35">
@@ -3817,32 +3821,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>0.00055</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>243</v>
+        <v>196</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.01228333333333333</v>
+        <v>0.007433333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.04161666666666667</v>
+        <v>0.07438333333333334</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.14195</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -3851,32 +3855,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
         <v>32</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>213</v>
+        <v>252</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.0094</v>
+        <v>0.01448333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.05509500000000001</v>
+        <v>0.04195</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.05140833333333333</v>
+        <v>0.1578833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3885,32 +3889,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>177</v>
+        <v>142</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.00085</v>
+        <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.03373333333333334</v>
+        <v>0.003483333333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.03453333333333333</v>
+        <v>0.07606666666666669</v>
       </c>
     </row>
     <row r="38">
@@ -3919,32 +3923,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E38" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>181</v>
+        <v>129</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.02203333333333333</v>
+        <v>0.0003666666666666667</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.02473333333333333</v>
+        <v>0.1532333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3953,32 +3957,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>192</v>
+        <v>165</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.0089</v>
+        <v>0.018525</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.1123083333333333</v>
+        <v>0.03788333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -3987,32 +3991,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>129</v>
+        <v>192</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.0006666666666666666</v>
+        <v>0.01158333333333333</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.2311416666666667</v>
+        <v>0.1403833333333333</v>
       </c>
     </row>
     <row r="41">
@@ -4025,28 +4029,28 @@
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D41" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.0008</v>
+        <v>0.00095</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00365</v>
+        <v>0.0053</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02789166666666667</v>
+        <v>0.02965</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.08975</v>
+        <v>0.06693333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -4068,7 +4072,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>110</v>
@@ -4077,10 +4081,10 @@
         <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.003766666666666667</v>
+        <v>0.003366666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2332083333333334</v>
+        <v>0.2715</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 17:23:10 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Round of 32: Iowa State over Kentucky</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T21:04:02.141168+00:00</t>
+          <t>2026-03-22T21:23:09.513266+00:00</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
@@ -2426,10 +2426,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8306909087400456</v>
+        <v>0.8312342764460491</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1693090912599544</v>
+        <v>0.1687657235539509</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2709,7 +2709,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4323083333333334</v>
+        <v>0.4324583333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>159</v>
@@ -2718,7 +2718,7 @@
         <v>313</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7574249999999999</v>
+        <v>0.7575249999999999</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>0.975725</v>
@@ -2743,7 +2743,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.05474166666666666</v>
+        <v>0.05469166666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>129</v>
@@ -2752,10 +2752,10 @@
         <v>260</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.2057583333333333</v>
+        <v>0.2056583333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.5801499999999999</v>
+        <v>0.58005</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2786,10 +2786,10 @@
         <v>298</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2641533333333334</v>
+        <v>0.2642533333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5877833333333334</v>
+        <v>0.5876833333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2845,7 +2845,7 @@
         <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.04978333333333333</v>
+        <v>0.04988333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>120</v>
@@ -2857,7 +2857,7 @@
         <v>0.1491033333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.4369683333333333</v>
+        <v>0.4370683333333333</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2888,10 +2888,10 @@
         <v>257</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.04401666666666666</v>
+        <v>0.04406666666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3795483333333334</v>
+        <v>0.3796483333333334</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2925,7 +2925,7 @@
         <v>0.12987</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5554333333333333</v>
+        <v>0.5552833333333334</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2947,7 +2947,7 @@
         <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03498333333333334</v>
+        <v>0.03468333333333334</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>110</v>
@@ -2956,10 +2956,10 @@
         <v>260</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.09213333333333337</v>
+        <v>0.09193333333333337</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3271400000000001</v>
+        <v>0.3269400000000001</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00015</v>
@@ -2990,10 +2990,10 @@
         <v>291</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1015083333333334</v>
+        <v>0.1015583333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5394866666666666</v>
+        <v>0.5393866666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3083,7 +3083,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.145625</v>
+        <v>0.145725</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>131</v>
@@ -3092,10 +3092,10 @@
         <v>277</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.291395</v>
+        <v>0.291445</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.6029166666666667</v>
+        <v>0.6031166666666666</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3126,7 +3126,7 @@
         <v>262</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.3095116666666667</v>
+        <v>0.3096616666666667</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>0.6615500000000002</v>
@@ -3163,7 +3163,7 @@
         <v>0.02902500000000001</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3858199999999999</v>
+        <v>0.38612</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3197,7 +3197,7 @@
         <v>0.07782500000000001</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.4056083333333333</v>
+        <v>0.4056583333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3228,10 +3228,10 @@
         <v>285</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.05011666666666666</v>
+        <v>0.05006666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2382666666666667</v>
+        <v>0.2380666666666667</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3262,10 +3262,10 @@
         <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01195</v>
+        <v>0.01185</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.09866666666666664</v>
+        <v>0.09841666666666664</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3296,7 +3296,7 @@
         <v>246</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03078333333333334</v>
+        <v>0.03073333333333334</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>0.2724816666666667</v>
@@ -3367,7 +3367,7 @@
         <v>0.02844166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3145566666666668</v>
+        <v>0.3146066666666668</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3435,7 +3435,7 @@
         <v>0.01348333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1170916666666667</v>
+        <v>0.1171916666666667</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.00025</v>
@@ -3469,7 +3469,7 @@
         <v>0.06420000000000002</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2431749999999999</v>
+        <v>0.243275</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -3506,7 +3506,7 @@
         <v>0.003066666666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.009266666666666666</v>
+        <v>0.009316666666666666</v>
       </c>
     </row>
     <row r="26">
@@ -3537,7 +3537,7 @@
         <v>0.02465833333333333</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2179750000000001</v>
+        <v>0.218075</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.0002</v>
@@ -3636,10 +3636,10 @@
         <v>231</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.007616666666666667</v>
+        <v>0.007666666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1108866666666666</v>
+        <v>0.1109866666666666</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.002016666666666667</v>
@@ -3673,7 +3673,7 @@
         <v>0.005033333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1008833333333333</v>
+        <v>0.1009833333333333</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0.01518333333333333</v>
@@ -3812,7 +3812,7 @@
         <v>0.03795</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02638333333333334</v>
+        <v>0.02633333333333334</v>
       </c>
     </row>
     <row r="35">
@@ -3880,7 +3880,7 @@
         <v>0.04195</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1578833333333333</v>
+        <v>0.1580833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3982,7 +3982,7 @@
         <v>0.018525</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.03788333333333333</v>
+        <v>0.03778333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -4016,7 +4016,7 @@
         <v>0.01158333333333333</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1403833333333333</v>
+        <v>0.1404833333333333</v>
       </c>
     </row>
     <row r="41">
@@ -4044,13 +4044,13 @@
         <v>246</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.0053</v>
+        <v>0.00525</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02965</v>
+        <v>0.02945</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.06693333333333333</v>
+        <v>0.06698333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -4084,7 +4084,7 @@
         <v>0.003366666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2715</v>
+        <v>0.27125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 17:43:30 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T21:23:09.513266+00:00</t>
+          <t>2026-03-22T21:43:29.568920+00:00</t>
         </is>
       </c>
     </row>
@@ -2426,10 +2426,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8312342764460491</v>
+        <v>0.8334476707168001</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1687657235539509</v>
+        <v>0.1665523292831999</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4324583333333334</v>
+        <v>0.4325583333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>159</v>
@@ -2718,10 +2718,10 @@
         <v>313</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7575249999999999</v>
+        <v>0.7577249999999999</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.975725</v>
+        <v>0.9758250000000001</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2752,7 +2752,7 @@
         <v>260</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.2056583333333333</v>
+        <v>0.2055583333333333</v>
       </c>
       <c r="I3" s="7" t="n">
         <v>0.58005</v>
@@ -2786,10 +2786,10 @@
         <v>298</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2642533333333333</v>
+        <v>0.2643533333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5876833333333334</v>
+        <v>0.5879833333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2823,7 +2823,7 @@
         <v>0.1393249999999999</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5732916666666665</v>
+        <v>0.5729916666666666</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2857,7 +2857,7 @@
         <v>0.1491033333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.4370683333333333</v>
+        <v>0.4371683333333333</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2888,10 +2888,10 @@
         <v>257</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.04406666666666666</v>
+        <v>0.04416666666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3796483333333334</v>
+        <v>0.3797483333333334</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.02319166666666667</v>
+        <v>0.023225</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>125</v>
@@ -2922,7 +2922,7 @@
         <v>291</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.12987</v>
+        <v>0.12967</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>0.5552833333333334</v>
@@ -2947,7 +2947,7 @@
         <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03468333333333334</v>
+        <v>0.03448333333333334</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>110</v>
@@ -2956,10 +2956,10 @@
         <v>260</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.09193333333333337</v>
+        <v>0.09163333333333336</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3269400000000001</v>
+        <v>0.3267900000000001</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00015</v>
@@ -2990,10 +2990,10 @@
         <v>291</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1015583333333333</v>
+        <v>0.1016083333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5393866666666666</v>
+        <v>0.5395366666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3027,7 +3027,7 @@
         <v>0.06686666666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.2408083333333334</v>
+        <v>0.2406083333333334</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3061,7 +3061,7 @@
         <v>0.0002333333333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.1367333333333333</v>
+        <v>0.1366666666666667</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0004</v>
@@ -3092,10 +3092,10 @@
         <v>277</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.291445</v>
+        <v>0.291545</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.6031166666666666</v>
+        <v>0.6032</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3117,7 +3117,7 @@
         <v>10</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.07591666666666665</v>
+        <v>0.07604999999999999</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>131</v>
@@ -3126,10 +3126,10 @@
         <v>262</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.3096616666666667</v>
+        <v>0.3101116666666667</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.6615500000000002</v>
+        <v>0.6621500000000001</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3163,7 +3163,7 @@
         <v>0.02902500000000001</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.38612</v>
+        <v>0.3864199999999999</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3185,7 +3185,7 @@
         <v>8</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.01436666666666667</v>
+        <v>0.0144</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>119</v>
@@ -3194,10 +3194,10 @@
         <v>288</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.07782500000000001</v>
+        <v>0.077875</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.4056583333333333</v>
+        <v>0.4057083333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3219,7 +3219,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.0105</v>
+        <v>0.0104</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>102</v>
@@ -3228,10 +3228,10 @@
         <v>285</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.05006666666666666</v>
+        <v>0.04971666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2380666666666667</v>
+        <v>0.2375</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3262,10 +3262,10 @@
         <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01185</v>
+        <v>0.01165</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.09841666666666664</v>
+        <v>0.09781666666666664</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3299,7 +3299,7 @@
         <v>0.03073333333333334</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2724816666666667</v>
+        <v>0.2720316666666667</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3333,7 +3333,7 @@
         <v>0.04966666666666666</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2301833333333333</v>
+        <v>0.2299333333333333</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.00035</v>
@@ -3364,10 +3364,10 @@
         <v>219</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02844166666666667</v>
+        <v>0.02854166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3146066666666668</v>
+        <v>0.3148066666666667</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3401,7 +3401,7 @@
         <v>0.0062</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.1019833333333333</v>
+        <v>0.1018833333333333</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0</v>
@@ -3435,7 +3435,7 @@
         <v>0.01348333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1171916666666667</v>
+        <v>0.1172916666666667</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.00025</v>
@@ -3534,10 +3534,10 @@
         <v>210</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02465833333333333</v>
+        <v>0.02475833333333333</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.218075</v>
+        <v>0.218375</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.0002</v>
@@ -3639,7 +3639,7 @@
         <v>0.007666666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1109866666666666</v>
+        <v>0.1110866666666666</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.002016666666666667</v>
@@ -3673,10 +3673,10 @@
         <v>0.005033333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1009833333333333</v>
+        <v>0.1010833333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.01518333333333333</v>
+        <v>0.01508333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -3741,7 +3741,7 @@
         <v>0.007766666666666667</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1573366666666667</v>
+        <v>0.1574366666666667</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.00155</v>
@@ -3809,10 +3809,10 @@
         <v>0.0027</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03795</v>
+        <v>0.03805</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02633333333333334</v>
+        <v>0.02628333333333334</v>
       </c>
     </row>
     <row r="35">
@@ -3843,7 +3843,7 @@
         <v>0.007433333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.07438333333333334</v>
+        <v>0.07448333333333333</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0</v>
@@ -3880,7 +3880,7 @@
         <v>0.04195</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1580833333333333</v>
+        <v>0.1579833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3982,7 +3982,7 @@
         <v>0.018525</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.03778333333333333</v>
+        <v>0.03783333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -4016,7 +4016,7 @@
         <v>0.01158333333333333</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1404833333333333</v>
+        <v>0.1408833333333333</v>
       </c>
     </row>
     <row r="41">
@@ -4044,13 +4044,13 @@
         <v>246</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00525</v>
+        <v>0.00515</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02945</v>
+        <v>0.02925</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.06698333333333333</v>
+        <v>0.06708333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -4084,7 +4084,7 @@
         <v>0.003366666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.27125</v>
+        <v>0.27095</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 18:07:24 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T21:43:29.568920+00:00</t>
+          <t>2026-03-22T22:01:43.891879+00:00</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
@@ -2426,10 +2426,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8334476707168001</v>
+        <v>0.8397760586647307</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1665523292831999</v>
+        <v>0.1602239413352693</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2709,7 +2709,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4325583333333334</v>
+        <v>0.4336583333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>159</v>
@@ -2718,10 +2718,10 @@
         <v>313</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7577249999999999</v>
+        <v>0.758975</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9758250000000001</v>
+        <v>0.975925</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2743,10 +2743,10 @@
         <v>8</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.05469166666666667</v>
+        <v>0.05459166666666666</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>260</v>
@@ -2755,7 +2755,7 @@
         <v>0.2055583333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.58005</v>
+        <v>0.5798999999999999</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2777,7 +2777,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.087675</v>
+        <v>0.08777500000000001</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>130</v>
@@ -2786,10 +2786,10 @@
         <v>298</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2643533333333333</v>
+        <v>0.2647533333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5879833333333334</v>
+        <v>0.5880333333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2811,7 +2811,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.01789166666666667</v>
+        <v>0.01779166666666667</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>126</v>
@@ -2820,10 +2820,10 @@
         <v>241</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1393249999999999</v>
+        <v>0.1391749999999999</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5729916666666666</v>
+        <v>0.5727916666666665</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2854,10 +2854,10 @@
         <v>251</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1491033333333333</v>
+        <v>0.1494033333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.4371683333333333</v>
+        <v>0.4380350000000001</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2888,10 +2888,10 @@
         <v>257</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.04416666666666666</v>
+        <v>0.04436666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3797483333333334</v>
+        <v>0.3804483333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2922,10 +2922,10 @@
         <v>291</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.12967</v>
+        <v>0.1295366666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5552833333333334</v>
+        <v>0.5550833333333333</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2947,7 +2947,7 @@
         <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03448333333333334</v>
+        <v>0.03313333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>110</v>
@@ -2956,10 +2956,10 @@
         <v>260</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.09163333333333336</v>
+        <v>0.08963333333333336</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3267900000000001</v>
+        <v>0.3253400000000001</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00015</v>
@@ -2990,10 +2990,10 @@
         <v>291</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1016083333333333</v>
+        <v>0.1017083333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5395366666666666</v>
+        <v>0.5403866666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3015,7 +3015,7 @@
         <v>7</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.008733333333333333</v>
+        <v>0.008633333333333333</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>99</v>
@@ -3024,10 +3024,10 @@
         <v>238</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.06686666666666666</v>
+        <v>0.06676666666666667</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.2406083333333334</v>
+        <v>0.2406750000000001</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3061,7 +3061,7 @@
         <v>0.0002333333333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.1366666666666667</v>
+        <v>0.1364666666666667</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0004</v>
@@ -3083,7 +3083,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.145725</v>
+        <v>0.146125</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>131</v>
@@ -3092,10 +3092,10 @@
         <v>277</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.291545</v>
+        <v>0.2918616666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.6032</v>
+        <v>0.6033499999999999</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3117,7 +3117,7 @@
         <v>10</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.07604999999999999</v>
+        <v>0.07639999999999998</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>131</v>
@@ -3126,10 +3126,10 @@
         <v>262</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.3101116666666667</v>
+        <v>0.3111116666666667</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.6621500000000001</v>
+        <v>0.6629500000000002</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3163,7 +3163,7 @@
         <v>0.02902500000000001</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3864199999999999</v>
+        <v>0.3868699999999999</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3194,10 +3194,10 @@
         <v>288</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.077875</v>
+        <v>0.07817499999999999</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.4057083333333333</v>
+        <v>0.4062083333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3219,19 +3219,19 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.0104</v>
+        <v>0.01</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>285</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04971666666666667</v>
+        <v>0.04871666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2375</v>
+        <v>0.23545</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3262,10 +3262,10 @@
         <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01165</v>
+        <v>0.01085</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.09781666666666664</v>
+        <v>0.09591666666666664</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3287,7 +3287,7 @@
         <v>7</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.002733333333333333</v>
+        <v>0.002633333333333333</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>112</v>
@@ -3296,10 +3296,10 @@
         <v>246</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03073333333333334</v>
+        <v>0.03068333333333334</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2720316666666667</v>
+        <v>0.2717816666666668</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3330,10 +3330,10 @@
         <v>198</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.04966666666666666</v>
+        <v>0.04963333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2299333333333333</v>
+        <v>0.2297333333333333</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.00035</v>
@@ -3364,10 +3364,10 @@
         <v>219</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02854166666666667</v>
+        <v>0.02864166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3148066666666667</v>
+        <v>0.3148566666666667</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3432,10 +3432,10 @@
         <v>185</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01348333333333333</v>
+        <v>0.01368333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1172916666666667</v>
+        <v>0.1174916666666667</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.00025</v>
@@ -3457,7 +3457,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.01376666666666667</v>
+        <v>0.01386666666666667</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>107</v>
@@ -3469,7 +3469,7 @@
         <v>0.06420000000000002</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.243275</v>
+        <v>0.2434749999999999</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -3525,7 +3525,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.00295</v>
+        <v>0.00305</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>105</v>
@@ -3534,10 +3534,10 @@
         <v>210</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02475833333333333</v>
+        <v>0.02495833333333334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.218375</v>
+        <v>0.219425</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.0002</v>
@@ -3571,10 +3571,10 @@
         <v>0.0005166666666666666</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.02998333333333334</v>
+        <v>0.02988333333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01151666666666667</v>
+        <v>0.01171666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3605,7 +3605,7 @@
         <v>0.006016666666666667</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1000166666666667</v>
+        <v>0.09956666666666668</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0</v>
@@ -3636,13 +3636,13 @@
         <v>231</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.007666666666666667</v>
+        <v>0.007716666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1110866666666666</v>
+        <v>0.1118866666666666</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.002016666666666667</v>
+        <v>0.001866666666666666</v>
       </c>
     </row>
     <row r="30">
@@ -3670,13 +3670,13 @@
         <v>212</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.005033333333333333</v>
+        <v>0.005183333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1010833333333333</v>
+        <v>0.1013333333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.01508333333333333</v>
+        <v>0.01498333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -3710,7 +3710,7 @@
         <v>0.001066666666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01676666666666667</v>
+        <v>0.01691666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3738,10 +3738,10 @@
         <v>229</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.007766666666666667</v>
+        <v>0.007866666666666668</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1574366666666667</v>
+        <v>0.1579866666666667</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.00155</v>
@@ -3809,10 +3809,10 @@
         <v>0.0027</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03805</v>
+        <v>0.03841666666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02628333333333334</v>
+        <v>0.02603333333333334</v>
       </c>
     </row>
     <row r="35">
@@ -3843,7 +3843,7 @@
         <v>0.007433333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.07448333333333333</v>
+        <v>0.07468333333333334</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0</v>
@@ -3877,10 +3877,10 @@
         <v>0.01448333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04195</v>
+        <v>0.042</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1579833333333333</v>
+        <v>0.1580333333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3914,7 +3914,7 @@
         <v>0.003483333333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.07606666666666669</v>
+        <v>0.07630000000000003</v>
       </c>
     </row>
     <row r="38">
@@ -3948,7 +3948,7 @@
         <v>0.0003666666666666667</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1532333333333333</v>
+        <v>0.1536166666666667</v>
       </c>
     </row>
     <row r="39">
@@ -3979,10 +3979,10 @@
         <v>0.0001</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.018525</v>
+        <v>0.018625</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.03783333333333333</v>
+        <v>0.03793333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -4016,7 +4016,7 @@
         <v>0.01158333333333333</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1408833333333333</v>
+        <v>0.1414333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -4044,13 +4044,13 @@
         <v>246</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00515</v>
+        <v>0.00475</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02925</v>
+        <v>0.02805</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.06708333333333333</v>
+        <v>0.06718333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -4084,7 +4084,7 @@
         <v>0.003366666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.27095</v>
+        <v>0.2696833333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 18:20:36 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T22:01:43.891879+00:00</t>
+          <t>2026-03-22T22:20:35.463999+00:00</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
@@ -2426,10 +2426,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8397760586647307</v>
+        <v>0.8418760199111757</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1602239413352693</v>
+        <v>0.1581239800888243</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4336583333333334</v>
+        <v>0.4340583333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>159</v>
@@ -2718,7 +2718,7 @@
         <v>313</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.758975</v>
+        <v>0.7591749999999999</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>0.975925</v>
@@ -2743,7 +2743,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.05459166666666666</v>
+        <v>0.05449166666666666</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>128</v>
@@ -2752,10 +2752,10 @@
         <v>260</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.2055583333333333</v>
+        <v>0.2054083333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.5798999999999999</v>
+        <v>0.5796999999999999</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2777,7 +2777,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.08777500000000001</v>
+        <v>0.087675</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>130</v>
@@ -2789,7 +2789,7 @@
         <v>0.2647533333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5880333333333334</v>
+        <v>0.5880833333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2820,10 +2820,10 @@
         <v>241</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1391749999999999</v>
+        <v>0.1391249999999999</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5727916666666665</v>
+        <v>0.5725916666666665</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2854,10 +2854,10 @@
         <v>251</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1494033333333333</v>
+        <v>0.1493033333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.4380350000000001</v>
+        <v>0.438285</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2888,10 +2888,10 @@
         <v>257</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.04436666666666667</v>
+        <v>0.04451666666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3804483333333333</v>
+        <v>0.380515</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.023225</v>
+        <v>0.023125</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>125</v>
@@ -2922,10 +2922,10 @@
         <v>291</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1295366666666667</v>
+        <v>0.1294866666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5550833333333333</v>
+        <v>0.5551333333333333</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2947,7 +2947,7 @@
         <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03313333333333333</v>
+        <v>0.03278333333333334</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>110</v>
@@ -2956,10 +2956,10 @@
         <v>260</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.08963333333333336</v>
+        <v>0.08928333333333335</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3253400000000001</v>
+        <v>0.32474</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00015</v>
@@ -2990,10 +2990,10 @@
         <v>291</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1017083333333333</v>
+        <v>0.1017583333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5403866666666666</v>
+        <v>0.5405866666666665</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3024,10 +3024,10 @@
         <v>238</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.06676666666666667</v>
+        <v>0.06681666666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.2406750000000001</v>
+        <v>0.2406416666666667</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3061,7 +3061,7 @@
         <v>0.0002333333333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.1364666666666667</v>
+        <v>0.1364166666666667</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0004</v>
@@ -3083,7 +3083,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.146125</v>
+        <v>0.146275</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>131</v>
@@ -3092,10 +3092,10 @@
         <v>277</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.2918616666666667</v>
+        <v>0.2919116666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.6033499999999999</v>
+        <v>0.6033999999999999</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3126,10 +3126,10 @@
         <v>262</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.3111116666666667</v>
+        <v>0.3113616666666667</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.6629500000000002</v>
+        <v>0.6634500000000002</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3160,10 +3160,10 @@
         <v>289</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.02902500000000001</v>
+        <v>0.02912500000000001</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3868699999999999</v>
+        <v>0.3869699999999999</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3219,7 +3219,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.01</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>101</v>
@@ -3228,10 +3228,10 @@
         <v>285</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04871666666666667</v>
+        <v>0.04851666666666667</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.23545</v>
+        <v>0.23475</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3265,7 +3265,7 @@
         <v>0.01085</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.09591666666666664</v>
+        <v>0.0955833333333333</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3299,7 +3299,7 @@
         <v>0.03068333333333334</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2717816666666668</v>
+        <v>0.2716816666666668</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3330,10 +3330,10 @@
         <v>198</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.04963333333333333</v>
+        <v>0.04953333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2297333333333333</v>
+        <v>0.2296333333333332</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.00035</v>
@@ -3364,10 +3364,10 @@
         <v>219</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02864166666666667</v>
+        <v>0.02869166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3148566666666667</v>
+        <v>0.3149566666666668</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3432,7 +3432,7 @@
         <v>185</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01368333333333333</v>
+        <v>0.01373333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>0.1174916666666667</v>
@@ -3457,7 +3457,7 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.01386666666666667</v>
+        <v>0.01396666666666667</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>107</v>
@@ -3469,7 +3469,7 @@
         <v>0.06420000000000002</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2434749999999999</v>
+        <v>0.243575</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -3525,7 +3525,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.00305</v>
+        <v>0.00315</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>105</v>
@@ -3534,10 +3534,10 @@
         <v>210</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02495833333333334</v>
+        <v>0.02505833333333334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.219425</v>
+        <v>0.2197250000000001</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.0002</v>
@@ -3574,7 +3574,7 @@
         <v>0.02988333333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01171666666666667</v>
+        <v>0.01191666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3602,10 +3602,10 @@
         <v>207</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.006016666666666667</v>
+        <v>0.005966666666666666</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.09956666666666668</v>
+        <v>0.09971666666666668</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0</v>
@@ -3639,7 +3639,7 @@
         <v>0.007716666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1118866666666666</v>
+        <v>0.1120866666666666</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.001866666666666666</v>
@@ -3673,7 +3673,7 @@
         <v>0.005183333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1013333333333333</v>
+        <v>0.1015333333333333</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0.01498333333333333</v>
@@ -3710,7 +3710,7 @@
         <v>0.001066666666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01691666666666667</v>
+        <v>0.01701666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3741,7 +3741,7 @@
         <v>0.007866666666666668</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1579866666666667</v>
+        <v>0.1582366666666667</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0.00155</v>
@@ -3778,7 +3778,7 @@
         <v>0.05215833333333333</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.01208333333333333</v>
+        <v>0.01198333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -3843,7 +3843,7 @@
         <v>0.007433333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.07468333333333334</v>
+        <v>0.07463333333333334</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0</v>
@@ -3880,7 +3880,7 @@
         <v>0.042</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1580333333333333</v>
+        <v>0.1578833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3914,7 +3914,7 @@
         <v>0.003483333333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.07630000000000003</v>
+        <v>0.07650000000000004</v>
       </c>
     </row>
     <row r="38">
@@ -4016,7 +4016,7 @@
         <v>0.01158333333333333</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1414333333333333</v>
+        <v>0.1415333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -4047,7 +4047,7 @@
         <v>0.00475</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02805</v>
+        <v>0.02785</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.06718333333333333</v>
@@ -4084,7 +4084,7 @@
         <v>0.003366666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2696833333333334</v>
+        <v>0.2693333333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 19:00:41 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T22:40:34.453729+00:00</t>
+          <t>2026-03-22T23:00:41.304946+00:00</t>
         </is>
       </c>
     </row>
@@ -2426,10 +2426,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8418760199111757</v>
+        <v>0.8426506766703782</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1581239800888243</v>
+        <v>0.1573493233296218</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4340583333333334</v>
+        <v>0.4341583333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>159</v>
@@ -2718,10 +2718,10 @@
         <v>313</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7591749999999999</v>
+        <v>0.7592749999999999</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.975925</v>
+        <v>0.976025</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2755,7 +2755,7 @@
         <v>0.2054083333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.5796999999999999</v>
+        <v>0.5796499999999999</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2823,7 +2823,7 @@
         <v>0.1391249999999999</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5725916666666665</v>
+        <v>0.5726916666666665</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2854,10 +2854,10 @@
         <v>251</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1493033333333333</v>
+        <v>0.1494033333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.438285</v>
+        <v>0.438385</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2888,10 +2888,10 @@
         <v>257</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.04451666666666666</v>
+        <v>0.04461666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.380515</v>
+        <v>0.380715</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.023125</v>
+        <v>0.023025</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>125</v>
@@ -2947,7 +2947,7 @@
         <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03278333333333334</v>
+        <v>0.03258333333333334</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>110</v>
@@ -2956,10 +2956,10 @@
         <v>260</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.08928333333333335</v>
+        <v>0.08898333333333336</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.32474</v>
+        <v>0.3244900000000001</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00015</v>
@@ -2993,7 +2993,7 @@
         <v>0.1017583333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5405866666666665</v>
+        <v>0.5407366666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3024,7 +3024,7 @@
         <v>238</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.06681666666666666</v>
+        <v>0.06686666666666666</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>0.2406416666666667</v>
@@ -3083,7 +3083,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.146275</v>
+        <v>0.146375</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>131</v>
@@ -3092,7 +3092,7 @@
         <v>277</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.2919116666666667</v>
+        <v>0.2920116666666667</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>0.6033999999999999</v>
@@ -3117,7 +3117,7 @@
         <v>10</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.07639999999999998</v>
+        <v>0.07649999999999998</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>131</v>
@@ -3126,10 +3126,10 @@
         <v>262</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.3113616666666667</v>
+        <v>0.3117616666666667</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.6634500000000002</v>
+        <v>0.6635500000000002</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3163,7 +3163,7 @@
         <v>0.02912500000000001</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3869699999999999</v>
+        <v>0.38717</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3197,7 +3197,7 @@
         <v>0.07817499999999999</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.4062083333333333</v>
+        <v>0.4064083333333334</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3228,10 +3228,10 @@
         <v>285</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04851666666666667</v>
+        <v>0.04811666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.23475</v>
+        <v>0.2343500000000001</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3262,10 +3262,10 @@
         <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01085</v>
+        <v>0.01075</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.0955833333333333</v>
+        <v>0.0953333333333333</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3299,7 +3299,7 @@
         <v>0.03068333333333334</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2716816666666668</v>
+        <v>0.2715816666666668</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3333,7 +3333,7 @@
         <v>0.04953333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2296333333333332</v>
+        <v>0.2295333333333333</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.00035</v>
@@ -3469,7 +3469,7 @@
         <v>0.06420000000000002</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.243575</v>
+        <v>0.2436749999999999</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -3534,7 +3534,7 @@
         <v>210</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02505833333333334</v>
+        <v>0.02510833333333333</v>
       </c>
       <c r="I26" s="5" t="n">
         <v>0.2197250000000001</v>
@@ -3639,7 +3639,7 @@
         <v>0.007716666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1120866666666666</v>
+        <v>0.1121866666666666</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.001866666666666666</v>
@@ -3775,7 +3775,7 @@
         <v>0.005383333333333333</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05215833333333333</v>
+        <v>0.05225833333333332</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0.01198333333333333</v>
@@ -3812,7 +3812,7 @@
         <v>0.03841666666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02603333333333334</v>
+        <v>0.02593333333333334</v>
       </c>
     </row>
     <row r="35">
@@ -3880,7 +3880,7 @@
         <v>0.042</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1578833333333333</v>
+        <v>0.1579833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3914,7 +3914,7 @@
         <v>0.003483333333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.07650000000000004</v>
+        <v>0.07665000000000004</v>
       </c>
     </row>
     <row r="38">
@@ -4016,7 +4016,7 @@
         <v>0.01158333333333333</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1415333333333333</v>
+        <v>0.1416333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -4044,13 +4044,13 @@
         <v>246</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00475</v>
+        <v>0.00465</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02785</v>
+        <v>0.02755</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.06718333333333333</v>
+        <v>0.06728333333333332</v>
       </c>
     </row>
     <row r="42">
@@ -4084,7 +4084,7 @@
         <v>0.003366666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2693333333333334</v>
+        <v>0.2689833333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 19:26:19 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T23:00:41.304946+00:00</t>
+          <t>2026-03-22T23:26:18.999458+00:00</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2426,10 +2426,10 @@
         <v>1</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.8426506766703782</v>
+        <v>0.8481569121456763</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.1573493233296218</v>
+        <v>0.1518430878543237</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4341583333333334</v>
+        <v>0.4347083333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>159</v>
@@ -2718,10 +2718,10 @@
         <v>313</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7592749999999999</v>
+        <v>0.7597749999999999</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.976025</v>
+        <v>0.976125</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2743,7 +2743,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.05449166666666666</v>
+        <v>0.05439166666666666</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>128</v>
@@ -2752,10 +2752,10 @@
         <v>260</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.2054083333333333</v>
+        <v>0.2053583333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.5796499999999999</v>
+        <v>0.5790666666666665</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2777,7 +2777,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.087675</v>
+        <v>0.087725</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>130</v>
@@ -2786,10 +2786,10 @@
         <v>298</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2647533333333333</v>
+        <v>0.2649533333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5880833333333334</v>
+        <v>0.5883833333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2820,10 +2820,10 @@
         <v>241</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1391249999999999</v>
+        <v>0.1390249999999999</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5726916666666665</v>
+        <v>0.5724083333333331</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2845,7 +2845,7 @@
         <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.04988333333333333</v>
+        <v>0.04998333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>120</v>
@@ -2854,10 +2854,10 @@
         <v>251</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1494033333333333</v>
+        <v>0.1495033333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.438385</v>
+        <v>0.438785</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2888,10 +2888,10 @@
         <v>257</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.04461666666666667</v>
+        <v>0.04466666666666666</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.380715</v>
+        <v>0.3813316666666667</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2913,7 +2913,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.023025</v>
+        <v>0.022975</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>125</v>
@@ -2922,10 +2922,10 @@
         <v>291</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1294866666666667</v>
+        <v>0.1291866666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5551333333333333</v>
+        <v>0.5545333333333333</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2947,7 +2947,7 @@
         <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03258333333333334</v>
+        <v>0.03168333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>110</v>
@@ -2956,10 +2956,10 @@
         <v>260</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.08898333333333336</v>
+        <v>0.08808333333333336</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3244900000000001</v>
+        <v>0.3223566666666667</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00015</v>
@@ -2981,7 +2981,7 @@
         <v>8</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0136</v>
+        <v>0.0138</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>124</v>
@@ -2990,10 +2990,10 @@
         <v>291</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1017583333333334</v>
+        <v>0.1021083333333333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5407366666666666</v>
+        <v>0.5414366666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3024,10 +3024,10 @@
         <v>238</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.06686666666666666</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.2406416666666667</v>
+        <v>0.2405916666666667</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3058,10 +3058,10 @@
         <v>284</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.0002333333333333334</v>
+        <v>0.0001833333333333333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.1364166666666667</v>
+        <v>0.1363666666666667</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0004</v>
@@ -3083,7 +3083,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.146375</v>
+        <v>0.146625</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>131</v>
@@ -3092,10 +3092,10 @@
         <v>277</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.2920116666666667</v>
+        <v>0.2925116666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.6033999999999999</v>
+        <v>0.6035999999999999</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3126,10 +3126,10 @@
         <v>262</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.3117616666666667</v>
+        <v>0.3122616666666667</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.6635500000000002</v>
+        <v>0.6645000000000002</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3160,10 +3160,10 @@
         <v>289</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.02912500000000001</v>
+        <v>0.029225</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.38717</v>
+        <v>0.38772</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3194,10 +3194,10 @@
         <v>288</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.07817499999999999</v>
+        <v>0.07857500000000001</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.4064083333333334</v>
+        <v>0.4069583333333334</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3219,7 +3219,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0097</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>101</v>
@@ -3228,10 +3228,10 @@
         <v>285</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04811666666666666</v>
+        <v>0.04721666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2343500000000001</v>
+        <v>0.2332</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3256,16 +3256,16 @@
         <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>209</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01075</v>
+        <v>0.01035</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.0953333333333333</v>
+        <v>0.09404999999999998</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3296,7 +3296,7 @@
         <v>246</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03068333333333334</v>
+        <v>0.03063333333333334</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>0.2715816666666668</v>
@@ -3330,10 +3330,10 @@
         <v>198</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.04953333333333333</v>
+        <v>0.04963333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2295333333333333</v>
+        <v>0.2293333333333333</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.00035</v>
@@ -3364,10 +3364,10 @@
         <v>219</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02869166666666667</v>
+        <v>0.02879166666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3149566666666668</v>
+        <v>0.3151566666666668</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3401,7 +3401,7 @@
         <v>0.0062</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.1018833333333333</v>
+        <v>0.1015833333333333</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0</v>
@@ -3432,10 +3432,10 @@
         <v>185</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01373333333333333</v>
+        <v>0.01368333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1174916666666667</v>
+        <v>0.1175416666666667</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0.00025</v>
@@ -3469,7 +3469,7 @@
         <v>0.06420000000000002</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2436749999999999</v>
+        <v>0.2439249999999999</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -3506,7 +3506,7 @@
         <v>0.003066666666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.009316666666666666</v>
+        <v>0.009516666666666666</v>
       </c>
     </row>
     <row r="26">
@@ -3525,7 +3525,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.00315</v>
+        <v>0.00325</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>105</v>
@@ -3534,10 +3534,10 @@
         <v>210</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02510833333333333</v>
+        <v>0.02530833333333334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2197250000000001</v>
+        <v>0.220325</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.0002</v>
@@ -3571,10 +3571,10 @@
         <v>0.0005166666666666666</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.02988333333333334</v>
+        <v>0.02983333333333334</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01191666666666667</v>
+        <v>0.01211666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3605,7 +3605,7 @@
         <v>0.005966666666666666</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.09971666666666668</v>
+        <v>0.09961666666666667</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0</v>
@@ -3639,7 +3639,7 @@
         <v>0.007716666666666667</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1121866666666666</v>
+        <v>0.1124866666666666</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.001866666666666666</v>
@@ -3673,10 +3673,10 @@
         <v>0.005183333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1015333333333333</v>
+        <v>0.1018833333333333</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.01498333333333333</v>
+        <v>0.01488333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -3707,7 +3707,7 @@
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.001066666666666667</v>
+        <v>0.001083333333333333</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0.01701666666666667</v>
@@ -3738,13 +3738,13 @@
         <v>229</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.007866666666666668</v>
+        <v>0.007966666666666667</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1582366666666667</v>
+        <v>0.1589866666666667</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00155</v>
+        <v>0.00145</v>
       </c>
     </row>
     <row r="33">
@@ -3775,10 +3775,10 @@
         <v>0.005383333333333333</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05225833333333332</v>
+        <v>0.05215833333333333</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.01198333333333333</v>
+        <v>0.01188333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -3809,10 +3809,10 @@
         <v>0.0027</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03841666666666667</v>
+        <v>0.03851666666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02593333333333334</v>
+        <v>0.02583333333333334</v>
       </c>
     </row>
     <row r="35">
@@ -3843,7 +3843,7 @@
         <v>0.007433333333333333</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.07463333333333334</v>
+        <v>0.07483333333333334</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0</v>
@@ -3877,10 +3877,10 @@
         <v>0.01448333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.042</v>
+        <v>0.0421</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1579833333333333</v>
+        <v>0.1576833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3914,7 +3914,7 @@
         <v>0.003483333333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.07665000000000004</v>
+        <v>0.07685000000000003</v>
       </c>
     </row>
     <row r="38">
@@ -3948,7 +3948,7 @@
         <v>0.0003666666666666667</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1536166666666667</v>
+        <v>0.1537166666666666</v>
       </c>
     </row>
     <row r="39">
@@ -3979,10 +3979,10 @@
         <v>0.0001</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.018625</v>
+        <v>0.018675</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.03793333333333333</v>
+        <v>0.03773333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -4013,10 +4013,10 @@
         <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.01158333333333333</v>
+        <v>0.01148333333333333</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1416333333333333</v>
+        <v>0.1417333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -4044,13 +4044,13 @@
         <v>246</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00465</v>
+        <v>0.00445</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.02755</v>
+        <v>0.0272</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.06728333333333332</v>
+        <v>0.06783333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -4084,7 +4084,7 @@
         <v>0.003366666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2689833333333334</v>
+        <v>0.2685333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 19:40:12 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T23:26:18.999458+00:00</t>
+          <t>2026-03-22T23:40:12.397623+00:00</t>
         </is>
       </c>
     </row>
@@ -2423,14 +2423,10 @@
       </c>
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G46" s="5" t="n">
-        <v>0.8481569121456763</v>
-      </c>
-      <c r="H46" s="5" t="n">
-        <v>0.1518430878543237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G46" s="5" t="inlineStr"/>
+      <c r="H46" s="5" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr">
         <is>
           <t>R32_W_01</t>
@@ -2709,7 +2705,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4347083333333334</v>
+        <v>0.4203083333333334</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>159</v>
@@ -2718,10 +2714,10 @@
         <v>313</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7597749999999999</v>
+        <v>0.7452916666666667</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.976125</v>
+        <v>0.974425</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2743,19 +2739,19 @@
         <v>8</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.05439166666666666</v>
+        <v>0.05514166666666667</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>260</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.2053583333333333</v>
+        <v>0.208475</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.5790666666666665</v>
+        <v>0.5829249999999999</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2777,19 +2773,19 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.087725</v>
+        <v>0.08762499999999999</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G4" s="8" t="n">
         <v>298</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2649533333333333</v>
+        <v>0.2622566666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5883833333333334</v>
+        <v>0.5849700000000002</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2811,19 +2807,19 @@
         <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.01779166666666667</v>
+        <v>0.01859166666666666</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>241</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1390249999999999</v>
+        <v>0.1422249999999999</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5724083333333331</v>
+        <v>0.5781416666666666</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2845,19 +2841,19 @@
         <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.04998333333333333</v>
+        <v>0.04828333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>251</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1495033333333333</v>
+        <v>0.1459066666666667</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.438785</v>
+        <v>0.4298933333333334</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2888,10 +2884,10 @@
         <v>257</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.04466666666666666</v>
+        <v>0.04198333333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3813316666666667</v>
+        <v>0.3691399999999999</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2913,19 +2909,19 @@
         <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.022975</v>
+        <v>0.024625</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>291</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1291866666666667</v>
+        <v>0.13169</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5545333333333333</v>
+        <v>0.56045</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2947,19 +2943,19 @@
         <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.03168333333333333</v>
+        <v>0.04868333333333334</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>260</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.08808333333333336</v>
+        <v>0.1152</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3223566666666667</v>
+        <v>0.3550233333333335</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0.00015</v>
@@ -2981,19 +2977,19 @@
         <v>8</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0138</v>
+        <v>0.013</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>291</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1021083333333333</v>
+        <v>0.09859166666666667</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5414366666666666</v>
+        <v>0.5297816666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3015,19 +3011,19 @@
         <v>7</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.008633333333333333</v>
+        <v>0.009233333333333333</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>99</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.06731666666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.2405916666666667</v>
+        <v>0.242825</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3052,16 +3048,16 @@
         <v>0</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>284</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.0001833333333333333</v>
+        <v>0.0003333333333333333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.1363666666666667</v>
+        <v>0.140525</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0.0004</v>
@@ -3083,19 +3079,19 @@
         <v>10</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.146625</v>
+        <v>0.1436083333333333</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G13" s="9" t="n">
         <v>277</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.2925116666666667</v>
+        <v>0.2854566666666666</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.6035999999999999</v>
+        <v>0.5944666666666667</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3117,7 +3113,7 @@
         <v>10</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.07649999999999998</v>
+        <v>0.07181666666666665</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>131</v>
@@ -3126,10 +3122,10 @@
         <v>262</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.3122616666666667</v>
+        <v>0.2926900000000001</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.6645000000000002</v>
+        <v>0.645275</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3160,10 +3156,10 @@
         <v>289</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.029225</v>
+        <v>0.02775833333333334</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.38772</v>
+        <v>0.3726233333333333</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3175,7 +3171,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
@@ -3185,19 +3181,19 @@
         <v>8</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0144</v>
+        <v>0.015</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.07857500000000001</v>
+        <v>0.06666666666666668</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.4069583333333334</v>
+        <v>0.2685</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3209,7 +3205,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
@@ -3219,19 +3215,19 @@
         <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.0097</v>
+        <v>0.01326666666666667</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.04721666666666666</v>
+        <v>0.07550833333333334</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2332</v>
+        <v>0.39677</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3256,16 +3252,16 @@
         <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.01035</v>
+        <v>0.0171</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.09404999999999998</v>
+        <v>0.1272666666666667</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3287,19 +3283,19 @@
         <v>7</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.002633333333333333</v>
+        <v>0.002933333333333333</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G19" s="9" t="n">
         <v>246</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03063333333333334</v>
+        <v>0.03126666666666667</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2715816666666668</v>
+        <v>0.2776733333333334</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3321,7 +3317,7 @@
         <v>7</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.00525</v>
+        <v>0.0053</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>109</v>
@@ -3330,10 +3326,10 @@
         <v>198</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.04963333333333333</v>
+        <v>0.05011666666666666</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2293333333333333</v>
+        <v>0.2324583333333333</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.00035</v>
@@ -3355,19 +3351,19 @@
         <v>8</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.0015</v>
+        <v>0.0013</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G21" s="9" t="n">
         <v>219</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02879166666666667</v>
+        <v>0.02763333333333334</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3151566666666668</v>
+        <v>0.3103983333333334</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3392,16 +3388,16 @@
         <v>0.00045</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>221</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.0062</v>
+        <v>0.00625</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.1015833333333333</v>
+        <v>0.1047333333333333</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0</v>
@@ -3423,7 +3419,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.001383333333333333</v>
+        <v>0.001183333333333333</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>90</v>
@@ -3432,13 +3428,13 @@
         <v>185</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01368333333333333</v>
+        <v>0.01278333333333333</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.1175416666666667</v>
+        <v>0.114925</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.00025</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="24">
@@ -3457,19 +3453,19 @@
         <v>8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.01396666666666667</v>
+        <v>0.01375</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>107</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.06420000000000002</v>
+        <v>0.06232500000000002</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2439249999999999</v>
+        <v>0.2379083333333334</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -3506,7 +3502,7 @@
         <v>0.003066666666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.009516666666666666</v>
+        <v>0.008816666666666665</v>
       </c>
     </row>
     <row r="26">
@@ -3525,7 +3521,7 @@
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.00325</v>
+        <v>0.00285</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>105</v>
@@ -3534,10 +3530,10 @@
         <v>210</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02530833333333334</v>
+        <v>0.02333333333333334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.220325</v>
+        <v>0.2052583333333333</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0.0002</v>
@@ -3562,19 +3558,19 @@
         <v>0</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G27" s="9" t="n">
         <v>164</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0005166666666666666</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.02983333333333334</v>
+        <v>0.03121666666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01211666666666667</v>
+        <v>0.01041666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -3602,10 +3598,10 @@
         <v>207</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.005966666666666666</v>
+        <v>0.00625</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.09961666666666667</v>
+        <v>0.1017166666666667</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0</v>
@@ -3630,19 +3626,19 @@
         <v>0.00025</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G29" s="9" t="n">
         <v>231</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.007716666666666667</v>
+        <v>0.007016666666666666</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1124866666666666</v>
+        <v>0.104515</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.001866666666666666</v>
+        <v>0.002966666666666666</v>
       </c>
     </row>
     <row r="30">
@@ -3664,19 +3660,19 @@
         <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>212</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.005183333333333333</v>
+        <v>0.004733333333333332</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.1018833333333333</v>
+        <v>0.09405833333333334</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.01488333333333333</v>
+        <v>0.01628333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -3698,7 +3694,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G31" s="9" t="n">
         <v>171</v>
@@ -3707,10 +3703,10 @@
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.001083333333333333</v>
+        <v>0.001116666666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01701666666666667</v>
+        <v>0.01601666666666667</v>
       </c>
     </row>
     <row r="32">
@@ -3729,22 +3725,22 @@
         <v>8</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00015</v>
+        <v>5e-05</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>229</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.007966666666666667</v>
+        <v>0.006266666666666666</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.1589866666666667</v>
+        <v>0.14932</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.00145</v>
+        <v>0.0019</v>
       </c>
     </row>
     <row r="33">
@@ -3769,16 +3765,16 @@
         <v>74</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.005383333333333333</v>
+        <v>0.004925</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05215833333333333</v>
+        <v>0.05085833333333333</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.01188333333333333</v>
+        <v>0.01308333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -3800,19 +3796,19 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>171</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0027</v>
+        <v>0.0026</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03851666666666667</v>
+        <v>0.03521666666666667</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02583333333333334</v>
+        <v>0.02948333333333333</v>
       </c>
     </row>
     <row r="35">
@@ -3834,16 +3830,16 @@
         <v>0.00055</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G35" s="9" t="n">
         <v>196</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.007433333333333333</v>
+        <v>0.007166666666666666</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.07483333333333334</v>
+        <v>0.07201666666666667</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>0</v>
@@ -3865,7 +3861,7 @@
         <v>5</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.0005</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="F36" s="8" t="n">
         <v>61</v>
@@ -3874,13 +3870,13 @@
         <v>252</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01448333333333333</v>
+        <v>0.01418333333333333</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.0421</v>
+        <v>0.04139999999999999</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1576833333333333</v>
+        <v>0.1597833333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3902,7 +3898,7 @@
         <v>0</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G37" s="9" t="n">
         <v>142</v>
@@ -3911,10 +3907,10 @@
         <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.003483333333333334</v>
+        <v>0.003683333333333334</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.07685000000000003</v>
+        <v>0.07066666666666668</v>
       </c>
     </row>
     <row r="38">
@@ -3948,7 +3944,7 @@
         <v>0.0003666666666666667</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1537166666666666</v>
+        <v>0.1512333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3979,10 +3975,10 @@
         <v>0.0001</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.018675</v>
+        <v>0.018075</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.03773333333333333</v>
+        <v>0.03658333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -4013,10 +4009,10 @@
         <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.01148333333333333</v>
+        <v>0.01203333333333334</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1417333333333333</v>
+        <v>0.1332833333333333</v>
       </c>
     </row>
     <row r="41">
@@ -4035,22 +4031,22 @@
         <v>7</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.00095</v>
+        <v>0.00135</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>246</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.00445</v>
+        <v>0.008</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.0272</v>
+        <v>0.04171666666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.06783333333333333</v>
+        <v>0.06153333333333333</v>
       </c>
     </row>
     <row r="42">
@@ -4081,10 +4077,10 @@
         <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.003366666666666666</v>
+        <v>0.003266666666666666</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2685333333333333</v>
+        <v>0.28655</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 20:00:10 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leaderboard'!$A$1:$J$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>d47a3783c781a135</t>
+          <t>c5094b59c8952f07</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>a02614466dbdf7f2</t>
+          <t>d47a3783c781a135</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Round of 32: St. John's over Kansas</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22T23:40:12.397623+00:00</t>
+          <t>2026-03-23T00:00:09.546659+00:00</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2031,10 +2031,14 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>St. John's</t>
+        </is>
+      </c>
       <c r="F35" s="6" t="b">
         <v>0</v>
       </c>
@@ -2552,12 +2556,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>East</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Illinois vs Houston</t>
+          <t>Duke vs St. John's</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -2573,7 +2577,7 @@
       <c r="H50" s="5" t="inlineStr"/>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>R16_S_02</t>
+          <t>R16_E_01</t>
         </is>
       </c>
     </row>
@@ -2585,12 +2589,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Texas vs Purdue</t>
+          <t>Illinois vs Houston</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2606,12 +2610,45 @@
       <c r="H51" s="7" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
+          <t>R16_S_02</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Sweet 16</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Texas vs Purdue</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G52" s="5" t="inlineStr"/>
+      <c r="H52" s="5" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
           <t>R16_W_02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I51"/>
+  <autoFilter ref="A1:I52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2705,19 +2742,19 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4203083333333334</v>
+        <v>0.4041166666666667</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>313</v>
+        <v>337</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7452916666666667</v>
+        <v>0.7354249999999998</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.974425</v>
+        <v>0.9643</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2736,22 +2773,22 @@
         <v>65</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.05514166666666667</v>
+        <v>0.02723333333333334</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.208475</v>
+        <v>0.1315416666666667</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.5829249999999999</v>
+        <v>0.4904866666666666</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2770,22 +2807,22 @@
         <v>64</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.08762499999999999</v>
+        <v>0.06431666666666667</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2622566666666667</v>
+        <v>0.1889333333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.5849700000000002</v>
+        <v>0.4997183333333335</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2797,29 +2834,29 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.01859166666666666</v>
+        <v>0.06755</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>127</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>241</v>
+        <v>258</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1422249999999999</v>
+        <v>0.1913666666666666</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5781416666666666</v>
+        <v>0.5107883333333332</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2831,29 +2868,29 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.04828333333333333</v>
+        <v>0.04585</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>251</v>
+        <v>292</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1459066666666667</v>
+        <v>0.1946583333333333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.4298933333333334</v>
+        <v>0.6565283333333333</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2865,29 +2902,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0</v>
+        <v>0.02148333333333333</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>257</v>
+        <v>238</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.04198333333333333</v>
+        <v>0.1411083333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3691399999999999</v>
+        <v>0.5622183333333334</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2899,29 +2936,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.024625</v>
+        <v>0.01895</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>291</v>
+        <v>243</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.13169</v>
+        <v>0.1045666666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.56045</v>
+        <v>0.294715</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2933,32 +2970,32 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.04868333333333334</v>
+        <v>0.1121666666666667</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1152</v>
+        <v>0.3610000000000001</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.3550233333333335</v>
+        <v>0.6995333333333336</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2967,29 +3004,29 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.013</v>
+        <v>0.02325</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.09859166666666667</v>
+        <v>0.0861</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.5297816666666666</v>
+        <v>0.3210416666666666</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3001,29 +3038,29 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.009233333333333333</v>
+        <v>0.01905</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>240</v>
+        <v>295</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.06731666666666666</v>
+        <v>0.101</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.242825</v>
+        <v>0.4821116666666669</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3035,32 +3072,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>284</v>
+        <v>250</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.0003333333333333333</v>
+        <v>0.02826666666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.140525</v>
+        <v>0.3488600000000001</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -3069,29 +3106,29 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.1436083333333333</v>
+        <v>0.00525</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>277</v>
+        <v>247</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.2854566666666666</v>
+        <v>0.05225833333333332</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.5944666666666667</v>
+        <v>0.3809583333333333</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3103,32 +3140,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.07181666666666665</v>
+        <v>0.03643333333333333</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.2926900000000001</v>
+        <v>0.08609166666666668</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.645275</v>
+        <v>0.2705066666666667</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0</v>
+        <v>0.0004666666666666666</v>
       </c>
     </row>
     <row r="15">
@@ -3137,29 +3174,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0</v>
+        <v>0.01273333333333333</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.02775833333333334</v>
+        <v>0.09213333333333333</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.3726233333333333</v>
+        <v>0.5114200000000001</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3171,29 +3208,29 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.015</v>
+        <v>0.0003</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>285</v>
+        <v>221</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.06666666666666668</v>
+        <v>0.0044</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2685</v>
+        <v>0.09553666666666666</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3205,32 +3242,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.01326666666666667</v>
+        <v>0</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>288</v>
+        <v>268</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.07550833333333334</v>
+        <v>5e-05</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.39677</v>
+        <v>0.1305366666666667</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0</v>
+        <v>0.0003666666666666667</v>
       </c>
     </row>
     <row r="18">
@@ -3239,29 +3276,29 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0</v>
+        <v>0.1042666666666666</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>221</v>
+        <v>255</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.0171</v>
+        <v>0.2189083333333334</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1272666666666667</v>
+        <v>0.5102150000000002</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3273,29 +3310,29 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.002933333333333333</v>
+        <v>0</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>246</v>
+        <v>282</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.03126666666666667</v>
+        <v>0.02335</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.2776733333333334</v>
+        <v>0.3582583333333333</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3307,32 +3344,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.0053</v>
+        <v>0.0204</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.05011666666666666</v>
+        <v>0.080225</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2324583333333333</v>
+        <v>0.3031416666666666</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.00035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -3341,29 +3378,29 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.0013</v>
+        <v>0</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02763333333333334</v>
+        <v>0.02006666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3103983333333334</v>
+        <v>0.1238116666666667</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3375,32 +3412,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.00045</v>
+        <v>0</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>221</v>
+        <v>173</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.00625</v>
+        <v>0</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.1047333333333333</v>
+        <v>0.007050000000000002</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0</v>
+        <v>0.004583333333333332</v>
       </c>
     </row>
     <row r="23">
@@ -3409,32 +3446,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.001183333333333333</v>
+        <v>0.00645</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01278333333333333</v>
+        <v>0.0488</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.114925</v>
+        <v>0.2218449999999999</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0003</v>
+        <v>0.00065</v>
       </c>
     </row>
     <row r="24">
@@ -3443,32 +3480,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.01375</v>
+        <v>5e-05</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.06232500000000002</v>
+        <v>0.00805</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.2379083333333334</v>
+        <v>0.2057216666666667</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="25">
@@ -3477,32 +3514,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0</v>
+        <v>0.0019</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0</v>
+        <v>0.01305</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.003066666666666667</v>
+        <v>0.11815</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.008816666666666665</v>
+        <v>0.0006833333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3511,32 +3548,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.00285</v>
+        <v>0.00035</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.02333333333333334</v>
+        <v>0.01036666666666667</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.2052583333333333</v>
+        <v>0.1385583333333333</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -3545,32 +3582,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0</v>
+        <v>0.00035</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>164</v>
+        <v>229</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0119</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.03121666666666667</v>
+        <v>0.1626950000000001</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.01041666666666667</v>
+        <v>0.001283333333333333</v>
       </c>
     </row>
     <row r="28">
@@ -3579,32 +3616,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>207</v>
+        <v>166</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.00625</v>
+        <v>0</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1017166666666667</v>
+        <v>0.001816666666666667</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0</v>
+        <v>0.008783333333333332</v>
       </c>
     </row>
     <row r="29">
@@ -3613,32 +3650,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.00025</v>
+        <v>0.0033</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.007016666666666666</v>
+        <v>0.02438333333333333</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.104515</v>
+        <v>0.1977550000000001</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.002966666666666666</v>
+        <v>0.00055</v>
       </c>
     </row>
     <row r="30">
@@ -3647,32 +3684,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>212</v>
+        <v>164</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.004733333333333332</v>
+        <v>0.0013</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.09405833333333334</v>
+        <v>0.02848333333333334</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.01628333333333333</v>
+        <v>0.01411666666666667</v>
       </c>
     </row>
     <row r="31">
@@ -3681,32 +3718,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
         <v>39</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0</v>
+        <v>0.002183333333333333</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.001116666666666667</v>
+        <v>0.05392333333333334</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.01601666666666667</v>
+        <v>0.03054999999999999</v>
       </c>
     </row>
     <row r="32">
@@ -3715,32 +3752,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>5e-05</v>
+        <v>0.00115</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>98</v>
+        <v>67</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>229</v>
+        <v>252</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.006266666666666666</v>
+        <v>0.01575</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.14932</v>
+        <v>0.05199500000000001</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0019</v>
+        <v>0.09896666666666668</v>
       </c>
     </row>
     <row r="33">
@@ -3749,32 +3786,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>176</v>
+        <v>129</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.004925</v>
+        <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.05085833333333333</v>
+        <v>0.0009333333333333334</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.01308333333333333</v>
+        <v>0.09396666666666667</v>
       </c>
     </row>
     <row r="34">
@@ -3783,11 +3820,11 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>7</v>
@@ -3796,19 +3833,19 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>171</v>
+        <v>212</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0026</v>
+        <v>0.00125</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.03521666666666667</v>
+        <v>0.07784166666666666</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.02948333333333333</v>
+        <v>0.004983333333333334</v>
       </c>
     </row>
     <row r="35">
@@ -3817,32 +3854,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.00055</v>
+        <v>0</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>196</v>
+        <v>177</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.007166666666666666</v>
+        <v>0.00095</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.07201666666666667</v>
+        <v>0.02795</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0</v>
+        <v>0.01835833333333333</v>
       </c>
     </row>
     <row r="36">
@@ -3851,32 +3888,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0001</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>252</v>
+        <v>176</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.01418333333333333</v>
+        <v>0.004683333333333334</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04139999999999999</v>
+        <v>0.04885</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1597833333333333</v>
+        <v>0.01666666666666667</v>
       </c>
     </row>
     <row r="37">
@@ -3885,14 +3922,14 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>0</v>
@@ -3901,16 +3938,16 @@
         <v>60</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>142</v>
+        <v>192</v>
       </c>
       <c r="H37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.003683333333333334</v>
+        <v>0.008633333333333333</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.07066666666666668</v>
+        <v>0.1732083333333333</v>
       </c>
     </row>
     <row r="38">
@@ -3919,32 +3956,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0</v>
+        <v>0.0027</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>129</v>
+        <v>246</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0</v>
+        <v>0.009849999999999999</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.0003666666666666667</v>
+        <v>0.05465833333333334</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1512333333333333</v>
+        <v>0.04763333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3953,32 +3990,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0.0001</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.018075</v>
+        <v>0.009416666666666667</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.03658333333333333</v>
+        <v>0.05066666666666667</v>
       </c>
     </row>
     <row r="40">
@@ -3987,32 +4024,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0</v>
+        <v>0.005933333333333333</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.01203333333333334</v>
+        <v>0.06567833333333335</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.1332833333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -4021,32 +4058,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D41" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.00135</v>
+        <v>0</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>246</v>
+        <v>142</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.04171666666666667</v>
+        <v>0.001066666666666667</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.06153333333333333</v>
+        <v>0.09630833333333334</v>
       </c>
     </row>
     <row r="42">
@@ -4068,7 +4105,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>110</v>
@@ -4077,10 +4114,10 @@
         <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.003266666666666666</v>
+        <v>0.002291666666666667</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.28655</v>
+        <v>0.3371083333333335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 20:21:05 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Round of 32: St. John's over Kansas</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T00:00:09.546659+00:00</t>
+          <t>2026-03-23T00:21:05.202832+00:00</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 20:40:09 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leaderboard'!$A$1:$J$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>c5094b59c8952f07</t>
+          <t>6cacbdc265ddc526</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>d47a3783c781a135</t>
+          <t>c5094b59c8952f07</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Round of 32: Tennessee over Virginia</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T00:21:05.202832+00:00</t>
+          <t>2026-03-23T00:40:09.153639+00:00</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>pre</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2208,10 +2208,14 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Tennessee</t>
+        </is>
+      </c>
       <c r="F40" s="4" t="b">
         <v>0</v>
       </c>
@@ -2241,7 +2245,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2278,7 +2282,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
@@ -2311,7 +2315,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2348,7 +2352,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2385,7 +2389,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2422,7 +2426,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
@@ -2455,7 +2459,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2492,7 +2496,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2529,7 +2533,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2589,12 +2593,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Illinois vs Houston</t>
+          <t>Tennessee vs Iowa State</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2610,7 +2614,7 @@
       <c r="H51" s="7" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>R16_S_02</t>
+          <t>R16_M_02</t>
         </is>
       </c>
     </row>
@@ -2622,12 +2626,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Texas vs Purdue</t>
+          <t>Illinois vs Houston</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2643,12 +2647,45 @@
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr">
         <is>
+          <t>R16_S_02</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Sweet 16</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Texas vs Purdue</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G53" s="7" t="inlineStr"/>
+      <c r="H53" s="7" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
           <t>R16_W_02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I52"/>
+  <autoFilter ref="A1:I53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2736,25 +2773,25 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4041166666666667</v>
+        <v>0.49545</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7354249999999998</v>
+        <v>0.8128249999999999</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9643</v>
+        <v>0.9850583333333333</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2766,29 +2803,29 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Ryan Evans</t>
+          <t>Stephen Mason</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.02723333333333334</v>
+        <v>0.07335</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>256</v>
+        <v>299</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.1315416666666667</v>
+        <v>0.2443666666666667</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.4904866666666666</v>
+        <v>0.59797</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2800,29 +2837,29 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Stephen Mason</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.06431666666666667</v>
+        <v>0.05671666666666667</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>310</v>
+        <v>294</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.1889333333333333</v>
+        <v>0.2559916666666667</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.4997183333333335</v>
+        <v>0.7691399999999999</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2834,29 +2871,29 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.06755</v>
+        <v>0.02723333333333333</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1913666666666666</v>
+        <v>0.1854083333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.5107883333333332</v>
+        <v>0.675145</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2868,29 +2905,29 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.04585</v>
+        <v>0.03431666666666667</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>292</v>
+        <v>307</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1946583333333333</v>
+        <v>0.1626</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.6565283333333333</v>
+        <v>0.6021283333333335</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2902,29 +2939,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.02148333333333333</v>
+        <v>0.00735</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1411083333333333</v>
+        <v>0.07646666666666667</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.5622183333333334</v>
+        <v>0.4933083333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2936,29 +2973,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>Ryan Evans</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.01895</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1045666666666667</v>
+        <v>0.08168333333333333</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.294715</v>
+        <v>0.3965833333333332</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -2970,29 +3007,29 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.1121666666666667</v>
+        <v>0.0203</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>136</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>264</v>
+        <v>292</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.3610000000000001</v>
+        <v>0.1361083333333334</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.6995333333333336</v>
+        <v>0.6259583333333331</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -3004,29 +3041,29 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.02325</v>
+        <v>0</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>297</v>
+        <v>272</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.0861</v>
+        <v>0.00015</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.3210416666666666</v>
+        <v>0.1866416666666667</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3038,29 +3075,29 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.01905</v>
+        <v>0.1386833333333333</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.101</v>
+        <v>0.2686416666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.4821116666666669</v>
+        <v>0.5854583333333335</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3072,29 +3109,29 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0</v>
+        <v>0.01258333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.02826666666666667</v>
+        <v>0.06866666666666667</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3488600000000001</v>
+        <v>0.3363099999999999</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0</v>
@@ -3106,29 +3143,29 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.00525</v>
+        <v>0</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>247</v>
+        <v>283</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.05225833333333332</v>
+        <v>0.04295</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.3809583333333333</v>
+        <v>0.4952766666666668</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3140,32 +3177,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.03643333333333333</v>
+        <v>0.01133333333333333</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>251</v>
+        <v>230</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.08609166666666668</v>
+        <v>0.084825</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.2705066666666667</v>
+        <v>0.2601416666666667</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.0004666666666666666</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3174,29 +3211,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.01273333333333333</v>
+        <v>0.05985</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>282</v>
+        <v>266</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.09213333333333333</v>
+        <v>0.2944083333333333</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.5114200000000001</v>
+        <v>0.6358166666666665</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3208,29 +3245,29 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0003</v>
+        <v>0.0157</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>221</v>
+        <v>282</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0044</v>
+        <v>0.06581666666666668</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.09553666666666666</v>
+        <v>0.2728083333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3242,32 +3279,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>5e-05</v>
+        <v>0.005183333333333333</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.1305366666666667</v>
+        <v>0.2646666666666667</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.0003666666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3276,29 +3313,29 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.1042666666666666</v>
+        <v>0.0012</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>255</v>
+        <v>238</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.2189083333333334</v>
+        <v>0.0186</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.5102150000000002</v>
+        <v>0.2384166666666666</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3310,32 +3347,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0</v>
+        <v>0.02491666666666667</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>282</v>
+        <v>247</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.02335</v>
+        <v>0.06288333333333332</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.3582583333333333</v>
+        <v>0.215525</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="20">
@@ -3344,29 +3381,29 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.0204</v>
+        <v>5e-05</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.080225</v>
+        <v>0.0023</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.3031416666666666</v>
+        <v>0.07544166666666666</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0</v>
@@ -3378,29 +3415,29 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0</v>
+        <v>0.00065</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>221</v>
+        <v>193</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.02006666666666667</v>
+        <v>0.01818333333333333</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.1238116666666667</v>
+        <v>0.1601666666666667</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3412,32 +3449,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>173</v>
+        <v>221</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0</v>
+        <v>0.01046666666666667</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.007050000000000002</v>
+        <v>0.08744166666666667</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.004583333333333332</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -3446,32 +3483,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.00645</v>
+        <v>0</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>110</v>
+        <v>77</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>204</v>
+        <v>173</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.0488</v>
+        <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.2218449999999999</v>
+        <v>0.005741666666666667</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.00065</v>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="24">
@@ -3480,32 +3517,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E24" s="5" t="n">
+        <v>0.002483333333333333</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>203</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>0.03316666666666666</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>0.1668116666666667</v>
+      </c>
+      <c r="J24" s="5" t="n">
         <v>5e-05</v>
-      </c>
-      <c r="F24" s="8" t="n">
-        <v>106</v>
-      </c>
-      <c r="G24" s="8" t="n">
-        <v>213</v>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>0.00805</v>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>0.2057216666666667</v>
-      </c>
-      <c r="J24" s="5" t="n">
-        <v>0.0001</v>
       </c>
     </row>
     <row r="25">
@@ -3514,32 +3551,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.0019</v>
+        <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.01305</v>
+        <v>0.0038</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.11815</v>
+        <v>0.08583999999999999</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.0006833333333333333</v>
+        <v>0.003533333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -3548,32 +3585,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.00035</v>
+        <v>0.0015</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>220</v>
+        <v>243</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.01036666666666667</v>
+        <v>0.0167</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1385583333333333</v>
+        <v>0.06772499999999999</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0</v>
+        <v>0.01513333333333333</v>
       </c>
     </row>
     <row r="27">
@@ -3582,32 +3619,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D27" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.00035</v>
+        <v>3.333333333333333e-05</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0119</v>
+        <v>0.002891666666666667</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1626950000000001</v>
+        <v>0.1508116666666666</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.001283333333333333</v>
+        <v>5e-05</v>
       </c>
     </row>
     <row r="28">
@@ -3616,32 +3653,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0</v>
+        <v>0.009675</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.001816666666666667</v>
+        <v>0.09574000000000001</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.008783333333333332</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="29">
@@ -3650,32 +3687,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>John Cash III</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.0033</v>
+        <v>0</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.02438333333333333</v>
+        <v>0.002616666666666666</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1977550000000001</v>
+        <v>0.1394416666666667</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.00055</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="30">
@@ -3684,32 +3721,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0</v>
+        <v>5e-05</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>164</v>
+        <v>210</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0013</v>
+        <v>0.001233333333333333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.02848333333333334</v>
+        <v>0.05612499999999999</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.01411666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -3718,32 +3755,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>190</v>
+        <v>167</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.002183333333333333</v>
+        <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.05392333333333334</v>
+        <v>0.001816666666666667</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.03054999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -3752,32 +3789,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00115</v>
+        <v>0.00615</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.01575</v>
+        <v>0.01336666666666667</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.05199500000000001</v>
+        <v>0.06710000000000001</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.09896666666666668</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -3786,32 +3823,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>John Cash III</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>58</v>
+        <v>104</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>129</v>
+        <v>211</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0</v>
+        <v>0.016875</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.0009333333333333334</v>
+        <v>0.1509166666666666</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>0.09396666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -3820,32 +3857,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E34" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>212</v>
+        <v>145</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.00125</v>
+        <v>0</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.07784166666666666</v>
+        <v>5.833333333333333e-05</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.004983333333333334</v>
+        <v>0.01781666666666667</v>
       </c>
     </row>
     <row r="35">
@@ -3854,32 +3891,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>177</v>
+        <v>125</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.00095</v>
+        <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.02795</v>
+        <v>0</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.01835833333333333</v>
+        <v>0.17375</v>
       </c>
     </row>
     <row r="36">
@@ -3888,32 +3925,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.004683333333333334</v>
+        <v>0</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.04885</v>
+        <v>0.0039</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.01666666666666667</v>
+        <v>0.02383333333333333</v>
       </c>
     </row>
     <row r="37">
@@ -3922,32 +3959,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
         <v>35</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.008633333333333333</v>
+        <v>0.01770833333333333</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.1732083333333333</v>
+        <v>0.02326666666666666</v>
       </c>
     </row>
     <row r="38">
@@ -3956,32 +3993,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.0027</v>
+        <v>0</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>246</v>
+        <v>192</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.009849999999999999</v>
+        <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.05465833333333334</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.04763333333333333</v>
+        <v>0.1581333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -3997,25 +4034,25 @@
         <v>34</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.009416666666666667</v>
+        <v>0.0013</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.05066666666666667</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="40">
@@ -4031,22 +4068,22 @@
         <v>33</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.005933333333333333</v>
+        <v>0.00055</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.06567833333333335</v>
+        <v>0.01941</v>
       </c>
       <c r="J40" s="5" t="n">
         <v>0</v>
@@ -4071,7 +4108,7 @@
         <v>0</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>142</v>
@@ -4080,10 +4117,10 @@
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.001066666666666667</v>
+        <v>0.00115</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.09630833333333334</v>
+        <v>0.08020000000000001</v>
       </c>
     </row>
     <row r="42">
@@ -4099,25 +4136,25 @@
         <v>18</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E42" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="H42" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.002291666666666667</v>
+        <v>0</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.3371083333333335</v>
+        <v>0.4259333333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 21:02:27 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Round of 32: Tennessee over Virginia</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T00:40:09.153639+00:00</t>
+          <t>2026-03-23T01:02:27.214347+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 21:20:17 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T01:02:27.214347+00:00</t>
+          <t>2026-03-23T01:20:16.863021+00:00</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 21:40:13 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leaderboard'!$A$1:$J$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>6cacbdc265ddc526</t>
+          <t>bee57d9ed3cd4c63</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>c5094b59c8952f07</t>
+          <t>6cacbdc265ddc526</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Round of 32: Iowa over Florida</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T01:20:16.863021+00:00</t>
+          <t>2026-03-23T01:40:13.069452+00:00</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2282,10 +2282,14 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Iowa</t>
+        </is>
+      </c>
       <c r="F42" s="4" t="b">
         <v>0</v>
       </c>
@@ -2631,7 +2635,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Illinois vs Houston</t>
+          <t>Iowa vs Nebraska</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2647,7 +2651,7 @@
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>R16_S_02</t>
+          <t>R16_S_01</t>
         </is>
       </c>
     </row>
@@ -2659,12 +2663,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Texas vs Purdue</t>
+          <t>Illinois vs Houston</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2680,12 +2684,45 @@
       <c r="H53" s="7" t="inlineStr"/>
       <c r="I53" s="2" t="inlineStr">
         <is>
+          <t>R16_S_02</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Sweet 16</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Texas vs Purdue</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G54" s="5" t="inlineStr"/>
+      <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
           <t>R16_W_02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I53"/>
+  <autoFilter ref="A1:I54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2779,19 +2816,19 @@
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.49545</v>
+        <v>0.3871833333333334</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.8128249999999999</v>
+        <v>0.7841000000000001</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9850583333333333</v>
+        <v>0.9829</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2807,25 +2844,25 @@
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.07335</v>
+        <v>0.2271333333333334</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>299</v>
+        <v>310</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.2443666666666667</v>
+        <v>0.4810866666666667</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.59797</v>
+        <v>0.7881083333333334</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2847,19 +2884,19 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.05671666666666667</v>
+        <v>0.05665</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>143</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2559916666666667</v>
+        <v>0.2350283333333333</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.7691399999999999</v>
+        <v>0.7815583333333334</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2881,19 +2918,19 @@
         <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.02723333333333333</v>
+        <v>0.01451666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1854083333333333</v>
+        <v>0.1709833333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.675145</v>
+        <v>0.6867916666666666</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2915,19 +2952,19 @@
         <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.03431666666666667</v>
+        <v>0.0314</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.1626</v>
+        <v>0.148975</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.6021283333333335</v>
+        <v>0.617138333333333</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2946,22 +2983,22 @@
         <v>66</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.00735</v>
+        <v>5e-05</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.07646666666666667</v>
+        <v>0.02595833333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.4933083333333333</v>
+        <v>0.3793216666666666</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -2980,22 +3017,22 @@
         <v>65</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0042</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.08168333333333333</v>
+        <v>0.04054166666666666</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3965833333333332</v>
+        <v>0.3189000000000001</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -3017,19 +3054,19 @@
         <v>8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.0203</v>
+        <v>0.01688333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1361083333333334</v>
+        <v>0.1163333333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.6259583333333331</v>
+        <v>0.6402333333333334</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -3054,16 +3091,16 @@
         <v>0</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.00015</v>
+        <v>0.0003</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.1866416666666667</v>
+        <v>0.1869083333333333</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3085,19 +3122,19 @@
         <v>9</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.1386833333333333</v>
+        <v>0.1351166666666667</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.2686416666666666</v>
+        <v>0.2757866666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.5854583333333335</v>
+        <v>0.6315666666666666</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3119,19 +3156,19 @@
         <v>7</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.01258333333333333</v>
+        <v>0.01693333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.06866666666666667</v>
+        <v>0.08732833333333333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3363099999999999</v>
+        <v>0.3781416666666666</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0</v>
@@ -3156,16 +3193,16 @@
         <v>0</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.04295</v>
+        <v>0.04091666666666666</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.4952766666666668</v>
+        <v>0.5158999999999999</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3184,22 +3221,22 @@
         <v>60</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.01133333333333333</v>
+        <v>0.0058</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.084825</v>
+        <v>0.05545</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.2601416666666667</v>
+        <v>0.214875</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3211,29 +3248,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.05985</v>
+        <v>0.00335</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>137</v>
+        <v>96</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.2944083333333333</v>
+        <v>0.056275</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.6358166666666665</v>
+        <v>0.1772333333333334</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3245,29 +3282,29 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0157</v>
+        <v>0.05538333333333333</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>110</v>
+        <v>136</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>282</v>
+        <v>267</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.06581666666666668</v>
+        <v>0.252095</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2728083333333333</v>
+        <v>0.6030300000000001</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3279,29 +3316,29 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
         <v>57</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0</v>
+        <v>0.01495</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>257</v>
+        <v>302</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.005183333333333333</v>
+        <v>0.06693333333333333</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2646666666666667</v>
+        <v>0.2763633333333334</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3313,29 +3350,29 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.0012</v>
+        <v>0</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.0186</v>
+        <v>0.00675</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.2384166666666666</v>
+        <v>0.2799083333333334</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3347,32 +3384,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.02491666666666667</v>
+        <v>0.00065</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>247</v>
+        <v>233</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.06288333333333332</v>
+        <v>0.0076</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.215525</v>
+        <v>0.1664833333333333</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -3381,29 +3418,29 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
         <v>54</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>5e-05</v>
+        <v>0.02546666666666667</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>221</v>
+        <v>247</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.0023</v>
+        <v>0.06511666666666667</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.07544166666666666</v>
+        <v>0.222825</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0</v>
@@ -3415,29 +3452,29 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.00065</v>
+        <v>0.0001833333333333333</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>193</v>
+        <v>221</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.01818333333333333</v>
+        <v>0.003675</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.1601666666666667</v>
+        <v>0.07509999999999999</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3449,29 +3486,29 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>221</v>
+        <v>193</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.01046666666666667</v>
+        <v>0.01346666666666666</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.08744166666666667</v>
+        <v>0.16475</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0</v>
@@ -3483,32 +3520,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>173</v>
+        <v>221</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0</v>
+        <v>0.01105</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.005741666666666667</v>
+        <v>0.09399999999999999</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>0.0035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -3517,32 +3554,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.002483333333333333</v>
+        <v>0</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>109</v>
+        <v>76</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>203</v>
+        <v>173</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.03316666666666666</v>
+        <v>0</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1668116666666667</v>
+        <v>0.005516666666666667</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>5e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -3551,7 +3588,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
@@ -3561,22 +3598,22 @@
         <v>6</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0</v>
+        <v>0.00015</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.0038</v>
+        <v>0.01575</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.08583999999999999</v>
+        <v>0.1141</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.003533333333333333</v>
+        <v>5e-05</v>
       </c>
     </row>
     <row r="26">
@@ -3585,32 +3622,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.0015</v>
+        <v>0</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>243</v>
+        <v>190</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.0167</v>
+        <v>0.005216666666666666</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.06772499999999999</v>
+        <v>0.1076916666666667</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.01513333333333333</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="27">
@@ -3629,22 +3666,22 @@
         <v>7</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>3.333333333333333e-05</v>
+        <v>0</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.002891666666666667</v>
+        <v>0.004158333333333332</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1508116666666666</v>
+        <v>0.1643</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>5e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -3663,22 +3700,22 @@
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.0003</v>
+        <v>0.00075</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.009675</v>
+        <v>0.01141666666666667</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.09574000000000001</v>
+        <v>0.1165416666666667</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3694,22 +3731,22 @@
         <v>47</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E29" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.002616666666666666</v>
+        <v>0</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1394416666666667</v>
+        <v>0.09124999999999998</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.0001</v>
@@ -3728,22 +3765,22 @@
         <v>46</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>5e-05</v>
+        <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.001233333333333333</v>
+        <v>0.0003</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.05612499999999999</v>
+        <v>0.02716666666666666</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0</v>
@@ -3762,22 +3799,22 @@
         <v>45</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="H31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.001816666666666667</v>
+        <v>0</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0</v>
@@ -3796,22 +3833,22 @@
         <v>44</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00615</v>
+        <v>0.00295</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.01336666666666667</v>
+        <v>0.0104</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.06710000000000001</v>
+        <v>0.05585833333333332</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0</v>
@@ -3830,22 +3867,22 @@
         <v>42</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.001</v>
+        <v>0.0001</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.016875</v>
+        <v>0.006308333333333332</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1509166666666666</v>
+        <v>0.09945</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0</v>
@@ -3870,7 +3907,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>145</v>
@@ -3879,10 +3916,10 @@
         <v>0</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>5.833333333333333e-05</v>
+        <v>8.000000000000001e-05</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.01781666666666667</v>
+        <v>0.008533333333333332</v>
       </c>
     </row>
     <row r="35">
@@ -3898,16 +3935,16 @@
         <v>38</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>0</v>
@@ -3916,7 +3953,7 @@
         <v>0</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.17375</v>
+        <v>0.2418</v>
       </c>
     </row>
     <row r="36">
@@ -3932,25 +3969,25 @@
         <v>36</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="H36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.0039</v>
+        <v>0.001983333333333333</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.02383333333333333</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="37">
@@ -3978,13 +4015,13 @@
         <v>172</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.01770833333333333</v>
+        <v>0.018375</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.02326666666666666</v>
+        <v>0.008683333333333333</v>
       </c>
     </row>
     <row r="38">
@@ -4015,10 +4052,10 @@
         <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0065</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.1581333333333333</v>
+        <v>0.06759999999999999</v>
       </c>
     </row>
     <row r="39">
@@ -4034,25 +4071,25 @@
         <v>34</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.0013</v>
+        <v>0.0002</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.074</v>
+        <v>0.07846666666666666</v>
       </c>
     </row>
     <row r="40">
@@ -4068,22 +4105,22 @@
         <v>33</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.00055</v>
+        <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.01941</v>
+        <v>0.00895</v>
       </c>
       <c r="J40" s="5" t="n">
         <v>0</v>
@@ -4102,25 +4139,25 @@
         <v>32</v>
       </c>
       <c r="D41" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="H41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.00115</v>
+        <v>0</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.08020000000000001</v>
+        <v>0.09003333333333335</v>
       </c>
     </row>
     <row r="42">
@@ -4136,16 +4173,16 @@
         <v>18</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E42" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="H42" s="5" t="n">
         <v>0</v>
@@ -4154,7 +4191,7 @@
         <v>0</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.4259333333333334</v>
+        <v>0.4755333333333335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 22:00:06 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Round of 32: Iowa over Florida</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T01:40:13.069452+00:00</t>
+          <t>2026-03-23T02:00:05.494737+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 22:20:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T02:00:05.494737+00:00</t>
+          <t>2026-03-23T02:20:08.023022+00:00</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>pre</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-22 22:40:23 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leaderboard'!$A$1:$J$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>bee57d9ed3cd4c63</t>
+          <t>377c1ef520c4154d</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>6cacbdc265ddc526</t>
+          <t>bee57d9ed3cd4c63</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T02:20:08.023022+00:00</t>
+          <t>2026-03-23T02:40:19.328651+00:00</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2430,10 +2430,14 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
       <c r="F46" s="4" t="b">
         <v>0</v>
       </c>
@@ -2701,7 +2705,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Texas vs Purdue</t>
+          <t>Arizona vs Arkansas</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -2717,12 +2721,45 @@
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr">
         <is>
+          <t>R16_W_01</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Sweet 16</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Texas vs Purdue</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G55" s="7" t="inlineStr"/>
+      <c r="H55" s="7" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
           <t>R16_W_02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I54"/>
+  <autoFilter ref="A1:I55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2810,25 +2847,25 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>9</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3871833333333334</v>
+        <v>0.4206000000000001</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>323</v>
+        <v>337</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7841000000000001</v>
+        <v>0.8282333333333334</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9829</v>
+        <v>0.9869166666666666</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2850,19 +2887,19 @@
         <v>7</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.2271333333333334</v>
+        <v>0.2217166666666666</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.4810866666666667</v>
+        <v>0.4938666666666667</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.7881083333333334</v>
+        <v>0.8047500000000001</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2884,19 +2921,19 @@
         <v>8</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.05665</v>
+        <v>0.05095</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.2350283333333333</v>
+        <v>0.230175</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.7815583333333334</v>
+        <v>0.76109</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2918,19 +2955,19 @@
         <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.01451666666666667</v>
+        <v>0.01105</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1709833333333333</v>
+        <v>0.1639333333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.6867916666666666</v>
+        <v>0.6734150000000001</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2946,25 +2983,25 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>8</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.0314</v>
+        <v>0.03621666666666667</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.148975</v>
+        <v>0.158225</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.617138333333333</v>
+        <v>0.6353783333333332</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -2976,29 +3013,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
         <v>66</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>5e-05</v>
+        <v>0.0206</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>243</v>
+        <v>300</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.02595833333333333</v>
+        <v>0.1274083333333333</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.3793216666666666</v>
+        <v>0.6623666666666667</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -3010,29 +3047,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ryan Evans</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0042</v>
+        <v>0</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.04054166666666666</v>
+        <v>0.02041666666666667</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3189000000000001</v>
+        <v>0.3659933333333332</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -3044,29 +3081,29 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.01688333333333333</v>
+        <v>0.14125</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>300</v>
+        <v>265</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.1163333333333333</v>
+        <v>0.2762833333333333</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.6402333333333334</v>
+        <v>0.6345916666666664</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -3078,29 +3115,29 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Frank Greer</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0</v>
+        <v>0.01533333333333333</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>278</v>
+        <v>253</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.0003</v>
+        <v>0.08964999999999999</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.1869083333333333</v>
+        <v>0.4099583333333334</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3112,29 +3149,29 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Ryan Evans</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.1351166666666667</v>
+        <v>0.00385</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>265</v>
+        <v>243</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.2757866666666666</v>
+        <v>0.03616666666666666</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.6315666666666666</v>
+        <v>0.2926983333333334</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3146,29 +3183,29 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Frank Greer</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.01693333333333333</v>
+        <v>0</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>125</v>
+        <v>130.5</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>253</v>
+        <v>287</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.08732833333333333</v>
+        <v>0.05010833333333334</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.3781416666666666</v>
+        <v>0.5610833333333333</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0</v>
@@ -3180,29 +3217,29 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.04091666666666666</v>
+        <v>0</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.5158999999999999</v>
+        <v>0.1758666666666666</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3214,29 +3251,29 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.0058</v>
+        <v>0.0631</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>231</v>
+        <v>271</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.05545</v>
+        <v>0.2929166666666667</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.214875</v>
+        <v>0.6552549999999999</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3248,29 +3285,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
         <v>60</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.00335</v>
+        <v>0.0059</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>249</v>
+        <v>230</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.056275</v>
+        <v>0.05335</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.1772333333333334</v>
+        <v>0.205775</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3282,29 +3319,29 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.05538333333333333</v>
+        <v>0.0026</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>136</v>
+        <v>96</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>267</v>
+        <v>252</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.252095</v>
+        <v>0.0615</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.6030300000000001</v>
+        <v>0.1829833333333334</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3316,29 +3353,29 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Thomas Stephens</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.01495</v>
+        <v>0</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>302</v>
+        <v>257</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.06693333333333333</v>
+        <v>0.00615</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2763633333333334</v>
+        <v>0.3101766666666667</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3350,29 +3387,29 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Thomas Stephens</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
         <v>57</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0</v>
+        <v>0.00065</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>257</v>
+        <v>233</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.00675</v>
+        <v>0.008783333333333332</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.2799083333333334</v>
+        <v>0.1955416666666667</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3384,29 +3421,29 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.00065</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>233</v>
+        <v>270</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.0076</v>
+        <v>0.01913333333333333</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1664833333333333</v>
+        <v>0.1898033333333333</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3425,22 +3462,22 @@
         <v>54</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.02546666666666667</v>
+        <v>0.003183333333333333</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>247</v>
+        <v>209</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.06511666666666667</v>
+        <v>0.01843333333333333</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.222825</v>
+        <v>0.155215</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0</v>
@@ -3452,29 +3489,29 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
         <v>54</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.0001833333333333333</v>
+        <v>0.0009</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>221</v>
+        <v>193</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.003675</v>
+        <v>0.01451666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.07509999999999999</v>
+        <v>0.1665</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3486,29 +3523,29 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.00015</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>193</v>
+        <v>221</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.01346666666666666</v>
+        <v>0.00365</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.16475</v>
+        <v>0.06734166666666666</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0</v>
@@ -3524,25 +3561,25 @@
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>221</v>
+        <v>175</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0.01105</v>
+        <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.09399999999999999</v>
+        <v>0.029</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0</v>
@@ -3554,32 +3591,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>173</v>
+        <v>190</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0</v>
+        <v>0.006233333333333334</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.005516666666666667</v>
+        <v>0.131355</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="25">
@@ -3588,32 +3625,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.01575</v>
+        <v>0</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1141</v>
+        <v>0.006033333333333333</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>5e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3622,7 +3659,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
@@ -3632,22 +3669,22 @@
         <v>6</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0</v>
+        <v>0.00025</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.005216666666666666</v>
+        <v>0.01493333333333333</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1076916666666667</v>
+        <v>0.1097416666666667</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -3656,32 +3693,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.004158333333333332</v>
+        <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1643</v>
+        <v>0.1107066666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="28">
@@ -3690,29 +3727,29 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00075</v>
+        <v>0.00015</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>185</v>
+        <v>213</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01141666666666667</v>
+        <v>0.006166666666666668</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1165416666666667</v>
+        <v>0.1883483333333334</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>0</v>
@@ -3724,32 +3761,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
         <v>47</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0</v>
+        <v>0.00085</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>214</v>
+        <v>185</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0</v>
+        <v>0.01125</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.09124999999999998</v>
+        <v>0.1244233333333334</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -3758,29 +3795,29 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Caroline Colson</t>
+          <t>Jimmy P</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
         <v>46</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0003</v>
+        <v>5e-05</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.02716666666666666</v>
+        <v>0.01373333333333333</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0</v>
@@ -3792,29 +3829,29 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Rob Blackwood</t>
+          <t>Caroline Colson</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>63</v>
+        <v>84</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>162</v>
+        <v>203</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0</v>
+        <v>0.026</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0</v>
@@ -3826,29 +3863,29 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Jimmy P</t>
+          <t>Rob Blackwood</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.00295</v>
+        <v>0</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>253</v>
+        <v>162</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.0104</v>
+        <v>0</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.05585833333333332</v>
+        <v>0.0003</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0</v>
@@ -3864,7 +3901,7 @@
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D33" s="9" t="n">
         <v>7</v>
@@ -3873,16 +3910,16 @@
         <v>0.0001</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G33" s="9" t="n">
         <v>209</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.006308333333333332</v>
+        <v>0.008016666666666667</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.09945</v>
+        <v>0.1282933333333333</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0</v>
@@ -3907,7 +3944,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>145</v>
@@ -3916,10 +3953,10 @@
         <v>0</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>8.000000000000001e-05</v>
+        <v>9.000000000000001e-05</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.008533333333333332</v>
+        <v>0.01196666666666667</v>
       </c>
     </row>
     <row r="35">
@@ -3953,7 +3990,7 @@
         <v>0</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.2418</v>
+        <v>0.2637333333333334</v>
       </c>
     </row>
     <row r="36">
@@ -3962,32 +3999,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0</v>
+        <v>0.00015</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.001983333333333333</v>
+        <v>0.02179166666666667</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.029</v>
+        <v>0.005916666666666666</v>
       </c>
     </row>
     <row r="37">
@@ -3996,32 +4033,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0.0007</v>
+        <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.018375</v>
+        <v>0.0003</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.008683333333333333</v>
+        <v>0.05738333333333333</v>
       </c>
     </row>
     <row r="38">
@@ -4030,32 +4067,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E38" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="H38" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.0065</v>
+        <v>0.0024</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.06759999999999999</v>
+        <v>0.03136666666666666</v>
       </c>
     </row>
     <row r="39">
@@ -4064,32 +4101,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.0002</v>
+        <v>0.007483333333333334</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.07846666666666666</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4098,32 +4135,32 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.00895</v>
+        <v>0.00705</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0</v>
+        <v>0.08575000000000001</v>
       </c>
     </row>
     <row r="41">
@@ -4145,7 +4182,7 @@
         <v>0</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>137</v>
@@ -4154,10 +4191,10 @@
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0</v>
+        <v>0.00025</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.09003333333333335</v>
+        <v>0.12215</v>
       </c>
     </row>
     <row r="42">
@@ -4170,7 +4207,7 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>4</v>
@@ -4179,7 +4216,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>82</v>
@@ -4191,7 +4228,7 @@
         <v>0</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.4755333333333335</v>
+        <v>0.4212333333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 00:30:39 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leaderboard'!$A$1:$J$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>377c1ef520c4154d</t>
+          <t>882601c8ddb9daf1</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>bee57d9ed3cd4c63</t>
+          <t>377c1ef520c4154d</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Round of 32: UConn over UCLA</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T03:20:22.820403+00:00</t>
+          <t>2026-03-23T04:15:36.902380+00:00</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2105,10 +2105,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>UConn</t>
+        </is>
+      </c>
       <c r="F37" s="6" t="b">
         <v>0</v>
       </c>
@@ -2601,12 +2605,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>East</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Tennessee vs Iowa State</t>
+          <t>Michigan State vs UConn</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2622,7 +2626,7 @@
       <c r="H51" s="7" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>R16_M_02</t>
+          <t>R16_E_02</t>
         </is>
       </c>
     </row>
@@ -2634,12 +2638,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Iowa vs Nebraska</t>
+          <t>Tennessee vs Iowa State</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2655,7 +2659,7 @@
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>R16_S_01</t>
+          <t>R16_M_02</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2676,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Illinois vs Houston</t>
+          <t>Iowa vs Nebraska</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2688,7 +2692,7 @@
       <c r="H53" s="7" t="inlineStr"/>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>R16_S_02</t>
+          <t>R16_S_01</t>
         </is>
       </c>
     </row>
@@ -2700,12 +2704,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Arizona vs Arkansas</t>
+          <t>Illinois vs Houston</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -2721,7 +2725,7 @@
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>R16_W_01</t>
+          <t>R16_S_02</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2742,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Texas vs Purdue</t>
+          <t>Arizona vs Arkansas</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2754,12 +2758,45 @@
       <c r="H55" s="7" t="inlineStr"/>
       <c r="I55" s="2" t="inlineStr">
         <is>
+          <t>R16_W_01</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Sweet 16</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Texas vs Purdue</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr"/>
+      <c r="F56" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G56" s="5" t="inlineStr"/>
+      <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
           <t>R16_W_02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
+  <autoFilter ref="A1:I56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2850,22 +2887,22 @@
         <v>89</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.4206000000000001</v>
+        <v>0.3180166666666667</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>337</v>
+        <v>297</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.8282333333333334</v>
+        <v>0.7721166666666665</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9869166666666666</v>
+        <v>0.9808333333333332</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2887,19 +2924,19 @@
         <v>7</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.2217166666666666</v>
+        <v>0.2776666666666667</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>154</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.4938666666666667</v>
+        <v>0.5634333333333333</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.8047500000000001</v>
+        <v>0.8327416666666668</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2918,22 +2955,22 @@
         <v>71</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.05095</v>
+        <v>0.03409999999999999</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>295</v>
+        <v>249</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.230175</v>
+        <v>0.15405</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.76109</v>
+        <v>0.6944416666666668</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2955,7 +2992,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.01105</v>
+        <v>0.01998333333333333</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>135</v>
@@ -2964,10 +3001,10 @@
         <v>245</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.1639333333333333</v>
+        <v>0.2297666666666666</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.6734150000000001</v>
+        <v>0.7593683333333332</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -2979,29 +3016,29 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Sid Cash Jr.</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
         <v>69</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.03621666666666667</v>
+        <v>0.2149</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>307</v>
+        <v>269</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.158225</v>
+        <v>0.3913833333333334</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.6353783333333332</v>
+        <v>0.7434733333333332</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -3013,29 +3050,29 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Sid Cash Jr.</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.0206</v>
+        <v>0.02476666666666667</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>300</v>
+        <v>267</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1274083333333333</v>
+        <v>0.1091</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.6623666666666667</v>
+        <v>0.5417116666666667</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -3047,29 +3084,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
         <v>66</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0</v>
+        <v>0.01515</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.02041666666666667</v>
+        <v>0.07421666666666668</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.3659933333333332</v>
+        <v>0.5359383333333334</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -3081,29 +3118,29 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.14125</v>
+        <v>0.0002333333333333333</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>265</v>
+        <v>243</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.2762833333333333</v>
+        <v>0.02871666666666666</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.6345916666666664</v>
+        <v>0.4099049999999999</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -3125,19 +3162,19 @@
         <v>7</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.01533333333333333</v>
+        <v>0.0197</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.08964999999999999</v>
+        <v>0.1002</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.4099583333333334</v>
+        <v>0.445235</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3159,19 +3196,19 @@
         <v>6</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.00385</v>
+        <v>0.00485</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.03616666666666666</v>
+        <v>0.04298333333333333</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.2926983333333334</v>
+        <v>0.3601166666666666</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3190,22 +3227,22 @@
         <v>65</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>130.5</v>
+        <v>121</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>287</v>
+        <v>229</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.05010833333333334</v>
+        <v>0.01378333333333333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.5610833333333333</v>
+        <v>0.4393816666666666</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0</v>
@@ -3217,7 +3254,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Cole Dalton</t>
+          <t>Morgan Anthony</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
@@ -3227,19 +3264,19 @@
         <v>5</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0</v>
+        <v>0.00585</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>278</v>
+        <v>252</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0</v>
+        <v>0.07896666666666667</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.1758666666666666</v>
+        <v>0.2339</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3251,29 +3288,29 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>John Fishback</t>
+          <t>Cole Dalton</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.0631</v>
+        <v>0</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>271</v>
+        <v>214</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.2929166666666667</v>
+        <v>0</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.6552549999999999</v>
+        <v>0.04551666666666666</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3285,29 +3322,29 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Morgan Fishback</t>
+          <t>John Fishback</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.0059</v>
+        <v>0.05026666666666666</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.05335</v>
+        <v>0.2396666666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.205775</v>
+        <v>0.5916549999999999</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3319,29 +3356,29 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Morgan Anthony</t>
+          <t>Morgan Fishback</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
         <v>60</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.0026</v>
+        <v>0.00755</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.0615</v>
+        <v>0.06503333333333335</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.1829833333333334</v>
+        <v>0.2376833333333333</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3360,22 +3397,22 @@
         <v>59</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>257</v>
+        <v>181</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.00615</v>
+        <v>0.0007666666666666666</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.3101766666666667</v>
+        <v>0.2062166666666667</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3387,29 +3424,29 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Bradley Duell</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.00065</v>
+        <v>0.00105</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>233</v>
+        <v>193</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.008783333333333332</v>
+        <v>0.02221666666666667</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.1955416666666667</v>
+        <v>0.2572016666666667</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3428,22 +3465,22 @@
         <v>57</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>270</v>
+        <v>208</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.01913333333333333</v>
+        <v>0.008633333333333333</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1898033333333333</v>
+        <v>0.1176383333333333</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3455,29 +3492,29 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.003183333333333333</v>
+        <v>0.00055</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>209</v>
+        <v>233</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.01843333333333333</v>
+        <v>0.0134</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.155215</v>
+        <v>0.2374566666666667</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0</v>
@@ -3489,29 +3526,29 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Bradley Duell</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
         <v>54</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.0009</v>
+        <v>0.0025</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.01451666666666667</v>
+        <v>0.01966666666666667</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.1665</v>
+        <v>0.1718166666666667</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3533,19 +3570,19 @@
         <v>5</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.00015</v>
+        <v>3.333333333333333e-05</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>100</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.00365</v>
+        <v>0.004483333333333334</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.06734166666666666</v>
+        <v>0.08471833333333334</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0</v>
@@ -3579,7 +3616,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.029</v>
+        <v>0.03577500000000001</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0</v>
@@ -3591,32 +3628,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Anthony</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
         <v>51</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0</v>
+        <v>0.001183333333333333</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.006233333333333334</v>
+        <v>0.02056666666666667</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.131355</v>
+        <v>0.1618633333333333</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -3625,32 +3662,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Jimmy Anthony</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0</v>
+        <v>0.009700000000000002</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.006033333333333333</v>
+        <v>0.1547</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="26">
@@ -3659,29 +3696,29 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.00025</v>
+        <v>0</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>198</v>
+        <v>173</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.01493333333333333</v>
+        <v>0</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.1097416666666667</v>
+        <v>0.008008333333333333</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0</v>
@@ -3693,7 +3730,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Dan Swatek</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
@@ -3709,16 +3746,16 @@
         <v>101</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>211</v>
+        <v>198</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0</v>
+        <v>0.0191</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1107066666666667</v>
+        <v>0.1336666666666667</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.0002</v>
+        <v>3.333333333333333e-05</v>
       </c>
     </row>
     <row r="28">
@@ -3727,32 +3764,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Ansley Duell</t>
+          <t>Dan Swatek</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.006166666666666668</v>
+        <v>0</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1883483333333334</v>
+        <v>0.1380916666666667</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="29">
@@ -3761,29 +3798,29 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Ansley Duell</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D29" s="9" t="n">
         <v>7</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.00085</v>
+        <v>0.00045</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>185</v>
+        <v>213</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.01125</v>
+        <v>0.00735</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1244233333333334</v>
+        <v>0.2034566666666667</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0</v>
@@ -3814,10 +3851,10 @@
         <v>193</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>5e-05</v>
+        <v>0</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.01373333333333333</v>
+        <v>0.02026666666666667</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0</v>
@@ -3842,16 +3879,16 @@
         <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.0003</v>
+        <v>0.0002166666666666667</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.026</v>
+        <v>0.03146666666666667</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0</v>
@@ -3876,7 +3913,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G32" s="8" t="n">
         <v>162</v>
@@ -3885,7 +3922,7 @@
         <v>0</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.0003</v>
+        <v>0.0002</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0</v>
@@ -3907,19 +3944,19 @@
         <v>7</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.0005</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.008016666666666667</v>
+        <v>0.009783333333333335</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1282933333333333</v>
+        <v>0.1459</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0</v>
@@ -3953,10 +3990,10 @@
         <v>0</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>0.0001883333333333333</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.01196666666666667</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="35">
@@ -3965,32 +4002,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>47</v>
+        <v>75</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>116</v>
+        <v>184</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0</v>
+        <v>0.01211666666666667</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0.2637333333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -3999,32 +4036,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.00015</v>
+        <v>0</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.02179166666666667</v>
+        <v>0.0002</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.005916666666666666</v>
+        <v>0.1254916666666667</v>
       </c>
     </row>
     <row r="37">
@@ -4033,32 +4070,32 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Linda Cash</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>153</v>
+        <v>116</v>
       </c>
       <c r="H37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.05738333333333333</v>
+        <v>0.306</v>
       </c>
     </row>
     <row r="38">
@@ -4067,32 +4104,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Adam Harris</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E38" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.0024</v>
+        <v>0.024675</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.03136666666666666</v>
+        <v>0.007333333333333333</v>
       </c>
     </row>
     <row r="39">
@@ -4101,32 +4138,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Wade Cuda</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>184</v>
+        <v>137</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.007483333333333334</v>
+        <v>6.666666666666666e-05</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0</v>
+        <v>0.08205833333333334</v>
       </c>
     </row>
     <row r="40">
@@ -4135,11 +4172,11 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Linda Cash</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D40" s="8" t="n">
         <v>4</v>
@@ -4148,19 +4185,19 @@
         <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>192</v>
+        <v>153</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.00705</v>
+        <v>0.00035</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.08575000000000001</v>
+        <v>0.08158333333333334</v>
       </c>
     </row>
     <row r="41">
@@ -4169,32 +4206,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Wade Cuda</t>
+          <t>Adam Harris</t>
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D41" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="H41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.00025</v>
+        <v>0.002058333333333333</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.12215</v>
+        <v>0.05289166666666666</v>
       </c>
     </row>
     <row r="42">
@@ -4207,7 +4244,7 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>4</v>
@@ -4216,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G42" s="8" t="n">
         <v>82</v>
@@ -4228,7 +4265,7 @@
         <v>0</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.4212333333333334</v>
+        <v>0.3252083333333335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 12:09:31 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$B$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Game State'!$A$1:$I$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leaderboard'!$A$1:$J$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-03-23</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/22/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/21/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/23/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/22/all-conf</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>52</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>882601c8ddb9daf1</t>
+          <t>684c3a7bbc5d8006</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>377c1ef520c4154d</t>
+          <t>882601c8ddb9daf1</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Round of 32: UConn over UCLA</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T04:15:36.902380+00:00</t>
+          <t>2026-03-23T16:09:26.480844+00:00</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2179,10 +2179,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr"/>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Alabama</t>
+        </is>
+      </c>
       <c r="F39" s="6" t="b">
         <v>0</v>
       </c>
@@ -2323,7 +2327,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2360,7 +2364,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2397,7 +2401,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2471,7 +2475,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2508,7 +2512,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2643,7 +2647,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Tennessee vs Iowa State</t>
+          <t>Michigan vs Alabama</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2659,7 +2663,7 @@
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>R16_M_02</t>
+          <t>R16_M_01</t>
         </is>
       </c>
     </row>
@@ -2671,12 +2675,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Iowa vs Nebraska</t>
+          <t>Tennessee vs Iowa State</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2692,7 +2696,7 @@
       <c r="H53" s="7" t="inlineStr"/>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>R16_S_01</t>
+          <t>R16_M_02</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2713,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Illinois vs Houston</t>
+          <t>Iowa vs Nebraska</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -2725,7 +2729,7 @@
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>R16_S_02</t>
+          <t>R16_S_01</t>
         </is>
       </c>
     </row>
@@ -2737,12 +2741,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Arizona vs Arkansas</t>
+          <t>Illinois vs Houston</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2758,7 +2762,7 @@
       <c r="H55" s="7" t="inlineStr"/>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>R16_W_01</t>
+          <t>R16_S_02</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2779,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Texas vs Purdue</t>
+          <t>Arizona vs Arkansas</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2791,12 +2795,45 @@
       <c r="H56" s="5" t="inlineStr"/>
       <c r="I56" s="3" t="inlineStr">
         <is>
+          <t>R16_W_01</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Sweet 16</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Texas vs Purdue</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G57" s="7" t="inlineStr"/>
+      <c r="H57" s="7" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
           <t>R16_W_02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I56"/>
+  <autoFilter ref="A1:I57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2890,19 +2927,19 @@
         <v>8</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.3180166666666667</v>
+        <v>0.3155833333333333</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>297</v>
+        <v>283</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.7721166666666665</v>
+        <v>0.8112000000000001</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0.9808333333333332</v>
+        <v>0.9919999999999998</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>0</v>
@@ -2924,19 +2961,19 @@
         <v>7</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.2776666666666667</v>
+        <v>0.2677333333333333</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0.5634333333333333</v>
+        <v>0.5857666666666667</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.8327416666666668</v>
+        <v>0.8725666666666668</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -2948,29 +2985,29 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Sydney Taylor</t>
+          <t>MK Anthony</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.03409999999999999</v>
+        <v>0.29245</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>249</v>
+        <v>269</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.15405</v>
+        <v>0.5064666666666666</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.6944416666666668</v>
+        <v>0.8480666666666667</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>0</v>
@@ -2982,7 +3019,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nick Garas</t>
+          <t>Sydney Taylor</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
@@ -2992,19 +3029,19 @@
         <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.01998333333333333</v>
+        <v>0.03646666666666667</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.2297666666666666</v>
+        <v>0.1780833333333333</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.7593683333333332</v>
+        <v>0.7495666666666667</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>0</v>
@@ -3016,29 +3053,29 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>MK Anthony</t>
+          <t>Nick Garas</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.2149</v>
+        <v>0.01553333333333333</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>269</v>
+        <v>245</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.3913833333333334</v>
+        <v>0.2380166666666667</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.7434733333333332</v>
+        <v>0.79975</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>0</v>
@@ -3057,22 +3094,22 @@
         <v>69</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.02476666666666667</v>
+        <v>0.00315</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>267</v>
+        <v>243</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.1091</v>
+        <v>0.04778333333333334</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.5417116666666667</v>
+        <v>0.4705733333333333</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>0</v>
@@ -3084,29 +3121,29 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Alec Piloto</t>
+          <t>Jack Reddeck</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
         <v>66</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.01515</v>
+        <v>0.00015</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.07421666666666668</v>
+        <v>0.03213333333333334</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.5359383333333334</v>
+        <v>0.4584566666666667</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>0</v>
@@ -3118,7 +3155,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Jack Reddeck</t>
+          <t>Alec Piloto</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
@@ -3128,19 +3165,19 @@
         <v>6</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.0002333333333333333</v>
+        <v>0</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.02871666666666666</v>
+        <v>0.01031666666666667</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.4099049999999999</v>
+        <v>0.4600416666666667</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>0</v>
@@ -3159,22 +3196,22 @@
         <v>65</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0197</v>
+        <v>0.0033</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>249</v>
+        <v>212</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0.1002</v>
+        <v>0.05608333333333334</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.445235</v>
+        <v>0.3560916666666668</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0</v>
@@ -3186,7 +3223,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Ryan Evans</t>
+          <t>Jake Anthony</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
@@ -3196,19 +3233,19 @@
         <v>6</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.00485</v>
+        <v>0</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.04298333333333333</v>
+        <v>0.01455</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.3601166666666666</v>
+        <v>0.4935249999999999</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
@@ -3220,29 +3257,29 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Jake Anthony</t>
+          <t>Ryan Evans</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
         <v>65</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>229</v>
+        <v>216</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.01378333333333333</v>
+        <v>0.009549999999999999</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.4393816666666666</v>
+        <v>0.2716833333333334</v>
       </c>
       <c r="J12" s="5" t="n">
         <v>0</v>
@@ -3264,7 +3301,7 @@
         <v>5</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.00585</v>
+        <v>0.00615</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>100</v>
@@ -3273,10 +3310,10 @@
         <v>252</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.07896666666666667</v>
+        <v>0.08173333333333332</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.2339</v>
+        <v>0.2576833333333333</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>0</v>
@@ -3310,7 +3347,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>0.04551666666666666</v>
+        <v>0.05961666666666665</v>
       </c>
       <c r="J14" s="5" t="n">
         <v>0</v>
@@ -3332,19 +3369,19 @@
         <v>8</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.05026666666666666</v>
+        <v>0.049</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>127</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.2396666666666667</v>
+        <v>0.2482166666666667</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.5916549999999999</v>
+        <v>0.6265400000000001</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -3366,19 +3403,19 @@
         <v>6</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.00755</v>
+        <v>0.007833333333333335</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>99</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.06503333333333335</v>
+        <v>0.07501666666666666</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.2376833333333333</v>
+        <v>0.2615750000000001</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>0</v>
@@ -3403,16 +3440,16 @@
         <v>0</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G17" s="9" t="n">
         <v>181</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.0007666666666666666</v>
+        <v>0.001033333333333333</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.2062166666666667</v>
+        <v>0.2466166666666667</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>0</v>
@@ -3434,7 +3471,7 @@
         <v>7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.00105</v>
+        <v>0.00095</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>112</v>
@@ -3443,10 +3480,10 @@
         <v>193</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.02221666666666667</v>
+        <v>0.03078333333333333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.2572016666666667</v>
+        <v>0.2929749999999999</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>0</v>
@@ -3458,7 +3495,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Sid Cash Sr.</t>
+          <t>Brant Fleming</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
@@ -3468,19 +3505,19 @@
         <v>6</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.0007</v>
+        <v>0.0012</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>208</v>
+        <v>230</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.008633333333333333</v>
+        <v>0.0148</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.1176383333333333</v>
+        <v>0.2635500000000001</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>0</v>
@@ -3492,29 +3529,29 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Brant Fleming</t>
+          <t>Sid Cash Sr.</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
         <v>57</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.00055</v>
+        <v>0</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>111</v>
+        <v>86</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>233</v>
+        <v>181</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.0134</v>
+        <v>0.00015</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>0.2374566666666667</v>
+        <v>0.06545666666666666</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0</v>
@@ -3526,29 +3563,29 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Dan Downs</t>
+          <t>Tyler Colson</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>6</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>0.01966666666666667</v>
+        <v>0.0366</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.1718166666666667</v>
+        <v>0.2336249999999999</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>0</v>
@@ -3560,7 +3597,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Tim Dwyer</t>
+          <t>Dan Downs</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
@@ -3570,19 +3607,19 @@
         <v>5</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>3.333333333333333e-05</v>
+        <v>0</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>215</v>
+        <v>174</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.004483333333333334</v>
+        <v>0.0015</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.08471833333333334</v>
+        <v>0.1024416666666667</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>0</v>
@@ -3594,29 +3631,29 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Tanner Downs</t>
+          <t>Tim Dwyer</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.03577500000000001</v>
+        <v>0.0318</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0</v>
@@ -3628,29 +3665,29 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Ben Hewitt</t>
+          <t>Tanner Downs</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.001183333333333333</v>
+        <v>0</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.02056666666666667</v>
+        <v>0</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.1618633333333333</v>
+        <v>0.04750833333333333</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -3678,16 +3715,16 @@
         <v>94</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>0.009700000000000002</v>
+        <v>0.009616666666666667</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.1547</v>
+        <v>0.1703916666666667</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3696,29 +3733,29 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Jack Anthony</t>
+          <t>Ben Hewitt</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E26" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>173</v>
+        <v>149</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0</v>
+        <v>0.0076</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>0.008008333333333333</v>
+        <v>0.1244166666666666</v>
       </c>
       <c r="J26" s="5" t="n">
         <v>0</v>
@@ -3730,32 +3767,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Tyler Colson</t>
+          <t>Jack Anthony</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D27" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>198</v>
+        <v>173</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0.0191</v>
+        <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.1336666666666667</v>
+        <v>0.009350000000000001</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>3.333333333333333e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -3786,10 +3823,10 @@
         <v>0</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>0.1380916666666667</v>
+        <v>0.1611833333333333</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3805,22 +3842,22 @@
         <v>48</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.00045</v>
+        <v>0</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>213</v>
+        <v>178</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0.00735</v>
+        <v>0.0001</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.2034566666666667</v>
+        <v>0.1208916666666666</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0</v>
@@ -3845,16 +3882,16 @@
         <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>193</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0</v>
+        <v>5e-05</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.02026666666666667</v>
+        <v>0.023</v>
       </c>
       <c r="J30" s="5" t="n">
         <v>0</v>
@@ -3873,22 +3910,22 @@
         <v>46</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>195</v>
+        <v>169</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>0.0002166666666666667</v>
+        <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.03146666666666667</v>
+        <v>0.003733333333333333</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>0</v>
@@ -3922,7 +3959,7 @@
         <v>0</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>0</v>
@@ -3941,22 +3978,22 @@
         <v>44</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.0005</v>
+        <v>0</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>212</v>
+        <v>174</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>0.009783333333333335</v>
+        <v>0.0001</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.1459</v>
+        <v>0.07047500000000001</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>0</v>
@@ -3968,32 +4005,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Bo Anthony</t>
+          <t>Shelley Anthony</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E34" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>145</v>
+        <v>172</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0</v>
+        <v>0.00215</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.0001883333333333333</v>
+        <v>0.0513</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.019</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -4002,32 +4039,32 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Luke Hurbanis</t>
+          <t>Bo Anthony</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>184</v>
+        <v>145</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.01211666666666667</v>
+        <v>0.00019</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>0</v>
+        <v>0.01591666666666667</v>
       </c>
     </row>
     <row r="36">
@@ -4036,32 +4073,32 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Lyles Downs</t>
+          <t>Luke Hurbanis</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
         <v>39</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.0002</v>
+        <v>0.002608333333333333</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1254916666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -4070,23 +4107,23 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Liz Cuda</t>
+          <t>Lyles Downs</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="H37" s="7" t="n">
         <v>0</v>
@@ -4095,7 +4132,7 @@
         <v>0</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0.306</v>
+        <v>0.12725</v>
       </c>
     </row>
     <row r="38">
@@ -4104,32 +4141,32 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Shelley Anthony</t>
+          <t>Liz Cuda</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E38" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>172</v>
+        <v>116</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>0.024675</v>
+        <v>0</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>0.007333333333333333</v>
+        <v>0.25405</v>
       </c>
     </row>
     <row r="39">
@@ -4160,10 +4197,10 @@
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>6.666666666666666e-05</v>
+        <v>0.00065</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>0.08205833333333334</v>
+        <v>0.07346666666666668</v>
       </c>
     </row>
     <row r="40">
@@ -4179,25 +4216,25 @@
         <v>36</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>153</v>
+        <v>103</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>0.00035</v>
+        <v>0</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>0.08158333333333334</v>
+        <v>0.1399</v>
       </c>
     </row>
     <row r="41">
@@ -4213,25 +4250,25 @@
         <v>36</v>
       </c>
       <c r="D41" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="H41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.002058333333333333</v>
+        <v>0</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>0.05289166666666666</v>
+        <v>0.08245</v>
       </c>
     </row>
     <row r="42">
@@ -4265,7 +4302,7 @@
         <v>0</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.3252083333333335</v>
+        <v>0.3069666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 13:01:16 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T16:50:31.880158+00:00</t>
+          <t>2026-03-23T17:01:10.824359+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 14:02:25 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T17:40:15.915361+00:00</t>
+          <t>2026-03-23T18:02:20.448528+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 15:34:15 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T19:00:18.634841+00:00</t>
+          <t>2026-03-23T19:34:09.244295+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 15:42:40 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23T19:34:09.244295+00:00</t>
+          <t>2026-03-23T19:42:36.557955+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 20:21:42 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24T00:01:57.680723+00:00</t>
+          <t>2026-03-24T00:21:38.631589+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 21:44:19 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24T01:26:25.299162+00:00</t>
+          <t>2026-03-24T01:44:07.924502+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 22:31:43 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24T02:06:27.510420+00:00</t>
+          <t>2026-03-24T02:31:39.217231+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 22:51:43 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24T02:31:39.217231+00:00</t>
+          <t>2026-03-24T02:51:39.947652+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-23 23:57:56 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24T03:11:22.001498+00:00</t>
+          <t>2026-03-24T03:42:05.549310+00:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-24 12:00:51 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/23/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/22/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/24/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/23/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24T03:42:05.549310+00:00</t>
+          <t>2026-03-24T16:00:47.525790+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-25 10:00:27 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/24/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/23/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/25/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/24/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-25T00:40:17.969024+00:00</t>
+          <t>2026-03-25T14:00:20.857988+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-28 15:39:38 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-28</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/25/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/24/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/28/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/27/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-25T21:00:50.340739+00:00</t>
+          <t>2026-03-28T19:39:34.108493+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-29 16:48:03 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/28/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/27/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/29/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/28/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-28T23:47:54.974254+00:00</t>
+          <t>2026-03-29T20:47:58.210572+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-03-31 20:15:18 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/29/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/28/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/31/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/30/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-03-29T20:47:58.210572+00:00</t>
+          <t>2026-04-01T00:15:13.836985+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-01 14:17:56 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/31/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/30/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/01/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/31/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01T03:47:14.183665+00:00</t>
+          <t>2026-04-01T18:17:27.008280+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-02 09:32:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/01/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/03/31/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/02/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/01/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02T00:25:24.571851+00:00</t>
+          <t>2026-04-02T13:31:56.481889+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-03 13:05:52 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/02/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/01/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/03/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/02/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-02T23:40:18.146969+00:00</t>
+          <t>2026-04-03T17:05:51.703667+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-08 13:29:29 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/03/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/02/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/08/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/07/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-04T03:41:11.857989+00:00</t>
+          <t>2026-04-08T17:29:29.106330+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-09 12:00:40 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-09</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/08/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/07/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/09/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/08/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-09T03:40:37.141681+00:00</t>
+          <t>2026-04-09T16:00:39.853954+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-10 12:00:07 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/09/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/08/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/10/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/09/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10T03:40:05.716763+00:00</t>
+          <t>2026-04-10T16:00:07.204661+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-11 12:00:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/10/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/09/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/11/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/10/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-11T04:04:50.878245+00:00</t>
+          <t>2026-04-11T16:00:07.942210+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-12 12:03:07 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/11/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/10/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/12/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/11/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-12T03:41:57.797207+00:00</t>
+          <t>2026-04-12T16:03:07.416855+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-13 12:00:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-13</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/12/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/11/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/13/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/12/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-13T03:40:08.465302+00:00</t>
+          <t>2026-04-13T16:00:08.002086+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-14 12:20:03 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/13/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/12/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/14/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/13/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-14T03:41:43.785140+00:00</t>
+          <t>2026-04-14T16:20:02.698287+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-15 12:00:09 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/14/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/13/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/15/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/14/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-15T03:35:04.370407+00:00</t>
+          <t>2026-04-15T16:00:08.468675+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-16 12:06:09 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/15/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/14/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/16/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/15/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-16T03:41:18.942621+00:00</t>
+          <t>2026-04-16T16:06:08.895536+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-17 11:26:00 CDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/16/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/15/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/17/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/16/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17T03:42:35.624443+00:00</t>
+          <t>2026-04-17T16:26:00.240230+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-17 23:18:24 CDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-18</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/17/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/16/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/18/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/17/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-18T03:33:32.971744+00:00</t>
+          <t>2026-04-18T04:06:20.092733+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-19 12:13:13 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-19</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/18/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/17/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/19/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/18/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-19T03:40:05.877424+00:00</t>
+          <t>2026-04-19T16:13:12.858996+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-20 12:08:20 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/19/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/18/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/20/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/19/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-20T03:49:36.163679+00:00</t>
+          <t>2026-04-20T16:08:19.770272+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-21 12:00:07 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/20/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/19/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/21/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/20/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21T03:43:46.637992+00:00</t>
+          <t>2026-04-21T16:00:07.386549+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-22 12:01:34 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-22</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/21/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/20/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/22/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/21/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22T03:40:27.170882+00:00</t>
+          <t>2026-04-22T16:01:33.982820+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-23 12:00:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/22/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/21/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/23/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/22/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23T03:42:32.382776+00:00</t>
+          <t>2026-04-23T16:00:07.577906+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-24 12:00:06 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/23/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/22/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/24/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/23/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24T03:48:32.815627+00:00</t>
+          <t>2026-04-24T16:00:05.554960+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-25 12:03:47 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/24/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/23/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/25/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/24/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-25T03:40:19.346708+00:00</t>
+          <t>2026-04-25T16:03:46.714633+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-26 12:14:59 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-26</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/25/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/24/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/26/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/25/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-26T03:46:43.402956+00:00</t>
+          <t>2026-04-26T16:14:58.510453+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-27 12:00:21 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/26/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/25/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/27/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/26/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27T03:40:10.891802+00:00</t>
+          <t>2026-04-27T16:00:20.947218+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-28 12:00:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/27/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/26/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/28/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/27/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28T03:40:34.680320+00:00</t>
+          <t>2026-04-28T16:00:08.037963+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-29 12:02:01 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-29</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/28/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/27/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/29/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/28/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29T03:47:05.593919+00:00</t>
+          <t>2026-04-29T16:02:00.326342+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-04-30 12:00:36 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/29/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/28/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/30/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/29/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30T03:47:47.539261+00:00</t>
+          <t>2026-04-30T16:00:36.027427+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-01 12:00:10 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/30/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/29/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/01/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/30/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01T03:52:03.039177+00:00</t>
+          <t>2026-05-01T16:00:09.189715+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-02 12:02:39 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-02</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/01/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/04/30/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/02/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/01/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02T03:50:37.747205+00:00</t>
+          <t>2026-05-02T16:02:38.893340+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-03 12:13:44 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/02/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/01/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/03/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/02/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03T03:43:01.477858+00:00</t>
+          <t>2026-05-03T16:13:43.902982+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-04 12:00:07 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/03/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/02/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/04/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/03/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04T03:46:02.117051+00:00</t>
+          <t>2026-05-04T16:00:07.240123+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-05 12:00:19 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/04/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/03/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/05/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/04/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05T03:43:28.033085+00:00</t>
+          <t>2026-05-05T16:00:18.667977+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-06 10:31:38 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/05/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/04/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/06/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/05/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05T22:20:05.670111+00:00</t>
+          <t>2026-05-06T14:31:35.631135+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-07 12:00:08 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/06/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/05/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/07/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/06/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07T03:50:36.336753+00:00</t>
+          <t>2026-05-07T16:00:07.581379+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-08 13:38:59 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/07/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/06/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/08/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/07/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08T03:41:42.959549+00:00</t>
+          <t>2026-05-08T17:38:54.675764+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-09 12:00:55 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/08/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/07/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/09/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/08/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09T03:42:44.003726+00:00</t>
+          <t>2026-05-09T16:00:55.223838+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-10 12:00:07 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/09/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/08/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/10/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/09/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10T03:45:18.686781+00:00</t>
+          <t>2026-05-10T16:00:07.122566+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-11 12:00:47 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/10/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/09/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/11/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/10/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11T03:53:16.842251+00:00</t>
+          <t>2026-05-11T16:00:47.260689+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-12 12:06:42 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/11/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/10/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/12/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/11/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12T03:40:07.333815+00:00</t>
+          <t>2026-05-12T16:06:42.316590+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish GitHub Pages bundle 2026-05-13 12:00:09 EDT
</commit_message>
<xml_diff>
--- a/live_pool_odds.xlsx
+++ b/live_pool_odds.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -522,8 +522,8 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/12/all-conf
-https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/11/all-conf</t>
+          <t>https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/13/all-conf
+https://ncaa-api.henrygd.me/scoreboard/basketball-men/d1/2026/05/12/all-conf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13T03:48:57.199911+00:00</t>
+          <t>2026-05-13T16:00:08.379919+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>